<commit_message>
Add job dispatch, resources and Gunbreaker rotation
Expand Paladin priorities and provide a dedicated FFXIV AHK script and multi-job spell configuration.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9041B4A6-5052-4A41-8AD0-6D602C38E5C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F18F0A45-21B9-4BD8-ADD3-799B5F2170AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="28800" windowHeight="15555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
+    <sheet name="GNB" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="89">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -178,6 +179,120 @@
   </si>
   <si>
     <t>Fight or Flight Buff;Goring Blade Ready</t>
+  </si>
+  <si>
+    <t>Keen Edge</t>
+  </si>
+  <si>
+    <t>Brutal Shell Ready</t>
+  </si>
+  <si>
+    <t>Brutal Shell</t>
+  </si>
+  <si>
+    <t>Solid Barrel Ready</t>
+  </si>
+  <si>
+    <t>Solid Barrel</t>
+  </si>
+  <si>
+    <t>Burst Strike</t>
+  </si>
+  <si>
+    <t>Ready To Blast</t>
+  </si>
+  <si>
+    <t>Hypervelocity</t>
+  </si>
+  <si>
+    <t>Double Down</t>
+  </si>
+  <si>
+    <t>Bloodfest</t>
+  </si>
+  <si>
+    <t>Ready To Reign</t>
+  </si>
+  <si>
+    <t>Reign of Beasts</t>
+  </si>
+  <si>
+    <t>Noble Blood Ready</t>
+  </si>
+  <si>
+    <t>Noble Blood</t>
+  </si>
+  <si>
+    <t>Lion Hearth Ready</t>
+  </si>
+  <si>
+    <t>Lion Hearth</t>
+  </si>
+  <si>
+    <t>Gnashing Fang</t>
+  </si>
+  <si>
+    <t>Ready to Rip</t>
+  </si>
+  <si>
+    <t>Jugular Rip</t>
+  </si>
+  <si>
+    <t>Savage Claw Ready</t>
+  </si>
+  <si>
+    <t>Savage Claw</t>
+  </si>
+  <si>
+    <t>Ready to Tear</t>
+  </si>
+  <si>
+    <t>Abdomen Tear</t>
+  </si>
+  <si>
+    <t>Wicked Talon Ready</t>
+  </si>
+  <si>
+    <t>Wicked Talon</t>
+  </si>
+  <si>
+    <t>Ready To Gouge</t>
+  </si>
+  <si>
+    <t>Eye Gouge</t>
+  </si>
+  <si>
+    <t>Blasting Zone</t>
+  </si>
+  <si>
+    <t>Bow Shock</t>
+  </si>
+  <si>
+    <t>Lighting Shot</t>
+  </si>
+  <si>
+    <t>No Mercy</t>
+  </si>
+  <si>
+    <t>Ready To Break</t>
+  </si>
+  <si>
+    <t>Sonic Break</t>
+  </si>
+  <si>
+    <t>stack_a</t>
+  </si>
+  <si>
+    <t>No Mercy Buff</t>
+  </si>
+  <si>
+    <t>Fated Circle</t>
+  </si>
+  <si>
+    <t>Royal Authority Ready;Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready</t>
+  </si>
+  <si>
+    <t>Riot Blade Ready;Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready</t>
   </si>
 </sst>
 </file>
@@ -551,7 +666,7 @@
         <v>31</v>
       </c>
       <c r="E2">
-        <v>2500</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -571,7 +686,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>2</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -602,7 +717,7 @@
         <v>2</v>
       </c>
       <c r="H5" t="s">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="I5" t="s">
         <v>47</v>
@@ -636,7 +751,7 @@
         <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>2</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -771,7 +886,7 @@
         <v>33</v>
       </c>
       <c r="F16">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="G16" t="s">
         <v>50</v>
@@ -1048,6 +1163,586 @@
       </c>
       <c r="D34" t="s">
         <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7762502F-9F7A-4AD9-AC88-345A2195334F}">
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9">
+        <v>10</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11">
+        <v>6</v>
+      </c>
+      <c r="D11" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11">
+        <v>60</v>
+      </c>
+      <c r="I11">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+      <c r="G14" t="s">
+        <v>63</v>
+      </c>
+      <c r="H14" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D15" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18">
+        <v>8</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="H18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19">
+        <v>4</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
+      </c>
+      <c r="G19" t="s">
+        <v>68</v>
+      </c>
+      <c r="I19">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>68</v>
+      </c>
+      <c r="D20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21">
+        <v>5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>33</v>
+      </c>
+      <c r="G21" t="s">
+        <v>70</v>
+      </c>
+      <c r="H21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23">
+        <v>4</v>
+      </c>
+      <c r="D23" t="s">
+        <v>30</v>
+      </c>
+      <c r="G23" t="s">
+        <v>72</v>
+      </c>
+      <c r="H23" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25">
+        <v>5</v>
+      </c>
+      <c r="D25" t="s">
+        <v>33</v>
+      </c>
+      <c r="G25" t="s">
+        <v>74</v>
+      </c>
+      <c r="H25" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>74</v>
+      </c>
+      <c r="D26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+      <c r="D27" t="s">
+        <v>30</v>
+      </c>
+      <c r="G27" t="s">
+        <v>76</v>
+      </c>
+      <c r="H27" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D28" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29">
+        <v>5</v>
+      </c>
+      <c r="D29" t="s">
+        <v>33</v>
+      </c>
+      <c r="H29" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30" t="s">
+        <v>33</v>
+      </c>
+      <c r="F30">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>79</v>
+      </c>
+      <c r="D31" t="s">
+        <v>33</v>
+      </c>
+      <c r="F31">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B32" t="s">
+        <v>29</v>
+      </c>
+      <c r="C32">
+        <v>4</v>
+      </c>
+      <c r="D32" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>81</v>
+      </c>
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33">
+        <v>2</v>
+      </c>
+      <c r="D33" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>85</v>
+      </c>
+      <c r="D34" t="s">
+        <v>32</v>
+      </c>
+      <c r="F34">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>82</v>
+      </c>
+      <c r="D35" t="s">
+        <v>32</v>
+      </c>
+      <c r="F35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>83</v>
+      </c>
+      <c r="B36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" t="s">
+        <v>29</v>
+      </c>
+      <c r="C37">
+        <v>8</v>
+      </c>
+      <c r="D37" t="s">
+        <v>30</v>
+      </c>
+      <c r="I37">
+        <v>-1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct Gunbreaker job lookup and combo selection
Use the GNB spell book, select Blasting Zone and finish active Gnashing Fang and Lion Heart combos.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F18F0A45-21B9-4BD8-ADD3-799B5F2170AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D51BB84-3D7B-48E7-BB35-04D2C978C76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
     <sheet name="GNB" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$37</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -26,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="102">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -199,9 +202,6 @@
     <t>Burst Strike</t>
   </si>
   <si>
-    <t>Ready To Blast</t>
-  </si>
-  <si>
     <t>Hypervelocity</t>
   </si>
   <si>
@@ -211,9 +211,6 @@
     <t>Bloodfest</t>
   </si>
   <si>
-    <t>Ready To Reign</t>
-  </si>
-  <si>
     <t>Reign of Beasts</t>
   </si>
   <si>
@@ -223,12 +220,6 @@
     <t>Noble Blood</t>
   </si>
   <si>
-    <t>Lion Hearth Ready</t>
-  </si>
-  <si>
-    <t>Lion Hearth</t>
-  </si>
-  <si>
     <t>Gnashing Fang</t>
   </si>
   <si>
@@ -256,9 +247,6 @@
     <t>Wicked Talon</t>
   </si>
   <si>
-    <t>Ready To Gouge</t>
-  </si>
-  <si>
     <t>Eye Gouge</t>
   </si>
   <si>
@@ -274,15 +262,9 @@
     <t>No Mercy</t>
   </si>
   <si>
-    <t>Ready To Break</t>
-  </si>
-  <si>
     <t>Sonic Break</t>
   </si>
   <si>
-    <t>stack_a</t>
-  </si>
-  <si>
     <t>No Mercy Buff</t>
   </si>
   <si>
@@ -293,6 +275,66 @@
   </si>
   <si>
     <t>Riot Blade Ready;Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready</t>
+  </si>
+  <si>
+    <t>Shield Bash</t>
+  </si>
+  <si>
+    <t>stacks_a</t>
+  </si>
+  <si>
+    <t>Ready to Rip; Savage Claw Ready</t>
+  </si>
+  <si>
+    <t>Ready to Tear;Wicked Talon Ready</t>
+  </si>
+  <si>
+    <t>Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Ready to Blast</t>
+  </si>
+  <si>
+    <t>Ready to Blast;Ready to Rip;Ready to Tear;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Ready to Reign</t>
+  </si>
+  <si>
+    <t>Ready to Break</t>
+  </si>
+  <si>
+    <t>Ready to Break;No Mercy Buff</t>
+  </si>
+  <si>
+    <t>Lion Heart Ready</t>
+  </si>
+  <si>
+    <t>Solid Barrel Ready;Ready to Blast;Noble Blood Ready;Lion Heart Ready;Ready to Rip;Savage Claw Ready;Ready to Tear;Wicked Talon Ready;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Brutal Shell Ready;Ready to Blast;Noble Blood Ready;Lion Heart Ready;Ready to Rip;Savage Claw Ready;Ready to Tear;Wicked Talon Ready;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Ready to Reign;Ready to Blast;Noble Blood Ready;Lion Heart Ready;Ready to Rip;Savage Claw Ready;Ready to Tear;Wicked Talon Ready;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Noble Blood Ready;Ready to Blast;Noble Blood Ready;Lion Heart Ready;Ready to Rip;Savage Claw Ready;Ready to Tear;Wicked Talon Ready;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Lion Heart</t>
+  </si>
+  <si>
+    <t>Lion Heart Ready;Ready to Blast;Noble Blood Ready;Lion Heart Ready;Ready to Rip;Savage Claw Ready;Ready to Tear;Wicked Talon Ready;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Ready to Blast;Noble Blood Ready;Lion Heart Ready;Ready to Rip;Savage Claw Ready;Ready to Tear;Wicked Talon Ready;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Savage Claw Ready;Ready to Blast;Noble Blood Ready;Lion Heart Ready;Ready to Rip;Savage Claw Ready;Ready to Tear;Wicked Talon Ready;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Wicked Talon Ready;Ready to Blast;Noble Blood Ready;Lion Heart Ready;Ready to Rip;Savage Claw Ready;Ready to Tear;Wicked Talon Ready;Ready to Gouge</t>
   </si>
 </sst>
 </file>
@@ -619,7 +661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -686,7 +728,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -717,7 +759,7 @@
         <v>2</v>
       </c>
       <c r="H5" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I5" t="s">
         <v>47</v>
@@ -751,7 +793,7 @@
         <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1162,6 +1204,20 @@
         <v>4</v>
       </c>
       <c r="D34" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B35" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1208,7 +1264,7 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -1239,7 +1295,7 @@
         <v>52</v>
       </c>
       <c r="H3" t="s">
-        <v>54</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1250,7 +1306,7 @@
         <v>31</v>
       </c>
       <c r="E4">
-        <v>30</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -1270,7 +1326,7 @@
         <v>54</v>
       </c>
       <c r="H5" t="s">
-        <v>52</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1281,7 +1337,7 @@
         <v>31</v>
       </c>
       <c r="E6">
-        <v>30</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1298,7 +1354,7 @@
         <v>30</v>
       </c>
       <c r="H7" t="s">
-        <v>54</v>
+        <v>93</v>
       </c>
       <c r="I7">
         <v>1</v>
@@ -1318,7 +1374,10 @@
         <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>57</v>
+        <v>87</v>
+      </c>
+      <c r="H8" t="s">
+        <v>88</v>
       </c>
       <c r="I8">
         <v>-1</v>
@@ -1326,21 +1385,18 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>87</v>
       </c>
       <c r="D9" t="s">
         <v>32</v>
       </c>
       <c r="E9">
-        <v>10</v>
-      </c>
-      <c r="H9" t="s">
-        <v>57</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
         <v>28</v>
@@ -1351,10 +1407,13 @@
       <c r="D10" t="s">
         <v>33</v>
       </c>
+      <c r="H10" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B11" t="s">
         <v>28</v>
@@ -1365,8 +1424,11 @@
       <c r="D11" t="s">
         <v>30</v>
       </c>
-      <c r="E11">
-        <v>60</v>
+      <c r="F11">
+        <v>60000</v>
+      </c>
+      <c r="H11" t="s">
+        <v>88</v>
       </c>
       <c r="I11">
         <v>-2</v>
@@ -1374,7 +1436,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
         <v>28</v>
@@ -1386,10 +1448,13 @@
         <v>33</v>
       </c>
       <c r="F12">
-        <v>60</v>
+        <v>120000</v>
       </c>
       <c r="G12" t="s">
-        <v>61</v>
+        <v>89</v>
+      </c>
+      <c r="H12" t="s">
+        <v>88</v>
       </c>
       <c r="I12">
         <v>3</v>
@@ -1397,18 +1462,18 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="D13" t="s">
         <v>32</v>
       </c>
       <c r="E13">
-        <v>30</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B14" t="s">
         <v>28</v>
@@ -1420,26 +1485,26 @@
         <v>30</v>
       </c>
       <c r="G14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H14" t="s">
-        <v>61</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
         <v>31</v>
       </c>
       <c r="E15">
-        <v>30</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s">
         <v>28</v>
@@ -1451,26 +1516,26 @@
         <v>30</v>
       </c>
       <c r="G16" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="H16" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="D17" t="s">
         <v>31</v>
       </c>
       <c r="E17">
-        <v>30</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>97</v>
       </c>
       <c r="B18" t="s">
         <v>28</v>
@@ -1482,12 +1547,12 @@
         <v>30</v>
       </c>
       <c r="H18" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B19" t="s">
         <v>28</v>
@@ -1498,8 +1563,14 @@
       <c r="D19" t="s">
         <v>30</v>
       </c>
+      <c r="E19">
+        <v>30000</v>
+      </c>
       <c r="G19" t="s">
-        <v>68</v>
+        <v>84</v>
+      </c>
+      <c r="H19" t="s">
+        <v>99</v>
       </c>
       <c r="I19">
         <v>-1</v>
@@ -1507,15 +1578,18 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
         <v>32</v>
       </c>
+      <c r="E20">
+        <v>10000</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B21" t="s">
         <v>28</v>
@@ -1526,24 +1600,24 @@
       <c r="D21" t="s">
         <v>33</v>
       </c>
-      <c r="G21" t="s">
-        <v>70</v>
-      </c>
       <c r="H21" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D22" t="s">
         <v>31</v>
       </c>
+      <c r="E22">
+        <v>30000</v>
+      </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B23" t="s">
         <v>28</v>
@@ -1555,23 +1629,26 @@
         <v>30</v>
       </c>
       <c r="G23" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="H23" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D24" t="s">
         <v>32</v>
       </c>
+      <c r="E24">
+        <v>10000</v>
+      </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B25" t="s">
         <v>28</v>
@@ -1582,24 +1659,24 @@
       <c r="D25" t="s">
         <v>33</v>
       </c>
-      <c r="G25" t="s">
-        <v>74</v>
-      </c>
       <c r="H25" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D26" t="s">
         <v>31</v>
       </c>
+      <c r="E26">
+        <v>30000</v>
+      </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B27" t="s">
         <v>28</v>
@@ -1611,23 +1688,26 @@
         <v>30</v>
       </c>
       <c r="G27" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H27" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D28" t="s">
         <v>32</v>
       </c>
+      <c r="E28">
+        <v>10000</v>
+      </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B29" t="s">
         <v>28</v>
@@ -1639,34 +1719,46 @@
         <v>33</v>
       </c>
       <c r="H29" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>78</v>
+        <v>73</v>
+      </c>
+      <c r="B30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30">
+        <v>9</v>
       </c>
       <c r="D30" t="s">
         <v>33</v>
       </c>
       <c r="F30">
-        <v>30</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>79</v>
+        <v>74</v>
+      </c>
+      <c r="B31" t="s">
+        <v>29</v>
+      </c>
+      <c r="C31">
+        <v>9</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
       </c>
       <c r="F31">
-        <v>60</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B32" t="s">
         <v>29</v>
@@ -1677,10 +1769,16 @@
       <c r="D32" t="s">
         <v>30</v>
       </c>
+      <c r="G32" t="s">
+        <v>86</v>
+      </c>
+      <c r="H32" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B33" t="s">
         <v>28</v>
@@ -1691,32 +1789,38 @@
       <c r="D33" t="s">
         <v>33</v>
       </c>
+      <c r="E33" t="s">
+        <v>91</v>
+      </c>
+      <c r="F33">
+        <v>60000</v>
+      </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="D34" t="s">
         <v>32</v>
       </c>
-      <c r="F34">
-        <v>20</v>
+      <c r="E34">
+        <v>20000</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D35" t="s">
         <v>32</v>
       </c>
-      <c r="F35">
-        <v>30</v>
+      <c r="E35">
+        <v>30000</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B36" t="s">
         <v>28</v>
@@ -1727,10 +1831,13 @@
       <c r="D36" t="s">
         <v>30</v>
       </c>
+      <c r="H36" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B37" t="s">
         <v>29</v>
@@ -1740,6 +1847,9 @@
       </c>
       <c r="D37" t="s">
         <v>30</v>
+      </c>
+      <c r="H37" t="s">
+        <v>101</v>
       </c>
       <c r="I37">
         <v>-1</v>

</xml_diff>

<commit_message>
Prioritize Double Down in the Gunbreaker rotation
Move Double Down ahead of combo follow-ups and prepare a Burst Strike burst helper.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D51BB84-3D7B-48E7-BB35-04D2C978C76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D968C7E-D3AC-447C-BC39-5746094F63D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="103">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -335,6 +335,9 @@
   </si>
   <si>
     <t>Wicked Talon Ready;Ready to Blast;Noble Blood Ready;Lion Heart Ready;Ready to Rip;Savage Claw Ready;Ready to Tear;Wicked Talon Ready;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>Ready to Break;Ready to Blast;Ready to Rip;Ready to Tear;Ready to Gouge</t>
   </si>
 </sst>
 </file>
@@ -1563,7 +1566,7 @@
       <c r="D19" t="s">
         <v>30</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <v>30000</v>
       </c>
       <c r="G19" t="s">
@@ -1789,11 +1792,11 @@
       <c r="D33" t="s">
         <v>33</v>
       </c>
-      <c r="E33" t="s">
-        <v>91</v>
-      </c>
       <c r="F33">
         <v>60000</v>
+      </c>
+      <c r="G33" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -1832,7 +1835,7 @@
         <v>30</v>
       </c>
       <c r="H36" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add an initial Summoner rotation and rename core modules
Introduce summon priorities and consolidate spell handling and character initialization modules.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D968C7E-D3AC-447C-BC39-5746094F63D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA835AF1-E65A-478F-8EAC-1FDDA22E0692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
     <sheet name="GNB" sheetId="2" r:id="rId2"/>
+    <sheet name="SMN" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$37</definedName>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="194">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -338,6 +339,279 @@
   </si>
   <si>
     <t>Ready to Break;Ready to Blast;Ready to Rip;Ready to Tear;Ready to Gouge</t>
+  </si>
+  <si>
+    <t>stacks_b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aetherflow </t>
+  </si>
+  <si>
+    <t>Attunments</t>
+  </si>
+  <si>
+    <t>Summon Carbuncle</t>
+  </si>
+  <si>
+    <t>Swiftcast Buff</t>
+  </si>
+  <si>
+    <t>Ruin III</t>
+  </si>
+  <si>
+    <t>Change during big summons</t>
+  </si>
+  <si>
+    <t>Astral Impulse</t>
+  </si>
+  <si>
+    <t>Fountain of Fire</t>
+  </si>
+  <si>
+    <t>Umbral Impulse</t>
+  </si>
+  <si>
+    <t>Tri-disaster</t>
+  </si>
+  <si>
+    <t>Astral Flare</t>
+  </si>
+  <si>
+    <t>aoe</t>
+  </si>
+  <si>
+    <t>Brand of Purgatory</t>
+  </si>
+  <si>
+    <t>Umbral Flare</t>
+  </si>
+  <si>
+    <t>Energy Drain</t>
+  </si>
+  <si>
+    <t>Further Ruin</t>
+  </si>
+  <si>
+    <t>If no stack only</t>
+  </si>
+  <si>
+    <t>Energy Siphon</t>
+  </si>
+  <si>
+    <t>Necrotize</t>
+  </si>
+  <si>
+    <t>Under Buff</t>
+  </si>
+  <si>
+    <t>Painflare</t>
+  </si>
+  <si>
+    <t>Ruin IV</t>
+  </si>
+  <si>
+    <t>Big Summon Cooldown</t>
+  </si>
+  <si>
+    <t>Big summon cast</t>
+  </si>
+  <si>
+    <t>Summon Bahamut</t>
+  </si>
+  <si>
+    <t>Dreadwyrm Trance;Garuda Ready;Ifrit Ready;Titan Ready;Big Summon Cooldown;Ekindle Ready;Flare Ready;Big Summon Cooldown</t>
+  </si>
+  <si>
+    <t>Garuda;Ifrit;Titan;Crimson Cyclone Ready;Crimson Strike Ready;Slipstream Ready;Mountain Buster Ready</t>
+  </si>
+  <si>
+    <t>Summon Phoenix</t>
+  </si>
+  <si>
+    <t>Firebird Trance;Garuda Ready;Ifrit Ready;Titan Ready;Big Summon Cooldown;Ekindle Ready;Flare Ready;Big Summon Cooldown</t>
+  </si>
+  <si>
+    <t>Summon Solar Bahamut</t>
+  </si>
+  <si>
+    <t>Lightwyrm Trance;Lux Solaris Ready;Garuda Ready;Ifrit Ready;Titan Ready;Big Summon Cooldown;Ekindle Ready;Flare Ready;Big Summon Cooldown</t>
+  </si>
+  <si>
+    <t>Dreadwyrm Trance</t>
+  </si>
+  <si>
+    <t>Firebird Trance</t>
+  </si>
+  <si>
+    <t>Lightwyrm Trance</t>
+  </si>
+  <si>
+    <t>Ekindle Ready</t>
+  </si>
+  <si>
+    <t>Enkindle Bahamut</t>
+  </si>
+  <si>
+    <t>Enkindle Phoenix</t>
+  </si>
+  <si>
+    <t>Enkindle Solar Bahamut</t>
+  </si>
+  <si>
+    <t>Flare Ready</t>
+  </si>
+  <si>
+    <t>Deathflare</t>
+  </si>
+  <si>
+    <t>Rekindle</t>
+  </si>
+  <si>
+    <t>heal - Auto cast end of summon</t>
+  </si>
+  <si>
+    <t>Sunflare</t>
+  </si>
+  <si>
+    <t>Lux Solaris Ready</t>
+  </si>
+  <si>
+    <t>Lux Solaris</t>
+  </si>
+  <si>
+    <t>Ifrit Ready</t>
+  </si>
+  <si>
+    <t>Summon Ifrit II</t>
+  </si>
+  <si>
+    <t>Ifrit;Crimson Cyclone Ready</t>
+  </si>
+  <si>
+    <t>Ifrit Ready;Garuda;Ifrit;Titan;Crimson Cyclone Ready;Crimson Strike Ready;Slipstream Ready;Mountain Buster Ready</t>
+  </si>
+  <si>
+    <t>Ifrit</t>
+  </si>
+  <si>
+    <t>Titan Ready</t>
+  </si>
+  <si>
+    <t>Summon Titan II</t>
+  </si>
+  <si>
+    <t>Titan</t>
+  </si>
+  <si>
+    <t>Titan Ready;Garuda;Ifrit;Titan;Crimson Cyclone Ready;Crimson Strike Ready;Slipstream Ready;Mountain Buster Ready</t>
+  </si>
+  <si>
+    <t>Garuda Ready</t>
+  </si>
+  <si>
+    <t>Summon Garuda II</t>
+  </si>
+  <si>
+    <t>Garuda;Slipstream Ready</t>
+  </si>
+  <si>
+    <t>Garuda Ready;Garuda;Ifrit;Titan;Crimson Cyclone Ready;Crimson Strike Ready;Slipstream Ready;Mountain Buster Ready</t>
+  </si>
+  <si>
+    <t>Garuda</t>
+  </si>
+  <si>
+    <t>Gemshine</t>
+  </si>
+  <si>
+    <t>Ruby Rite</t>
+  </si>
+  <si>
+    <t>Require attunments stacks</t>
+  </si>
+  <si>
+    <t>Topaz Rite</t>
+  </si>
+  <si>
+    <t>Mountain Buster Ready</t>
+  </si>
+  <si>
+    <t>Emerald Rite</t>
+  </si>
+  <si>
+    <t>Precious Brilliance</t>
+  </si>
+  <si>
+    <t>Ruby Catastrophe</t>
+  </si>
+  <si>
+    <t>Topaz Catastrophe</t>
+  </si>
+  <si>
+    <t>Emerald Catastrophe</t>
+  </si>
+  <si>
+    <t>Astral Flow</t>
+  </si>
+  <si>
+    <t>Crimson Cyclone Ready</t>
+  </si>
+  <si>
+    <t>Crimson Cyclone</t>
+  </si>
+  <si>
+    <t>Crimson Strike Ready</t>
+  </si>
+  <si>
+    <t>Crimson Strike</t>
+  </si>
+  <si>
+    <t>Mountain Buster</t>
+  </si>
+  <si>
+    <t>Slipstream Ready</t>
+  </si>
+  <si>
+    <t>Slipstream</t>
+  </si>
+  <si>
+    <t>Slipstream Ready;Swiftcast Buff</t>
+  </si>
+  <si>
+    <t>Searing Light</t>
+  </si>
+  <si>
+    <t>Searing Light Buff;Ruby's Glimmer</t>
+  </si>
+  <si>
+    <t>Searing Light Buff</t>
+  </si>
+  <si>
+    <t>Ruby's Glimmer</t>
+  </si>
+  <si>
+    <t>Searing Flash</t>
+  </si>
+  <si>
+    <t>Swiftcast</t>
+  </si>
+  <si>
+    <t>Addle</t>
+  </si>
+  <si>
+    <t>Physick</t>
+  </si>
+  <si>
+    <t>Resurrection</t>
+  </si>
+  <si>
+    <t>Sleep</t>
+  </si>
+  <si>
+    <t>Lucid Dreaming</t>
+  </si>
+  <si>
+    <t>Radiant Aegis</t>
   </si>
 </sst>
 </file>
@@ -361,12 +635,48 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFECD9FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -381,9 +691,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1861,4 +2178,1184 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E11AA6E-3A21-4E4D-BBE2-CBF8D1A645C0}">
+  <dimension ref="A1:K92"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>104</v>
+      </c>
+      <c r="J2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" t="s">
+        <v>107</v>
+      </c>
+      <c r="K8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13">
+        <v>5</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K14" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15">
+        <v>5</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+      <c r="K15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="K16" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18">
+        <v>60000</v>
+      </c>
+      <c r="G18" t="s">
+        <v>119</v>
+      </c>
+      <c r="I18">
+        <v>2</v>
+      </c>
+      <c r="K18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>121</v>
+      </c>
+      <c r="B19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19">
+        <v>6</v>
+      </c>
+      <c r="D19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" t="s">
+        <v>119</v>
+      </c>
+      <c r="I19">
+        <v>2</v>
+      </c>
+      <c r="K19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20">
+        <v>9</v>
+      </c>
+      <c r="D20" t="s">
+        <v>33</v>
+      </c>
+      <c r="I20">
+        <v>-1</v>
+      </c>
+      <c r="K20" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>124</v>
+      </c>
+      <c r="B21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>33</v>
+      </c>
+      <c r="I21">
+        <v>-1</v>
+      </c>
+      <c r="K21" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>119</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23">
+        <v>5</v>
+      </c>
+      <c r="D23" t="s">
+        <v>30</v>
+      </c>
+      <c r="H23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>126</v>
+      </c>
+      <c r="D26" t="s">
+        <v>31</v>
+      </c>
+      <c r="E26">
+        <v>60000</v>
+      </c>
+      <c r="K26" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28">
+        <v>8</v>
+      </c>
+      <c r="D28" t="s">
+        <v>30</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="H28" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29">
+        <v>8</v>
+      </c>
+      <c r="D29" t="s">
+        <v>30</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="H29" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30">
+        <v>8</v>
+      </c>
+      <c r="D30" t="s">
+        <v>30</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="H30" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D32" t="s">
+        <v>32</v>
+      </c>
+      <c r="E32">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D33" t="s">
+        <v>32</v>
+      </c>
+      <c r="E33">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34" t="s">
+        <v>32</v>
+      </c>
+      <c r="E34">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>138</v>
+      </c>
+      <c r="D36" t="s">
+        <v>31</v>
+      </c>
+      <c r="E36">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37">
+        <v>8</v>
+      </c>
+      <c r="D37" t="s">
+        <v>33</v>
+      </c>
+      <c r="H37" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B38" t="s">
+        <v>28</v>
+      </c>
+      <c r="C38">
+        <v>8</v>
+      </c>
+      <c r="D38" t="s">
+        <v>33</v>
+      </c>
+      <c r="H38" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B39" t="s">
+        <v>28</v>
+      </c>
+      <c r="C39">
+        <v>8</v>
+      </c>
+      <c r="D39" t="s">
+        <v>33</v>
+      </c>
+      <c r="H39" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>142</v>
+      </c>
+      <c r="D41" t="s">
+        <v>31</v>
+      </c>
+      <c r="E41">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B42" t="s">
+        <v>28</v>
+      </c>
+      <c r="C42">
+        <v>4</v>
+      </c>
+      <c r="D42" t="s">
+        <v>33</v>
+      </c>
+      <c r="H42" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B43" t="s">
+        <v>28</v>
+      </c>
+      <c r="C43">
+        <v>4</v>
+      </c>
+      <c r="D43" t="s">
+        <v>33</v>
+      </c>
+      <c r="H43" t="s">
+        <v>142</v>
+      </c>
+      <c r="K43" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B44" t="s">
+        <v>28</v>
+      </c>
+      <c r="C44">
+        <v>4</v>
+      </c>
+      <c r="D44" t="s">
+        <v>33</v>
+      </c>
+      <c r="H44" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D46" t="s">
+        <v>31</v>
+      </c>
+      <c r="E46">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B47" t="s">
+        <v>27</v>
+      </c>
+      <c r="C47">
+        <v>12</v>
+      </c>
+      <c r="D47" t="s">
+        <v>33</v>
+      </c>
+      <c r="H47" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="K47" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="D50" t="s">
+        <v>31</v>
+      </c>
+      <c r="E50">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B51" t="s">
+        <v>28</v>
+      </c>
+      <c r="C51">
+        <v>7</v>
+      </c>
+      <c r="D51" t="s">
+        <v>30</v>
+      </c>
+      <c r="G51" t="s">
+        <v>151</v>
+      </c>
+      <c r="H51" t="s">
+        <v>152</v>
+      </c>
+      <c r="K51">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D52" t="s">
+        <v>31</v>
+      </c>
+      <c r="E52">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="D53" t="s">
+        <v>31</v>
+      </c>
+      <c r="E53">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B54" t="s">
+        <v>27</v>
+      </c>
+      <c r="C54">
+        <v>7</v>
+      </c>
+      <c r="D54" t="s">
+        <v>30</v>
+      </c>
+      <c r="G54" t="s">
+        <v>156</v>
+      </c>
+      <c r="H54" t="s">
+        <v>157</v>
+      </c>
+      <c r="K54">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D55" t="s">
+        <v>31</v>
+      </c>
+      <c r="E55">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="D56" t="s">
+        <v>31</v>
+      </c>
+      <c r="E56">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="B57" t="s">
+        <v>29</v>
+      </c>
+      <c r="C57">
+        <v>7</v>
+      </c>
+      <c r="D57" t="s">
+        <v>30</v>
+      </c>
+      <c r="G57" t="s">
+        <v>160</v>
+      </c>
+      <c r="H57" t="s">
+        <v>161</v>
+      </c>
+      <c r="K57">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="D58" t="s">
+        <v>31</v>
+      </c>
+      <c r="E58">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>163</v>
+      </c>
+      <c r="B60" t="s">
+        <v>27</v>
+      </c>
+      <c r="C60">
+        <v>4</v>
+      </c>
+      <c r="D60" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B61" t="s">
+        <v>27</v>
+      </c>
+      <c r="C61">
+        <v>4</v>
+      </c>
+      <c r="D61" t="s">
+        <v>30</v>
+      </c>
+      <c r="H61" t="s">
+        <v>107</v>
+      </c>
+      <c r="J61">
+        <v>-1</v>
+      </c>
+      <c r="K61" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B62" t="s">
+        <v>27</v>
+      </c>
+      <c r="C62">
+        <v>4</v>
+      </c>
+      <c r="D62" t="s">
+        <v>30</v>
+      </c>
+      <c r="G62" t="s">
+        <v>167</v>
+      </c>
+      <c r="J62">
+        <v>-1</v>
+      </c>
+      <c r="K62" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="B63" t="s">
+        <v>27</v>
+      </c>
+      <c r="C63">
+        <v>4</v>
+      </c>
+      <c r="D63" t="s">
+        <v>30</v>
+      </c>
+      <c r="J63">
+        <v>-1</v>
+      </c>
+      <c r="K63" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>169</v>
+      </c>
+      <c r="B65" t="s">
+        <v>29</v>
+      </c>
+      <c r="C65">
+        <v>4</v>
+      </c>
+      <c r="D65" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B66" t="s">
+        <v>29</v>
+      </c>
+      <c r="C66">
+        <v>4</v>
+      </c>
+      <c r="D66" t="s">
+        <v>30</v>
+      </c>
+      <c r="H66" t="s">
+        <v>107</v>
+      </c>
+      <c r="J66">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B67" t="s">
+        <v>29</v>
+      </c>
+      <c r="C67">
+        <v>4</v>
+      </c>
+      <c r="D67" t="s">
+        <v>30</v>
+      </c>
+      <c r="J67">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B68" t="s">
+        <v>29</v>
+      </c>
+      <c r="C68">
+        <v>4</v>
+      </c>
+      <c r="D68" t="s">
+        <v>30</v>
+      </c>
+      <c r="J68">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D71" t="s">
+        <v>31</v>
+      </c>
+      <c r="E71">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A72" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B72" t="s">
+        <v>28</v>
+      </c>
+      <c r="C72">
+        <v>4</v>
+      </c>
+      <c r="D72" t="s">
+        <v>30</v>
+      </c>
+      <c r="G72" t="s">
+        <v>176</v>
+      </c>
+      <c r="H72" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A73" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D73" t="s">
+        <v>31</v>
+      </c>
+      <c r="E73">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A74" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B74" t="s">
+        <v>28</v>
+      </c>
+      <c r="C74">
+        <v>4</v>
+      </c>
+      <c r="D74" t="s">
+        <v>30</v>
+      </c>
+      <c r="H74" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A75" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D75" t="s">
+        <v>31</v>
+      </c>
+      <c r="E75">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A76" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B76" t="s">
+        <v>28</v>
+      </c>
+      <c r="C76">
+        <v>4</v>
+      </c>
+      <c r="D76" t="s">
+        <v>33</v>
+      </c>
+      <c r="H76" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A77" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D77" t="s">
+        <v>31</v>
+      </c>
+      <c r="E77">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A78" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="B78" t="s">
+        <v>28</v>
+      </c>
+      <c r="C78">
+        <v>4</v>
+      </c>
+      <c r="D78" t="s">
+        <v>30</v>
+      </c>
+      <c r="H78" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>182</v>
+      </c>
+      <c r="B80" t="s">
+        <v>28</v>
+      </c>
+      <c r="C80">
+        <v>2</v>
+      </c>
+      <c r="D80" t="s">
+        <v>33</v>
+      </c>
+      <c r="F80">
+        <v>120000</v>
+      </c>
+      <c r="G80" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>184</v>
+      </c>
+      <c r="D81" t="s">
+        <v>32</v>
+      </c>
+      <c r="E81">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>185</v>
+      </c>
+      <c r="D82" t="s">
+        <v>32</v>
+      </c>
+      <c r="E82">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>186</v>
+      </c>
+      <c r="B83" t="s">
+        <v>28</v>
+      </c>
+      <c r="C83">
+        <v>2</v>
+      </c>
+      <c r="D83" t="s">
+        <v>33</v>
+      </c>
+      <c r="H83" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>187</v>
+      </c>
+      <c r="B85" t="s">
+        <v>27</v>
+      </c>
+      <c r="C85">
+        <v>11</v>
+      </c>
+      <c r="D85" t="s">
+        <v>33</v>
+      </c>
+      <c r="F85">
+        <v>40000</v>
+      </c>
+      <c r="G85" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>107</v>
+      </c>
+      <c r="D86" t="s">
+        <v>31</v>
+      </c>
+      <c r="E86">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>188</v>
+      </c>
+      <c r="B87" t="s">
+        <v>28</v>
+      </c>
+      <c r="C87">
+        <v>12</v>
+      </c>
+      <c r="D87" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>189</v>
+      </c>
+      <c r="B88" t="s">
+        <v>28</v>
+      </c>
+      <c r="C88">
+        <v>10</v>
+      </c>
+      <c r="D88" t="s">
+        <v>30</v>
+      </c>
+      <c r="H88" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>190</v>
+      </c>
+      <c r="B89" t="s">
+        <v>29</v>
+      </c>
+      <c r="C89">
+        <v>11</v>
+      </c>
+      <c r="D89" t="s">
+        <v>30</v>
+      </c>
+      <c r="H89" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>191</v>
+      </c>
+      <c r="B90" t="s">
+        <v>28</v>
+      </c>
+      <c r="C90">
+        <v>3</v>
+      </c>
+      <c r="D90" t="s">
+        <v>30</v>
+      </c>
+      <c r="H90" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>192</v>
+      </c>
+      <c r="B91" t="s">
+        <v>29</v>
+      </c>
+      <c r="C91">
+        <v>3</v>
+      </c>
+      <c r="D91" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>193</v>
+      </c>
+      <c r="B92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C92">
+        <v>10</v>
+      </c>
+      <c r="D92" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refine Summoner and Gunbreaker and wire Scholar dispatch
Fix Summoner resource bounds and oGCD choices, adjust Gunbreaker priorities and add SCH routing.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA835AF1-E65A-478F-8EAC-1FDDA22E0692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1B12F6-D70D-4F5E-9394-7B268BC6DFA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
     <sheet name="GNB" sheetId="2" r:id="rId2"/>
     <sheet name="SMN" sheetId="3" r:id="rId3"/>
+    <sheet name="SCH" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$37</definedName>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="200">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -612,6 +613,24 @@
   </si>
   <si>
     <t>Radiant Aegis</t>
+  </si>
+  <si>
+    <t>Biolysis</t>
+  </si>
+  <si>
+    <t>Broil IV</t>
+  </si>
+  <si>
+    <t>Ruin II</t>
+  </si>
+  <si>
+    <t>Chain Stratagem</t>
+  </si>
+  <si>
+    <t>Impact imminent</t>
+  </si>
+  <si>
+    <t>Baneful Impaction</t>
   </si>
 </sst>
 </file>
@@ -691,7 +710,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -700,7 +719,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2240,7 +2258,7 @@
         <v>31</v>
       </c>
       <c r="E4">
-        <v>2450</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -2318,6 +2336,9 @@
       <c r="C11">
         <v>5</v>
       </c>
+      <c r="D11" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -2746,7 +2767,7 @@
         <v>31</v>
       </c>
       <c r="E46">
-        <v>30</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -2762,7 +2783,7 @@
       <c r="D47" t="s">
         <v>33</v>
       </c>
-      <c r="H47" s="8" t="s">
+      <c r="H47" t="s">
         <v>147</v>
       </c>
       <c r="K47" t="s">
@@ -3140,7 +3161,7 @@
       <c r="D76" t="s">
         <v>33</v>
       </c>
-      <c r="H76" s="8" t="s">
+      <c r="H76" t="s">
         <v>167</v>
       </c>
     </row>
@@ -3353,6 +3374,174 @@
       </c>
       <c r="D92" t="s">
         <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF394502-4A59-4E3D-B4CF-5A5D5E1CBE54}">
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>194</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6">
+        <v>28500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>195</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>196</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>197</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9">
+        <v>120000</v>
+      </c>
+      <c r="G9" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>198</v>
+      </c>
+      <c r="D10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11" t="s">
+        <v>33</v>
+      </c>
+      <c r="H11" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>192</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12">
+        <v>60000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adjust GCD configuration and weave timing
Update the spell workbook and raise the minimum oGCD window from 650 to 675 ms.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1B12F6-D70D-4F5E-9394-7B268BC6DFA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6009D0DE-B81C-43C8-9359-6571A73D8DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -1046,7 +1046,7 @@
         <v>31</v>
       </c>
       <c r="E2">
-        <v>2460</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1613,7 +1613,7 @@
         <v>31</v>
       </c>
       <c r="E2">
-        <v>2460</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -2258,7 +2258,7 @@
         <v>31</v>
       </c>
       <c r="E4">
-        <v>2440</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add Dark Knight rotation and resource handling
Introduce DRK action priorities, spell data and additional resource diagnostics.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6009D0DE-B81C-43C8-9359-6571A73D8DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3995CE7C-4696-4AE4-A244-2B7710995162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
     <sheet name="GNB" sheetId="2" r:id="rId2"/>
-    <sheet name="SMN" sheetId="3" r:id="rId3"/>
-    <sheet name="SCH" sheetId="4" r:id="rId4"/>
+    <sheet name="DRK" sheetId="5" r:id="rId3"/>
+    <sheet name="SMN" sheetId="3" r:id="rId4"/>
+    <sheet name="SCH" sheetId="4" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$37</definedName>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="233">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -631,6 +632,105 @@
   </si>
   <si>
     <t>Baneful Impaction</t>
+  </si>
+  <si>
+    <t>Hard Slash</t>
+  </si>
+  <si>
+    <t>Syphon Strike</t>
+  </si>
+  <si>
+    <t>Syphon Strike Ready</t>
+  </si>
+  <si>
+    <t>Souleater</t>
+  </si>
+  <si>
+    <t>Souleater Ready</t>
+  </si>
+  <si>
+    <t>Delirium</t>
+  </si>
+  <si>
+    <t>Blood Gauge</t>
+  </si>
+  <si>
+    <t>Abyssal Drain</t>
+  </si>
+  <si>
+    <t>Quietus</t>
+  </si>
+  <si>
+    <t>Scarlet Delirium</t>
+  </si>
+  <si>
+    <t>Shadowbringer</t>
+  </si>
+  <si>
+    <t>Unmend</t>
+  </si>
+  <si>
+    <t>Unleash</t>
+  </si>
+  <si>
+    <t>Stalwart Soul</t>
+  </si>
+  <si>
+    <t>Living Shadow</t>
+  </si>
+  <si>
+    <t>Scorn</t>
+  </si>
+  <si>
+    <t>Disesteem</t>
+  </si>
+  <si>
+    <t>Clone</t>
+  </si>
+  <si>
+    <t>2m Burst</t>
+  </si>
+  <si>
+    <t>Salted Earth</t>
+  </si>
+  <si>
+    <t>Salt and Darkness</t>
+  </si>
+  <si>
+    <t>Salt and Darkness Ready</t>
+  </si>
+  <si>
+    <t>Edge of Shadow</t>
+  </si>
+  <si>
+    <t>Flood of Shadow</t>
+  </si>
+  <si>
+    <t>Blood gauge : 3 free cast et 30 given by blood weapon</t>
+  </si>
+  <si>
+    <t>1m Burst</t>
+  </si>
+  <si>
+    <t>Comeuppance</t>
+  </si>
+  <si>
+    <t>Torcleaver</t>
+  </si>
+  <si>
+    <t>Recent EoS</t>
+  </si>
+  <si>
+    <t>secondary_bar</t>
+  </si>
+  <si>
+    <t>Bloodspiller</t>
+  </si>
+  <si>
+    <t>Scorn;Clone;2m Burst</t>
+  </si>
+  <si>
+    <t>Carve and Spit</t>
   </si>
 </sst>
 </file>
@@ -2199,6 +2299,569 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0983F4B6-DA2C-422A-9A48-B565C13F35E9}">
+  <dimension ref="A1:M38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>202</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>204</v>
+      </c>
+      <c r="H6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>204</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" t="s">
+        <v>204</v>
+      </c>
+      <c r="K8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>232</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13">
+        <v>60000</v>
+      </c>
+      <c r="G13" t="s">
+        <v>225</v>
+      </c>
+      <c r="J13">
+        <v>3</v>
+      </c>
+      <c r="K13">
+        <v>180</v>
+      </c>
+      <c r="M13" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>225</v>
+      </c>
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>230</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+      <c r="K15">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>209</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="K16">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17">
+        <v>8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+      <c r="K17">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>227</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18">
+        <v>8</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="K18">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>208</v>
+      </c>
+      <c r="B19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19">
+        <v>8</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
+      </c>
+      <c r="K19">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21">
+        <v>4</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>212</v>
+      </c>
+      <c r="B22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+      <c r="D22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>213</v>
+      </c>
+      <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23">
+        <v>6</v>
+      </c>
+      <c r="D23" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>214</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25">
+        <v>7</v>
+      </c>
+      <c r="D25" t="s">
+        <v>33</v>
+      </c>
+      <c r="F25">
+        <v>120000</v>
+      </c>
+      <c r="G25" t="s">
+        <v>231</v>
+      </c>
+      <c r="I25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>215</v>
+      </c>
+      <c r="D26" t="s">
+        <v>32</v>
+      </c>
+      <c r="E26">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>216</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27">
+        <v>7</v>
+      </c>
+      <c r="D27" t="s">
+        <v>30</v>
+      </c>
+      <c r="H27" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>217</v>
+      </c>
+      <c r="D28" t="s">
+        <v>31</v>
+      </c>
+      <c r="E28">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>218</v>
+      </c>
+      <c r="D29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>219</v>
+      </c>
+      <c r="B31" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31">
+        <v>5</v>
+      </c>
+      <c r="D31" t="s">
+        <v>33</v>
+      </c>
+      <c r="F31">
+        <v>90000</v>
+      </c>
+      <c r="G31" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>221</v>
+      </c>
+      <c r="D32" t="s">
+        <v>31</v>
+      </c>
+      <c r="E32">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>220</v>
+      </c>
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33">
+        <v>5</v>
+      </c>
+      <c r="D33" t="s">
+        <v>33</v>
+      </c>
+      <c r="H33" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>222</v>
+      </c>
+      <c r="B35" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35">
+        <v>9</v>
+      </c>
+      <c r="D35" t="s">
+        <v>33</v>
+      </c>
+      <c r="F35">
+        <v>1750</v>
+      </c>
+      <c r="G35" t="s">
+        <v>228</v>
+      </c>
+      <c r="J35">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>210</v>
+      </c>
+      <c r="B36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36">
+        <v>9</v>
+      </c>
+      <c r="D36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F36">
+        <v>1750</v>
+      </c>
+      <c r="I36">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>223</v>
+      </c>
+      <c r="B37" t="s">
+        <v>29</v>
+      </c>
+      <c r="C37">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F37">
+        <v>1750</v>
+      </c>
+      <c r="G37" t="s">
+        <v>228</v>
+      </c>
+      <c r="J37">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>228</v>
+      </c>
+      <c r="D38" t="s">
+        <v>31</v>
+      </c>
+      <c r="E38">
+        <v>45000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E11AA6E-3A21-4E4D-BBE2-CBF8D1A645C0}">
   <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3381,7 +4044,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF394502-4A59-4E3D-B4CF-5A5D5E1CBE54}">
   <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Add Dancer and receive job gauges and buffs
Route gauge and buff messages, add a rotation template and expand common status handling.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3995CE7C-4696-4AE4-A244-2B7710995162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17B14328-8E49-456B-B9DD-D291C1B5650A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="DRK" sheetId="5" r:id="rId3"/>
     <sheet name="SMN" sheetId="3" r:id="rId4"/>
     <sheet name="SCH" sheetId="4" r:id="rId5"/>
+    <sheet name="DNC" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$37</definedName>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="283">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -731,6 +732,156 @@
   </si>
   <si>
     <t>Carve and Spit</t>
+  </si>
+  <si>
+    <t>Cascade</t>
+  </si>
+  <si>
+    <t>Fountain</t>
+  </si>
+  <si>
+    <t>Fountain Ready</t>
+  </si>
+  <si>
+    <t>Windmill</t>
+  </si>
+  <si>
+    <t>Bladeshower</t>
+  </si>
+  <si>
+    <t>Reverse Cascade</t>
+  </si>
+  <si>
+    <t>Fountainfall</t>
+  </si>
+  <si>
+    <t>Rising Windmill</t>
+  </si>
+  <si>
+    <t>Bloodshower</t>
+  </si>
+  <si>
+    <t>Fan Dance</t>
+  </si>
+  <si>
+    <t>Fan Dance II</t>
+  </si>
+  <si>
+    <t>Fan Dance III</t>
+  </si>
+  <si>
+    <t>Fan Dance IV</t>
+  </si>
+  <si>
+    <t>Saber Dance</t>
+  </si>
+  <si>
+    <t>Devilement</t>
+  </si>
+  <si>
+    <t>Devilment Buff</t>
+  </si>
+  <si>
+    <t>Starfall Dance</t>
+  </si>
+  <si>
+    <t>Flourishing Starfall</t>
+  </si>
+  <si>
+    <t>Silken Symmetry</t>
+  </si>
+  <si>
+    <t>Silken Flow</t>
+  </si>
+  <si>
+    <t>Technical Step</t>
+  </si>
+  <si>
+    <t>Technical Dancing</t>
+  </si>
+  <si>
+    <t>Last Dance Ready</t>
+  </si>
+  <si>
+    <t>Last Dance</t>
+  </si>
+  <si>
+    <t>To be retrieved</t>
+  </si>
+  <si>
+    <t>Emboite</t>
+  </si>
+  <si>
+    <t>Entrechat</t>
+  </si>
+  <si>
+    <t>Jete</t>
+  </si>
+  <si>
+    <t>Pirouette</t>
+  </si>
+  <si>
+    <t>Special</t>
+  </si>
+  <si>
+    <t>Fans</t>
+  </si>
+  <si>
+    <t>Spirit</t>
+  </si>
+  <si>
+    <t>Flourishing Finish</t>
+  </si>
+  <si>
+    <t>Tillana</t>
+  </si>
+  <si>
+    <t>Threefold Fan Dance</t>
+  </si>
+  <si>
+    <t>Fourfold Fan Dance</t>
+  </si>
+  <si>
+    <t>Flourish</t>
+  </si>
+  <si>
+    <t>Standard Step</t>
+  </si>
+  <si>
+    <t>Standard Dancing</t>
+  </si>
+  <si>
+    <t>Standard Finish</t>
+  </si>
+  <si>
+    <t>Quadruple Technical Finish</t>
+  </si>
+  <si>
+    <t>Double Standard Finish</t>
+  </si>
+  <si>
+    <t>Triple Technical Finish</t>
+  </si>
+  <si>
+    <t>Single Standard Finish</t>
+  </si>
+  <si>
+    <t>Technical Step on CD</t>
+  </si>
+  <si>
+    <t>Flourishing Finish;Technical Step on CD</t>
+  </si>
+  <si>
+    <t>Single Technical Finish</t>
+  </si>
+  <si>
+    <t>Double Technical Finish</t>
+  </si>
+  <si>
+    <t>Standard Step on CD</t>
+  </si>
+  <si>
+    <t>Last Dance Ready;Standard Step on CD</t>
   </si>
 </sst>
 </file>
@@ -1146,7 +1297,7 @@
         <v>31</v>
       </c>
       <c r="E2">
-        <v>2480</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1713,7 +1864,7 @@
         <v>31</v>
       </c>
       <c r="E2">
-        <v>2480</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -2375,7 +2526,7 @@
         <v>31</v>
       </c>
       <c r="E3">
-        <v>2480</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -4210,4 +4361,753 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
+  <dimension ref="A1:K55"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" customWidth="1"/>
+    <col min="3" max="3" width="6.140625" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>263</v>
+      </c>
+      <c r="J2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>235</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>237</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>30</v>
+      </c>
+      <c r="H10" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11">
+        <v>30000</v>
+      </c>
+      <c r="K11" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>238</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12">
+        <v>7</v>
+      </c>
+      <c r="D12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>240</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>252</v>
+      </c>
+      <c r="D14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14">
+        <v>30000</v>
+      </c>
+      <c r="K14" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>239</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+      <c r="H15" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>241</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>270</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18">
+        <v>30000</v>
+      </c>
+      <c r="G18" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>271</v>
+      </c>
+      <c r="D19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>272</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20">
+        <v>9</v>
+      </c>
+      <c r="D20" t="s">
+        <v>262</v>
+      </c>
+      <c r="G20" t="s">
+        <v>282</v>
+      </c>
+      <c r="H20" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>276</v>
+      </c>
+      <c r="D21" t="s">
+        <v>262</v>
+      </c>
+      <c r="G21" t="s">
+        <v>282</v>
+      </c>
+      <c r="H21" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>274</v>
+      </c>
+      <c r="D22" t="s">
+        <v>262</v>
+      </c>
+      <c r="G22" t="s">
+        <v>282</v>
+      </c>
+      <c r="H22" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>281</v>
+      </c>
+      <c r="D23" t="s">
+        <v>31</v>
+      </c>
+      <c r="E23">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>255</v>
+      </c>
+      <c r="D24" t="s">
+        <v>32</v>
+      </c>
+      <c r="E24">
+        <v>30000</v>
+      </c>
+      <c r="H24" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>256</v>
+      </c>
+      <c r="B25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25">
+        <v>9</v>
+      </c>
+      <c r="D25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>253</v>
+      </c>
+      <c r="B26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26">
+        <v>9</v>
+      </c>
+      <c r="D26" t="s">
+        <v>30</v>
+      </c>
+      <c r="G26" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>254</v>
+      </c>
+      <c r="D27" t="s">
+        <v>31</v>
+      </c>
+      <c r="E27">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>279</v>
+      </c>
+      <c r="D28" t="s">
+        <v>262</v>
+      </c>
+      <c r="G28" t="s">
+        <v>278</v>
+      </c>
+      <c r="H28" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>280</v>
+      </c>
+      <c r="D29" t="s">
+        <v>262</v>
+      </c>
+      <c r="G29" t="s">
+        <v>278</v>
+      </c>
+      <c r="H29" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>275</v>
+      </c>
+      <c r="D30" t="s">
+        <v>262</v>
+      </c>
+      <c r="G30" t="s">
+        <v>278</v>
+      </c>
+      <c r="H30" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>273</v>
+      </c>
+      <c r="D31" t="s">
+        <v>262</v>
+      </c>
+      <c r="G31" t="s">
+        <v>278</v>
+      </c>
+      <c r="H31" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>277</v>
+      </c>
+      <c r="D32" t="s">
+        <v>31</v>
+      </c>
+      <c r="E32">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>265</v>
+      </c>
+      <c r="D33" t="s">
+        <v>32</v>
+      </c>
+      <c r="E33">
+        <v>30000</v>
+      </c>
+      <c r="G33" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>266</v>
+      </c>
+      <c r="B34" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34">
+        <v>9</v>
+      </c>
+      <c r="D34" t="s">
+        <v>30</v>
+      </c>
+      <c r="H34" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>258</v>
+      </c>
+      <c r="B35" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35">
+        <v>4</v>
+      </c>
+      <c r="D35" t="s">
+        <v>262</v>
+      </c>
+      <c r="F35">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>259</v>
+      </c>
+      <c r="B36" t="s">
+        <v>27</v>
+      </c>
+      <c r="C36">
+        <v>5</v>
+      </c>
+      <c r="D36" t="s">
+        <v>262</v>
+      </c>
+      <c r="F36">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>260</v>
+      </c>
+      <c r="B37" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37">
+        <v>7</v>
+      </c>
+      <c r="D37" t="s">
+        <v>262</v>
+      </c>
+      <c r="F37">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>261</v>
+      </c>
+      <c r="B38" t="s">
+        <v>27</v>
+      </c>
+      <c r="C38">
+        <v>8</v>
+      </c>
+      <c r="D38" t="s">
+        <v>262</v>
+      </c>
+      <c r="F38">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>242</v>
+      </c>
+      <c r="B41" t="s">
+        <v>27</v>
+      </c>
+      <c r="C41">
+        <v>6</v>
+      </c>
+      <c r="D41" t="s">
+        <v>33</v>
+      </c>
+      <c r="E41">
+        <v>1000</v>
+      </c>
+      <c r="F41">
+        <v>1000</v>
+      </c>
+      <c r="I41">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>243</v>
+      </c>
+      <c r="B42" t="s">
+        <v>29</v>
+      </c>
+      <c r="C42">
+        <v>6</v>
+      </c>
+      <c r="D42" t="s">
+        <v>33</v>
+      </c>
+      <c r="F42">
+        <v>1000</v>
+      </c>
+      <c r="I42">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>267</v>
+      </c>
+      <c r="D43" t="s">
+        <v>32</v>
+      </c>
+      <c r="E43">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>244</v>
+      </c>
+      <c r="B44" t="s">
+        <v>28</v>
+      </c>
+      <c r="C44">
+        <v>6</v>
+      </c>
+      <c r="D44" t="s">
+        <v>33</v>
+      </c>
+      <c r="F44">
+        <v>1000</v>
+      </c>
+      <c r="H44" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>268</v>
+      </c>
+      <c r="D45" t="s">
+        <v>32</v>
+      </c>
+      <c r="E45">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>245</v>
+      </c>
+      <c r="B46" t="s">
+        <v>28</v>
+      </c>
+      <c r="C46">
+        <v>5</v>
+      </c>
+      <c r="D46" t="s">
+        <v>33</v>
+      </c>
+      <c r="F46">
+        <v>1000</v>
+      </c>
+      <c r="H46" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>246</v>
+      </c>
+      <c r="B48" t="s">
+        <v>28</v>
+      </c>
+      <c r="C48">
+        <v>4</v>
+      </c>
+      <c r="D48" t="s">
+        <v>30</v>
+      </c>
+      <c r="J48">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>247</v>
+      </c>
+      <c r="B50" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50">
+        <v>2</v>
+      </c>
+      <c r="D50" t="s">
+        <v>33</v>
+      </c>
+      <c r="F50">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>248</v>
+      </c>
+      <c r="D51" t="s">
+        <v>31</v>
+      </c>
+      <c r="E51">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>250</v>
+      </c>
+      <c r="D52" t="s">
+        <v>32</v>
+      </c>
+      <c r="E52">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>249</v>
+      </c>
+      <c r="B53" t="s">
+        <v>28</v>
+      </c>
+      <c r="C53">
+        <v>7</v>
+      </c>
+      <c r="D53" t="s">
+        <v>30</v>
+      </c>
+      <c r="H53" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>269</v>
+      </c>
+      <c r="B55" t="s">
+        <v>27</v>
+      </c>
+      <c r="C55">
+        <v>12</v>
+      </c>
+      <c r="D55" t="s">
+        <v>33</v>
+      </c>
+      <c r="F55">
+        <v>60000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Expand Dancer priorities and gauge timing
Refine dance and burst decisions, reorder gauge bytes and add status checks at a future time.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17B14328-8E49-456B-B9DD-D291C1B5650A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4824F2AA-D62A-449C-8275-66F554CC2426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="288">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -776,9 +776,6 @@
     <t>Saber Dance</t>
   </si>
   <si>
-    <t>Devilement</t>
-  </si>
-  <si>
     <t>Devilment Buff</t>
   </si>
   <si>
@@ -809,6 +806,9 @@
     <t>To be retrieved</t>
   </si>
   <si>
+    <t>Technical Finish</t>
+  </si>
+  <si>
     <t>Emboite</t>
   </si>
   <si>
@@ -827,9 +827,6 @@
     <t>Fans</t>
   </si>
   <si>
-    <t>Spirit</t>
-  </si>
-  <si>
     <t>Flourishing Finish</t>
   </si>
   <si>
@@ -869,9 +866,6 @@
     <t>Technical Step on CD</t>
   </si>
   <si>
-    <t>Flourishing Finish;Technical Step on CD</t>
-  </si>
-  <si>
     <t>Single Technical Finish</t>
   </si>
   <si>
@@ -881,7 +875,28 @@
     <t>Standard Step on CD</t>
   </si>
   <si>
-    <t>Last Dance Ready;Standard Step on CD</t>
+    <t>Esprit</t>
+  </si>
+  <si>
+    <t>Technical Finish Buff</t>
+  </si>
+  <si>
+    <t>Flourishing Starfall;Devilment Buff</t>
+  </si>
+  <si>
+    <t>Devilment</t>
+  </si>
+  <si>
+    <t>Silken Symmetry;Silken Flow;Threefold Fan Dance;Fourfold Fan Dance</t>
+  </si>
+  <si>
+    <t>Flourishing Finish;Technical Finish Buff</t>
+  </si>
+  <si>
+    <t>Technical Dancing;;Technical Step on CD</t>
+  </si>
+  <si>
+    <t>Standard Dancing;Standard Step on CD</t>
   </si>
 </sst>
 </file>
@@ -4365,7 +4380,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -4411,7 +4426,7 @@
         <v>263</v>
       </c>
       <c r="J2" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -4506,7 +4521,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D11" t="s">
         <v>32</v>
@@ -4515,7 +4530,7 @@
         <v>30000</v>
       </c>
       <c r="K11" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -4532,7 +4547,7 @@
         <v>30</v>
       </c>
       <c r="H12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -4549,12 +4564,12 @@
         <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D14" t="s">
         <v>32</v>
@@ -4563,7 +4578,7 @@
         <v>30000</v>
       </c>
       <c r="K14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -4580,7 +4595,7 @@
         <v>30</v>
       </c>
       <c r="H15" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -4597,12 +4612,12 @@
         <v>30</v>
       </c>
       <c r="H16" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B18" t="s">
         <v>27</v>
@@ -4617,12 +4632,12 @@
         <v>30000</v>
       </c>
       <c r="G18" t="s">
-        <v>271</v>
+        <v>287</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D19" t="s">
         <v>31</v>
@@ -4633,7 +4648,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
@@ -4645,43 +4660,43 @@
         <v>262</v>
       </c>
       <c r="G20" t="s">
-        <v>282</v>
+        <v>254</v>
       </c>
       <c r="H20" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D21" t="s">
         <v>262</v>
       </c>
       <c r="G21" t="s">
-        <v>282</v>
+        <v>254</v>
       </c>
       <c r="H21" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D22" t="s">
         <v>262</v>
       </c>
       <c r="G22" t="s">
-        <v>282</v>
+        <v>254</v>
       </c>
       <c r="H22" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D23" t="s">
         <v>31</v>
@@ -4692,7 +4707,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D24" t="s">
         <v>32</v>
@@ -4700,13 +4715,10 @@
       <c r="E24">
         <v>30000</v>
       </c>
-      <c r="H24" t="s">
-        <v>255</v>
-      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B25" t="s">
         <v>29</v>
@@ -4717,193 +4729,176 @@
       <c r="D25" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>253</v>
-      </c>
-      <c r="B26" t="s">
-        <v>28</v>
-      </c>
-      <c r="C26">
-        <v>9</v>
-      </c>
-      <c r="D26" t="s">
-        <v>30</v>
-      </c>
-      <c r="G26" t="s">
+      <c r="H25" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>254</v>
+        <v>252</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27">
+        <v>9</v>
       </c>
       <c r="D27" t="s">
-        <v>31</v>
-      </c>
-      <c r="E27">
-        <v>15000</v>
+        <v>30</v>
+      </c>
+      <c r="G27" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>279</v>
+        <v>253</v>
       </c>
       <c r="D28" t="s">
-        <v>262</v>
-      </c>
-      <c r="G28" t="s">
-        <v>278</v>
-      </c>
-      <c r="H28" t="s">
-        <v>254</v>
+        <v>31</v>
+      </c>
+      <c r="E28">
+        <v>15000</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>280</v>
+        <v>257</v>
+      </c>
+      <c r="B29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29">
+        <v>9</v>
       </c>
       <c r="D29" t="s">
         <v>262</v>
       </c>
       <c r="G29" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="H29" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D30" t="s">
         <v>262</v>
       </c>
       <c r="G30" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="H30" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D31" t="s">
         <v>262</v>
       </c>
       <c r="G31" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="H31" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D32" t="s">
+        <v>262</v>
+      </c>
+      <c r="G32" t="s">
+        <v>285</v>
+      </c>
+      <c r="H32" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>272</v>
+      </c>
+      <c r="D33" t="s">
+        <v>262</v>
+      </c>
+      <c r="G33" t="s">
+        <v>285</v>
+      </c>
+      <c r="H33" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>276</v>
+      </c>
+      <c r="D34" t="s">
         <v>31</v>
       </c>
-      <c r="E32">
+      <c r="E34">
         <v>120000</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>281</v>
+      </c>
+      <c r="D35" t="s">
+        <v>31</v>
+      </c>
+      <c r="E35">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>264</v>
+      </c>
+      <c r="D36" t="s">
+        <v>32</v>
+      </c>
+      <c r="E36">
+        <v>30000</v>
+      </c>
+      <c r="G36" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>265</v>
       </c>
-      <c r="D33" t="s">
-        <v>32</v>
-      </c>
-      <c r="E33">
-        <v>30000</v>
-      </c>
-      <c r="G33" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>266</v>
-      </c>
-      <c r="B34" t="s">
-        <v>28</v>
-      </c>
-      <c r="C34">
+      <c r="B37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37">
         <v>9</v>
       </c>
-      <c r="D34" t="s">
-        <v>30</v>
-      </c>
-      <c r="H34" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="D37" t="s">
+        <v>30</v>
+      </c>
+      <c r="H37" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>258</v>
       </c>
-      <c r="B35" t="s">
-        <v>27</v>
-      </c>
-      <c r="C35">
+      <c r="B38" t="s">
+        <v>27</v>
+      </c>
+      <c r="C38">
         <v>4</v>
-      </c>
-      <c r="D35" t="s">
-        <v>262</v>
-      </c>
-      <c r="F35">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>259</v>
-      </c>
-      <c r="B36" t="s">
-        <v>27</v>
-      </c>
-      <c r="C36">
-        <v>5</v>
-      </c>
-      <c r="D36" t="s">
-        <v>262</v>
-      </c>
-      <c r="F36">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>260</v>
-      </c>
-      <c r="B37" t="s">
-        <v>27</v>
-      </c>
-      <c r="C37">
-        <v>7</v>
-      </c>
-      <c r="D37" t="s">
-        <v>262</v>
-      </c>
-      <c r="F37">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>261</v>
-      </c>
-      <c r="B38" t="s">
-        <v>27</v>
-      </c>
-      <c r="C38">
-        <v>8</v>
       </c>
       <c r="D38" t="s">
         <v>262</v>
@@ -4912,66 +4907,63 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>259</v>
+      </c>
+      <c r="B39" t="s">
+        <v>27</v>
+      </c>
+      <c r="C39">
+        <v>5</v>
+      </c>
+      <c r="D39" t="s">
+        <v>262</v>
+      </c>
+      <c r="F39">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>260</v>
+      </c>
+      <c r="B40" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40">
+        <v>7</v>
+      </c>
+      <c r="D40" t="s">
+        <v>262</v>
+      </c>
+      <c r="F40">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="B41" t="s">
         <v>27</v>
       </c>
       <c r="C41">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D41" t="s">
-        <v>33</v>
-      </c>
-      <c r="E41">
-        <v>1000</v>
+        <v>262</v>
       </c>
       <c r="F41">
         <v>1000</v>
       </c>
-      <c r="I41">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>243</v>
-      </c>
-      <c r="B42" t="s">
-        <v>29</v>
-      </c>
-      <c r="C42">
-        <v>6</v>
-      </c>
-      <c r="D42" t="s">
-        <v>33</v>
-      </c>
-      <c r="F42">
-        <v>1000</v>
-      </c>
-      <c r="I42">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>267</v>
-      </c>
-      <c r="D43" t="s">
-        <v>32</v>
-      </c>
-      <c r="E43">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B44" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C44">
         <v>6</v>
@@ -4979,132 +4971,192 @@
       <c r="D44" t="s">
         <v>33</v>
       </c>
+      <c r="E44">
+        <v>1000</v>
+      </c>
       <c r="F44">
         <v>1000</v>
       </c>
-      <c r="H44" t="s">
+      <c r="I44">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>243</v>
+      </c>
+      <c r="B45" t="s">
+        <v>29</v>
+      </c>
+      <c r="C45">
+        <v>6</v>
+      </c>
+      <c r="D45" t="s">
+        <v>33</v>
+      </c>
+      <c r="F45">
+        <v>1000</v>
+      </c>
+      <c r="I45">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>266</v>
+      </c>
+      <c r="D46" t="s">
+        <v>32</v>
+      </c>
+      <c r="E46">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>244</v>
+      </c>
+      <c r="B47" t="s">
+        <v>28</v>
+      </c>
+      <c r="C47">
+        <v>6</v>
+      </c>
+      <c r="D47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F47">
+        <v>1000</v>
+      </c>
+      <c r="H47" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+      <c r="D48" t="s">
+        <v>32</v>
+      </c>
+      <c r="E48">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>245</v>
+      </c>
+      <c r="B49" t="s">
+        <v>28</v>
+      </c>
+      <c r="C49">
+        <v>5</v>
+      </c>
+      <c r="D49" t="s">
+        <v>33</v>
+      </c>
+      <c r="F49">
+        <v>1000</v>
+      </c>
+      <c r="H49" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>246</v>
+      </c>
+      <c r="B51" t="s">
+        <v>28</v>
+      </c>
+      <c r="C51">
+        <v>4</v>
+      </c>
+      <c r="D51" t="s">
+        <v>30</v>
+      </c>
+      <c r="J51">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>283</v>
+      </c>
+      <c r="B53" t="s">
+        <v>28</v>
+      </c>
+      <c r="C53">
+        <v>2</v>
+      </c>
+      <c r="D53" t="s">
+        <v>33</v>
+      </c>
+      <c r="F53">
+        <v>120000</v>
+      </c>
+      <c r="G53" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>247</v>
+      </c>
+      <c r="D54" t="s">
+        <v>31</v>
+      </c>
+      <c r="E54">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>249</v>
+      </c>
+      <c r="D55" t="s">
+        <v>32</v>
+      </c>
+      <c r="E55">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>248</v>
+      </c>
+      <c r="B56" t="s">
+        <v>28</v>
+      </c>
+      <c r="C56">
+        <v>7</v>
+      </c>
+      <c r="D56" t="s">
+        <v>30</v>
+      </c>
+      <c r="H56" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>268</v>
       </c>
-      <c r="D45" t="s">
-        <v>32</v>
-      </c>
-      <c r="E45">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>245</v>
-      </c>
-      <c r="B46" t="s">
-        <v>28</v>
-      </c>
-      <c r="C46">
-        <v>5</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="B58" t="s">
+        <v>27</v>
+      </c>
+      <c r="C58">
+        <v>12</v>
+      </c>
+      <c r="D58" t="s">
         <v>33</v>
       </c>
-      <c r="F46">
-        <v>1000</v>
-      </c>
-      <c r="H46" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>246</v>
-      </c>
-      <c r="B48" t="s">
-        <v>28</v>
-      </c>
-      <c r="C48">
-        <v>4</v>
-      </c>
-      <c r="D48" t="s">
-        <v>30</v>
-      </c>
-      <c r="J48">
-        <v>-50</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>247</v>
-      </c>
-      <c r="B50" t="s">
-        <v>28</v>
-      </c>
-      <c r="C50">
-        <v>2</v>
-      </c>
-      <c r="D50" t="s">
-        <v>33</v>
-      </c>
-      <c r="F50">
-        <v>120000</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>248</v>
-      </c>
-      <c r="D51" t="s">
-        <v>31</v>
-      </c>
-      <c r="E51">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>250</v>
-      </c>
-      <c r="D52" t="s">
-        <v>32</v>
-      </c>
-      <c r="E52">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>249</v>
-      </c>
-      <c r="B53" t="s">
-        <v>28</v>
-      </c>
-      <c r="C53">
-        <v>7</v>
-      </c>
-      <c r="D53" t="s">
-        <v>30</v>
-      </c>
-      <c r="H53" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>269</v>
-      </c>
-      <c r="B55" t="s">
-        <v>27</v>
-      </c>
-      <c r="C55">
-        <v>12</v>
-      </c>
-      <c r="D55" t="s">
-        <v>33</v>
-      </c>
-      <c r="F55">
+      <c r="F58">
         <v>60000</v>
+      </c>
+      <c r="G58" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine Dancer step and finisher priorities
Add Standard Step timing rules, prioritize Last Dance and lower the Esprit spending threshold.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4824F2AA-D62A-449C-8275-66F554CC2426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90F2110-FCB1-4FEF-8C14-C78F6F57063E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="297">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -887,16 +887,43 @@
     <t>Devilment</t>
   </si>
   <si>
-    <t>Silken Symmetry;Silken Flow;Threefold Fan Dance;Fourfold Fan Dance</t>
-  </si>
-  <si>
-    <t>Flourishing Finish;Technical Finish Buff</t>
-  </si>
-  <si>
     <t>Technical Dancing;;Technical Step on CD</t>
   </si>
   <si>
     <t>Standard Dancing;Standard Step on CD</t>
+  </si>
+  <si>
+    <t>Follow up high level</t>
+  </si>
+  <si>
+    <t>Flourishing Symmetry</t>
+  </si>
+  <si>
+    <t>Flourishing Flow</t>
+  </si>
+  <si>
+    <t>Ignord</t>
+  </si>
+  <si>
+    <t>Finishing Move Ready</t>
+  </si>
+  <si>
+    <t>Silken Symmetry;Silken Flow;Threefold Fan Dance;Fourfold Fan Dance;Finishing Move Ready</t>
+  </si>
+  <si>
+    <t>Finishing Move</t>
+  </si>
+  <si>
+    <t>Standard Step on CD;Last Dance Ready</t>
+  </si>
+  <si>
+    <t>Dance of the Dawn</t>
+  </si>
+  <si>
+    <t>Dance of the Dawn Ready</t>
+  </si>
+  <si>
+    <t>Flourishing Finish;Technical Finish Buff;Dance of the Dawn Ready</t>
   </si>
 </sst>
 </file>
@@ -4380,7 +4407,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -4535,27 +4562,24 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>238</v>
-      </c>
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12">
-        <v>7</v>
+        <v>287</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
-      </c>
-      <c r="H12" t="s">
-        <v>250</v>
+        <v>32</v>
+      </c>
+      <c r="E12">
+        <v>30000</v>
+      </c>
+      <c r="K12" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C13">
         <v>7</v>
@@ -4569,86 +4593,86 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>251</v>
+        <v>240</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14">
+        <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14">
-        <v>30000</v>
-      </c>
-      <c r="K14" t="s">
-        <v>256</v>
+        <v>30</v>
+      </c>
+      <c r="H14" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>239</v>
-      </c>
-      <c r="B15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15">
-        <v>8</v>
+        <v>251</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
-      </c>
-      <c r="H15" t="s">
-        <v>251</v>
+        <v>32</v>
+      </c>
+      <c r="E15">
+        <v>30000</v>
+      </c>
+      <c r="K15" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>288</v>
+      </c>
+      <c r="D16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16">
+        <v>30000</v>
+      </c>
+      <c r="K16" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>239</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17">
+        <v>8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H17" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>241</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B18" t="s">
         <v>29</v>
       </c>
-      <c r="C16">
+      <c r="C18">
         <v>8</v>
       </c>
-      <c r="D16" t="s">
-        <v>30</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="H18" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>269</v>
-      </c>
-      <c r="B18" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18">
-        <v>9</v>
-      </c>
-      <c r="D18" t="s">
-        <v>30</v>
-      </c>
-      <c r="F18">
-        <v>30000</v>
-      </c>
-      <c r="G18" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>270</v>
-      </c>
-      <c r="D19" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>271</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
@@ -4657,181 +4681,190 @@
         <v>9</v>
       </c>
       <c r="D20" t="s">
+        <v>30</v>
+      </c>
+      <c r="F20">
+        <v>30000</v>
+      </c>
+      <c r="G20" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>292</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+      <c r="F21">
+        <v>30000</v>
+      </c>
+      <c r="G21" t="s">
+        <v>293</v>
+      </c>
+      <c r="H21" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>270</v>
+      </c>
+      <c r="D22" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>271</v>
+      </c>
+      <c r="B23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23">
+        <v>9</v>
+      </c>
+      <c r="D23" t="s">
         <v>262</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G23" t="s">
         <v>254</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H23" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>275</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D24" t="s">
         <v>262</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G24" t="s">
         <v>254</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H24" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>273</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D25" t="s">
         <v>262</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G25" t="s">
         <v>254</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H25" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>279</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D26" t="s">
         <v>31</v>
       </c>
-      <c r="E23">
+      <c r="E26">
         <v>30000</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>254</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D27" t="s">
         <v>32</v>
       </c>
-      <c r="E24">
+      <c r="E27">
         <v>30000</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>255</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B28" t="s">
         <v>29</v>
       </c>
-      <c r="C25">
+      <c r="C28">
         <v>9</v>
       </c>
-      <c r="D25" t="s">
-        <v>30</v>
-      </c>
-      <c r="H25" t="s">
+      <c r="D28" t="s">
+        <v>30</v>
+      </c>
+      <c r="H28" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>252</v>
       </c>
-      <c r="B27" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27">
+      <c r="B30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30">
         <v>9</v>
       </c>
-      <c r="D27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G27" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="D30" t="s">
+        <v>30</v>
+      </c>
+      <c r="G30" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>253</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D31" t="s">
         <v>31</v>
       </c>
-      <c r="E28">
+      <c r="E31">
         <v>15000</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>257</v>
       </c>
-      <c r="B29" t="s">
-        <v>28</v>
-      </c>
-      <c r="C29">
+      <c r="B32" t="s">
+        <v>28</v>
+      </c>
+      <c r="C32">
         <v>9</v>
-      </c>
-      <c r="D29" t="s">
-        <v>262</v>
-      </c>
-      <c r="G29" t="s">
-        <v>285</v>
-      </c>
-      <c r="H29" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>277</v>
-      </c>
-      <c r="D30" t="s">
-        <v>262</v>
-      </c>
-      <c r="G30" t="s">
-        <v>285</v>
-      </c>
-      <c r="H30" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>278</v>
-      </c>
-      <c r="D31" t="s">
-        <v>262</v>
-      </c>
-      <c r="G31" t="s">
-        <v>285</v>
-      </c>
-      <c r="H31" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>274</v>
       </c>
       <c r="D32" t="s">
         <v>262</v>
       </c>
       <c r="G32" t="s">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="H32" t="s">
         <v>253</v>
       </c>
+      <c r="K32" t="s">
+        <v>286</v>
+      </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D33" t="s">
         <v>262</v>
       </c>
       <c r="G33" t="s">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="H33" t="s">
         <v>253</v>
@@ -4839,117 +4872,105 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D34" t="s">
-        <v>31</v>
-      </c>
-      <c r="E34">
-        <v>120000</v>
+        <v>262</v>
+      </c>
+      <c r="G34" t="s">
+        <v>296</v>
+      </c>
+      <c r="H34" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="D35" t="s">
-        <v>31</v>
-      </c>
-      <c r="E35">
-        <v>20000</v>
+        <v>262</v>
+      </c>
+      <c r="G35" t="s">
+        <v>296</v>
+      </c>
+      <c r="H35" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D36" t="s">
-        <v>32</v>
-      </c>
-      <c r="E36">
-        <v>30000</v>
+        <v>262</v>
       </c>
       <c r="G36" t="s">
-        <v>264</v>
+        <v>296</v>
+      </c>
+      <c r="H36" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>265</v>
-      </c>
-      <c r="B37" t="s">
-        <v>28</v>
-      </c>
-      <c r="C37">
-        <v>9</v>
+        <v>276</v>
       </c>
       <c r="D37" t="s">
-        <v>30</v>
-      </c>
-      <c r="H37" t="s">
-        <v>264</v>
+        <v>31</v>
+      </c>
+      <c r="E37">
+        <v>120000</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>258</v>
-      </c>
-      <c r="B38" t="s">
-        <v>27</v>
-      </c>
-      <c r="C38">
-        <v>4</v>
+        <v>281</v>
       </c>
       <c r="D38" t="s">
-        <v>262</v>
-      </c>
-      <c r="F38">
-        <v>1000</v>
+        <v>31</v>
+      </c>
+      <c r="E38">
+        <v>20000</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>259</v>
-      </c>
-      <c r="B39" t="s">
-        <v>27</v>
-      </c>
-      <c r="C39">
-        <v>5</v>
+        <v>264</v>
       </c>
       <c r="D39" t="s">
-        <v>262</v>
-      </c>
-      <c r="F39">
-        <v>1000</v>
+        <v>32</v>
+      </c>
+      <c r="E39">
+        <v>30000</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B40" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C40">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D40" t="s">
-        <v>262</v>
-      </c>
-      <c r="F40">
-        <v>1000</v>
+        <v>30</v>
+      </c>
+      <c r="H40" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B41" t="s">
         <v>27</v>
       </c>
       <c r="C41">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D41" t="s">
         <v>262</v>
@@ -4958,66 +4979,63 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>259</v>
+      </c>
+      <c r="B42" t="s">
+        <v>27</v>
+      </c>
+      <c r="C42">
+        <v>5</v>
+      </c>
+      <c r="D42" t="s">
+        <v>262</v>
+      </c>
+      <c r="F42">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>260</v>
+      </c>
+      <c r="B43" t="s">
+        <v>27</v>
+      </c>
+      <c r="C43">
+        <v>7</v>
+      </c>
+      <c r="D43" t="s">
+        <v>262</v>
+      </c>
+      <c r="F43">
+        <v>1000</v>
+      </c>
+    </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="B44" t="s">
         <v>27</v>
       </c>
       <c r="C44">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D44" t="s">
-        <v>33</v>
-      </c>
-      <c r="E44">
-        <v>1000</v>
+        <v>262</v>
       </c>
       <c r="F44">
         <v>1000</v>
       </c>
-      <c r="I44">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>243</v>
-      </c>
-      <c r="B45" t="s">
-        <v>29</v>
-      </c>
-      <c r="C45">
-        <v>6</v>
-      </c>
-      <c r="D45" t="s">
-        <v>33</v>
-      </c>
-      <c r="F45">
-        <v>1000</v>
-      </c>
-      <c r="I45">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>266</v>
-      </c>
-      <c r="D46" t="s">
-        <v>32</v>
-      </c>
-      <c r="E46">
-        <v>30000</v>
-      </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B47" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C47">
         <v>6</v>
@@ -5025,138 +5043,234 @@
       <c r="D47" t="s">
         <v>33</v>
       </c>
+      <c r="E47">
+        <v>1000</v>
+      </c>
       <c r="F47">
         <v>1000</v>
       </c>
-      <c r="H47" t="s">
-        <v>266</v>
+      <c r="I47">
+        <v>-1</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>267</v>
+        <v>243</v>
+      </c>
+      <c r="B48" t="s">
+        <v>29</v>
+      </c>
+      <c r="C48">
+        <v>6</v>
       </c>
       <c r="D48" t="s">
-        <v>32</v>
-      </c>
-      <c r="E48">
-        <v>30000</v>
+        <v>33</v>
+      </c>
+      <c r="F48">
+        <v>1000</v>
+      </c>
+      <c r="I48">
+        <v>-1</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>245</v>
-      </c>
-      <c r="B49" t="s">
-        <v>28</v>
-      </c>
-      <c r="C49">
-        <v>5</v>
+        <v>266</v>
       </c>
       <c r="D49" t="s">
+        <v>32</v>
+      </c>
+      <c r="E49">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>244</v>
+      </c>
+      <c r="B50" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50">
+        <v>6</v>
+      </c>
+      <c r="D50" t="s">
         <v>33</v>
       </c>
-      <c r="F49">
+      <c r="F50">
         <v>1000</v>
       </c>
-      <c r="H49" t="s">
-        <v>267</v>
+      <c r="H50" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>246</v>
-      </c>
-      <c r="B51" t="s">
-        <v>28</v>
-      </c>
-      <c r="C51">
-        <v>4</v>
+        <v>267</v>
       </c>
       <c r="D51" t="s">
-        <v>30</v>
-      </c>
-      <c r="J51">
-        <v>-50</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>283</v>
-      </c>
-      <c r="B53" t="s">
-        <v>28</v>
-      </c>
-      <c r="C53">
-        <v>2</v>
-      </c>
-      <c r="D53" t="s">
+        <v>32</v>
+      </c>
+      <c r="E51">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>245</v>
+      </c>
+      <c r="B52" t="s">
+        <v>28</v>
+      </c>
+      <c r="C52">
+        <v>5</v>
+      </c>
+      <c r="D52" t="s">
         <v>33</v>
       </c>
-      <c r="F53">
-        <v>120000</v>
-      </c>
-      <c r="G53" t="s">
-        <v>282</v>
+      <c r="F52">
+        <v>1000</v>
+      </c>
+      <c r="H52" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>247</v>
+        <v>246</v>
+      </c>
+      <c r="B54" t="s">
+        <v>28</v>
+      </c>
+      <c r="C54">
+        <v>4</v>
       </c>
       <c r="D54" t="s">
-        <v>31</v>
-      </c>
-      <c r="E54">
-        <v>20000</v>
+        <v>30</v>
+      </c>
+      <c r="J54">
+        <v>-50</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>249</v>
+        <v>295</v>
       </c>
       <c r="D55" t="s">
         <v>32</v>
       </c>
       <c r="E55">
-        <v>20000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>248</v>
+        <v>294</v>
       </c>
       <c r="B56" t="s">
         <v>28</v>
       </c>
       <c r="C56">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D56" t="s">
         <v>30</v>
       </c>
       <c r="H56" t="s">
-        <v>249</v>
+        <v>295</v>
+      </c>
+      <c r="J56">
+        <v>-50</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>268</v>
+        <v>283</v>
       </c>
       <c r="B58" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C58">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D58" t="s">
         <v>33</v>
       </c>
       <c r="F58">
+        <v>120000</v>
+      </c>
+      <c r="G58" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>247</v>
+      </c>
+      <c r="D59" t="s">
+        <v>31</v>
+      </c>
+      <c r="E59">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>249</v>
+      </c>
+      <c r="D60" t="s">
+        <v>32</v>
+      </c>
+      <c r="E60">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>248</v>
+      </c>
+      <c r="B61" t="s">
+        <v>28</v>
+      </c>
+      <c r="C61">
+        <v>7</v>
+      </c>
+      <c r="D61" t="s">
+        <v>30</v>
+      </c>
+      <c r="H61" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>268</v>
+      </c>
+      <c r="B63" t="s">
+        <v>27</v>
+      </c>
+      <c r="C63">
+        <v>12</v>
+      </c>
+      <c r="D63" t="s">
+        <v>33</v>
+      </c>
+      <c r="F63">
         <v>60000</v>
       </c>
-      <c r="G58" t="s">
-        <v>284</v>
+      <c r="G63" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>290</v>
+      </c>
+      <c r="D64" t="s">
+        <v>32</v>
+      </c>
+      <c r="E64">
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Read Gunbreaker cartridges from the job gauge
Use gauge data for cartridge counts and remove the burst-delay condition from Double Down.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90F2110-FCB1-4FEF-8C14-C78F6F57063E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1005B5FA-FFDD-489E-A8AB-952AEA66239D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="298">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -924,6 +924,9 @@
   </si>
   <si>
     <t>Flourishing Finish;Technical Finish Buff;Dance of the Dawn Ready</t>
+  </si>
+  <si>
+    <t>stacks_a_obsolete</t>
   </si>
 </sst>
 </file>
@@ -1895,7 +1898,7 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add the initial Bard rotation and gauge dispatch
Introduce BRD priorities and strengthen status checks around the next GCD.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1005B5FA-FFDD-489E-A8AB-952AEA66239D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9D947FF-FAC2-4D38-B744-A9C9483E5A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14160" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="DRK" sheetId="5" r:id="rId3"/>
     <sheet name="SMN" sheetId="3" r:id="rId4"/>
     <sheet name="SCH" sheetId="4" r:id="rId5"/>
-    <sheet name="DNC" sheetId="6" r:id="rId6"/>
+    <sheet name="BRD" sheetId="7" r:id="rId6"/>
+    <sheet name="DNC" sheetId="6" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$37</definedName>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="367">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -927,6 +928,213 @@
   </si>
   <si>
     <t>stacks_a_obsolete</t>
+  </si>
+  <si>
+    <t>Burst Shot</t>
+  </si>
+  <si>
+    <t>Refulgent Arrow</t>
+  </si>
+  <si>
+    <t>Stormbite</t>
+  </si>
+  <si>
+    <t>Caustic Bite</t>
+  </si>
+  <si>
+    <t>Iron Jaws</t>
+  </si>
+  <si>
+    <t>Apex Arrow</t>
+  </si>
+  <si>
+    <t>Blast Arrow</t>
+  </si>
+  <si>
+    <t>Resonant Arrow</t>
+  </si>
+  <si>
+    <t>Radiant Encore</t>
+  </si>
+  <si>
+    <t>Ladonsbite</t>
+  </si>
+  <si>
+    <t>Shadowbite</t>
+  </si>
+  <si>
+    <t>Pitch Perfect</t>
+  </si>
+  <si>
+    <t>Mage’s Ballad</t>
+  </si>
+  <si>
+    <t>Heartbreak Shot</t>
+  </si>
+  <si>
+    <t>Rain of Death</t>
+  </si>
+  <si>
+    <t>Army’s Paeon</t>
+  </si>
+  <si>
+    <t>Enhanced Army’s Paeon</t>
+  </si>
+  <si>
+    <t>Empyreal Arrow</t>
+  </si>
+  <si>
+    <t>Barrage</t>
+  </si>
+  <si>
+    <t>Raging Strikes</t>
+  </si>
+  <si>
+    <t>Sidewinder</t>
+  </si>
+  <si>
+    <t>Battle Voice</t>
+  </si>
+  <si>
+    <t>Radiant Finale</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>prio song</t>
+  </si>
+  <si>
+    <t>at 3 stack unless end of buff / minuet</t>
+  </si>
+  <si>
+    <t>Use if close to 3 or under buff</t>
+  </si>
+  <si>
+    <t>AOE HBS</t>
+  </si>
+  <si>
+    <t>High priority oGCD</t>
+  </si>
+  <si>
+    <t>Song 2</t>
+  </si>
+  <si>
+    <t>Song 3</t>
+  </si>
+  <si>
+    <t>buff</t>
+  </si>
+  <si>
+    <t>The Wanderer's Minuet</t>
+  </si>
+  <si>
+    <t>Custom Buff</t>
+  </si>
+  <si>
+    <t>Filler</t>
+  </si>
+  <si>
+    <t>Bloodletter</t>
+  </si>
+  <si>
+    <t>Low level HBS</t>
+  </si>
+  <si>
+    <t>Refresh Dots</t>
+  </si>
+  <si>
+    <t>DoT</t>
+  </si>
+  <si>
+    <t>Hawk’s Eye procs</t>
+  </si>
+  <si>
+    <t>80+, No overcap unless 2m burst soon</t>
+  </si>
+  <si>
+    <t>Apex Arrow follow up at 80+</t>
+  </si>
+  <si>
+    <t>Lvl 96, barrage follow up</t>
+  </si>
+  <si>
+    <t>Lvl 100, Radiant Finale follow up</t>
+  </si>
+  <si>
+    <t>AoE Refulgent Arrow</t>
+  </si>
+  <si>
+    <t>Filler AOE</t>
+  </si>
+  <si>
+    <t>During 2m Buffs</t>
+  </si>
+  <si>
+    <t>Main 2m buff, after minuet</t>
+  </si>
+  <si>
+    <t>Battle Voice Buff</t>
+  </si>
+  <si>
+    <t>Raging Strikes Buff</t>
+  </si>
+  <si>
+    <t>Radiant Finale Buff</t>
+  </si>
+  <si>
+    <t>Barrage Buff</t>
+  </si>
+  <si>
+    <t>simple  oGCD - on CD</t>
+  </si>
+  <si>
+    <t>Blast Arrow Ready</t>
+  </si>
+  <si>
+    <t>Only if 80+</t>
+  </si>
+  <si>
+    <t>Resonant Arrow Ready</t>
+  </si>
+  <si>
+    <t>Radiant Encore Ready</t>
+  </si>
+  <si>
+    <t>Storm DoT</t>
+  </si>
+  <si>
+    <t>Caustic DoT</t>
+  </si>
+  <si>
+    <t>Storm DoT;Caustic DoT</t>
+  </si>
+  <si>
+    <t>Wanderer song</t>
+  </si>
+  <si>
+    <t>Mage song</t>
+  </si>
+  <si>
+    <t>Army song</t>
+  </si>
+  <si>
+    <t>Wanderer song;Mage song</t>
+  </si>
+  <si>
+    <t>Wanderer song;Army song</t>
+  </si>
+  <si>
+    <t>Mage song;Army song</t>
+  </si>
+  <si>
+    <t>Apex</t>
+  </si>
+  <si>
+    <t>Hawk's Eye</t>
+  </si>
+  <si>
+    <t>Ref Arrow ready</t>
   </si>
 </sst>
 </file>
@@ -1296,19 +1504,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -1334,7 +1542,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -1345,7 +1553,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1365,7 +1573,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1376,7 +1584,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1399,7 +1607,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1410,7 +1618,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1430,7 +1638,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>41</v>
       </c>
@@ -1441,7 +1649,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -1461,7 +1669,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1472,7 +1680,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -1492,7 +1700,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -1503,7 +1711,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -1520,7 +1728,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1531,7 +1739,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -1548,7 +1756,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -1568,7 +1776,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -1579,7 +1787,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -1590,7 +1798,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -1607,7 +1815,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -1627,7 +1835,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1638,7 +1846,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -1658,7 +1866,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -1669,7 +1877,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -1689,7 +1897,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -1700,7 +1908,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>46</v>
       </c>
@@ -1720,7 +1928,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>16</v>
       </c>
@@ -1731,7 +1939,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>17</v>
       </c>
@@ -1751,7 +1959,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -1762,7 +1970,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>19</v>
       </c>
@@ -1779,7 +1987,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>20</v>
       </c>
@@ -1796,7 +2004,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -1813,7 +2021,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>22</v>
       </c>
@@ -1827,7 +2035,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -1841,7 +2049,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>82</v>
       </c>
@@ -1863,16 +2071,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7762502F-9F7A-4AD9-AC88-345A2195334F}">
   <dimension ref="A1:I37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -1901,7 +2109,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -1912,7 +2120,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -1932,7 +2140,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -1943,7 +2151,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -1963,7 +2171,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -1974,7 +2182,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>55</v>
       </c>
@@ -1994,7 +2202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>56</v>
       </c>
@@ -2017,7 +2225,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>87</v>
       </c>
@@ -2028,7 +2236,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>57</v>
       </c>
@@ -2045,7 +2253,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -2068,7 +2276,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -2094,7 +2302,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>89</v>
       </c>
@@ -2105,7 +2313,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>60</v>
       </c>
@@ -2125,7 +2333,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>61</v>
       </c>
@@ -2136,7 +2344,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>62</v>
       </c>
@@ -2156,7 +2364,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>92</v>
       </c>
@@ -2167,7 +2375,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>97</v>
       </c>
@@ -2184,7 +2392,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>63</v>
       </c>
@@ -2210,7 +2418,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>64</v>
       </c>
@@ -2221,7 +2429,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>65</v>
       </c>
@@ -2238,7 +2446,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>66</v>
       </c>
@@ -2249,7 +2457,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>67</v>
       </c>
@@ -2269,7 +2477,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>68</v>
       </c>
@@ -2280,7 +2488,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -2297,7 +2505,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -2308,7 +2516,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>71</v>
       </c>
@@ -2328,7 +2536,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>86</v>
       </c>
@@ -2339,7 +2547,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>72</v>
       </c>
@@ -2356,7 +2564,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>73</v>
       </c>
@@ -2373,7 +2581,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>74</v>
       </c>
@@ -2390,7 +2598,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>75</v>
       </c>
@@ -2410,7 +2618,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>76</v>
       </c>
@@ -2430,7 +2638,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>78</v>
       </c>
@@ -2441,7 +2649,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>90</v>
       </c>
@@ -2452,7 +2660,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -2469,7 +2677,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>79</v>
       </c>
@@ -2497,19 +2705,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0983F4B6-DA2C-422A-9A48-B565C13F35E9}">
   <dimension ref="A1:M38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.1796875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -2544,7 +2752,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2563,7 +2771,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -2574,7 +2782,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>200</v>
       </c>
@@ -2591,7 +2799,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>202</v>
       </c>
@@ -2602,7 +2810,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>201</v>
       </c>
@@ -2622,7 +2830,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>204</v>
       </c>
@@ -2633,7 +2841,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>203</v>
       </c>
@@ -2653,7 +2861,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>232</v>
       </c>
@@ -2670,7 +2878,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>207</v>
       </c>
@@ -2687,7 +2895,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>205</v>
       </c>
@@ -2716,7 +2924,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>225</v>
       </c>
@@ -2727,7 +2935,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>230</v>
       </c>
@@ -2744,7 +2952,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>209</v>
       </c>
@@ -2761,7 +2969,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>226</v>
       </c>
@@ -2778,7 +2986,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>227</v>
       </c>
@@ -2795,7 +3003,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>208</v>
       </c>
@@ -2812,7 +3020,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>211</v>
       </c>
@@ -2826,7 +3034,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>212</v>
       </c>
@@ -2840,7 +3048,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>213</v>
       </c>
@@ -2854,7 +3062,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>214</v>
       </c>
@@ -2877,7 +3085,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>215</v>
       </c>
@@ -2888,7 +3096,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>216</v>
       </c>
@@ -2905,7 +3113,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>217</v>
       </c>
@@ -2916,7 +3124,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>218</v>
       </c>
@@ -2927,7 +3135,7 @@
         <v>24000</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>219</v>
       </c>
@@ -2947,7 +3155,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>221</v>
       </c>
@@ -2958,7 +3166,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>220</v>
       </c>
@@ -2975,7 +3183,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>222</v>
       </c>
@@ -2998,7 +3206,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>210</v>
       </c>
@@ -3018,7 +3226,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>223</v>
       </c>
@@ -3041,7 +3249,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>228</v>
       </c>
@@ -3060,16 +3268,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E11AA6E-3A21-4E4D-BBE2-CBF8D1A645C0}">
   <dimension ref="A1:K92"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -3101,7 +3309,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="I2" t="s">
         <v>104</v>
       </c>
@@ -3109,7 +3317,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -3120,7 +3328,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>106</v>
       </c>
@@ -3137,7 +3345,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>108</v>
       </c>
@@ -3157,7 +3365,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>110</v>
       </c>
@@ -3171,7 +3379,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>111</v>
       </c>
@@ -3185,7 +3393,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>112</v>
       </c>
@@ -3199,7 +3407,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>113</v>
       </c>
@@ -3216,7 +3424,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>114</v>
       </c>
@@ -3233,7 +3441,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>116</v>
       </c>
@@ -3250,7 +3458,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>117</v>
       </c>
@@ -3267,7 +3475,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>118</v>
       </c>
@@ -3293,7 +3501,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>121</v>
       </c>
@@ -3316,7 +3524,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>122</v>
       </c>
@@ -3336,7 +3544,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>124</v>
       </c>
@@ -3356,7 +3564,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>119</v>
       </c>
@@ -3367,7 +3575,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>125</v>
       </c>
@@ -3384,7 +3592,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>126</v>
       </c>
@@ -3398,7 +3606,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>128</v>
       </c>
@@ -3418,7 +3626,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>131</v>
       </c>
@@ -3438,7 +3646,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>133</v>
       </c>
@@ -3458,7 +3666,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>135</v>
       </c>
@@ -3469,7 +3677,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>136</v>
       </c>
@@ -3480,7 +3688,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
         <v>137</v>
       </c>
@@ -3491,7 +3699,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>138</v>
       </c>
@@ -3502,7 +3710,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>139</v>
       </c>
@@ -3519,7 +3727,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>140</v>
       </c>
@@ -3536,7 +3744,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
         <v>141</v>
       </c>
@@ -3553,7 +3761,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>142</v>
       </c>
@@ -3564,7 +3772,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>143</v>
       </c>
@@ -3581,7 +3789,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>144</v>
       </c>
@@ -3601,7 +3809,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
         <v>146</v>
       </c>
@@ -3618,7 +3826,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
         <v>147</v>
       </c>
@@ -3629,7 +3837,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
         <v>148</v>
       </c>
@@ -3649,7 +3857,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>149</v>
       </c>
@@ -3660,7 +3868,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>150</v>
       </c>
@@ -3683,7 +3891,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>153</v>
       </c>
@@ -3694,7 +3902,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="6" t="s">
         <v>154</v>
       </c>
@@ -3705,7 +3913,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="6" t="s">
         <v>155</v>
       </c>
@@ -3728,7 +3936,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="6" t="s">
         <v>156</v>
       </c>
@@ -3739,7 +3947,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="7" t="s">
         <v>158</v>
       </c>
@@ -3750,7 +3958,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="7" t="s">
         <v>159</v>
       </c>
@@ -3773,7 +3981,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="7" t="s">
         <v>162</v>
       </c>
@@ -3784,7 +3992,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>163</v>
       </c>
@@ -3798,7 +4006,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>164</v>
       </c>
@@ -3821,7 +4029,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" s="6" t="s">
         <v>166</v>
       </c>
@@ -3844,7 +4052,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" s="7" t="s">
         <v>168</v>
       </c>
@@ -3864,7 +4072,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>169</v>
       </c>
@@ -3878,7 +4086,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
         <v>170</v>
       </c>
@@ -3898,7 +4106,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" s="6" t="s">
         <v>171</v>
       </c>
@@ -3915,7 +4123,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="7" t="s">
         <v>172</v>
       </c>
@@ -3932,12 +4140,12 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
         <v>174</v>
       </c>
@@ -3948,7 +4156,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
         <v>175</v>
       </c>
@@ -3968,7 +4176,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>176</v>
       </c>
@@ -3979,7 +4187,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
         <v>177</v>
       </c>
@@ -3996,7 +4204,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" s="6" t="s">
         <v>167</v>
       </c>
@@ -4007,7 +4215,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A76" s="6" t="s">
         <v>178</v>
       </c>
@@ -4024,7 +4232,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" s="7" t="s">
         <v>179</v>
       </c>
@@ -4035,7 +4243,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="7" t="s">
         <v>180</v>
       </c>
@@ -4052,7 +4260,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>182</v>
       </c>
@@ -4072,7 +4280,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>184</v>
       </c>
@@ -4083,7 +4291,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>185</v>
       </c>
@@ -4094,7 +4302,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>186</v>
       </c>
@@ -4111,7 +4319,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>187</v>
       </c>
@@ -4131,7 +4339,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>107</v>
       </c>
@@ -4142,7 +4350,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>188</v>
       </c>
@@ -4156,7 +4364,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>189</v>
       </c>
@@ -4173,7 +4381,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>190</v>
       </c>
@@ -4190,7 +4398,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>191</v>
       </c>
@@ -4207,7 +4415,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>192</v>
       </c>
@@ -4221,7 +4429,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>193</v>
       </c>
@@ -4243,12 +4451,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF394502-4A59-4E3D-B4CF-5A5D5E1CBE54}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -4277,12 +4485,12 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="I2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -4293,7 +4501,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>194</v>
       </c>
@@ -4310,7 +4518,7 @@
         <v>28500</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>195</v>
       </c>
@@ -4324,7 +4532,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>196</v>
       </c>
@@ -4338,7 +4546,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>197</v>
       </c>
@@ -4358,7 +4566,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>198</v>
       </c>
@@ -4369,7 +4577,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>199</v>
       </c>
@@ -4386,7 +4594,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>192</v>
       </c>
@@ -4409,17 +4617,716 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD84FEA-D0D3-4F98-B644-3E9C52C4A2B7}">
+  <dimension ref="A1:L51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6328125" customWidth="1"/>
+    <col min="8" max="8" width="14.08984375" customWidth="1"/>
+    <col min="9" max="9" width="18.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="J2" t="s">
+        <v>333</v>
+      </c>
+      <c r="K2" t="s">
+        <v>309</v>
+      </c>
+      <c r="L2" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>298</v>
+      </c>
+      <c r="B6" t="s">
+        <v>332</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>365</v>
+      </c>
+      <c r="B7" t="s">
+        <v>366</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>299</v>
+      </c>
+      <c r="B8" t="s">
+        <v>337</v>
+      </c>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8">
+        <v>9</v>
+      </c>
+      <c r="E8" t="s">
+        <v>30</v>
+      </c>
+      <c r="I8" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>303</v>
+      </c>
+      <c r="B9" t="s">
+        <v>338</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="L9">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>351</v>
+      </c>
+      <c r="B10" t="s">
+        <v>352</v>
+      </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B11" t="s">
+        <v>339</v>
+      </c>
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>30</v>
+      </c>
+      <c r="I11" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>307</v>
+      </c>
+      <c r="B12" t="s">
+        <v>343</v>
+      </c>
+      <c r="E12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>308</v>
+      </c>
+      <c r="B13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13">
+        <v>9</v>
+      </c>
+      <c r="E13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>353</v>
+      </c>
+      <c r="E15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>305</v>
+      </c>
+      <c r="B16" t="s">
+        <v>340</v>
+      </c>
+      <c r="E16" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>354</v>
+      </c>
+      <c r="E17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>306</v>
+      </c>
+      <c r="B18" t="s">
+        <v>341</v>
+      </c>
+      <c r="E18" t="s">
+        <v>30</v>
+      </c>
+      <c r="I18" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>300</v>
+      </c>
+      <c r="B20" t="s">
+        <v>336</v>
+      </c>
+      <c r="C20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20">
+        <v>4</v>
+      </c>
+      <c r="E20" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>355</v>
+      </c>
+      <c r="E21" t="s">
+        <v>331</v>
+      </c>
+      <c r="F21">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>301</v>
+      </c>
+      <c r="B22" t="s">
+        <v>336</v>
+      </c>
+      <c r="C22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22" t="s">
+        <v>30</v>
+      </c>
+      <c r="H22" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>356</v>
+      </c>
+      <c r="E23" t="s">
+        <v>331</v>
+      </c>
+      <c r="F23">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>302</v>
+      </c>
+      <c r="B24" t="s">
+        <v>335</v>
+      </c>
+      <c r="C24" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24" t="s">
+        <v>30</v>
+      </c>
+      <c r="H24" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>330</v>
+      </c>
+      <c r="B26" t="s">
+        <v>322</v>
+      </c>
+      <c r="C26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26">
+        <v>8</v>
+      </c>
+      <c r="E26" t="s">
+        <v>33</v>
+      </c>
+      <c r="G26">
+        <v>120000</v>
+      </c>
+      <c r="H26" t="s">
+        <v>358</v>
+      </c>
+      <c r="I26" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>358</v>
+      </c>
+      <c r="E27" t="s">
+        <v>331</v>
+      </c>
+      <c r="F27">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>309</v>
+      </c>
+      <c r="B28" t="s">
+        <v>323</v>
+      </c>
+      <c r="C28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28">
+        <v>8</v>
+      </c>
+      <c r="E28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>310</v>
+      </c>
+      <c r="B30" t="s">
+        <v>327</v>
+      </c>
+      <c r="C30" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30">
+        <v>8</v>
+      </c>
+      <c r="E30" t="s">
+        <v>33</v>
+      </c>
+      <c r="G30">
+        <v>120000</v>
+      </c>
+      <c r="H30" t="s">
+        <v>359</v>
+      </c>
+      <c r="I30" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>359</v>
+      </c>
+      <c r="E31" t="s">
+        <v>331</v>
+      </c>
+      <c r="F31">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>333</v>
+      </c>
+      <c r="B32" t="s">
+        <v>334</v>
+      </c>
+      <c r="C32" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32">
+        <v>6</v>
+      </c>
+      <c r="E32" t="s">
+        <v>33</v>
+      </c>
+      <c r="G32">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>311</v>
+      </c>
+      <c r="B33" t="s">
+        <v>324</v>
+      </c>
+      <c r="C33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33">
+        <v>6</v>
+      </c>
+      <c r="E33" t="s">
+        <v>33</v>
+      </c>
+      <c r="G33">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>312</v>
+      </c>
+      <c r="B34" t="s">
+        <v>325</v>
+      </c>
+      <c r="C34" t="s">
+        <v>29</v>
+      </c>
+      <c r="D34">
+        <v>6</v>
+      </c>
+      <c r="E34" t="s">
+        <v>33</v>
+      </c>
+      <c r="G34">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>313</v>
+      </c>
+      <c r="B36" t="s">
+        <v>328</v>
+      </c>
+      <c r="C36" t="s">
+        <v>29</v>
+      </c>
+      <c r="D36">
+        <v>8</v>
+      </c>
+      <c r="E36" t="s">
+        <v>33</v>
+      </c>
+      <c r="G36">
+        <v>120000</v>
+      </c>
+      <c r="H36" t="s">
+        <v>360</v>
+      </c>
+      <c r="I36" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>360</v>
+      </c>
+      <c r="E37" t="s">
+        <v>331</v>
+      </c>
+      <c r="F37">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>314</v>
+      </c>
+      <c r="B38" t="s">
+        <v>329</v>
+      </c>
+      <c r="E38" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>316</v>
+      </c>
+      <c r="B41" t="s">
+        <v>344</v>
+      </c>
+      <c r="C41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D41">
+        <v>7</v>
+      </c>
+      <c r="E41" t="s">
+        <v>33</v>
+      </c>
+      <c r="G41">
+        <v>120000</v>
+      </c>
+      <c r="H41" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>349</v>
+      </c>
+      <c r="F42">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>319</v>
+      </c>
+      <c r="B43" t="s">
+        <v>345</v>
+      </c>
+      <c r="C43" t="s">
+        <v>28</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43" t="s">
+        <v>33</v>
+      </c>
+      <c r="G43">
+        <v>120000</v>
+      </c>
+      <c r="H43" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>346</v>
+      </c>
+      <c r="F44">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>317</v>
+      </c>
+      <c r="B45" t="s">
+        <v>344</v>
+      </c>
+      <c r="C45" t="s">
+        <v>29</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45" t="s">
+        <v>33</v>
+      </c>
+      <c r="G45">
+        <v>120000</v>
+      </c>
+      <c r="H45" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>347</v>
+      </c>
+      <c r="F46">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>320</v>
+      </c>
+      <c r="B47" t="s">
+        <v>344</v>
+      </c>
+      <c r="C47" t="s">
+        <v>28</v>
+      </c>
+      <c r="D47">
+        <v>7</v>
+      </c>
+      <c r="E47" t="s">
+        <v>33</v>
+      </c>
+      <c r="G47">
+        <v>110000</v>
+      </c>
+      <c r="H47" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>348</v>
+      </c>
+      <c r="F48">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>318</v>
+      </c>
+      <c r="B50" t="s">
+        <v>350</v>
+      </c>
+      <c r="C50" t="s">
+        <v>28</v>
+      </c>
+      <c r="D50">
+        <v>6</v>
+      </c>
+      <c r="E50" t="s">
+        <v>33</v>
+      </c>
+      <c r="G50">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>315</v>
+      </c>
+      <c r="B51" t="s">
+        <v>326</v>
+      </c>
+      <c r="C51" t="s">
+        <v>28</v>
+      </c>
+      <c r="D51">
+        <v>5</v>
+      </c>
+      <c r="E51" t="s">
+        <v>33</v>
+      </c>
+      <c r="G51">
+        <v>15000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
   <dimension ref="A1:K64"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" customWidth="1"/>
-    <col min="3" max="3" width="6.140625" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7265625" customWidth="1"/>
+    <col min="3" max="3" width="6.1796875" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -4451,7 +5358,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="I2" t="s">
         <v>263</v>
       </c>
@@ -4459,7 +5366,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -4470,7 +5377,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>233</v>
       </c>
@@ -4487,7 +5394,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>236</v>
       </c>
@@ -4504,7 +5411,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>235</v>
       </c>
@@ -4515,7 +5422,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>234</v>
       </c>
@@ -4532,7 +5439,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>237</v>
       </c>
@@ -4549,7 +5456,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>250</v>
       </c>
@@ -4563,7 +5470,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>287</v>
       </c>
@@ -4577,7 +5484,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>238</v>
       </c>
@@ -4594,7 +5501,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>240</v>
       </c>
@@ -4611,7 +5518,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>251</v>
       </c>
@@ -4625,7 +5532,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>288</v>
       </c>
@@ -4639,7 +5546,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>239</v>
       </c>
@@ -4656,7 +5563,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>241</v>
       </c>
@@ -4673,7 +5580,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>269</v>
       </c>
@@ -4693,7 +5600,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>292</v>
       </c>
@@ -4710,7 +5617,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>270</v>
       </c>
@@ -4721,7 +5628,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>271</v>
       </c>
@@ -4741,7 +5648,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>275</v>
       </c>
@@ -4755,7 +5662,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>273</v>
       </c>
@@ -4769,7 +5676,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>279</v>
       </c>
@@ -4780,7 +5687,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>254</v>
       </c>
@@ -4791,7 +5698,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>255</v>
       </c>
@@ -4808,7 +5715,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>252</v>
       </c>
@@ -4825,7 +5732,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>253</v>
       </c>
@@ -4836,7 +5743,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>257</v>
       </c>
@@ -4859,7 +5766,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>277</v>
       </c>
@@ -4873,7 +5780,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>278</v>
       </c>
@@ -4887,7 +5794,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>274</v>
       </c>
@@ -4901,7 +5808,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>272</v>
       </c>
@@ -4915,7 +5822,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>276</v>
       </c>
@@ -4926,7 +5833,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>281</v>
       </c>
@@ -4937,7 +5844,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>264</v>
       </c>
@@ -4948,7 +5855,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>265</v>
       </c>
@@ -4965,7 +5872,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>258</v>
       </c>
@@ -4982,7 +5889,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>259</v>
       </c>
@@ -4999,7 +5906,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>260</v>
       </c>
@@ -5016,7 +5923,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>261</v>
       </c>
@@ -5033,7 +5940,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>242</v>
       </c>
@@ -5056,7 +5963,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>243</v>
       </c>
@@ -5076,7 +5983,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>266</v>
       </c>
@@ -5087,7 +5994,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>244</v>
       </c>
@@ -5107,7 +6014,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>267</v>
       </c>
@@ -5118,7 +6025,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>245</v>
       </c>
@@ -5138,7 +6045,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>246</v>
       </c>
@@ -5155,7 +6062,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>295</v>
       </c>
@@ -5166,7 +6073,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>294</v>
       </c>
@@ -5186,7 +6093,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>283</v>
       </c>
@@ -5206,7 +6113,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>247</v>
       </c>
@@ -5217,7 +6124,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>249</v>
       </c>
@@ -5228,7 +6135,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>248</v>
       </c>
@@ -5245,7 +6152,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>268</v>
       </c>
@@ -5265,7 +6172,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>290</v>
       </c>

</xml_diff>

<commit_message>
Expand Bard songs, burst and damage priorities
Add song cycling, raid buffs, Pitch Perfect, gauge spending and DoT refresh decisions.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9D947FF-FAC2-4D38-B744-A9C9483E5A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9056D4-4722-4B5E-B538-898991132CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14160" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="370">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -966,18 +966,12 @@
     <t>Pitch Perfect</t>
   </si>
   <si>
-    <t>Mage’s Ballad</t>
-  </si>
-  <si>
     <t>Heartbreak Shot</t>
   </si>
   <si>
     <t>Rain of Death</t>
   </si>
   <si>
-    <t>Army’s Paeon</t>
-  </si>
-  <si>
     <t>Enhanced Army’s Paeon</t>
   </si>
   <si>
@@ -1026,9 +1020,6 @@
     <t>buff</t>
   </si>
   <si>
-    <t>The Wanderer's Minuet</t>
-  </si>
-  <si>
     <t>Custom Buff</t>
   </si>
   <si>
@@ -1135,6 +1126,24 @@
   </si>
   <si>
     <t>Ref Arrow ready</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>na</t>
+  </si>
+  <si>
+    <t>the Wanderer's Minuet</t>
+  </si>
+  <si>
+    <t>Mage's Ballad</t>
+  </si>
+  <si>
+    <t>Army's Paeon</t>
   </si>
 </sst>
 </file>
@@ -4618,700 +4627,805 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD84FEA-D0D3-4F98-B644-3E9C52C4A2B7}">
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6328125" customWidth="1"/>
-    <col min="8" max="8" width="14.08984375" customWidth="1"/>
-    <col min="9" max="9" width="18.6328125" customWidth="1"/>
+    <col min="3" max="3" width="8.36328125" customWidth="1"/>
+    <col min="6" max="6" width="13.6328125" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.08984375" customWidth="1"/>
+    <col min="10" max="10" width="18.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="J2" t="s">
-        <v>333</v>
-      </c>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="K2" t="s">
         <v>309</v>
       </c>
       <c r="L2" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+      <c r="M2" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>31</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>2450</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>298</v>
       </c>
       <c r="B6" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="C6" t="s">
+        <v>365</v>
+      </c>
+      <c r="D6" t="s">
         <v>27</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>5</v>
       </c>
-      <c r="E6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="F6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B7" t="s">
+        <v>363</v>
+      </c>
+      <c r="C7" t="s">
         <v>365</v>
       </c>
-      <c r="B7" t="s">
-        <v>366</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>32</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>30000</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>299</v>
       </c>
       <c r="B8" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="C8" t="s">
+        <v>365</v>
+      </c>
+      <c r="D8" t="s">
         <v>27</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>9</v>
       </c>
-      <c r="E8" t="s">
-        <v>30</v>
-      </c>
-      <c r="I8" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J8" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>303</v>
       </c>
       <c r="B9" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C9" t="s">
+        <v>365</v>
+      </c>
+      <c r="D9" t="s">
         <v>27</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>12</v>
       </c>
-      <c r="E9" t="s">
-        <v>30</v>
-      </c>
-      <c r="L9">
+      <c r="F9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M9">
         <v>-100</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B10" t="s">
-        <v>352</v>
-      </c>
-      <c r="E10" t="s">
+        <v>349</v>
+      </c>
+      <c r="C10" t="s">
+        <v>365</v>
+      </c>
+      <c r="F10" t="s">
         <v>32</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>304</v>
       </c>
       <c r="B11" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C11" t="s">
+        <v>365</v>
+      </c>
+      <c r="D11" t="s">
         <v>27</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>12</v>
       </c>
-      <c r="E11" t="s">
-        <v>30</v>
-      </c>
-      <c r="I11" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="F11" t="s">
+        <v>30</v>
+      </c>
+      <c r="J11" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>307</v>
       </c>
       <c r="B12" t="s">
-        <v>343</v>
-      </c>
-      <c r="E12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+        <v>340</v>
+      </c>
+      <c r="C12" t="s">
+        <v>366</v>
+      </c>
+      <c r="F12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>308</v>
       </c>
       <c r="B13" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C13" t="s">
+        <v>366</v>
+      </c>
+      <c r="D13" t="s">
         <v>29</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>9</v>
       </c>
-      <c r="E13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="F13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>353</v>
-      </c>
-      <c r="E15" t="s">
+        <v>350</v>
+      </c>
+      <c r="F15" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>305</v>
       </c>
       <c r="B16" t="s">
-        <v>340</v>
-      </c>
-      <c r="E16" t="s">
-        <v>30</v>
-      </c>
-      <c r="I16" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+        <v>337</v>
+      </c>
+      <c r="F16" t="s">
+        <v>30</v>
+      </c>
+      <c r="J16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>354</v>
-      </c>
-      <c r="E17" t="s">
+        <v>351</v>
+      </c>
+      <c r="F17" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>306</v>
       </c>
       <c r="B18" t="s">
-        <v>341</v>
-      </c>
-      <c r="E18" t="s">
-        <v>30</v>
-      </c>
-      <c r="I18" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+        <v>338</v>
+      </c>
+      <c r="F18" t="s">
+        <v>30</v>
+      </c>
+      <c r="J18" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>300</v>
       </c>
       <c r="B20" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C20" t="s">
+        <v>365</v>
+      </c>
+      <c r="D20" t="s">
         <v>28</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>4</v>
       </c>
-      <c r="E20" t="s">
-        <v>30</v>
-      </c>
-      <c r="H20" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="F20" t="s">
+        <v>30</v>
+      </c>
+      <c r="I20" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>355</v>
-      </c>
-      <c r="E21" t="s">
-        <v>331</v>
-      </c>
-      <c r="F21">
+        <v>352</v>
+      </c>
+      <c r="C21" t="s">
+        <v>365</v>
+      </c>
+      <c r="F21" t="s">
+        <v>328</v>
+      </c>
+      <c r="G21">
         <v>45000</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>301</v>
       </c>
       <c r="B22" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C22" t="s">
+        <v>365</v>
+      </c>
+      <c r="D22" t="s">
         <v>27</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>4</v>
       </c>
-      <c r="E22" t="s">
-        <v>30</v>
-      </c>
-      <c r="H22" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="F22" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>356</v>
-      </c>
-      <c r="E23" t="s">
-        <v>331</v>
-      </c>
-      <c r="F23">
+        <v>353</v>
+      </c>
+      <c r="C23" t="s">
+        <v>365</v>
+      </c>
+      <c r="F23" t="s">
+        <v>328</v>
+      </c>
+      <c r="G23">
         <v>45000</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>302</v>
       </c>
       <c r="B24" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C24" t="s">
+        <v>365</v>
+      </c>
+      <c r="D24" t="s">
         <v>29</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>4</v>
       </c>
-      <c r="E24" t="s">
-        <v>30</v>
-      </c>
-      <c r="H24" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="F24" t="s">
+        <v>30</v>
+      </c>
+      <c r="I24" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>330</v>
+        <v>367</v>
       </c>
       <c r="B26" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C26" t="s">
+        <v>365</v>
+      </c>
+      <c r="D26" t="s">
         <v>27</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>8</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>33</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>120000</v>
       </c>
-      <c r="H26" t="s">
-        <v>358</v>
-      </c>
       <c r="I26" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+        <v>355</v>
+      </c>
+      <c r="J26" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>358</v>
-      </c>
-      <c r="E27" t="s">
-        <v>331</v>
-      </c>
-      <c r="F27">
+        <v>355</v>
+      </c>
+      <c r="C27" t="s">
+        <v>365</v>
+      </c>
+      <c r="F27" t="s">
+        <v>328</v>
+      </c>
+      <c r="G27">
         <v>45000</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>309</v>
       </c>
       <c r="B28" t="s">
+        <v>321</v>
+      </c>
+      <c r="D28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>368</v>
+      </c>
+      <c r="B30" t="s">
+        <v>325</v>
+      </c>
+      <c r="C30" t="s">
+        <v>365</v>
+      </c>
+      <c r="D30" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30">
+        <v>8</v>
+      </c>
+      <c r="F30" t="s">
+        <v>33</v>
+      </c>
+      <c r="H30">
+        <v>120000</v>
+      </c>
+      <c r="I30" t="s">
+        <v>356</v>
+      </c>
+      <c r="J30" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>356</v>
+      </c>
+      <c r="C31" t="s">
+        <v>365</v>
+      </c>
+      <c r="F31" t="s">
+        <v>328</v>
+      </c>
+      <c r="G31">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>330</v>
+      </c>
+      <c r="B32" t="s">
+        <v>331</v>
+      </c>
+      <c r="C32" t="s">
+        <v>365</v>
+      </c>
+      <c r="D32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E32">
+        <v>6</v>
+      </c>
+      <c r="F32" t="s">
+        <v>33</v>
+      </c>
+      <c r="H32">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>310</v>
+      </c>
+      <c r="B33" t="s">
+        <v>322</v>
+      </c>
+      <c r="C33" t="s">
+        <v>365</v>
+      </c>
+      <c r="D33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E33">
+        <v>6</v>
+      </c>
+      <c r="F33" t="s">
+        <v>33</v>
+      </c>
+      <c r="H33">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>311</v>
+      </c>
+      <c r="B34" t="s">
         <v>323</v>
       </c>
-      <c r="C28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28">
+      <c r="C34" t="s">
+        <v>366</v>
+      </c>
+      <c r="D34" t="s">
+        <v>29</v>
+      </c>
+      <c r="E34">
+        <v>6</v>
+      </c>
+      <c r="F34" t="s">
+        <v>33</v>
+      </c>
+      <c r="H34">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>369</v>
+      </c>
+      <c r="B36" t="s">
+        <v>326</v>
+      </c>
+      <c r="C36" t="s">
+        <v>365</v>
+      </c>
+      <c r="D36" t="s">
+        <v>29</v>
+      </c>
+      <c r="E36">
         <v>8</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F36" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>310</v>
-      </c>
-      <c r="B30" t="s">
+      <c r="H36">
+        <v>120000</v>
+      </c>
+      <c r="I36" t="s">
+        <v>357</v>
+      </c>
+      <c r="J36" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>357</v>
+      </c>
+      <c r="C37" t="s">
+        <v>365</v>
+      </c>
+      <c r="F37" t="s">
+        <v>328</v>
+      </c>
+      <c r="G37">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>312</v>
+      </c>
+      <c r="B38" t="s">
         <v>327</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C38" t="s">
+        <v>366</v>
+      </c>
+      <c r="F38" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>314</v>
+      </c>
+      <c r="B41" t="s">
+        <v>341</v>
+      </c>
+      <c r="C41" t="s">
+        <v>365</v>
+      </c>
+      <c r="D41" t="s">
+        <v>29</v>
+      </c>
+      <c r="E41">
+        <v>7</v>
+      </c>
+      <c r="F41" t="s">
+        <v>33</v>
+      </c>
+      <c r="H41">
+        <v>120000</v>
+      </c>
+      <c r="I41" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>346</v>
+      </c>
+      <c r="C42" t="s">
+        <v>365</v>
+      </c>
+      <c r="G42">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>317</v>
+      </c>
+      <c r="B43" t="s">
+        <v>342</v>
+      </c>
+      <c r="C43" t="s">
+        <v>365</v>
+      </c>
+      <c r="D43" t="s">
         <v>28</v>
       </c>
-      <c r="D30">
-        <v>8</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="E43">
+        <v>2</v>
+      </c>
+      <c r="F43" t="s">
         <v>33</v>
       </c>
-      <c r="G30">
+      <c r="H43">
         <v>120000</v>
       </c>
-      <c r="H30" t="s">
-        <v>359</v>
-      </c>
-      <c r="I30" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>359</v>
-      </c>
-      <c r="E31" t="s">
-        <v>331</v>
-      </c>
-      <c r="F31">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>333</v>
-      </c>
-      <c r="B32" t="s">
-        <v>334</v>
-      </c>
-      <c r="C32" t="s">
-        <v>27</v>
-      </c>
-      <c r="D32">
+      <c r="I43" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>343</v>
+      </c>
+      <c r="C44" t="s">
+        <v>365</v>
+      </c>
+      <c r="G44">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>315</v>
+      </c>
+      <c r="B45" t="s">
+        <v>341</v>
+      </c>
+      <c r="C45" t="s">
+        <v>365</v>
+      </c>
+      <c r="D45" t="s">
+        <v>29</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45" t="s">
+        <v>33</v>
+      </c>
+      <c r="H45">
+        <v>120000</v>
+      </c>
+      <c r="I45" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>344</v>
+      </c>
+      <c r="C46" t="s">
+        <v>365</v>
+      </c>
+      <c r="G46">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>318</v>
+      </c>
+      <c r="B47" t="s">
+        <v>341</v>
+      </c>
+      <c r="C47" t="s">
+        <v>365</v>
+      </c>
+      <c r="D47" t="s">
+        <v>28</v>
+      </c>
+      <c r="E47">
+        <v>7</v>
+      </c>
+      <c r="F47" t="s">
+        <v>33</v>
+      </c>
+      <c r="H47">
+        <v>110000</v>
+      </c>
+      <c r="I47" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>345</v>
+      </c>
+      <c r="C48" t="s">
+        <v>365</v>
+      </c>
+      <c r="G48">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>316</v>
+      </c>
+      <c r="B50" t="s">
+        <v>347</v>
+      </c>
+      <c r="C50" t="s">
+        <v>365</v>
+      </c>
+      <c r="D50" t="s">
+        <v>28</v>
+      </c>
+      <c r="E50">
         <v>6</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F50" t="s">
         <v>33</v>
       </c>
-      <c r="G32">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>311</v>
-      </c>
-      <c r="B33" t="s">
+      <c r="H50">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>313</v>
+      </c>
+      <c r="B51" t="s">
         <v>324</v>
       </c>
-      <c r="C33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D33">
-        <v>6</v>
-      </c>
-      <c r="E33" t="s">
+      <c r="C51" t="s">
+        <v>365</v>
+      </c>
+      <c r="D51" t="s">
+        <v>28</v>
+      </c>
+      <c r="E51">
+        <v>5</v>
+      </c>
+      <c r="F51" t="s">
         <v>33</v>
       </c>
-      <c r="G33">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>312</v>
-      </c>
-      <c r="B34" t="s">
-        <v>325</v>
-      </c>
-      <c r="C34" t="s">
-        <v>29</v>
-      </c>
-      <c r="D34">
-        <v>6</v>
-      </c>
-      <c r="E34" t="s">
-        <v>33</v>
-      </c>
-      <c r="G34">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>313</v>
-      </c>
-      <c r="B36" t="s">
-        <v>328</v>
-      </c>
-      <c r="C36" t="s">
-        <v>29</v>
-      </c>
-      <c r="D36">
-        <v>8</v>
-      </c>
-      <c r="E36" t="s">
-        <v>33</v>
-      </c>
-      <c r="G36">
-        <v>120000</v>
-      </c>
-      <c r="H36" t="s">
-        <v>360</v>
-      </c>
-      <c r="I36" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>360</v>
-      </c>
-      <c r="E37" t="s">
-        <v>331</v>
-      </c>
-      <c r="F37">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>314</v>
-      </c>
-      <c r="B38" t="s">
-        <v>329</v>
-      </c>
-      <c r="E38" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>316</v>
-      </c>
-      <c r="B41" t="s">
-        <v>344</v>
-      </c>
-      <c r="C41" t="s">
-        <v>29</v>
-      </c>
-      <c r="D41">
-        <v>7</v>
-      </c>
-      <c r="E41" t="s">
-        <v>33</v>
-      </c>
-      <c r="G41">
-        <v>120000</v>
-      </c>
-      <c r="H41" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>349</v>
-      </c>
-      <c r="F42">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>319</v>
-      </c>
-      <c r="B43" t="s">
-        <v>345</v>
-      </c>
-      <c r="C43" t="s">
-        <v>28</v>
-      </c>
-      <c r="D43">
-        <v>2</v>
-      </c>
-      <c r="E43" t="s">
-        <v>33</v>
-      </c>
-      <c r="G43">
-        <v>120000</v>
-      </c>
-      <c r="H43" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>346</v>
-      </c>
-      <c r="F44">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>317</v>
-      </c>
-      <c r="B45" t="s">
-        <v>344</v>
-      </c>
-      <c r="C45" t="s">
-        <v>29</v>
-      </c>
-      <c r="D45">
-        <v>2</v>
-      </c>
-      <c r="E45" t="s">
-        <v>33</v>
-      </c>
-      <c r="G45">
-        <v>120000</v>
-      </c>
-      <c r="H45" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>347</v>
-      </c>
-      <c r="F46">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>320</v>
-      </c>
-      <c r="B47" t="s">
-        <v>344</v>
-      </c>
-      <c r="C47" t="s">
-        <v>28</v>
-      </c>
-      <c r="D47">
-        <v>7</v>
-      </c>
-      <c r="E47" t="s">
-        <v>33</v>
-      </c>
-      <c r="G47">
-        <v>110000</v>
-      </c>
-      <c r="H47" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>348</v>
-      </c>
-      <c r="F48">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>318</v>
-      </c>
-      <c r="B50" t="s">
-        <v>350</v>
-      </c>
-      <c r="C50" t="s">
-        <v>28</v>
-      </c>
-      <c r="D50">
-        <v>6</v>
-      </c>
-      <c r="E50" t="s">
-        <v>33</v>
-      </c>
-      <c r="G50">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>315</v>
-      </c>
-      <c r="B51" t="s">
-        <v>326</v>
-      </c>
-      <c r="C51" t="s">
-        <v>28</v>
-      </c>
-      <c r="D51">
-        <v>5</v>
-      </c>
-      <c r="E51" t="s">
-        <v>33</v>
-      </c>
-      <c r="G51">
+      <c r="H51">
         <v>15000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Adjust Double Down cost and add a joystick hotkey
Require one cartridge for Double Down and add Joy3 input to the standalone AHK script.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9056D4-4722-4B5E-B538-898991132CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79742670-E61E-4890-817F-D020D6BA8A16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14160" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14160" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -2282,7 +2282,7 @@
         <v>88</v>
       </c>
       <c r="I11">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update Gunbreaker and Scholar for patch 7.2
Refine Gunbreaker priorities, read Scholar Aetherflow from the gauge and add future-GCD availability checks.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79742670-E61E-4890-817F-D020D6BA8A16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{806DA1EC-306D-4EF9-85C0-54BD07F8E160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14160" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="375">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -630,9 +630,6 @@
     <t>Chain Stratagem</t>
   </si>
   <si>
-    <t>Impact imminent</t>
-  </si>
-  <si>
     <t>Baneful Impaction</t>
   </si>
   <si>
@@ -1144,6 +1141,24 @@
   </si>
   <si>
     <t>Army's Paeon</t>
+  </si>
+  <si>
+    <t>Impact Imminent</t>
+  </si>
+  <si>
+    <t>Aetherflow</t>
+  </si>
+  <si>
+    <t>Dissipation</t>
+  </si>
+  <si>
+    <t>Dot</t>
+  </si>
+  <si>
+    <t>Burst</t>
+  </si>
+  <si>
+    <t>Impact Imminent;Burst</t>
   </si>
 </sst>
 </file>
@@ -1513,19 +1528,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -1551,7 +1566,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -1562,7 +1577,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1582,7 +1597,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1593,7 +1608,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1616,7 +1631,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1627,7 +1642,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1647,7 +1662,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>41</v>
       </c>
@@ -1658,7 +1673,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -1678,7 +1693,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1689,7 +1704,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -1709,7 +1724,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -1720,7 +1735,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -1737,7 +1752,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1748,7 +1763,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -1765,7 +1780,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -1785,7 +1800,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -1796,7 +1811,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -1807,7 +1822,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -1824,7 +1839,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -1844,7 +1859,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1855,7 +1870,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -1875,7 +1890,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -1886,7 +1901,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -1906,7 +1921,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -1917,7 +1932,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>46</v>
       </c>
@@ -1937,7 +1952,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>16</v>
       </c>
@@ -1948,7 +1963,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>17</v>
       </c>
@@ -1968,7 +1983,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -1979,7 +1994,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>19</v>
       </c>
@@ -1996,7 +2011,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>20</v>
       </c>
@@ -2013,7 +2028,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -2030,7 +2045,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>22</v>
       </c>
@@ -2044,7 +2059,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -2058,7 +2073,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>82</v>
       </c>
@@ -2080,16 +2095,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7762502F-9F7A-4AD9-AC88-345A2195334F}">
   <dimension ref="A1:I37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -2115,10 +2130,10 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -2129,7 +2144,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -2149,7 +2164,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -2160,7 +2175,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -2180,7 +2195,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -2191,7 +2206,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>55</v>
       </c>
@@ -2211,7 +2226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>56</v>
       </c>
@@ -2234,7 +2249,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>87</v>
       </c>
@@ -2245,7 +2260,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>57</v>
       </c>
@@ -2262,7 +2277,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -2285,7 +2300,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -2311,7 +2326,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>89</v>
       </c>
@@ -2322,7 +2337,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>60</v>
       </c>
@@ -2342,7 +2357,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>61</v>
       </c>
@@ -2353,7 +2368,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>62</v>
       </c>
@@ -2373,7 +2388,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>92</v>
       </c>
@@ -2384,7 +2399,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>97</v>
       </c>
@@ -2401,7 +2416,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>63</v>
       </c>
@@ -2427,7 +2442,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>64</v>
       </c>
@@ -2438,7 +2453,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>65</v>
       </c>
@@ -2455,7 +2470,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>66</v>
       </c>
@@ -2466,7 +2481,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>67</v>
       </c>
@@ -2486,7 +2501,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>68</v>
       </c>
@@ -2497,7 +2512,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -2514,7 +2529,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -2525,7 +2540,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>71</v>
       </c>
@@ -2545,7 +2560,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>86</v>
       </c>
@@ -2556,7 +2571,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>72</v>
       </c>
@@ -2573,7 +2588,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>73</v>
       </c>
@@ -2590,7 +2605,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>74</v>
       </c>
@@ -2607,7 +2622,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>75</v>
       </c>
@@ -2627,7 +2642,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>76</v>
       </c>
@@ -2647,7 +2662,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>78</v>
       </c>
@@ -2658,7 +2673,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>90</v>
       </c>
@@ -2669,7 +2684,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -2686,7 +2701,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>79</v>
       </c>
@@ -2714,19 +2729,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0983F4B6-DA2C-422A-9A48-B565C13F35E9}">
   <dimension ref="A1:M38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="22.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -2758,10 +2773,10 @@
         <v>103</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2771,16 +2786,16 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -2791,9 +2806,9 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B4" t="s">
         <v>27</v>
@@ -2805,12 +2820,12 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -2819,9 +2834,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
@@ -2833,15 +2848,15 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H6" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -2850,9 +2865,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
@@ -2864,15 +2879,15 @@
         <v>30</v>
       </c>
       <c r="H8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K8">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B10" t="s">
         <v>27</v>
@@ -2887,9 +2902,9 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B11" t="s">
         <v>29</v>
@@ -2904,9 +2919,9 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B13" t="s">
         <v>28</v>
@@ -2921,7 +2936,7 @@
         <v>60000</v>
       </c>
       <c r="G13" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J13">
         <v>3</v>
@@ -2930,12 +2945,12 @@
         <v>180</v>
       </c>
       <c r="M13" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>224</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>225</v>
       </c>
       <c r="D14" t="s">
         <v>31</v>
@@ -2944,9 +2959,9 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B15" t="s">
         <v>27</v>
@@ -2961,9 +2976,9 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B16" t="s">
         <v>27</v>
@@ -2978,9 +2993,9 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B17" t="s">
         <v>27</v>
@@ -2995,9 +3010,9 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B18" t="s">
         <v>27</v>
@@ -3012,9 +3027,9 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B19" t="s">
         <v>29</v>
@@ -3029,9 +3044,9 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B21" t="s">
         <v>29</v>
@@ -3043,9 +3058,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
@@ -3057,9 +3072,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B23" t="s">
         <v>29</v>
@@ -3071,9 +3086,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B25" t="s">
         <v>28</v>
@@ -3088,15 +3103,15 @@
         <v>120000</v>
       </c>
       <c r="G25" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I25">
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D26" t="s">
         <v>32</v>
@@ -3105,9 +3120,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B27" t="s">
         <v>28</v>
@@ -3119,12 +3134,12 @@
         <v>30</v>
       </c>
       <c r="H27" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D28" t="s">
         <v>31</v>
@@ -3133,9 +3148,9 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -3144,9 +3159,9 @@
         <v>24000</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B31" t="s">
         <v>28</v>
@@ -3161,12 +3176,12 @@
         <v>90000</v>
       </c>
       <c r="G31" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D32" t="s">
         <v>31</v>
@@ -3175,9 +3190,9 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B33" t="s">
         <v>28</v>
@@ -3189,12 +3204,12 @@
         <v>33</v>
       </c>
       <c r="H33" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>221</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>222</v>
       </c>
       <c r="B35" t="s">
         <v>27</v>
@@ -3209,15 +3224,15 @@
         <v>1750</v>
       </c>
       <c r="G35" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J35">
         <v>-1</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B36" t="s">
         <v>28</v>
@@ -3235,9 +3250,9 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B37" t="s">
         <v>29</v>
@@ -3252,15 +3267,15 @@
         <v>1750</v>
       </c>
       <c r="G37" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J37">
         <v>-1</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D38" t="s">
         <v>31</v>
@@ -3277,16 +3292,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E11AA6E-3A21-4E4D-BBE2-CBF8D1A645C0}">
   <dimension ref="A1:K92"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -3318,7 +3333,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
         <v>104</v>
       </c>
@@ -3326,7 +3341,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -3337,7 +3352,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>106</v>
       </c>
@@ -3354,7 +3369,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>108</v>
       </c>
@@ -3374,7 +3389,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>110</v>
       </c>
@@ -3388,7 +3403,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>111</v>
       </c>
@@ -3402,7 +3417,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>112</v>
       </c>
@@ -3416,7 +3431,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>113</v>
       </c>
@@ -3433,7 +3448,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>114</v>
       </c>
@@ -3450,7 +3465,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>116</v>
       </c>
@@ -3467,7 +3482,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>117</v>
       </c>
@@ -3484,7 +3499,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>118</v>
       </c>
@@ -3510,7 +3525,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>121</v>
       </c>
@@ -3533,7 +3548,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>122</v>
       </c>
@@ -3553,7 +3568,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>124</v>
       </c>
@@ -3573,7 +3588,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>119</v>
       </c>
@@ -3584,7 +3599,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>125</v>
       </c>
@@ -3601,7 +3616,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>126</v>
       </c>
@@ -3615,7 +3630,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>128</v>
       </c>
@@ -3635,7 +3650,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>131</v>
       </c>
@@ -3655,7 +3670,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>133</v>
       </c>
@@ -3675,7 +3690,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>135</v>
       </c>
@@ -3686,7 +3701,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>136</v>
       </c>
@@ -3697,7 +3712,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>137</v>
       </c>
@@ -3708,7 +3723,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>138</v>
       </c>
@@ -3719,7 +3734,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>139</v>
       </c>
@@ -3736,7 +3751,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>140</v>
       </c>
@@ -3753,7 +3768,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>141</v>
       </c>
@@ -3770,7 +3785,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>142</v>
       </c>
@@ -3781,7 +3796,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>143</v>
       </c>
@@ -3798,7 +3813,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>144</v>
       </c>
@@ -3818,7 +3833,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>146</v>
       </c>
@@ -3835,7 +3850,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>147</v>
       </c>
@@ -3846,7 +3861,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>148</v>
       </c>
@@ -3866,7 +3881,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>149</v>
       </c>
@@ -3877,7 +3892,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>150</v>
       </c>
@@ -3900,7 +3915,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>153</v>
       </c>
@@ -3911,7 +3926,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>154</v>
       </c>
@@ -3922,7 +3937,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>155</v>
       </c>
@@ -3945,7 +3960,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>156</v>
       </c>
@@ -3956,7 +3971,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
         <v>158</v>
       </c>
@@ -3967,7 +3982,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>159</v>
       </c>
@@ -3990,7 +4005,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
         <v>162</v>
       </c>
@@ -4001,7 +4016,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>163</v>
       </c>
@@ -4015,7 +4030,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>164</v>
       </c>
@@ -4038,7 +4053,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>166</v>
       </c>
@@ -4061,7 +4076,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>168</v>
       </c>
@@ -4081,7 +4096,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>169</v>
       </c>
@@ -4095,7 +4110,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>170</v>
       </c>
@@ -4115,7 +4130,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>171</v>
       </c>
@@ -4132,7 +4147,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>172</v>
       </c>
@@ -4149,12 +4164,12 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>174</v>
       </c>
@@ -4165,7 +4180,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>175</v>
       </c>
@@ -4185,7 +4200,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
         <v>176</v>
       </c>
@@ -4196,7 +4211,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
         <v>177</v>
       </c>
@@ -4213,7 +4228,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>167</v>
       </c>
@@ -4224,7 +4239,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>178</v>
       </c>
@@ -4241,7 +4256,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
         <v>179</v>
       </c>
@@ -4252,7 +4267,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
         <v>180</v>
       </c>
@@ -4269,7 +4284,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>182</v>
       </c>
@@ -4289,7 +4304,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>184</v>
       </c>
@@ -4300,7 +4315,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>185</v>
       </c>
@@ -4311,7 +4326,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>186</v>
       </c>
@@ -4328,7 +4343,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>187</v>
       </c>
@@ -4348,7 +4363,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>107</v>
       </c>
@@ -4359,7 +4374,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>188</v>
       </c>
@@ -4373,7 +4388,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>189</v>
       </c>
@@ -4390,7 +4405,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>190</v>
       </c>
@@ -4407,7 +4422,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>191</v>
       </c>
@@ -4424,7 +4439,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>192</v>
       </c>
@@ -4438,7 +4453,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>193</v>
       </c>
@@ -4459,13 +4474,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF394502-4A59-4E3D-B4CF-5A5D5E1CBE54}">
-  <dimension ref="A1:I12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -4494,12 +4510,12 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -4507,10 +4523,10 @@
         <v>31</v>
       </c>
       <c r="E4">
-        <v>2450</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>194</v>
       </c>
@@ -4526,27 +4542,27 @@
       <c r="F6">
         <v>28500</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="G6" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>372</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>195</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>27</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
-      </c>
-      <c r="D7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>196</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
       </c>
       <c r="C8">
         <v>5</v>
@@ -4555,69 +4571,145 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B9" t="s">
         <v>28</v>
       </c>
       <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10">
         <v>2</v>
       </c>
-      <c r="D9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9">
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10">
         <v>120000</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G10" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>373</v>
+      </c>
+      <c r="D11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>369</v>
+      </c>
+      <c r="D12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>198</v>
-      </c>
-      <c r="D10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>199</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="B13" t="s">
         <v>28</v>
       </c>
-      <c r="C11">
+      <c r="C13">
         <v>2</v>
       </c>
-      <c r="D11" t="s">
-        <v>33</v>
-      </c>
-      <c r="H11" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>192</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B14" t="s">
         <v>29</v>
       </c>
-      <c r="C12">
+      <c r="C14">
         <v>3</v>
       </c>
-      <c r="D12" t="s">
-        <v>33</v>
-      </c>
-      <c r="F12">
+      <c r="D14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14">
         <v>60000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>370</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15">
+        <v>6</v>
+      </c>
+      <c r="D15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>371</v>
+      </c>
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17">
+        <v>6</v>
+      </c>
+      <c r="D17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F17">
+        <v>180000</v>
       </c>
     </row>
   </sheetData>
@@ -4628,26 +4720,26 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD84FEA-D0D3-4F98-B644-3E9C52C4A2B7}">
   <dimension ref="A1:M51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.36328125" customWidth="1"/>
-    <col min="6" max="6" width="13.6328125" customWidth="1"/>
-    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.08984375" customWidth="1"/>
-    <col min="10" max="10" width="18.6328125" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>25</v>
@@ -4677,21 +4769,21 @@
         <v>103</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="L2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="M2" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -4702,15 +4794,15 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C6" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D6" t="s">
         <v>27</v>
@@ -4722,15 +4814,15 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>361</v>
+      </c>
+      <c r="B7" t="s">
         <v>362</v>
       </c>
-      <c r="B7" t="s">
-        <v>363</v>
-      </c>
       <c r="C7" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F7" t="s">
         <v>32</v>
@@ -4739,15 +4831,15 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B8" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D8" t="s">
         <v>27</v>
@@ -4759,18 +4851,18 @@
         <v>30</v>
       </c>
       <c r="J8" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C9" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D9" t="s">
         <v>27</v>
@@ -4785,15 +4877,15 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>347</v>
+      </c>
+      <c r="B10" t="s">
         <v>348</v>
       </c>
-      <c r="B10" t="s">
-        <v>349</v>
-      </c>
       <c r="C10" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F10" t="s">
         <v>32</v>
@@ -4802,15 +4894,15 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B11" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C11" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D11" t="s">
         <v>27</v>
@@ -4822,32 +4914,32 @@
         <v>30</v>
       </c>
       <c r="J11" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>306</v>
+      </c>
+      <c r="B12" t="s">
+        <v>339</v>
+      </c>
+      <c r="C12" t="s">
+        <v>365</v>
+      </c>
+      <c r="F12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>307</v>
       </c>
-      <c r="B12" t="s">
-        <v>340</v>
-      </c>
-      <c r="C12" t="s">
-        <v>366</v>
-      </c>
-      <c r="F12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>308</v>
-      </c>
       <c r="B13" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C13" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D13" t="s">
         <v>29</v>
@@ -4859,59 +4951,59 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="F15" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B16" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F16" t="s">
         <v>30</v>
       </c>
       <c r="J16" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>350</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>351</v>
       </c>
       <c r="F17" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B18" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F18" t="s">
         <v>30</v>
       </c>
       <c r="J18" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B20" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C20" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D20" t="s">
         <v>28</v>
@@ -4923,32 +5015,32 @@
         <v>30</v>
       </c>
       <c r="I20" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C21" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F21" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G21">
         <v>45000</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B22" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C22" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D22" t="s">
         <v>27</v>
@@ -4960,32 +5052,32 @@
         <v>30</v>
       </c>
       <c r="I22" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C23" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F23" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G23">
         <v>45000</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B24" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C24" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D24" t="s">
         <v>29</v>
@@ -4997,18 +5089,18 @@
         <v>30</v>
       </c>
       <c r="I24" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B26" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C26" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D26" t="s">
         <v>27</v>
@@ -5023,32 +5115,32 @@
         <v>120000</v>
       </c>
       <c r="I26" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J26" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C27" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F27" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G27">
         <v>45000</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B28" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D28" t="s">
         <v>27</v>
@@ -5060,15 +5152,15 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B30" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C30" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D30" t="s">
         <v>28</v>
@@ -5083,35 +5175,35 @@
         <v>120000</v>
       </c>
       <c r="I30" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J30" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C31" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F31" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G31">
         <v>45000</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>329</v>
+      </c>
+      <c r="B32" t="s">
         <v>330</v>
       </c>
-      <c r="B32" t="s">
-        <v>331</v>
-      </c>
       <c r="C32" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D32" t="s">
         <v>27</v>
@@ -5126,15 +5218,15 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B33" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C33" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D33" t="s">
         <v>27</v>
@@ -5149,15 +5241,15 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B34" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C34" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D34" t="s">
         <v>29</v>
@@ -5172,15 +5264,15 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B36" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C36" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D36" t="s">
         <v>29</v>
@@ -5195,49 +5287,49 @@
         <v>120000</v>
       </c>
       <c r="I36" t="s">
+        <v>356</v>
+      </c>
+      <c r="J36" t="s">
         <v>357</v>
       </c>
-      <c r="J36" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C37" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F37" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G37">
         <v>45000</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B38" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C38" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F38" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B41" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C41" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D41" t="s">
         <v>29</v>
@@ -5252,29 +5344,29 @@
         <v>120000</v>
       </c>
       <c r="I41" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C42" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G42">
         <v>10000</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B43" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C43" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D43" t="s">
         <v>28</v>
@@ -5289,29 +5381,29 @@
         <v>120000</v>
       </c>
       <c r="I43" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C44" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G44">
         <v>20000</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B45" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C45" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D45" t="s">
         <v>29</v>
@@ -5326,29 +5418,29 @@
         <v>120000</v>
       </c>
       <c r="I45" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C46" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G46">
         <v>20000</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B47" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C47" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D47" t="s">
         <v>28</v>
@@ -5363,29 +5455,29 @@
         <v>110000</v>
       </c>
       <c r="I47" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C48" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G48">
         <v>20000</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B50" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C50" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D50" t="s">
         <v>28</v>
@@ -5400,15 +5492,15 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B51" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C51" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D51" t="s">
         <v>28</v>
@@ -5432,15 +5524,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
   <dimension ref="A1:K64"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.7265625" customWidth="1"/>
-    <col min="3" max="3" width="6.1796875" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" customWidth="1"/>
+    <col min="3" max="3" width="6.140625" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -5469,18 +5561,18 @@
         <v>83</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J2" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -5491,9 +5583,9 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
@@ -5505,12 +5597,12 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>235</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>236</v>
       </c>
       <c r="B7" t="s">
         <v>29</v>
@@ -5522,12 +5614,12 @@
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D8" t="s">
         <v>31</v>
@@ -5536,9 +5628,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B9" t="s">
         <v>27</v>
@@ -5550,12 +5642,12 @@
         <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B10" t="s">
         <v>29</v>
@@ -5567,12 +5659,12 @@
         <v>30</v>
       </c>
       <c r="H10" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D11" t="s">
         <v>32</v>
@@ -5581,12 +5673,12 @@
         <v>30000</v>
       </c>
       <c r="K11" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D12" t="s">
         <v>32</v>
@@ -5595,12 +5687,12 @@
         <v>30000</v>
       </c>
       <c r="K12" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B13" t="s">
         <v>27</v>
@@ -5612,12 +5704,12 @@
         <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
@@ -5629,12 +5721,12 @@
         <v>30</v>
       </c>
       <c r="H14" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>250</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>251</v>
       </c>
       <c r="D15" t="s">
         <v>32</v>
@@ -5643,12 +5735,12 @@
         <v>30000</v>
       </c>
       <c r="K15" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D16" t="s">
         <v>32</v>
@@ -5657,12 +5749,12 @@
         <v>30000</v>
       </c>
       <c r="K16" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B17" t="s">
         <v>27</v>
@@ -5674,12 +5766,12 @@
         <v>30</v>
       </c>
       <c r="H17" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B18" t="s">
         <v>29</v>
@@ -5691,12 +5783,12 @@
         <v>30</v>
       </c>
       <c r="H18" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
@@ -5711,12 +5803,12 @@
         <v>30000</v>
       </c>
       <c r="G20" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D21" t="s">
         <v>30</v>
@@ -5725,15 +5817,15 @@
         <v>30000</v>
       </c>
       <c r="G21" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H21" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D22" t="s">
         <v>31</v>
@@ -5742,9 +5834,9 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B23" t="s">
         <v>27</v>
@@ -5753,46 +5845,46 @@
         <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G23" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G24" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H24" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D25" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G25" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H25" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D26" t="s">
         <v>31</v>
@@ -5801,9 +5893,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D27" t="s">
         <v>32</v>
@@ -5812,9 +5904,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B28" t="s">
         <v>29</v>
@@ -5826,12 +5918,12 @@
         <v>30</v>
       </c>
       <c r="H28" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B30" t="s">
         <v>28</v>
@@ -5843,12 +5935,12 @@
         <v>30</v>
       </c>
       <c r="G30" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D31" t="s">
         <v>31</v>
@@ -5857,9 +5949,9 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B32" t="s">
         <v>28</v>
@@ -5868,77 +5960,77 @@
         <v>9</v>
       </c>
       <c r="D32" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G32" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H32" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="K32" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>276</v>
+      </c>
+      <c r="D33" t="s">
+        <v>261</v>
+      </c>
+      <c r="G33" t="s">
+        <v>295</v>
+      </c>
+      <c r="H33" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>277</v>
       </c>
-      <c r="D33" t="s">
-        <v>262</v>
-      </c>
-      <c r="G33" t="s">
-        <v>296</v>
-      </c>
-      <c r="H33" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>278</v>
-      </c>
       <c r="D34" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G34" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H34" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D35" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G35" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H35" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G36" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H36" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D37" t="s">
         <v>31</v>
@@ -5947,9 +6039,9 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D38" t="s">
         <v>31</v>
@@ -5958,9 +6050,9 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D39" t="s">
         <v>32</v>
@@ -5969,9 +6061,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B40" t="s">
         <v>28</v>
@@ -5983,12 +6075,12 @@
         <v>30</v>
       </c>
       <c r="H40" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B41" t="s">
         <v>27</v>
@@ -5997,15 +6089,15 @@
         <v>4</v>
       </c>
       <c r="D41" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F41">
         <v>1000</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B42" t="s">
         <v>27</v>
@@ -6014,15 +6106,15 @@
         <v>5</v>
       </c>
       <c r="D42" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F42">
         <v>1000</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B43" t="s">
         <v>27</v>
@@ -6031,15 +6123,15 @@
         <v>7</v>
       </c>
       <c r="D43" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F43">
         <v>1000</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B44" t="s">
         <v>27</v>
@@ -6048,15 +6140,15 @@
         <v>8</v>
       </c>
       <c r="D44" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F44">
         <v>1000</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B47" t="s">
         <v>27</v>
@@ -6077,9 +6169,9 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B48" t="s">
         <v>29</v>
@@ -6097,9 +6189,9 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D49" t="s">
         <v>32</v>
@@ -6108,9 +6200,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B50" t="s">
         <v>28</v>
@@ -6125,12 +6217,12 @@
         <v>1000</v>
       </c>
       <c r="H50" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>266</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>267</v>
       </c>
       <c r="D51" t="s">
         <v>32</v>
@@ -6139,9 +6231,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B52" t="s">
         <v>28</v>
@@ -6156,12 +6248,12 @@
         <v>1000</v>
       </c>
       <c r="H52" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B54" t="s">
         <v>28</v>
@@ -6176,9 +6268,9 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D55" t="s">
         <v>32</v>
@@ -6187,9 +6279,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B56" t="s">
         <v>28</v>
@@ -6201,15 +6293,15 @@
         <v>30</v>
       </c>
       <c r="H56" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J56">
         <v>-50</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B58" t="s">
         <v>28</v>
@@ -6224,12 +6316,12 @@
         <v>120000</v>
       </c>
       <c r="G58" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D59" t="s">
         <v>31</v>
@@ -6238,9 +6330,9 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D60" t="s">
         <v>32</v>
@@ -6249,9 +6341,9 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B61" t="s">
         <v>28</v>
@@ -6263,12 +6355,12 @@
         <v>30</v>
       </c>
       <c r="H61" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B63" t="s">
         <v>27</v>
@@ -6283,12 +6375,12 @@
         <v>60000</v>
       </c>
       <c r="G63" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D64" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Prepare AoE rotation support and count weaves
Add an AoE parameter to job rotations and track oGCD usage between GCDs.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{806DA1EC-306D-4EF9-85C0-54BD07F8E160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5818F66-DA9C-4304-BA16-7DB9C4327EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4380" yWindow="4380" windowWidth="28800" windowHeight="15375" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -4523,7 +4523,7 @@
         <v>31</v>
       </c>
       <c r="E4">
-        <v>2400</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -4677,6 +4677,9 @@
       <c r="F15">
         <v>60000</v>
       </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -4695,7 +4698,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>371</v>
       </c>
@@ -4710,6 +4713,9 @@
       </c>
       <c r="F17">
         <v>180000</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand AoE rotations and decode the Summoner gauge
Add Dancer and Paladin AoE choices and Summoner gauge diagnostics. Attunement handling remains in progress.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5818F66-DA9C-4304-BA16-7DB9C4327EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C237964-E20C-439D-9042-DA1A8B2EDFEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4380" yWindow="4380" windowWidth="28800" windowHeight="15375" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="385">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -276,12 +276,6 @@
     <t>Fated Circle</t>
   </si>
   <si>
-    <t>Royal Authority Ready;Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready</t>
-  </si>
-  <si>
-    <t>Riot Blade Ready;Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready</t>
-  </si>
-  <si>
     <t>Shield Bash</t>
   </si>
   <si>
@@ -1159,6 +1153,42 @@
   </si>
   <si>
     <t>Impact Imminent;Burst</t>
+  </si>
+  <si>
+    <t>weird temp fix</t>
+  </si>
+  <si>
+    <t>Holy Circle</t>
+  </si>
+  <si>
+    <t>Prominence</t>
+  </si>
+  <si>
+    <t>Prominence Ready</t>
+  </si>
+  <si>
+    <t>Total Eclipse</t>
+  </si>
+  <si>
+    <t>Royal Authority Ready;Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready;Prominence Ready</t>
+  </si>
+  <si>
+    <t>Riot Blade Ready;Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready;Prominence Ready</t>
+  </si>
+  <si>
+    <t>Riot Blade Ready;Royal Authority Ready;Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready</t>
+  </si>
+  <si>
+    <t>Riot Blade Ready;Royal Authority Ready;Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready;Prominence Ready</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>Clemency</t>
+  </si>
+  <si>
+    <t>Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready</t>
   </si>
 </sst>
 </file>
@@ -1182,7 +1212,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1225,6 +1255,30 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1238,7 +1292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1247,6 +1301,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1527,7 +1587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -1578,7 +1638,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B3" t="s">
@@ -1594,11 +1654,11 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>80</v>
+        <v>378</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="8" t="s">
         <v>1</v>
       </c>
       <c r="D4" t="s">
@@ -1609,7 +1669,7 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="8" t="s">
         <v>43</v>
       </c>
       <c r="B5" t="s">
@@ -1625,14 +1685,14 @@
         <v>2</v>
       </c>
       <c r="H5" t="s">
-        <v>81</v>
+        <v>379</v>
       </c>
       <c r="I5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="8" t="s">
         <v>2</v>
       </c>
       <c r="D6" t="s">
@@ -1643,7 +1703,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
@@ -1659,11 +1719,11 @@
         <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>80</v>
+        <v>378</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="8" t="s">
         <v>41</v>
       </c>
       <c r="D8" t="s">
@@ -1674,7 +1734,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="8" t="s">
         <v>40</v>
       </c>
       <c r="B9" t="s">
@@ -1694,7 +1754,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D10" t="s">
@@ -1705,7 +1765,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B11" t="s">
@@ -1725,7 +1785,7 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="A12" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D12" t="s">
@@ -1736,7 +1796,7 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B13" t="s">
@@ -1753,101 +1813,110 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="A14" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="H14" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="D15" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15">
+        <v>30000</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" t="s">
         <v>8</v>
       </c>
-      <c r="D14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" t="s">
-        <v>28</v>
-      </c>
-      <c r="C15">
+      <c r="H16" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
         <v>8</v>
-      </c>
-      <c r="D15" t="s">
-        <v>30</v>
-      </c>
-      <c r="H15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16">
-        <v>2</v>
-      </c>
-      <c r="D16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16">
-        <v>60000</v>
-      </c>
-      <c r="G16" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>49</v>
       </c>
       <c r="D17" t="s">
         <v>32</v>
       </c>
       <c r="E17">
-        <v>20000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>11</v>
+      <c r="A18" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18">
+        <v>8</v>
       </c>
       <c r="D18" t="s">
-        <v>32</v>
-      </c>
-      <c r="E18">
-        <v>30000</v>
+        <v>30</v>
+      </c>
+      <c r="H18" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>10</v>
+      <c r="A19" s="5" t="s">
+        <v>374</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C19">
-        <v>2</v>
-      </c>
-      <c r="D19" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="H19" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>12</v>
+      <c r="A20" s="10" t="s">
+        <v>48</v>
       </c>
       <c r="B20" t="s">
         <v>28</v>
       </c>
       <c r="C20">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D20" t="s">
         <v>33</v>
@@ -1856,85 +1925,82 @@
         <v>60000</v>
       </c>
       <c r="G20" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>13</v>
+      <c r="A21" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="D21" t="s">
         <v>32</v>
       </c>
       <c r="E21">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22">
         <v>30000</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22">
-        <v>7</v>
-      </c>
-      <c r="D22" t="s">
-        <v>30</v>
-      </c>
-      <c r="G22" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" t="s">
-        <v>13</v>
-      </c>
-    </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>15</v>
+      <c r="A23" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>31</v>
-      </c>
-      <c r="E23">
-        <v>30000</v>
+        <v>30</v>
+      </c>
+      <c r="H23" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>44</v>
+      <c r="A24" s="10" t="s">
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C24">
         <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>30</v>
+        <v>33</v>
+      </c>
+      <c r="F24">
+        <v>60000</v>
       </c>
       <c r="G24" t="s">
-        <v>45</v>
-      </c>
-      <c r="H24" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>45</v>
+      <c r="A25" s="10" t="s">
+        <v>13</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E25">
         <v>30000</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>46</v>
+      <c r="A26" s="10" t="s">
+        <v>14</v>
       </c>
       <c r="B26" t="s">
         <v>29</v>
@@ -1946,15 +2012,15 @@
         <v>30</v>
       </c>
       <c r="G26" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H26" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>16</v>
+      <c r="A27" s="10" t="s">
+        <v>15</v>
       </c>
       <c r="D27" t="s">
         <v>31</v>
@@ -1964,8 +2030,8 @@
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>17</v>
+      <c r="A28" s="10" t="s">
+        <v>44</v>
       </c>
       <c r="B28" t="s">
         <v>29</v>
@@ -1977,118 +2043,218 @@
         <v>30</v>
       </c>
       <c r="G28" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="H28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>18</v>
+      <c r="A29" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="D29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E29">
         <v>30000</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>19</v>
+      <c r="A30" s="10" t="s">
+        <v>46</v>
       </c>
       <c r="B30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C30">
         <v>7</v>
       </c>
       <c r="D30" t="s">
-        <v>33</v>
+        <v>30</v>
+      </c>
+      <c r="G30" t="s">
+        <v>16</v>
       </c>
       <c r="H30" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E31">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B32" t="s">
+        <v>29</v>
+      </c>
+      <c r="C32">
+        <v>7</v>
+      </c>
+      <c r="D32" t="s">
+        <v>30</v>
+      </c>
+      <c r="G32" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="H32" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" t="s">
+        <v>32</v>
+      </c>
+      <c r="E33">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B34" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34">
+        <v>7</v>
+      </c>
+      <c r="D34" t="s">
+        <v>33</v>
+      </c>
+      <c r="H34" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B35" t="s">
         <v>28</v>
       </c>
-      <c r="C31">
+      <c r="C35">
         <v>4</v>
       </c>
-      <c r="D31" t="s">
-        <v>33</v>
-      </c>
-      <c r="F31">
+      <c r="D35" t="s">
+        <v>33</v>
+      </c>
+      <c r="F35">
         <v>30000</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B36" t="s">
         <v>28</v>
       </c>
-      <c r="C32">
+      <c r="C36">
         <v>5</v>
       </c>
-      <c r="D32" t="s">
-        <v>33</v>
-      </c>
-      <c r="F32">
+      <c r="D36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F36">
         <v>30000</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B37" t="s">
         <v>28</v>
       </c>
-      <c r="C33">
+      <c r="C37">
         <v>1</v>
       </c>
-      <c r="D33" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="D37" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>23</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B38" t="s">
         <v>29</v>
       </c>
-      <c r="C34">
+      <c r="C38">
         <v>4</v>
       </c>
-      <c r="D34" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>82</v>
-      </c>
-      <c r="B35" t="s">
+      <c r="D38" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>80</v>
+      </c>
+      <c r="B39" t="s">
         <v>27</v>
       </c>
-      <c r="C35">
+      <c r="C39">
         <v>3</v>
       </c>
-      <c r="D35" t="s">
-        <v>30</v>
+      <c r="D39" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="12" t="s">
+        <v>382</v>
+      </c>
+      <c r="B40" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40">
+        <v>1</v>
+      </c>
+      <c r="D40" t="s">
+        <v>33</v>
+      </c>
+      <c r="E40">
+        <v>10000</v>
+      </c>
+      <c r="F40">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="13" t="s">
+        <v>383</v>
+      </c>
+      <c r="B41" t="s">
+        <v>27</v>
+      </c>
+      <c r="C41">
+        <v>7</v>
+      </c>
+      <c r="D41" t="s">
+        <v>30</v>
+      </c>
+      <c r="H41" t="s">
+        <v>384</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2130,7 +2296,7 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -2161,7 +2327,7 @@
         <v>52</v>
       </c>
       <c r="H3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -2192,7 +2358,7 @@
         <v>54</v>
       </c>
       <c r="H5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -2220,7 +2386,7 @@
         <v>30</v>
       </c>
       <c r="H7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I7">
         <v>1</v>
@@ -2240,10 +2406,10 @@
         <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I8">
         <v>-1</v>
@@ -2251,7 +2417,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
         <v>32</v>
@@ -2274,7 +2440,7 @@
         <v>33</v>
       </c>
       <c r="H10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -2294,7 +2460,7 @@
         <v>60000</v>
       </c>
       <c r="H11" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I11">
         <v>-1</v>
@@ -2317,10 +2483,10 @@
         <v>120000</v>
       </c>
       <c r="G12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I12">
         <v>3</v>
@@ -2328,7 +2494,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D13" t="s">
         <v>32</v>
@@ -2354,7 +2520,7 @@
         <v>61</v>
       </c>
       <c r="H14" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -2382,15 +2548,15 @@
         <v>30</v>
       </c>
       <c r="G16" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H16" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
         <v>31</v>
@@ -2401,7 +2567,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B18" t="s">
         <v>28</v>
@@ -2413,7 +2579,7 @@
         <v>30</v>
       </c>
       <c r="H18" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -2433,10 +2599,10 @@
         <v>30000</v>
       </c>
       <c r="G19" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H19" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I19">
         <v>-1</v>
@@ -2467,7 +2633,7 @@
         <v>33</v>
       </c>
       <c r="H21" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -2495,10 +2661,10 @@
         <v>30</v>
       </c>
       <c r="G23" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -2526,7 +2692,7 @@
         <v>33</v>
       </c>
       <c r="H25" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -2554,15 +2720,15 @@
         <v>30</v>
       </c>
       <c r="G27" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H27" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D28" t="s">
         <v>32</v>
@@ -2585,7 +2751,7 @@
         <v>33</v>
       </c>
       <c r="H29" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -2636,10 +2802,10 @@
         <v>30</v>
       </c>
       <c r="G32" t="s">
+        <v>84</v>
+      </c>
+      <c r="H32" t="s">
         <v>86</v>
-      </c>
-      <c r="H32" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -2659,7 +2825,7 @@
         <v>60000</v>
       </c>
       <c r="G33" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -2675,7 +2841,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D35" t="s">
         <v>32</v>
@@ -2698,7 +2864,7 @@
         <v>30</v>
       </c>
       <c r="H36" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -2715,7 +2881,7 @@
         <v>30</v>
       </c>
       <c r="H37" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I37">
         <v>-1</v>
@@ -2767,13 +2933,13 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
@@ -2786,13 +2952,13 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2808,7 +2974,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B4" t="s">
         <v>27</v>
@@ -2820,12 +2986,12 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -2836,7 +3002,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
@@ -2848,15 +3014,15 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -2867,7 +3033,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
@@ -2879,7 +3045,7 @@
         <v>30</v>
       </c>
       <c r="H8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K8">
         <v>20</v>
@@ -2887,7 +3053,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B10" t="s">
         <v>27</v>
@@ -2904,7 +3070,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B11" t="s">
         <v>29</v>
@@ -2921,7 +3087,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B13" t="s">
         <v>28</v>
@@ -2936,7 +3102,7 @@
         <v>60000</v>
       </c>
       <c r="G13" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="J13">
         <v>3</v>
@@ -2945,12 +3111,12 @@
         <v>180</v>
       </c>
       <c r="M13" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D14" t="s">
         <v>31</v>
@@ -2961,7 +3127,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B15" t="s">
         <v>27</v>
@@ -2978,7 +3144,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B16" t="s">
         <v>27</v>
@@ -2995,7 +3161,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B17" t="s">
         <v>27</v>
@@ -3012,7 +3178,7 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B18" t="s">
         <v>27</v>
@@ -3029,7 +3195,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B19" t="s">
         <v>29</v>
@@ -3046,7 +3212,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B21" t="s">
         <v>29</v>
@@ -3060,7 +3226,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
@@ -3074,7 +3240,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B23" t="s">
         <v>29</v>
@@ -3088,7 +3254,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B25" t="s">
         <v>28</v>
@@ -3103,7 +3269,7 @@
         <v>120000</v>
       </c>
       <c r="G25" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="I25">
         <v>2</v>
@@ -3111,7 +3277,7 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D26" t="s">
         <v>32</v>
@@ -3122,7 +3288,7 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B27" t="s">
         <v>28</v>
@@ -3134,12 +3300,12 @@
         <v>30</v>
       </c>
       <c r="H27" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D28" t="s">
         <v>31</v>
@@ -3150,7 +3316,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -3161,7 +3327,7 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B31" t="s">
         <v>28</v>
@@ -3176,12 +3342,12 @@
         <v>90000</v>
       </c>
       <c r="G31" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D32" t="s">
         <v>31</v>
@@ -3192,7 +3358,7 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B33" t="s">
         <v>28</v>
@@ -3204,12 +3370,12 @@
         <v>33</v>
       </c>
       <c r="H33" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B35" t="s">
         <v>27</v>
@@ -3224,7 +3390,7 @@
         <v>1750</v>
       </c>
       <c r="G35" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="J35">
         <v>-1</v>
@@ -3232,7 +3398,7 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B36" t="s">
         <v>28</v>
@@ -3252,7 +3418,7 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B37" t="s">
         <v>29</v>
@@ -3267,7 +3433,7 @@
         <v>1750</v>
       </c>
       <c r="G37" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="J37">
         <v>-1</v>
@@ -3275,7 +3441,7 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D38" t="s">
         <v>31</v>
@@ -3291,7 +3457,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E11AA6E-3A21-4E4D-BBE2-CBF8D1A645C0}">
-  <dimension ref="A1:K92"/>
+  <dimension ref="A1:M92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
@@ -3327,18 +3493,18 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -3354,7 +3520,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
@@ -3366,12 +3532,12 @@
         <v>30</v>
       </c>
       <c r="H6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
@@ -3383,15 +3549,15 @@
         <v>30</v>
       </c>
       <c r="H8" t="s">
+        <v>105</v>
+      </c>
+      <c r="K8" t="s">
         <v>107</v>
-      </c>
-      <c r="K8" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B9" t="s">
         <v>27</v>
@@ -3405,7 +3571,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B10" t="s">
         <v>27</v>
@@ -3419,7 +3585,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -3433,7 +3599,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B13" t="s">
         <v>29</v>
@@ -3445,12 +3611,12 @@
         <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
@@ -3462,12 +3628,12 @@
         <v>30</v>
       </c>
       <c r="K14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B15" t="s">
         <v>29</v>
@@ -3479,12 +3645,12 @@
         <v>30</v>
       </c>
       <c r="K15" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
@@ -3496,12 +3662,12 @@
         <v>30</v>
       </c>
       <c r="K16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B18" t="s">
         <v>27</v>
@@ -3516,18 +3682,18 @@
         <v>60000</v>
       </c>
       <c r="G18" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I18">
         <v>2</v>
       </c>
       <c r="K18" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B19" t="s">
         <v>29</v>
@@ -3539,18 +3705,18 @@
         <v>33</v>
       </c>
       <c r="G19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
@@ -3565,12 +3731,12 @@
         <v>-1</v>
       </c>
       <c r="K20" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B21" t="s">
         <v>29</v>
@@ -3585,12 +3751,12 @@
         <v>-1</v>
       </c>
       <c r="K21" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D22" t="s">
         <v>32</v>
@@ -3601,7 +3767,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B23" t="s">
         <v>28</v>
@@ -3613,12 +3779,12 @@
         <v>30</v>
       </c>
       <c r="H23" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D26" t="s">
         <v>31</v>
@@ -3627,12 +3793,12 @@
         <v>60000</v>
       </c>
       <c r="K26" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B28" t="s">
         <v>27</v>
@@ -3644,15 +3810,15 @@
         <v>30</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H28" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B29" t="s">
         <v>27</v>
@@ -3664,15 +3830,15 @@
         <v>30</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H29" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B30" t="s">
         <v>27</v>
@@ -3684,15 +3850,15 @@
         <v>30</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H30" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D32" t="s">
         <v>32</v>
@@ -3703,7 +3869,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D33" t="s">
         <v>32</v>
@@ -3714,7 +3880,7 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D34" t="s">
         <v>32</v>
@@ -3725,7 +3891,7 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D36" t="s">
         <v>31</v>
@@ -3736,7 +3902,7 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B37" t="s">
         <v>28</v>
@@ -3748,12 +3914,12 @@
         <v>33</v>
       </c>
       <c r="H37" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B38" t="s">
         <v>28</v>
@@ -3765,12 +3931,12 @@
         <v>33</v>
       </c>
       <c r="H38" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B39" t="s">
         <v>28</v>
@@ -3782,12 +3948,12 @@
         <v>33</v>
       </c>
       <c r="H39" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D41" t="s">
         <v>31</v>
@@ -3798,7 +3964,7 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B42" t="s">
         <v>28</v>
@@ -3810,12 +3976,12 @@
         <v>33</v>
       </c>
       <c r="H42" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B43" t="s">
         <v>28</v>
@@ -3827,15 +3993,15 @@
         <v>33</v>
       </c>
       <c r="H43" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K43" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B44" t="s">
         <v>28</v>
@@ -3847,12 +4013,12 @@
         <v>33</v>
       </c>
       <c r="H44" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D46" t="s">
         <v>31</v>
@@ -3863,7 +4029,7 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B47" t="s">
         <v>27</v>
@@ -3875,15 +4041,15 @@
         <v>33</v>
       </c>
       <c r="H47" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="K47" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D50" t="s">
         <v>31</v>
@@ -3894,7 +4060,7 @@
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B51" t="s">
         <v>28</v>
@@ -3906,10 +4072,10 @@
         <v>30</v>
       </c>
       <c r="G51" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H51" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="K51">
         <v>2</v>
@@ -3917,7 +4083,7 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D52" t="s">
         <v>31</v>
@@ -3928,7 +4094,7 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D53" t="s">
         <v>31</v>
@@ -3939,7 +4105,7 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B54" t="s">
         <v>27</v>
@@ -3951,10 +4117,10 @@
         <v>30</v>
       </c>
       <c r="G54" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H54" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="K54">
         <v>4</v>
@@ -3962,7 +4128,7 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D55" t="s">
         <v>31</v>
@@ -3973,7 +4139,7 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D56" t="s">
         <v>31</v>
@@ -3984,7 +4150,7 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B57" t="s">
         <v>29</v>
@@ -3996,10 +4162,10 @@
         <v>30</v>
       </c>
       <c r="G57" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H57" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K57">
         <v>4</v>
@@ -4007,7 +4173,7 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D58" t="s">
         <v>31</v>
@@ -4018,7 +4184,7 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B60" t="s">
         <v>27</v>
@@ -4032,7 +4198,7 @@
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B61" t="s">
         <v>27</v>
@@ -4044,18 +4210,18 @@
         <v>30</v>
       </c>
       <c r="H61" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J61">
         <v>-1</v>
       </c>
       <c r="K61" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B62" t="s">
         <v>27</v>
@@ -4067,18 +4233,18 @@
         <v>30</v>
       </c>
       <c r="G62" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="J62">
         <v>-1</v>
       </c>
       <c r="K62" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B63" t="s">
         <v>27</v>
@@ -4093,12 +4259,12 @@
         <v>-1</v>
       </c>
       <c r="K63" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B65" t="s">
         <v>29</v>
@@ -4110,9 +4276,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B66" t="s">
         <v>29</v>
@@ -4124,15 +4290,18 @@
         <v>30</v>
       </c>
       <c r="H66" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J66">
         <v>-1</v>
       </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M66" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B67" t="s">
         <v>29</v>
@@ -4143,13 +4312,19 @@
       <c r="D67" t="s">
         <v>30</v>
       </c>
+      <c r="G67" t="s">
+        <v>165</v>
+      </c>
       <c r="J67">
         <v>-1</v>
       </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M67" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B68" t="s">
         <v>29</v>
@@ -4163,15 +4338,18 @@
       <c r="J68">
         <v>-1</v>
       </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="M68" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D71" t="s">
         <v>31</v>
@@ -4180,9 +4358,9 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B72" t="s">
         <v>28</v>
@@ -4194,15 +4372,15 @@
         <v>30</v>
       </c>
       <c r="G72" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H72" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A73" s="5" t="s">
         <v>174</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A73" s="5" t="s">
-        <v>176</v>
       </c>
       <c r="D73" t="s">
         <v>31</v>
@@ -4211,9 +4389,9 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B74" t="s">
         <v>28</v>
@@ -4225,12 +4403,12 @@
         <v>30</v>
       </c>
       <c r="H74" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D75" t="s">
         <v>31</v>
@@ -4239,9 +4417,9 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B76" t="s">
         <v>28</v>
@@ -4253,12 +4431,12 @@
         <v>33</v>
       </c>
       <c r="H76" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D77" t="s">
         <v>31</v>
@@ -4267,9 +4445,9 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B78" t="s">
         <v>28</v>
@@ -4281,12 +4459,12 @@
         <v>30</v>
       </c>
       <c r="H78" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B80" t="s">
         <v>28</v>
@@ -4301,12 +4479,12 @@
         <v>120000</v>
       </c>
       <c r="G80" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D81" t="s">
         <v>32</v>
@@ -4317,7 +4495,7 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D82" t="s">
         <v>32</v>
@@ -4328,7 +4506,7 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B83" t="s">
         <v>28</v>
@@ -4340,12 +4518,12 @@
         <v>33</v>
       </c>
       <c r="H83" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B85" t="s">
         <v>27</v>
@@ -4360,12 +4538,12 @@
         <v>40000</v>
       </c>
       <c r="G85" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D86" t="s">
         <v>31</v>
@@ -4376,7 +4554,7 @@
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B87" t="s">
         <v>28</v>
@@ -4390,7 +4568,7 @@
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B88" t="s">
         <v>28</v>
@@ -4402,12 +4580,12 @@
         <v>30</v>
       </c>
       <c r="H88" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B89" t="s">
         <v>29</v>
@@ -4419,12 +4597,12 @@
         <v>30</v>
       </c>
       <c r="H89" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B90" t="s">
         <v>28</v>
@@ -4436,12 +4614,12 @@
         <v>30</v>
       </c>
       <c r="H90" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B91" t="s">
         <v>29</v>
@@ -4455,7 +4633,7 @@
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B92" t="s">
         <v>27</v>
@@ -4507,12 +4685,12 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -4528,7 +4706,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
@@ -4543,12 +4721,12 @@
         <v>28500</v>
       </c>
       <c r="G6" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -4559,7 +4737,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
@@ -4573,7 +4751,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B9" t="s">
         <v>28</v>
@@ -4587,7 +4765,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B10" t="s">
         <v>28</v>
@@ -4602,12 +4780,12 @@
         <v>120000</v>
       </c>
       <c r="G10" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D11" t="s">
         <v>31</v>
@@ -4618,7 +4796,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D12" t="s">
         <v>32</v>
@@ -4629,7 +4807,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B13" t="s">
         <v>28</v>
@@ -4641,12 +4819,12 @@
         <v>33</v>
       </c>
       <c r="H13" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
@@ -4663,7 +4841,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B15" t="s">
         <v>27</v>
@@ -4683,7 +4861,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B16" t="s">
         <v>28</v>
@@ -4700,7 +4878,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B17" t="s">
         <v>29</v>
@@ -4742,10 +4920,10 @@
         <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>25</v>
@@ -4769,24 +4947,24 @@
         <v>39</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K2" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="L2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="M2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -4802,13 +4980,13 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B6" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C6" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D6" t="s">
         <v>27</v>
@@ -4822,13 +5000,13 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C7" t="s">
         <v>362</v>
-      </c>
-      <c r="C7" t="s">
-        <v>364</v>
       </c>
       <c r="F7" t="s">
         <v>32</v>
@@ -4839,13 +5017,13 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C8" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D8" t="s">
         <v>27</v>
@@ -4857,18 +5035,18 @@
         <v>30</v>
       </c>
       <c r="J8" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B9" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C9" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D9" t="s">
         <v>27</v>
@@ -4885,13 +5063,13 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B10" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C10" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="F10" t="s">
         <v>32</v>
@@ -4902,13 +5080,13 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B11" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C11" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D11" t="s">
         <v>27</v>
@@ -4920,18 +5098,18 @@
         <v>30</v>
       </c>
       <c r="J11" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B12" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C12" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="F12" t="s">
         <v>30</v>
@@ -4939,13 +5117,13 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B13" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C13" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="D13" t="s">
         <v>29</v>
@@ -4959,7 +5137,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="F15" t="s">
         <v>32</v>
@@ -4967,21 +5145,21 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B16" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="F16" t="s">
         <v>30</v>
       </c>
       <c r="J16" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="F17" t="s">
         <v>32</v>
@@ -4989,27 +5167,27 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B18" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F18" t="s">
         <v>30</v>
       </c>
       <c r="J18" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C20" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D20" t="s">
         <v>28</v>
@@ -5021,18 +5199,18 @@
         <v>30</v>
       </c>
       <c r="I20" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C21" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="F21" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="G21">
         <v>45000</v>
@@ -5040,13 +5218,13 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B22" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C22" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D22" t="s">
         <v>27</v>
@@ -5058,18 +5236,18 @@
         <v>30</v>
       </c>
       <c r="I22" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C23" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="F23" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="G23">
         <v>45000</v>
@@ -5077,13 +5255,13 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B24" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C24" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D24" t="s">
         <v>29</v>
@@ -5095,18 +5273,18 @@
         <v>30</v>
       </c>
       <c r="I24" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B26" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C26" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D26" t="s">
         <v>27</v>
@@ -5121,21 +5299,21 @@
         <v>120000</v>
       </c>
       <c r="I26" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="J26" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C27" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="F27" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="G27">
         <v>45000</v>
@@ -5143,10 +5321,10 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B28" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D28" t="s">
         <v>27</v>
@@ -5160,13 +5338,13 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B30" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C30" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D30" t="s">
         <v>28</v>
@@ -5181,21 +5359,21 @@
         <v>120000</v>
       </c>
       <c r="I30" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="J30" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C31" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="F31" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="G31">
         <v>45000</v>
@@ -5203,13 +5381,13 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B32" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C32" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D32" t="s">
         <v>27</v>
@@ -5226,13 +5404,13 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B33" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C33" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D33" t="s">
         <v>27</v>
@@ -5249,13 +5427,13 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B34" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C34" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="D34" t="s">
         <v>29</v>
@@ -5272,13 +5450,13 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B36" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C36" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D36" t="s">
         <v>29</v>
@@ -5293,21 +5471,21 @@
         <v>120000</v>
       </c>
       <c r="I36" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="J36" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C37" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="F37" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="G37">
         <v>45000</v>
@@ -5315,13 +5493,13 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B38" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C38" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="F38" t="s">
         <v>32</v>
@@ -5329,13 +5507,13 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B41" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C41" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D41" t="s">
         <v>29</v>
@@ -5350,15 +5528,15 @@
         <v>120000</v>
       </c>
       <c r="I41" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C42" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="G42">
         <v>10000</v>
@@ -5366,13 +5544,13 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B43" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C43" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D43" t="s">
         <v>28</v>
@@ -5387,15 +5565,15 @@
         <v>120000</v>
       </c>
       <c r="I43" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C44" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="G44">
         <v>20000</v>
@@ -5403,13 +5581,13 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B45" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C45" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D45" t="s">
         <v>29</v>
@@ -5424,15 +5602,15 @@
         <v>120000</v>
       </c>
       <c r="I45" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C46" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="G46">
         <v>20000</v>
@@ -5440,13 +5618,13 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B47" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C47" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D47" t="s">
         <v>28</v>
@@ -5461,15 +5639,15 @@
         <v>110000</v>
       </c>
       <c r="I47" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C48" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="G48">
         <v>20000</v>
@@ -5477,13 +5655,13 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B50" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C50" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D50" t="s">
         <v>28</v>
@@ -5500,13 +5678,13 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B51" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C51" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D51" t="s">
         <v>28</v>
@@ -5564,18 +5742,18 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="J2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -5591,7 +5769,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
@@ -5603,12 +5781,12 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B7" t="s">
         <v>29</v>
@@ -5620,12 +5798,12 @@
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D8" t="s">
         <v>31</v>
@@ -5636,7 +5814,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B9" t="s">
         <v>27</v>
@@ -5648,12 +5826,12 @@
         <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B10" t="s">
         <v>29</v>
@@ -5665,12 +5843,12 @@
         <v>30</v>
       </c>
       <c r="H10" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D11" t="s">
         <v>32</v>
@@ -5679,12 +5857,12 @@
         <v>30000</v>
       </c>
       <c r="K11" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D12" t="s">
         <v>32</v>
@@ -5693,12 +5871,12 @@
         <v>30000</v>
       </c>
       <c r="K12" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B13" t="s">
         <v>27</v>
@@ -5710,12 +5888,12 @@
         <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
@@ -5727,12 +5905,12 @@
         <v>30</v>
       </c>
       <c r="H14" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D15" t="s">
         <v>32</v>
@@ -5741,12 +5919,12 @@
         <v>30000</v>
       </c>
       <c r="K15" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D16" t="s">
         <v>32</v>
@@ -5755,12 +5933,12 @@
         <v>30000</v>
       </c>
       <c r="K16" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B17" t="s">
         <v>27</v>
@@ -5772,12 +5950,12 @@
         <v>30</v>
       </c>
       <c r="H17" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B18" t="s">
         <v>29</v>
@@ -5789,12 +5967,12 @@
         <v>30</v>
       </c>
       <c r="H18" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
@@ -5809,12 +5987,12 @@
         <v>30000</v>
       </c>
       <c r="G20" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D21" t="s">
         <v>30</v>
@@ -5823,15 +6001,15 @@
         <v>30000</v>
       </c>
       <c r="G21" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="H21" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D22" t="s">
         <v>31</v>
@@ -5842,7 +6020,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B23" t="s">
         <v>27</v>
@@ -5851,46 +6029,46 @@
         <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G23" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H23" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D24" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G24" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H24" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D25" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G25" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H25" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D26" t="s">
         <v>31</v>
@@ -5901,7 +6079,7 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D27" t="s">
         <v>32</v>
@@ -5912,7 +6090,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B28" t="s">
         <v>29</v>
@@ -5924,12 +6102,12 @@
         <v>30</v>
       </c>
       <c r="H28" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B30" t="s">
         <v>28</v>
@@ -5941,12 +6119,12 @@
         <v>30</v>
       </c>
       <c r="G30" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D31" t="s">
         <v>31</v>
@@ -5957,7 +6135,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B32" t="s">
         <v>28</v>
@@ -5966,77 +6144,77 @@
         <v>9</v>
       </c>
       <c r="D32" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G32" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="H32" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="K32" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D33" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G33" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="H33" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D34" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G34" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="H34" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D35" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G35" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="H35" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D36" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G36" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="H36" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D37" t="s">
         <v>31</v>
@@ -6047,7 +6225,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D38" t="s">
         <v>31</v>
@@ -6058,7 +6236,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D39" t="s">
         <v>32</v>
@@ -6069,7 +6247,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B40" t="s">
         <v>28</v>
@@ -6081,12 +6259,12 @@
         <v>30</v>
       </c>
       <c r="H40" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B41" t="s">
         <v>27</v>
@@ -6095,7 +6273,7 @@
         <v>4</v>
       </c>
       <c r="D41" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F41">
         <v>1000</v>
@@ -6103,7 +6281,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B42" t="s">
         <v>27</v>
@@ -6112,7 +6290,7 @@
         <v>5</v>
       </c>
       <c r="D42" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F42">
         <v>1000</v>
@@ -6120,7 +6298,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B43" t="s">
         <v>27</v>
@@ -6129,7 +6307,7 @@
         <v>7</v>
       </c>
       <c r="D43" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F43">
         <v>1000</v>
@@ -6137,7 +6315,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B44" t="s">
         <v>27</v>
@@ -6146,7 +6324,7 @@
         <v>8</v>
       </c>
       <c r="D44" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F44">
         <v>1000</v>
@@ -6154,7 +6332,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B47" t="s">
         <v>27</v>
@@ -6177,7 +6355,7 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B48" t="s">
         <v>29</v>
@@ -6197,7 +6375,7 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D49" t="s">
         <v>32</v>
@@ -6208,7 +6386,7 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B50" t="s">
         <v>28</v>
@@ -6223,12 +6401,12 @@
         <v>1000</v>
       </c>
       <c r="H50" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D51" t="s">
         <v>32</v>
@@ -6239,7 +6417,7 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B52" t="s">
         <v>28</v>
@@ -6254,12 +6432,12 @@
         <v>1000</v>
       </c>
       <c r="H52" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B54" t="s">
         <v>28</v>
@@ -6276,7 +6454,7 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D55" t="s">
         <v>32</v>
@@ -6287,7 +6465,7 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B56" t="s">
         <v>28</v>
@@ -6299,7 +6477,7 @@
         <v>30</v>
       </c>
       <c r="H56" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J56">
         <v>-50</v>
@@ -6307,7 +6485,7 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B58" t="s">
         <v>28</v>
@@ -6322,12 +6500,12 @@
         <v>120000</v>
       </c>
       <c r="G58" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D59" t="s">
         <v>31</v>
@@ -6338,7 +6516,7 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D60" t="s">
         <v>32</v>
@@ -6349,7 +6527,7 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B61" t="s">
         <v>28</v>
@@ -6361,12 +6539,12 @@
         <v>30</v>
       </c>
       <c r="H61" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B63" t="s">
         <v>27</v>
@@ -6381,12 +6559,12 @@
         <v>60000</v>
       </c>
       <c r="G63" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D64" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Enable alternate rotations and refine weaving
Add Scholar instant and AoE choices, Paladin burst suppression and Dancer dance guards and Improvisation handling. Update BRD for weaves
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C237964-E20C-439D-9042-DA1A8B2EDFEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED1FD71C-9092-4FBA-AD74-1E8C6C026904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="390">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1189,6 +1189,21 @@
   </si>
   <si>
     <t>Blade of Faith Ready;Blade of Truth Ready;Blade of Valor Ready</t>
+  </si>
+  <si>
+    <t>Art of War</t>
+  </si>
+  <si>
+    <t>Summon Eos</t>
+  </si>
+  <si>
+    <t>Improvisation</t>
+  </si>
+  <si>
+    <t>Improvised Finish</t>
+  </si>
+  <si>
+    <t>Improvised Dancing</t>
   </si>
 </sst>
 </file>
@@ -1292,7 +1307,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1305,8 +1320,6 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1825,7 +1838,7 @@
       <c r="D14" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="G14" t="s">
         <v>376</v>
       </c>
       <c r="H14" t="s">
@@ -1842,7 +1855,7 @@
       <c r="E15">
         <v>30000</v>
       </c>
-      <c r="H15" s="12" t="s">
+      <c r="H15" t="s">
         <v>376</v>
       </c>
     </row>
@@ -2216,7 +2229,7 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="12" t="s">
+      <c r="A40" t="s">
         <v>382</v>
       </c>
       <c r="B40" t="s">
@@ -2236,7 +2249,7 @@
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="13" t="s">
+      <c r="A41" t="s">
         <v>383</v>
       </c>
       <c r="B41" t="s">
@@ -4652,7 +4665,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF394502-4A59-4E3D-B4CF-5A5D5E1CBE54}">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -4765,89 +4778,86 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>195</v>
+        <v>385</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10">
-        <v>120000</v>
-      </c>
-      <c r="G10" t="s">
-        <v>372</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>371</v>
+        <v>195</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11">
-        <v>20000</v>
+        <v>33</v>
+      </c>
+      <c r="F11">
+        <v>120000</v>
+      </c>
+      <c r="G11" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E12">
-        <v>30000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>196</v>
-      </c>
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13">
-        <v>2</v>
+        <v>367</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" t="s">
-        <v>367</v>
+        <v>32</v>
+      </c>
+      <c r="E13">
+        <v>30000</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" t="s">
         <v>33</v>
       </c>
-      <c r="F14">
-        <v>60000</v>
+      <c r="H14" t="s">
+        <v>367</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>368</v>
+        <v>190</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C15">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D15" t="s">
         <v>33</v>
@@ -4855,16 +4865,13 @@
       <c r="F15">
         <v>60000</v>
       </c>
-      <c r="I15">
-        <v>3</v>
-      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>116</v>
+        <v>368</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C16">
         <v>6</v>
@@ -4873,15 +4880,18 @@
         <v>33</v>
       </c>
       <c r="F16">
-        <v>1000</v>
+        <v>60000</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>369</v>
+        <v>116</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C17">
         <v>6</v>
@@ -4890,10 +4900,41 @@
         <v>33</v>
       </c>
       <c r="F17">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>369</v>
+      </c>
+      <c r="B18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18">
         <v>180000</v>
       </c>
-      <c r="I17">
+      <c r="I18">
         <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>386</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -5707,7 +5748,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -6573,7 +6614,53 @@
         <v>30000</v>
       </c>
     </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>387</v>
+      </c>
+      <c r="B66" t="s">
+        <v>28</v>
+      </c>
+      <c r="C66">
+        <v>11</v>
+      </c>
+      <c r="D66" t="s">
+        <v>33</v>
+      </c>
+      <c r="G66" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>389</v>
+      </c>
+      <c r="D67" t="s">
+        <v>31</v>
+      </c>
+      <c r="E67">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>388</v>
+      </c>
+      <c r="B68" t="s">
+        <v>28</v>
+      </c>
+      <c r="C68">
+        <v>11</v>
+      </c>
+      <c r="D68" t="s">
+        <v>33</v>
+      </c>
+      <c r="H68" t="s">
+        <v>389</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adjust Dancer AoE actions and start Monk spell data
Use Fan Dance II in AoE, remove automatic Improvised Finish and expand the spell workbook.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED1FD71C-9092-4FBA-AD74-1E8C6C026904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09449B43-E920-4419-86CF-8A710B52D6D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="SCH" sheetId="4" r:id="rId5"/>
     <sheet name="BRD" sheetId="7" r:id="rId6"/>
     <sheet name="DNC" sheetId="6" r:id="rId7"/>
+    <sheet name="MNK" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$37</definedName>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="460">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1204,13 +1205,223 @@
   </si>
   <si>
     <t>Improvised Dancing</t>
+  </si>
+  <si>
+    <t>Leaping Opo</t>
+  </si>
+  <si>
+    <t>Dragon Kick</t>
+  </si>
+  <si>
+    <t>Shadow of the Destroyer</t>
+  </si>
+  <si>
+    <t>Rising Raptor</t>
+  </si>
+  <si>
+    <t>Twin Snakes</t>
+  </si>
+  <si>
+    <t>Demolish</t>
+  </si>
+  <si>
+    <t>Four-point Fury</t>
+  </si>
+  <si>
+    <t>Pouncing Coeurl</t>
+  </si>
+  <si>
+    <t>Base Opo</t>
+  </si>
+  <si>
+    <t>Boosted Opo</t>
+  </si>
+  <si>
+    <t>AOE Opo - min 4 targets</t>
+  </si>
+  <si>
+    <t>Rockbreaker</t>
+  </si>
+  <si>
+    <t>Base raprot</t>
+  </si>
+  <si>
+    <t>Boost Raptor</t>
+  </si>
+  <si>
+    <t>AOE Raptor - min 4 targets</t>
+  </si>
+  <si>
+    <t>Base Coeurl - FLANK</t>
+  </si>
+  <si>
+    <t>Botts Coeurl - REAR</t>
+  </si>
+  <si>
+    <t>AOE Coeurl - min 4 targets</t>
+  </si>
+  <si>
+    <t>Enlightened Meditation</t>
+  </si>
+  <si>
+    <t>Enlightenment</t>
+  </si>
+  <si>
+    <t>Out of range filler</t>
+  </si>
+  <si>
+    <t>Chackra spender</t>
+  </si>
+  <si>
+    <t>Besoin de suivre le nombre de chackra</t>
+  </si>
+  <si>
+    <t>Besoin de savoir la forme actuelle</t>
+  </si>
+  <si>
+    <t>Besoin de suivre les boosted buff</t>
+  </si>
+  <si>
+    <t>Six-sided star</t>
+  </si>
+  <si>
+    <t>Disengage tool</t>
+  </si>
+  <si>
+    <t>Manual</t>
+  </si>
+  <si>
+    <t>Perfect Balance</t>
+  </si>
+  <si>
+    <t>Start special sequence</t>
+  </si>
+  <si>
+    <t>Besoin de suivre les sequences - laquelle faire, lesquelles faites, dans laquelle on est …</t>
+  </si>
+  <si>
+    <t>En particulier - il y a une barre pour les 3 forme de la sequence du moment. Voir toutes les possibilités</t>
+  </si>
+  <si>
+    <t>Besoin d'une catégorie "en perfectr balance"</t>
+  </si>
+  <si>
+    <t>Besoin dune categorie "burst &amp;m" et "burst 2m"</t>
+  </si>
+  <si>
+    <t>Riddle of Fire</t>
+  </si>
+  <si>
+    <t>Riddle of Wind</t>
+  </si>
+  <si>
+    <t>Masterful Blitz</t>
+  </si>
+  <si>
+    <t>Form shift</t>
+  </si>
+  <si>
+    <t>Force boost</t>
+  </si>
+  <si>
+    <t>1 m burst 1</t>
+  </si>
+  <si>
+    <t>90s burst 2</t>
+  </si>
+  <si>
+    <t>Brotherhood</t>
+  </si>
+  <si>
+    <t>Fire Buff</t>
+  </si>
+  <si>
+    <t>Wind Buff</t>
+  </si>
+  <si>
+    <t>Brother Buff</t>
+  </si>
+  <si>
+    <t>Wind's Rumination</t>
+  </si>
+  <si>
+    <t>Mantra</t>
+  </si>
+  <si>
+    <t>Riddle of Earth</t>
+  </si>
+  <si>
+    <t>Arm's Length</t>
+  </si>
+  <si>
+    <t>Bloodbath</t>
+  </si>
+  <si>
+    <t>Feint</t>
+  </si>
+  <si>
+    <t>Earth Buff</t>
+  </si>
+  <si>
+    <t>Fire's Rumination</t>
+  </si>
+  <si>
+    <t>Wind's Rumination;Wind Buff</t>
+  </si>
+  <si>
+    <t>Fire's Rumination;Fire Buff</t>
+  </si>
+  <si>
+    <t>Earth's Rumination</t>
+  </si>
+  <si>
+    <t>Formless Shift</t>
+  </si>
+  <si>
+    <t>Leg Sweep</t>
+  </si>
+  <si>
+    <t>Thunderclap</t>
+  </si>
+  <si>
+    <t>True North</t>
+  </si>
+  <si>
+    <t>Need to have a potential over on it</t>
+  </si>
+  <si>
+    <t>Opo-opo Form</t>
+  </si>
+  <si>
+    <t>Raptor Form</t>
+  </si>
+  <si>
+    <t>Coeurl Form</t>
+  </si>
+  <si>
+    <t>Give 2 stacks</t>
+  </si>
+  <si>
+    <t>Give 1 stack</t>
+  </si>
+  <si>
+    <t>Give one stack</t>
+  </si>
+  <si>
+    <t>Formless Shift;Opo-opo Form</t>
+  </si>
+  <si>
+    <t>Formless Shift;Raptor Form</t>
+  </si>
+  <si>
+    <t>SI on a des stack de formeless, ca ne donne pas de forme…</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1221,6 +1432,15 @@
     <font>
       <b/>
       <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1307,7 +1527,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1320,6 +1540,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6663,4 +6884,720 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3261DB23-C434-4F35-8B4F-998D4295A585}">
+  <dimension ref="A1:N55"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3">
+        <v>1950</v>
+      </c>
+      <c r="K3" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>451</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>452</v>
+      </c>
+      <c r="H6" t="s">
+        <v>457</v>
+      </c>
+      <c r="K6" t="s">
+        <v>398</v>
+      </c>
+      <c r="N6" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>391</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" t="s">
+        <v>452</v>
+      </c>
+      <c r="H7" t="s">
+        <v>457</v>
+      </c>
+      <c r="K7" t="s">
+        <v>399</v>
+      </c>
+      <c r="M7" t="s">
+        <v>456</v>
+      </c>
+      <c r="N7" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>392</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>452</v>
+      </c>
+      <c r="H8" t="s">
+        <v>457</v>
+      </c>
+      <c r="K8" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>452</v>
+      </c>
+      <c r="D10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>393</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s">
+        <v>453</v>
+      </c>
+      <c r="H11" t="s">
+        <v>458</v>
+      </c>
+      <c r="K11" t="s">
+        <v>402</v>
+      </c>
+      <c r="N11" s="12" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>394</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" t="s">
+        <v>453</v>
+      </c>
+      <c r="H12" t="s">
+        <v>458</v>
+      </c>
+      <c r="K12" t="s">
+        <v>403</v>
+      </c>
+      <c r="M12" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>396</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13">
+        <v>5</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="G13" t="s">
+        <v>453</v>
+      </c>
+      <c r="H13" t="s">
+        <v>458</v>
+      </c>
+      <c r="K13" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>453</v>
+      </c>
+      <c r="D15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E15">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>397</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" t="s">
+        <v>451</v>
+      </c>
+      <c r="H16" t="s">
+        <v>457</v>
+      </c>
+      <c r="K16" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>395</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17">
+        <v>6</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G17" t="s">
+        <v>451</v>
+      </c>
+      <c r="H17" t="s">
+        <v>457</v>
+      </c>
+      <c r="K17" t="s">
+        <v>406</v>
+      </c>
+      <c r="M17" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>401</v>
+      </c>
+      <c r="B18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="G18" t="s">
+        <v>451</v>
+      </c>
+      <c r="H18" t="s">
+        <v>457</v>
+      </c>
+      <c r="K18" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>415</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20">
+        <v>3</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K20" t="s">
+        <v>416</v>
+      </c>
+      <c r="N20" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>408</v>
+      </c>
+      <c r="B21" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21">
+        <v>7</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+      <c r="K21" t="s">
+        <v>410</v>
+      </c>
+      <c r="N21" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>409</v>
+      </c>
+      <c r="B22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22">
+        <v>7</v>
+      </c>
+      <c r="D22" t="s">
+        <v>30</v>
+      </c>
+      <c r="K22" t="s">
+        <v>411</v>
+      </c>
+      <c r="N22" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N23" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>418</v>
+      </c>
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24">
+        <v>8</v>
+      </c>
+      <c r="K24" t="s">
+        <v>419</v>
+      </c>
+      <c r="N24" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>426</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25">
+        <v>8</v>
+      </c>
+      <c r="N25" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>427</v>
+      </c>
+      <c r="B27" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
+        <v>30</v>
+      </c>
+      <c r="G27" t="s">
+        <v>446</v>
+      </c>
+      <c r="K27" t="s">
+        <v>428</v>
+      </c>
+      <c r="N27" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>446</v>
+      </c>
+      <c r="D28" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N29" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>424</v>
+      </c>
+      <c r="B30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30">
+        <v>9</v>
+      </c>
+      <c r="F30">
+        <v>60000</v>
+      </c>
+      <c r="G30" t="s">
+        <v>444</v>
+      </c>
+      <c r="K30" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>442</v>
+      </c>
+      <c r="B31" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31">
+        <v>9</v>
+      </c>
+      <c r="E31">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>432</v>
+      </c>
+      <c r="E32">
+        <v>20000</v>
+      </c>
+      <c r="K32" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>425</v>
+      </c>
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33">
+        <v>9</v>
+      </c>
+      <c r="F33">
+        <v>90000</v>
+      </c>
+      <c r="G33" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>435</v>
+      </c>
+      <c r="E34">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>433</v>
+      </c>
+      <c r="E35">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>431</v>
+      </c>
+      <c r="B37" t="s">
+        <v>29</v>
+      </c>
+      <c r="C37">
+        <v>9</v>
+      </c>
+      <c r="F37">
+        <v>120000</v>
+      </c>
+      <c r="G37" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>434</v>
+      </c>
+      <c r="E38">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>439</v>
+      </c>
+      <c r="B41" t="s">
+        <v>27</v>
+      </c>
+      <c r="C41">
+        <v>10</v>
+      </c>
+      <c r="F41">
+        <v>90000</v>
+      </c>
+      <c r="M41">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>437</v>
+      </c>
+      <c r="B42" t="s">
+        <v>27</v>
+      </c>
+      <c r="C42">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>445</v>
+      </c>
+      <c r="E43">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>441</v>
+      </c>
+      <c r="E44">
+        <v>15000</v>
+      </c>
+      <c r="F44">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>436</v>
+      </c>
+      <c r="B45" t="s">
+        <v>28</v>
+      </c>
+      <c r="C45">
+        <v>11</v>
+      </c>
+      <c r="F45">
+        <v>90000</v>
+      </c>
+      <c r="M45">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>438</v>
+      </c>
+      <c r="B46" t="s">
+        <v>29</v>
+      </c>
+      <c r="C46">
+        <v>11</v>
+      </c>
+      <c r="F46">
+        <v>120000</v>
+      </c>
+      <c r="M46">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>440</v>
+      </c>
+      <c r="B47" t="s">
+        <v>28</v>
+      </c>
+      <c r="C47">
+        <v>12</v>
+      </c>
+      <c r="F47">
+        <v>90000</v>
+      </c>
+      <c r="M47">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D50" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>382</v>
+      </c>
+      <c r="B52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>448</v>
+      </c>
+      <c r="B53" t="s">
+        <v>28</v>
+      </c>
+      <c r="C53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>449</v>
+      </c>
+      <c r="B54" t="s">
+        <v>27</v>
+      </c>
+      <c r="C54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>447</v>
+      </c>
+      <c r="B55" t="s">
+        <v>28</v>
+      </c>
+      <c r="C55">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Handle overlapping Dancer procs and scaffold Monk
Consume the oldest matching Dancer proc and add the initial Monk rotation file.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09449B43-E920-4419-86CF-8A710B52D6D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A2C309D-80C0-419D-9FBC-F68D77E5DF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8385" yWindow="1635" windowWidth="25605" windowHeight="13935" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -25,17 +25,26 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$37</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1250" uniqueCount="463">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -796,9 +805,6 @@
     <t>Last Dance</t>
   </si>
   <si>
-    <t>To be retrieved</t>
-  </si>
-  <si>
     <t>Technical Finish</t>
   </si>
   <si>
@@ -895,15 +901,9 @@
     <t>Flourishing Flow</t>
   </si>
   <si>
-    <t>Ignord</t>
-  </si>
-  <si>
     <t>Finishing Move Ready</t>
   </si>
   <si>
-    <t>Silken Symmetry;Silken Flow;Threefold Fan Dance;Fourfold Fan Dance;Finishing Move Ready</t>
-  </si>
-  <si>
     <t>Finishing Move</t>
   </si>
   <si>
@@ -1415,6 +1415,24 @@
   </si>
   <si>
     <t>SI on a des stack de formeless, ca ne donne pas de forme…</t>
+  </si>
+  <si>
+    <t>Balance Buff</t>
+  </si>
+  <si>
+    <t>Fixme</t>
+  </si>
+  <si>
+    <t>Silken Symmetry;Flourishing Symmetry</t>
+  </si>
+  <si>
+    <t>Silken Flow;Flourishing Flow</t>
+  </si>
+  <si>
+    <t>FIXME On erase des buffs au lieu d'utiliser les 2</t>
+  </si>
+  <si>
+    <t>Flourishing Symmetry;Flourishing Flow;Threefold Fan Dance;Fourfold Fan Dance;Finishing Move Ready</t>
   </si>
 </sst>
 </file>
@@ -1888,7 +1906,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1919,7 +1937,7 @@
         <v>2</v>
       </c>
       <c r="H5" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="I5" t="s">
         <v>47</v>
@@ -1953,7 +1971,7 @@
         <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -2048,7 +2066,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
@@ -2060,15 +2078,15 @@
         <v>30</v>
       </c>
       <c r="G14" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="H14" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="D15" t="s">
         <v>31</v>
@@ -2077,12 +2095,12 @@
         <v>30000</v>
       </c>
       <c r="H15" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
@@ -2097,7 +2115,7 @@
         <v>8</v>
       </c>
       <c r="H16" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -2130,7 +2148,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B19" t="s">
         <v>29</v>
@@ -2451,7 +2469,7 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B40" t="s">
         <v>27</v>
@@ -2471,7 +2489,7 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="B41" t="s">
         <v>27</v>
@@ -2483,7 +2501,7 @@
         <v>30</v>
       </c>
       <c r="H41" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>
@@ -2530,7 +2548,7 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -4530,7 +4548,7 @@
         <v>-1</v>
       </c>
       <c r="M66" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.25">
@@ -4553,7 +4571,7 @@
         <v>-1</v>
       </c>
       <c r="M67" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.25">
@@ -4573,7 +4591,7 @@
         <v>-1</v>
       </c>
       <c r="M68" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.25">
@@ -4955,12 +4973,12 @@
         <v>28500</v>
       </c>
       <c r="G6" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -4999,7 +5017,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B10" t="s">
         <v>29</v>
@@ -5028,12 +5046,12 @@
         <v>120000</v>
       </c>
       <c r="G11" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D12" t="s">
         <v>31</v>
@@ -5044,7 +5062,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D13" t="s">
         <v>32</v>
@@ -5067,7 +5085,7 @@
         <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -5089,7 +5107,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B16" t="s">
         <v>27</v>
@@ -5126,7 +5144,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B18" t="s">
         <v>29</v>
@@ -5146,7 +5164,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="B19" t="s">
         <v>27</v>
@@ -5182,10 +5200,10 @@
         <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>25</v>
@@ -5220,13 +5238,13 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="L2" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="M2" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -5242,13 +5260,13 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B6" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="C6" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D6" t="s">
         <v>27</v>
@@ -5262,13 +5280,13 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>356</v>
+      </c>
+      <c r="B7" t="s">
+        <v>357</v>
+      </c>
+      <c r="C7" t="s">
         <v>359</v>
-      </c>
-      <c r="B7" t="s">
-        <v>360</v>
-      </c>
-      <c r="C7" t="s">
-        <v>362</v>
       </c>
       <c r="F7" t="s">
         <v>32</v>
@@ -5279,13 +5297,13 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B8" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C8" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D8" t="s">
         <v>27</v>
@@ -5297,18 +5315,18 @@
         <v>30</v>
       </c>
       <c r="J8" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B9" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="C9" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D9" t="s">
         <v>27</v>
@@ -5325,13 +5343,13 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B10" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C10" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F10" t="s">
         <v>32</v>
@@ -5342,13 +5360,13 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="B11" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C11" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D11" t="s">
         <v>27</v>
@@ -5360,18 +5378,18 @@
         <v>30</v>
       </c>
       <c r="J11" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B12" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="C12" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="F12" t="s">
         <v>30</v>
@@ -5379,13 +5397,13 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B13" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C13" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D13" t="s">
         <v>29</v>
@@ -5399,7 +5417,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="F15" t="s">
         <v>32</v>
@@ -5407,21 +5425,21 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B16" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F16" t="s">
         <v>30</v>
       </c>
       <c r="J16" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F17" t="s">
         <v>32</v>
@@ -5429,27 +5447,27 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B18" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="F18" t="s">
         <v>30</v>
       </c>
       <c r="J18" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B20" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C20" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D20" t="s">
         <v>28</v>
@@ -5461,18 +5479,18 @@
         <v>30</v>
       </c>
       <c r="I20" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C21" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F21" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="G21">
         <v>45000</v>
@@ -5480,13 +5498,13 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B22" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C22" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D22" t="s">
         <v>27</v>
@@ -5498,18 +5516,18 @@
         <v>30</v>
       </c>
       <c r="I22" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C23" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F23" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="G23">
         <v>45000</v>
@@ -5517,13 +5535,13 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B24" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="C24" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D24" t="s">
         <v>29</v>
@@ -5535,18 +5553,18 @@
         <v>30</v>
       </c>
       <c r="I24" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B26" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="C26" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D26" t="s">
         <v>27</v>
@@ -5561,21 +5579,21 @@
         <v>120000</v>
       </c>
       <c r="I26" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="J26" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C27" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F27" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="G27">
         <v>45000</v>
@@ -5583,10 +5601,10 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B28" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="D28" t="s">
         <v>27</v>
@@ -5600,13 +5618,13 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B30" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C30" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D30" t="s">
         <v>28</v>
@@ -5621,21 +5639,21 @@
         <v>120000</v>
       </c>
       <c r="I30" t="s">
+        <v>350</v>
+      </c>
+      <c r="J30" t="s">
         <v>353</v>
-      </c>
-      <c r="J30" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C31" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F31" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="G31">
         <v>45000</v>
@@ -5643,13 +5661,13 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B32" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="C32" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D32" t="s">
         <v>27</v>
@@ -5666,13 +5684,13 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B33" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C33" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D33" t="s">
         <v>27</v>
@@ -5689,13 +5707,13 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B34" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C34" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D34" t="s">
         <v>29</v>
@@ -5712,13 +5730,13 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B36" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C36" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D36" t="s">
         <v>29</v>
@@ -5733,21 +5751,21 @@
         <v>120000</v>
       </c>
       <c r="I36" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="J36" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="C37" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F37" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="G37">
         <v>45000</v>
@@ -5755,13 +5773,13 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B38" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C38" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="F38" t="s">
         <v>32</v>
@@ -5769,13 +5787,13 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B41" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C41" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D41" t="s">
         <v>29</v>
@@ -5790,15 +5808,15 @@
         <v>120000</v>
       </c>
       <c r="I41" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C42" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="G42">
         <v>10000</v>
@@ -5806,13 +5824,13 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B43" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C43" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D43" t="s">
         <v>28</v>
@@ -5827,15 +5845,15 @@
         <v>120000</v>
       </c>
       <c r="I43" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="C44" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="G44">
         <v>20000</v>
@@ -5843,13 +5861,13 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B45" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C45" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D45" t="s">
         <v>29</v>
@@ -5864,15 +5882,15 @@
         <v>120000</v>
       </c>
       <c r="I45" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C46" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="G46">
         <v>20000</v>
@@ -5880,13 +5898,13 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="B47" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C47" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D47" t="s">
         <v>28</v>
@@ -5901,15 +5919,15 @@
         <v>110000</v>
       </c>
       <c r="I47" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C48" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="G48">
         <v>20000</v>
@@ -5917,13 +5935,13 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="B50" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="C50" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D50" t="s">
         <v>28</v>
@@ -5940,13 +5958,13 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B51" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="C51" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D51" t="s">
         <v>28</v>
@@ -5969,16 +5987,17 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
-  <dimension ref="A1:K68"/>
+  <dimension ref="A1:P68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.7109375" customWidth="1"/>
     <col min="3" max="3" width="6.140625" customWidth="1"/>
     <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -6010,15 +6029,15 @@
         <v>226</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J2" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -6029,7 +6048,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>230</v>
       </c>
@@ -6046,7 +6065,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>233</v>
       </c>
@@ -6063,7 +6082,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>232</v>
       </c>
@@ -6074,7 +6093,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>231</v>
       </c>
@@ -6091,7 +6110,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>234</v>
       </c>
@@ -6108,7 +6127,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>247</v>
       </c>
@@ -6118,13 +6137,10 @@
       <c r="E11">
         <v>30000</v>
       </c>
-      <c r="K11" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D12" t="s">
         <v>32</v>
@@ -6132,11 +6148,8 @@
       <c r="E12">
         <v>30000</v>
       </c>
-      <c r="K12" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>235</v>
       </c>
@@ -6149,11 +6162,11 @@
       <c r="D13" t="s">
         <v>30</v>
       </c>
-      <c r="H13" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P13" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>237</v>
       </c>
@@ -6166,11 +6179,14 @@
       <c r="D14" t="s">
         <v>30</v>
       </c>
-      <c r="H14" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="O14" t="s">
+        <v>461</v>
+      </c>
+      <c r="P14" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>248</v>
       </c>
@@ -6180,13 +6196,10 @@
       <c r="E15">
         <v>30000</v>
       </c>
-      <c r="K15" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D16" t="s">
         <v>32</v>
@@ -6194,11 +6207,8 @@
       <c r="E16">
         <v>30000</v>
       </c>
-      <c r="K16" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>236</v>
       </c>
@@ -6211,11 +6221,11 @@
       <c r="D17" t="s">
         <v>30</v>
       </c>
-      <c r="H17" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P17" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>238</v>
       </c>
@@ -6228,13 +6238,13 @@
       <c r="D18" t="s">
         <v>30</v>
       </c>
-      <c r="H18" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P18" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
@@ -6249,12 +6259,12 @@
         <v>30000</v>
       </c>
       <c r="G20" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D21" t="s">
         <v>30</v>
@@ -6263,15 +6273,15 @@
         <v>30000</v>
       </c>
       <c r="G21" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="H21" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D22" t="s">
         <v>31</v>
@@ -6280,9 +6290,9 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B23" t="s">
         <v>27</v>
@@ -6291,46 +6301,46 @@
         <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G23" t="s">
         <v>251</v>
       </c>
       <c r="H23" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D24" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G24" t="s">
         <v>251</v>
       </c>
       <c r="H24" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D25" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G25" t="s">
         <v>251</v>
       </c>
       <c r="H25" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D26" t="s">
         <v>31</v>
@@ -6339,7 +6349,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>251</v>
       </c>
@@ -6350,7 +6360,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>252</v>
       </c>
@@ -6367,7 +6377,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>249</v>
       </c>
@@ -6381,10 +6391,10 @@
         <v>30</v>
       </c>
       <c r="G30" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>250</v>
       </c>
@@ -6395,9 +6405,9 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B32" t="s">
         <v>28</v>
@@ -6406,27 +6416,27 @@
         <v>9</v>
       </c>
       <c r="D32" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G32" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H32" t="s">
         <v>250</v>
       </c>
       <c r="K32" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D33" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G33" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H33" t="s">
         <v>250</v>
@@ -6434,13 +6444,13 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D34" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G34" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H34" t="s">
         <v>250</v>
@@ -6448,13 +6458,13 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D35" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G35" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H35" t="s">
         <v>250</v>
@@ -6462,13 +6472,13 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G36" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H36" t="s">
         <v>250</v>
@@ -6476,7 +6486,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D37" t="s">
         <v>31</v>
@@ -6487,7 +6497,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D38" t="s">
         <v>31</v>
@@ -6498,7 +6508,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D39" t="s">
         <v>32</v>
@@ -6509,7 +6519,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B40" t="s">
         <v>28</v>
@@ -6521,12 +6531,12 @@
         <v>30</v>
       </c>
       <c r="H40" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B41" t="s">
         <v>27</v>
@@ -6535,7 +6545,7 @@
         <v>4</v>
       </c>
       <c r="D41" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F41">
         <v>1000</v>
@@ -6543,7 +6553,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B42" t="s">
         <v>27</v>
@@ -6552,7 +6562,7 @@
         <v>5</v>
       </c>
       <c r="D42" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F42">
         <v>1000</v>
@@ -6560,7 +6570,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B43" t="s">
         <v>27</v>
@@ -6569,7 +6579,7 @@
         <v>7</v>
       </c>
       <c r="D43" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F43">
         <v>1000</v>
@@ -6577,7 +6587,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B44" t="s">
         <v>27</v>
@@ -6586,7 +6596,7 @@
         <v>8</v>
       </c>
       <c r="D44" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F44">
         <v>1000</v>
@@ -6637,7 +6647,7 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D49" t="s">
         <v>32</v>
@@ -6663,12 +6673,12 @@
         <v>1000</v>
       </c>
       <c r="H50" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D51" t="s">
         <v>32</v>
@@ -6694,7 +6704,7 @@
         <v>1000</v>
       </c>
       <c r="H52" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
@@ -6716,7 +6726,7 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D55" t="s">
         <v>32</v>
@@ -6727,7 +6737,7 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B56" t="s">
         <v>28</v>
@@ -6739,7 +6749,7 @@
         <v>30</v>
       </c>
       <c r="H56" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="J56">
         <v>-50</v>
@@ -6747,7 +6757,7 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B58" t="s">
         <v>28</v>
@@ -6762,7 +6772,7 @@
         <v>120000</v>
       </c>
       <c r="G58" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
@@ -6806,7 +6816,7 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B63" t="s">
         <v>27</v>
@@ -6821,12 +6831,12 @@
         <v>60000</v>
       </c>
       <c r="G63" t="s">
-        <v>288</v>
+        <v>462</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D64" t="s">
         <v>32</v>
@@ -6837,7 +6847,7 @@
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B66" t="s">
         <v>28</v>
@@ -6849,12 +6859,12 @@
         <v>33</v>
       </c>
       <c r="G66" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="D67" t="s">
         <v>31</v>
@@ -6865,7 +6875,7 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B68" t="s">
         <v>28</v>
@@ -6877,7 +6887,7 @@
         <v>33</v>
       </c>
       <c r="H68" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>
@@ -6888,7 +6898,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3261DB23-C434-4F35-8B4F-998D4295A585}">
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -6928,7 +6938,7 @@
         <v>226</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -6942,12 +6952,12 @@
         <v>1950</v>
       </c>
       <c r="K3" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="D5" t="s">
         <v>32</v>
@@ -6958,7 +6968,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
@@ -6970,21 +6980,21 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="H6" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="K6" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="N6" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="B7" t="s">
         <v>28</v>
@@ -6996,24 +7006,24 @@
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="H7" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="K7" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="M7" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="N7" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="B8" t="s">
         <v>29</v>
@@ -7025,18 +7035,18 @@
         <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="H8" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="K8" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="D10" t="s">
         <v>32</v>
@@ -7047,7 +7057,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -7059,21 +7069,21 @@
         <v>30</v>
       </c>
       <c r="G11" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="H11" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="K11" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="N11" s="12" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="B12" t="s">
         <v>28</v>
@@ -7085,21 +7095,21 @@
         <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="H12" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="K12" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="M12" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="B13" t="s">
         <v>29</v>
@@ -7111,18 +7121,18 @@
         <v>30</v>
       </c>
       <c r="G13" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="H13" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="K13" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="D15" t="s">
         <v>32</v>
@@ -7133,7 +7143,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="B16" t="s">
         <v>27</v>
@@ -7145,18 +7155,18 @@
         <v>30</v>
       </c>
       <c r="G16" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="H16" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="K16" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="B17" t="s">
         <v>28</v>
@@ -7168,21 +7178,21 @@
         <v>30</v>
       </c>
       <c r="G17" t="s">
+        <v>448</v>
+      </c>
+      <c r="H17" t="s">
+        <v>454</v>
+      </c>
+      <c r="K17" t="s">
+        <v>403</v>
+      </c>
+      <c r="M17" t="s">
         <v>451</v>
-      </c>
-      <c r="H17" t="s">
-        <v>457</v>
-      </c>
-      <c r="K17" t="s">
-        <v>406</v>
-      </c>
-      <c r="M17" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="B18" t="s">
         <v>29</v>
@@ -7194,18 +7204,18 @@
         <v>30</v>
       </c>
       <c r="G18" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="H18" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="K18" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
@@ -7216,16 +7226,20 @@
       <c r="D20" t="s">
         <v>30</v>
       </c>
+      <c r="E20">
+        <f>2*E3</f>
+        <v>3900</v>
+      </c>
       <c r="K20" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="N20" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="B21" t="s">
         <v>27</v>
@@ -7237,15 +7251,15 @@
         <v>30</v>
       </c>
       <c r="K21" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="N21" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
@@ -7257,20 +7271,20 @@
         <v>30</v>
       </c>
       <c r="K22" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="N22" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N23" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B24" t="s">
         <v>27</v>
@@ -7278,89 +7292,83 @@
       <c r="C24">
         <v>8</v>
       </c>
+      <c r="D24" t="s">
+        <v>33</v>
+      </c>
       <c r="K24" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="N24" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>426</v>
-      </c>
-      <c r="B25" t="s">
+        <v>457</v>
+      </c>
+      <c r="D25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>423</v>
+      </c>
+      <c r="B26" t="s">
         <v>28</v>
       </c>
-      <c r="C25">
+      <c r="C26">
         <v>8</v>
       </c>
-      <c r="N25" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>427</v>
-      </c>
-      <c r="B27" t="s">
-        <v>29</v>
-      </c>
-      <c r="C27">
-        <v>8</v>
-      </c>
-      <c r="D27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G27" t="s">
-        <v>446</v>
-      </c>
-      <c r="K27" t="s">
-        <v>428</v>
-      </c>
-      <c r="N27" t="s">
-        <v>417</v>
+      <c r="D26" t="s">
+        <v>458</v>
+      </c>
+      <c r="N26" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>446</v>
+        <v>424</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28">
+        <v>8</v>
       </c>
       <c r="D28" t="s">
+        <v>30</v>
+      </c>
+      <c r="G28" t="s">
+        <v>443</v>
+      </c>
+      <c r="K28" t="s">
+        <v>425</v>
+      </c>
+      <c r="N28" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>443</v>
+      </c>
+      <c r="D29" t="s">
         <v>32</v>
       </c>
-      <c r="E28">
+      <c r="E29">
         <v>30000</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N29" t="s">
-        <v>423</v>
-      </c>
-    </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>424</v>
-      </c>
-      <c r="B30" t="s">
-        <v>27</v>
-      </c>
-      <c r="C30">
-        <v>9</v>
-      </c>
-      <c r="F30">
-        <v>60000</v>
-      </c>
-      <c r="G30" t="s">
-        <v>444</v>
-      </c>
-      <c r="K30" t="s">
-        <v>429</v>
+      <c r="N30" t="s">
+        <v>420</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>442</v>
+        <v>421</v>
       </c>
       <c r="B31" t="s">
         <v>27</v>
@@ -7368,231 +7376,304 @@
       <c r="C31">
         <v>9</v>
       </c>
-      <c r="E31">
-        <v>20000</v>
+      <c r="D31" t="s">
+        <v>458</v>
+      </c>
+      <c r="F31">
+        <v>60000</v>
+      </c>
+      <c r="G31" t="s">
+        <v>441</v>
+      </c>
+      <c r="K31" t="s">
+        <v>426</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>432</v>
+        <v>439</v>
+      </c>
+      <c r="B32" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32">
+        <v>9</v>
+      </c>
+      <c r="D32" t="s">
+        <v>458</v>
       </c>
       <c r="E32">
         <v>20000</v>
       </c>
-      <c r="K32" t="s">
-        <v>430</v>
-      </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>425</v>
-      </c>
-      <c r="B33" t="s">
-        <v>28</v>
-      </c>
-      <c r="C33">
-        <v>9</v>
-      </c>
-      <c r="F33">
-        <v>90000</v>
-      </c>
-      <c r="G33" t="s">
-        <v>443</v>
+        <v>429</v>
+      </c>
+      <c r="D33" t="s">
+        <v>31</v>
+      </c>
+      <c r="E33">
+        <v>20000</v>
+      </c>
+      <c r="K33" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>435</v>
-      </c>
-      <c r="E34">
-        <v>15000</v>
+        <v>422</v>
+      </c>
+      <c r="B34" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34">
+        <v>9</v>
+      </c>
+      <c r="D34" t="s">
+        <v>458</v>
+      </c>
+      <c r="F34">
+        <v>90000</v>
+      </c>
+      <c r="G34" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>433</v>
+        <v>432</v>
+      </c>
+      <c r="B35" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35">
+        <v>9</v>
+      </c>
+      <c r="D35" t="s">
+        <v>458</v>
       </c>
       <c r="E35">
         <v>15000</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
-        <v>28</v>
-      </c>
-      <c r="C36">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>431</v>
-      </c>
-      <c r="B37" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37">
-        <v>9</v>
-      </c>
-      <c r="F37">
-        <v>120000</v>
-      </c>
-      <c r="G37" t="s">
-        <v>434</v>
+      <c r="A36" t="s">
+        <v>430</v>
+      </c>
+      <c r="D36" t="s">
+        <v>31</v>
+      </c>
+      <c r="E36">
+        <v>15000</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>434</v>
-      </c>
-      <c r="E38">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>439</v>
-      </c>
-      <c r="B41" t="s">
-        <v>27</v>
-      </c>
-      <c r="C41">
-        <v>10</v>
-      </c>
-      <c r="F41">
-        <v>90000</v>
-      </c>
-      <c r="M41">
+        <v>428</v>
+      </c>
+      <c r="B38" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38">
+        <v>9</v>
+      </c>
+      <c r="D38" t="s">
+        <v>458</v>
+      </c>
+      <c r="F38">
+        <v>120000</v>
+      </c>
+      <c r="G38" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>431</v>
+      </c>
+      <c r="D39" t="s">
+        <v>31</v>
+      </c>
+      <c r="E39">
         <v>20000</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B42" t="s">
         <v>27</v>
       </c>
       <c r="C42">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="D42" t="s">
+        <v>33</v>
+      </c>
+      <c r="F42">
+        <v>90000</v>
+      </c>
+      <c r="M42">
+        <v>20000</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>445</v>
-      </c>
-      <c r="E43">
-        <v>30000</v>
+        <v>434</v>
+      </c>
+      <c r="B43" t="s">
+        <v>27</v>
+      </c>
+      <c r="C43">
+        <v>11</v>
+      </c>
+      <c r="D43" t="s">
+        <v>458</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>441</v>
+        <v>442</v>
+      </c>
+      <c r="B44" t="s">
+        <v>27</v>
+      </c>
+      <c r="C44">
+        <v>11</v>
+      </c>
+      <c r="D44" t="s">
+        <v>458</v>
       </c>
       <c r="E44">
-        <v>15000</v>
-      </c>
-      <c r="F44">
-        <v>120000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>436</v>
-      </c>
-      <c r="B45" t="s">
-        <v>28</v>
-      </c>
-      <c r="C45">
-        <v>11</v>
+        <v>438</v>
+      </c>
+      <c r="D45" t="s">
+        <v>31</v>
+      </c>
+      <c r="E45">
+        <v>15000</v>
       </c>
       <c r="F45">
-        <v>90000</v>
-      </c>
-      <c r="M45">
-        <v>15000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="B46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C46">
         <v>11</v>
       </c>
+      <c r="D46" t="s">
+        <v>33</v>
+      </c>
       <c r="F46">
-        <v>120000</v>
+        <v>90000</v>
       </c>
       <c r="M46">
-        <v>6000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="B47" t="s">
+        <v>29</v>
+      </c>
+      <c r="C47">
+        <v>11</v>
+      </c>
+      <c r="D47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F47">
+        <v>120000</v>
+      </c>
+      <c r="M47">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>437</v>
+      </c>
+      <c r="B48" t="s">
         <v>28</v>
       </c>
-      <c r="C47">
+      <c r="C48">
         <v>12</v>
       </c>
-      <c r="F47">
+      <c r="D48" t="s">
+        <v>33</v>
+      </c>
+      <c r="F48">
         <v>90000</v>
       </c>
-      <c r="M47">
+      <c r="M48">
         <v>10000</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D50" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>382</v>
-      </c>
-      <c r="B52" t="s">
-        <v>27</v>
-      </c>
-      <c r="C52">
-        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>448</v>
+        <v>379</v>
       </c>
       <c r="B53" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
+      <c r="D53" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="B54" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C54">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D54" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B55" t="s">
+        <v>27</v>
+      </c>
+      <c r="C55">
+        <v>2</v>
+      </c>
+      <c r="D55" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>444</v>
+      </c>
+      <c r="B56" t="s">
         <v>28</v>
       </c>
-      <c r="C55">
+      <c r="C56">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire the Monk rotation and expand status helpers
Add MNK job and gauge dispatch, refine action priorities and generalize oldest-status consumption.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A2C309D-80C0-419D-9FBC-F68D77E5DF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76861B9F-8125-4074-AEF9-ACCA23766F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8385" yWindow="1635" windowWidth="25605" windowHeight="13935" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="14160" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1250" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="478">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1273,9 +1273,6 @@
     <t>Chackra spender</t>
   </si>
   <si>
-    <t>Besoin de suivre le nombre de chackra</t>
-  </si>
-  <si>
     <t>Besoin de savoir la forme actuelle</t>
   </si>
   <si>
@@ -1417,9 +1414,6 @@
     <t>SI on a des stack de formeless, ca ne donne pas de forme…</t>
   </si>
   <si>
-    <t>Balance Buff</t>
-  </si>
-  <si>
     <t>Fixme</t>
   </si>
   <si>
@@ -1433,6 +1427,57 @@
   </si>
   <si>
     <t>Flourishing Symmetry;Flourishing Flow;Threefold Fan Dance;Fourfold Fan Dance;Finishing Move Ready</t>
+  </si>
+  <si>
+    <t>Formless Shift;Coeurl Form</t>
+  </si>
+  <si>
+    <t>Opo-opo's Fury</t>
+  </si>
+  <si>
+    <t>Raptor's Fury</t>
+  </si>
+  <si>
+    <t>Coeurl's Fury</t>
+  </si>
+  <si>
+    <t>Formless Shift;Opo-opo Form;Opo-opo's Fury</t>
+  </si>
+  <si>
+    <t>Raptor Form;Opo-opo's Fury</t>
+  </si>
+  <si>
+    <t>Formless Shift;Raptor Form;Raptor's Fury</t>
+  </si>
+  <si>
+    <t>Coeurl Form;Raptor's Fury</t>
+  </si>
+  <si>
+    <t>Balance Buff 1</t>
+  </si>
+  <si>
+    <t>Besoin d egérer les charges … Pour le moment Perfect balance reste le seul truc manuel</t>
+  </si>
+  <si>
+    <t>Balance Buff 2</t>
+  </si>
+  <si>
+    <t>Balance Buff 3</t>
+  </si>
+  <si>
+    <t>Forbidden Meditation</t>
+  </si>
+  <si>
+    <t>The Forbidden Chakra</t>
+  </si>
+  <si>
+    <t>FIXME FIRE BUFF AT LVL 100</t>
+  </si>
+  <si>
+    <t>Wind's Reply</t>
+  </si>
+  <si>
+    <t>Fire's Reply</t>
   </si>
 </sst>
 </file>
@@ -6163,7 +6208,7 @@
         <v>30</v>
       </c>
       <c r="P13" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -6180,10 +6225,10 @@
         <v>30</v>
       </c>
       <c r="O14" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="P14" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
@@ -6222,7 +6267,7 @@
         <v>30</v>
       </c>
       <c r="P17" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
@@ -6239,7 +6284,7 @@
         <v>30</v>
       </c>
       <c r="P18" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
@@ -6831,7 +6876,7 @@
         <v>60000</v>
       </c>
       <c r="G63" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
@@ -6898,7 +6943,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3261DB23-C434-4F35-8B4F-998D4295A585}">
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:P64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -6941,6 +6986,11 @@
         <v>313</v>
       </c>
     </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>464</v>
+      </c>
+    </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
@@ -6952,12 +7002,12 @@
         <v>1950</v>
       </c>
       <c r="K3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="D5" t="s">
         <v>32</v>
@@ -6968,36 +7018,21 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>387</v>
-      </c>
-      <c r="B6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6">
-        <v>4</v>
+        <v>462</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" t="s">
-        <v>449</v>
-      </c>
-      <c r="H6" t="s">
-        <v>454</v>
-      </c>
-      <c r="K6" t="s">
-        <v>395</v>
-      </c>
-      <c r="N6" t="s">
-        <v>410</v>
+        <v>31</v>
+      </c>
+      <c r="E6">
+        <v>3600000</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7">
         <v>4</v>
@@ -7006,27 +7041,24 @@
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H7" t="s">
-        <v>454</v>
+        <v>465</v>
       </c>
       <c r="K7" t="s">
-        <v>396</v>
-      </c>
-      <c r="M7" t="s">
-        <v>453</v>
+        <v>395</v>
       </c>
       <c r="N7" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8">
         <v>4</v>
@@ -7035,84 +7067,72 @@
         <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>449</v>
+        <v>466</v>
       </c>
       <c r="H8" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="K8" t="s">
+        <v>396</v>
+      </c>
+      <c r="M8" t="s">
+        <v>452</v>
+      </c>
+      <c r="N8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>389</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9">
+        <v>4</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" t="s">
+        <v>448</v>
+      </c>
+      <c r="H9" t="s">
+        <v>453</v>
+      </c>
+      <c r="K9" t="s">
         <v>397</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>449</v>
-      </c>
-      <c r="D10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10">
-        <v>30000</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>390</v>
-      </c>
-      <c r="B11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11">
-        <v>5</v>
+        <v>448</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
-      </c>
-      <c r="G11" t="s">
-        <v>450</v>
-      </c>
-      <c r="H11" t="s">
-        <v>455</v>
-      </c>
-      <c r="K11" t="s">
-        <v>399</v>
-      </c>
-      <c r="N11" s="12" t="s">
-        <v>456</v>
+        <v>32</v>
+      </c>
+      <c r="E11">
+        <v>30000</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>391</v>
-      </c>
-      <c r="B12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12">
-        <v>5</v>
+        <v>463</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
-      </c>
-      <c r="G12" t="s">
-        <v>450</v>
-      </c>
-      <c r="H12" t="s">
-        <v>455</v>
-      </c>
-      <c r="K12" t="s">
-        <v>400</v>
-      </c>
-      <c r="M12" t="s">
-        <v>452</v>
+        <v>31</v>
+      </c>
+      <c r="E12">
+        <v>3600000</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C13">
         <v>5</v>
@@ -7121,81 +7141,84 @@
         <v>30</v>
       </c>
       <c r="G13" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="H13" t="s">
+        <v>467</v>
+      </c>
+      <c r="K13" t="s">
+        <v>399</v>
+      </c>
+      <c r="N13" s="12" t="s">
         <v>455</v>
       </c>
-      <c r="K13" t="s">
-        <v>401</v>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>391</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+      <c r="G14" t="s">
+        <v>468</v>
+      </c>
+      <c r="H14" t="s">
+        <v>454</v>
+      </c>
+      <c r="K14" t="s">
+        <v>400</v>
+      </c>
+      <c r="M14" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>450</v>
+        <v>393</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15">
+        <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>394</v>
-      </c>
-      <c r="B16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16">
-        <v>6</v>
-      </c>
-      <c r="D16" t="s">
-        <v>30</v>
-      </c>
-      <c r="G16" t="s">
-        <v>448</v>
-      </c>
-      <c r="H16" t="s">
+        <v>30</v>
+      </c>
+      <c r="G15" t="s">
+        <v>449</v>
+      </c>
+      <c r="H15" t="s">
         <v>454</v>
       </c>
-      <c r="K16" t="s">
-        <v>402</v>
+      <c r="K15" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>392</v>
-      </c>
-      <c r="B17" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17">
-        <v>6</v>
+        <v>449</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
-      </c>
-      <c r="G17" t="s">
-        <v>448</v>
-      </c>
-      <c r="H17" t="s">
-        <v>454</v>
-      </c>
-      <c r="K17" t="s">
-        <v>403</v>
-      </c>
-      <c r="M17" t="s">
-        <v>451</v>
+        <v>32</v>
+      </c>
+      <c r="E17">
+        <v>30000</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C18">
         <v>6</v>
@@ -7204,293 +7227,325 @@
         <v>30</v>
       </c>
       <c r="G18" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H18" t="s">
-        <v>454</v>
+        <v>461</v>
+      </c>
+      <c r="I18">
+        <v>-1</v>
       </c>
       <c r="K18" t="s">
-        <v>404</v>
+        <v>402</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>392</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19">
+        <v>6</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
+      </c>
+      <c r="G19" t="s">
+        <v>447</v>
+      </c>
+      <c r="H19" t="s">
+        <v>461</v>
+      </c>
+      <c r="I19">
+        <v>2</v>
+      </c>
+      <c r="K19" t="s">
+        <v>403</v>
+      </c>
+      <c r="M19" t="s">
+        <v>450</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C20">
+        <v>6</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+      <c r="G20" t="s">
+        <v>447</v>
+      </c>
+      <c r="H20" t="s">
+        <v>461</v>
+      </c>
+      <c r="K20" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>411</v>
+      </c>
+      <c r="B22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22">
         <v>3</v>
       </c>
-      <c r="D20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E20">
+      <c r="D22" t="s">
+        <v>30</v>
+      </c>
+      <c r="F22">
         <f>2*E3</f>
         <v>3900</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K22" t="s">
+        <v>412</v>
+      </c>
+      <c r="N22" t="s">
         <v>413</v>
       </c>
-      <c r="N20" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>405</v>
-      </c>
-      <c r="B21" t="s">
-        <v>27</v>
-      </c>
-      <c r="C21">
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>473</v>
+      </c>
+      <c r="B23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23">
         <v>7</v>
       </c>
-      <c r="D21" t="s">
-        <v>30</v>
-      </c>
-      <c r="K21" t="s">
+      <c r="D23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23">
+        <v>1000</v>
+      </c>
+      <c r="K23" t="s">
         <v>407</v>
       </c>
-      <c r="N21" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>406</v>
-      </c>
-      <c r="B22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22">
-        <v>7</v>
-      </c>
-      <c r="D22" t="s">
-        <v>30</v>
-      </c>
-      <c r="K22" t="s">
-        <v>408</v>
-      </c>
-      <c r="N22" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N23" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>415</v>
+        <v>474</v>
       </c>
       <c r="B24" t="s">
         <v>27</v>
       </c>
       <c r="C24">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D24" t="s">
         <v>33</v>
       </c>
       <c r="K24" t="s">
-        <v>416</v>
-      </c>
-      <c r="N24" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>457</v>
+        <v>405</v>
+      </c>
+      <c r="B25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25">
+        <v>7</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="F25">
+        <v>1000</v>
+      </c>
+      <c r="K25" t="s">
+        <v>407</v>
+      </c>
+      <c r="N25" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>423</v>
+        <v>406</v>
       </c>
       <c r="B26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D26" t="s">
-        <v>458</v>
-      </c>
-      <c r="N26" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26" t="s">
+        <v>29</v>
+      </c>
+      <c r="K26" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N27" t="s">
         <v>418</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>424</v>
+        <v>414</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C28">
         <v>8</v>
       </c>
       <c r="D28" t="s">
-        <v>30</v>
-      </c>
-      <c r="G28" t="s">
-        <v>443</v>
+        <v>33</v>
       </c>
       <c r="K28" t="s">
-        <v>425</v>
+        <v>415</v>
       </c>
       <c r="N28" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>443</v>
+        <v>469</v>
       </c>
       <c r="D29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E29">
         <v>30000</v>
       </c>
+      <c r="N29" t="s">
+        <v>470</v>
+      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N30" t="s">
-        <v>420</v>
+      <c r="A30" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>421</v>
-      </c>
-      <c r="B31" t="s">
-        <v>27</v>
-      </c>
-      <c r="C31">
-        <v>9</v>
-      </c>
-      <c r="D31" t="s">
-        <v>458</v>
-      </c>
-      <c r="F31">
-        <v>60000</v>
-      </c>
-      <c r="G31" t="s">
-        <v>441</v>
-      </c>
-      <c r="K31" t="s">
-        <v>426</v>
+        <v>472</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>439</v>
+        <v>422</v>
       </c>
       <c r="B32" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C32">
+        <v>8</v>
+      </c>
+      <c r="D32" t="s">
+        <v>456</v>
+      </c>
+      <c r="N32" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>423</v>
+      </c>
+      <c r="B34" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34">
+        <v>8</v>
+      </c>
+      <c r="D34" t="s">
+        <v>30</v>
+      </c>
+      <c r="G34" t="s">
+        <v>442</v>
+      </c>
+      <c r="K34" t="s">
+        <v>424</v>
+      </c>
+      <c r="N34" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>442</v>
+      </c>
+      <c r="D35" t="s">
+        <v>32</v>
+      </c>
+      <c r="E35">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N36" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>420</v>
+      </c>
+      <c r="B37" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37">
         <v>9</v>
       </c>
-      <c r="D32" t="s">
-        <v>458</v>
-      </c>
-      <c r="E32">
+      <c r="D37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F37">
+        <v>60000</v>
+      </c>
+      <c r="G37" t="s">
+        <v>428</v>
+      </c>
+      <c r="K37" t="s">
+        <v>425</v>
+      </c>
+      <c r="N37" t="s">
+        <v>440</v>
+      </c>
+      <c r="P37" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>438</v>
+      </c>
+      <c r="D38" t="s">
+        <v>32</v>
+      </c>
+      <c r="E38">
         <v>20000</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>429</v>
-      </c>
-      <c r="D33" t="s">
-        <v>31</v>
-      </c>
-      <c r="E33">
-        <v>20000</v>
-      </c>
-      <c r="K33" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>422</v>
-      </c>
-      <c r="B34" t="s">
-        <v>28</v>
-      </c>
-      <c r="C34">
-        <v>9</v>
-      </c>
-      <c r="D34" t="s">
-        <v>458</v>
-      </c>
-      <c r="F34">
-        <v>90000</v>
-      </c>
-      <c r="G34" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>432</v>
-      </c>
-      <c r="B35" t="s">
-        <v>28</v>
-      </c>
-      <c r="C35">
-        <v>9</v>
-      </c>
-      <c r="D35" t="s">
-        <v>458</v>
-      </c>
-      <c r="E35">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>430</v>
-      </c>
-      <c r="D36" t="s">
-        <v>31</v>
-      </c>
-      <c r="E36">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>428</v>
-      </c>
-      <c r="B38" t="s">
-        <v>29</v>
-      </c>
-      <c r="C38">
-        <v>9</v>
-      </c>
-      <c r="D38" t="s">
-        <v>458</v>
-      </c>
-      <c r="F38">
-        <v>120000</v>
-      </c>
-      <c r="G38" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>431</v>
       </c>
       <c r="D39" t="s">
         <v>31</v>
@@ -7498,182 +7553,292 @@
       <c r="E39">
         <v>20000</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K39" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>477</v>
+      </c>
+      <c r="B40" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40">
+        <v>9</v>
+      </c>
+      <c r="D40" t="s">
+        <v>30</v>
+      </c>
+      <c r="H40" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>421</v>
+      </c>
+      <c r="B41" t="s">
+        <v>28</v>
+      </c>
+      <c r="C41">
+        <v>9</v>
+      </c>
+      <c r="D41" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41">
+        <v>90000</v>
+      </c>
+      <c r="G41" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>436</v>
-      </c>
-      <c r="B42" t="s">
-        <v>27</v>
-      </c>
-      <c r="C42">
+        <v>431</v>
+      </c>
+      <c r="D42" t="s">
+        <v>32</v>
+      </c>
+      <c r="E42">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>429</v>
+      </c>
+      <c r="D43" t="s">
+        <v>31</v>
+      </c>
+      <c r="E43">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>476</v>
+      </c>
+      <c r="B44" t="s">
+        <v>28</v>
+      </c>
+      <c r="C44">
+        <v>9</v>
+      </c>
+      <c r="D44" t="s">
+        <v>30</v>
+      </c>
+      <c r="H44" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>427</v>
+      </c>
+      <c r="B46" t="s">
+        <v>29</v>
+      </c>
+      <c r="C46">
+        <v>9</v>
+      </c>
+      <c r="D46" t="s">
+        <v>456</v>
+      </c>
+      <c r="F46">
+        <v>120000</v>
+      </c>
+      <c r="G46" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>430</v>
+      </c>
+      <c r="D47" t="s">
+        <v>31</v>
+      </c>
+      <c r="E47">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>435</v>
+      </c>
+      <c r="B50" t="s">
+        <v>27</v>
+      </c>
+      <c r="C50">
         <v>10</v>
       </c>
-      <c r="D42" t="s">
-        <v>33</v>
-      </c>
-      <c r="F42">
+      <c r="D50" t="s">
+        <v>33</v>
+      </c>
+      <c r="F50">
         <v>90000</v>
       </c>
-      <c r="M42">
+      <c r="M50">
         <v>20000</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>434</v>
-      </c>
-      <c r="B43" t="s">
-        <v>27</v>
-      </c>
-      <c r="C43">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>433</v>
+      </c>
+      <c r="B51" t="s">
+        <v>27</v>
+      </c>
+      <c r="C51">
         <v>11</v>
       </c>
-      <c r="D43" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>442</v>
-      </c>
-      <c r="B44" t="s">
-        <v>27</v>
-      </c>
-      <c r="C44">
+      <c r="D51" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>441</v>
+      </c>
+      <c r="B52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C52">
         <v>11</v>
       </c>
-      <c r="D44" t="s">
-        <v>458</v>
-      </c>
-      <c r="E44">
+      <c r="D52" t="s">
+        <v>456</v>
+      </c>
+      <c r="E52">
         <v>30000</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>438</v>
-      </c>
-      <c r="D45" t="s">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>437</v>
+      </c>
+      <c r="D53" t="s">
         <v>31</v>
       </c>
-      <c r="E45">
+      <c r="E53">
         <v>15000</v>
       </c>
-      <c r="F45">
+      <c r="F53">
         <v>120000</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>433</v>
-      </c>
-      <c r="B46" t="s">
-        <v>28</v>
-      </c>
-      <c r="C46">
-        <v>11</v>
-      </c>
-      <c r="D46" t="s">
-        <v>33</v>
-      </c>
-      <c r="F46">
-        <v>90000</v>
-      </c>
-      <c r="M46">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>435</v>
-      </c>
-      <c r="B47" t="s">
-        <v>29</v>
-      </c>
-      <c r="C47">
-        <v>11</v>
-      </c>
-      <c r="D47" t="s">
-        <v>33</v>
-      </c>
-      <c r="F47">
-        <v>120000</v>
-      </c>
-      <c r="M47">
-        <v>6000</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>437</v>
-      </c>
-      <c r="B48" t="s">
-        <v>28</v>
-      </c>
-      <c r="C48">
-        <v>12</v>
-      </c>
-      <c r="D48" t="s">
-        <v>33</v>
-      </c>
-      <c r="F48">
-        <v>90000</v>
-      </c>
-      <c r="M48">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>379</v>
-      </c>
-      <c r="B53" t="s">
-        <v>27</v>
-      </c>
-      <c r="C53">
-        <v>1</v>
-      </c>
-      <c r="D53" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>445</v>
+        <v>432</v>
       </c>
       <c r="B54" t="s">
         <v>28</v>
       </c>
       <c r="C54">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D54" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F54">
+        <v>90000</v>
+      </c>
+      <c r="M54">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>446</v>
+        <v>434</v>
       </c>
       <c r="B55" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C55">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D55" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F55">
+        <v>120000</v>
+      </c>
+      <c r="M55">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="B56" t="s">
         <v>28</v>
       </c>
       <c r="C56">
+        <v>12</v>
+      </c>
+      <c r="D56" t="s">
+        <v>33</v>
+      </c>
+      <c r="F56">
+        <v>90000</v>
+      </c>
+      <c r="M56">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>379</v>
+      </c>
+      <c r="B61" t="s">
+        <v>27</v>
+      </c>
+      <c r="C61">
+        <v>1</v>
+      </c>
+      <c r="D61" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>444</v>
+      </c>
+      <c r="B62" t="s">
+        <v>28</v>
+      </c>
+      <c r="C62">
+        <v>1</v>
+      </c>
+      <c r="D62" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>445</v>
+      </c>
+      <c r="B63" t="s">
+        <v>27</v>
+      </c>
+      <c r="C63">
+        <v>2</v>
+      </c>
+      <c r="D63" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>443</v>
+      </c>
+      <c r="B64" t="s">
+        <v>28</v>
+      </c>
+      <c r="C64">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Monk Nadi tracking and Perfect Balance priorities
Introduce Nadi helpers and reduce the minimum weave duration to 750 ms. Opener handling remains incomplete.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76861B9F-8125-4074-AEF9-ACCA23766F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9CC7CB4-7E19-44AC-8F5C-B534BAB1E9EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="14160" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9870" yWindow="5055" windowWidth="20865" windowHeight="12240" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1299" uniqueCount="487">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1453,15 +1453,9 @@
     <t>Coeurl Form;Raptor's Fury</t>
   </si>
   <si>
-    <t>Balance Buff 1</t>
-  </si>
-  <si>
     <t>Besoin d egérer les charges … Pour le moment Perfect balance reste le seul truc manuel</t>
   </si>
   <si>
-    <t>Balance Buff 2</t>
-  </si>
-  <si>
     <t>Balance Buff 3</t>
   </si>
   <si>
@@ -1478,6 +1472,39 @@
   </si>
   <si>
     <t>Fire's Reply</t>
+  </si>
+  <si>
+    <t>To be triggered</t>
+  </si>
+  <si>
+    <t>Lunar Start Action</t>
+  </si>
+  <si>
+    <t>Solar Start Action</t>
+  </si>
+  <si>
+    <t>Lunar Start Buff</t>
+  </si>
+  <si>
+    <t>Solar Start Buff</t>
+  </si>
+  <si>
+    <t>Balance Buff</t>
+  </si>
+  <si>
+    <t>Finisher Buff</t>
+  </si>
+  <si>
+    <t>Celestial</t>
+  </si>
+  <si>
+    <t>Phantom Rush</t>
+  </si>
+  <si>
+    <t>Elixir Burst</t>
+  </si>
+  <si>
+    <t>Rising Phoenix</t>
   </si>
 </sst>
 </file>
@@ -6943,7 +6970,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3261DB23-C434-4F35-8B4F-998D4295A585}">
-  <dimension ref="A1:P64"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -7317,7 +7344,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B23" t="s">
         <v>27</v>
@@ -7340,7 +7367,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B24" t="s">
         <v>27</v>
@@ -7416,6 +7443,9 @@
       <c r="D28" t="s">
         <v>33</v>
       </c>
+      <c r="G28" t="s">
+        <v>481</v>
+      </c>
       <c r="K28" t="s">
         <v>415</v>
       </c>
@@ -7425,26 +7455,32 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>469</v>
+        <v>481</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
       </c>
       <c r="E29">
-        <v>30000</v>
+        <v>20000</v>
       </c>
       <c r="N29" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>471</v>
+        <v>482</v>
+      </c>
+      <c r="D30" t="s">
+        <v>31</v>
+      </c>
+      <c r="E30">
+        <v>20000</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
@@ -7458,18 +7494,32 @@
         <v>8</v>
       </c>
       <c r="D32" t="s">
-        <v>456</v>
+        <v>30</v>
       </c>
       <c r="N32" t="s">
         <v>417</v>
       </c>
     </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>485</v>
+      </c>
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33">
+        <v>8</v>
+      </c>
+      <c r="D33" t="s">
+        <v>30</v>
+      </c>
+    </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>423</v>
+        <v>486</v>
       </c>
       <c r="B34" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C34">
         <v>8</v>
@@ -7477,109 +7527,80 @@
       <c r="D34" t="s">
         <v>30</v>
       </c>
-      <c r="G34" t="s">
-        <v>442</v>
-      </c>
-      <c r="K34" t="s">
-        <v>424</v>
-      </c>
-      <c r="N34" t="s">
-        <v>413</v>
-      </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>442</v>
+        <v>483</v>
+      </c>
+      <c r="B35" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35">
+        <v>8</v>
       </c>
       <c r="D35" t="s">
-        <v>32</v>
-      </c>
-      <c r="E35">
-        <v>30000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="N36" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>420</v>
-      </c>
-      <c r="B37" t="s">
-        <v>27</v>
-      </c>
-      <c r="C37">
-        <v>9</v>
-      </c>
-      <c r="D37" t="s">
-        <v>33</v>
-      </c>
-      <c r="F37">
-        <v>60000</v>
-      </c>
-      <c r="G37" t="s">
-        <v>428</v>
-      </c>
-      <c r="K37" t="s">
-        <v>425</v>
-      </c>
-      <c r="N37" t="s">
-        <v>440</v>
-      </c>
-      <c r="P37" t="s">
-        <v>475</v>
+      <c r="A36" t="s">
+        <v>484</v>
+      </c>
+      <c r="B36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36">
+        <v>8</v>
+      </c>
+      <c r="D36" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>438</v>
+        <v>423</v>
+      </c>
+      <c r="B38" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38">
+        <v>8</v>
       </c>
       <c r="D38" t="s">
-        <v>32</v>
-      </c>
-      <c r="E38">
-        <v>20000</v>
+        <v>30</v>
+      </c>
+      <c r="G38" t="s">
+        <v>442</v>
+      </c>
+      <c r="K38" t="s">
+        <v>424</v>
+      </c>
+      <c r="N38" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>428</v>
+        <v>442</v>
       </c>
       <c r="D39" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E39">
-        <v>20000</v>
-      </c>
-      <c r="K39" t="s">
-        <v>426</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>477</v>
-      </c>
-      <c r="B40" t="s">
-        <v>27</v>
-      </c>
-      <c r="C40">
-        <v>9</v>
-      </c>
-      <c r="D40" t="s">
-        <v>30</v>
-      </c>
-      <c r="H40" t="s">
-        <v>438</v>
+      <c r="N40" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C41">
         <v>9</v>
@@ -7588,40 +7609,52 @@
         <v>33</v>
       </c>
       <c r="F41">
-        <v>90000</v>
+        <v>60000</v>
       </c>
       <c r="G41" t="s">
-        <v>439</v>
+        <v>428</v>
+      </c>
+      <c r="K41" t="s">
+        <v>425</v>
+      </c>
+      <c r="N41" t="s">
+        <v>440</v>
+      </c>
+      <c r="P41" t="s">
+        <v>473</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="D42" t="s">
         <v>32</v>
       </c>
       <c r="E42">
-        <v>15000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D43" t="s">
         <v>31</v>
       </c>
       <c r="E43">
-        <v>15000</v>
+        <v>20000</v>
+      </c>
+      <c r="K43" t="s">
+        <v>426</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B44" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C44">
         <v>9</v>
@@ -7630,114 +7663,108 @@
         <v>30</v>
       </c>
       <c r="H44" t="s">
-        <v>431</v>
+        <v>438</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>421</v>
+      </c>
+      <c r="B45" t="s">
+        <v>28</v>
+      </c>
+      <c r="C45">
+        <v>9</v>
+      </c>
+      <c r="D45" t="s">
+        <v>33</v>
+      </c>
+      <c r="F45">
+        <v>90000</v>
+      </c>
+      <c r="G45" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>427</v>
-      </c>
-      <c r="B46" t="s">
-        <v>29</v>
-      </c>
-      <c r="C46">
-        <v>9</v>
+        <v>431</v>
       </c>
       <c r="D46" t="s">
-        <v>456</v>
-      </c>
-      <c r="F46">
-        <v>120000</v>
-      </c>
-      <c r="G46" t="s">
-        <v>430</v>
+        <v>32</v>
+      </c>
+      <c r="E46">
+        <v>15000</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="D47" t="s">
         <v>31</v>
       </c>
       <c r="E47">
-        <v>20000</v>
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>474</v>
+      </c>
+      <c r="B48" t="s">
+        <v>28</v>
+      </c>
+      <c r="C48">
+        <v>9</v>
+      </c>
+      <c r="D48" t="s">
+        <v>30</v>
+      </c>
+      <c r="H48" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="B50" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C50">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D50" t="s">
-        <v>33</v>
+        <v>456</v>
       </c>
       <c r="F50">
-        <v>90000</v>
-      </c>
-      <c r="M50">
-        <v>20000</v>
+        <v>120000</v>
+      </c>
+      <c r="G50" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>433</v>
-      </c>
-      <c r="B51" t="s">
-        <v>27</v>
-      </c>
-      <c r="C51">
-        <v>11</v>
+        <v>430</v>
       </c>
       <c r="D51" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>441</v>
-      </c>
-      <c r="B52" t="s">
-        <v>27</v>
-      </c>
-      <c r="C52">
-        <v>11</v>
-      </c>
-      <c r="D52" t="s">
-        <v>456</v>
-      </c>
-      <c r="E52">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>437</v>
-      </c>
-      <c r="D53" t="s">
         <v>31</v>
       </c>
-      <c r="E53">
-        <v>15000</v>
-      </c>
-      <c r="F53">
-        <v>120000</v>
+      <c r="E51">
+        <v>20000</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B54" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C54">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D54" t="s">
         <v>33</v>
@@ -7746,100 +7773,209 @@
         <v>90000</v>
       </c>
       <c r="M54">
-        <v>15000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B55" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C55">
         <v>11</v>
       </c>
       <c r="D55" t="s">
-        <v>33</v>
-      </c>
-      <c r="F55">
-        <v>120000</v>
-      </c>
-      <c r="M55">
-        <v>6000</v>
+        <v>456</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>441</v>
+      </c>
+      <c r="B56" t="s">
+        <v>27</v>
+      </c>
+      <c r="C56">
+        <v>11</v>
+      </c>
+      <c r="D56" t="s">
+        <v>456</v>
+      </c>
+      <c r="E56">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>437</v>
+      </c>
+      <c r="D57" t="s">
+        <v>31</v>
+      </c>
+      <c r="E57">
+        <v>15000</v>
+      </c>
+      <c r="F57">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>432</v>
+      </c>
+      <c r="B58" t="s">
+        <v>28</v>
+      </c>
+      <c r="C58">
+        <v>11</v>
+      </c>
+      <c r="D58" t="s">
+        <v>33</v>
+      </c>
+      <c r="F58">
+        <v>90000</v>
+      </c>
+      <c r="M58">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>434</v>
+      </c>
+      <c r="B59" t="s">
+        <v>29</v>
+      </c>
+      <c r="C59">
+        <v>11</v>
+      </c>
+      <c r="D59" t="s">
+        <v>33</v>
+      </c>
+      <c r="F59">
+        <v>120000</v>
+      </c>
+      <c r="M59">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>436</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B60" t="s">
         <v>28</v>
       </c>
-      <c r="C56">
+      <c r="C60">
         <v>12</v>
       </c>
-      <c r="D56" t="s">
-        <v>33</v>
-      </c>
-      <c r="F56">
+      <c r="D60" t="s">
+        <v>33</v>
+      </c>
+      <c r="F60">
         <v>90000</v>
       </c>
-      <c r="M56">
+      <c r="M60">
         <v>10000</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>379</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B65" t="s">
         <v>27</v>
       </c>
-      <c r="C61">
+      <c r="C65">
         <v>1</v>
       </c>
-      <c r="D61" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+      <c r="D65" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>444</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B66" t="s">
         <v>28</v>
       </c>
-      <c r="C62">
+      <c r="C66">
         <v>1</v>
       </c>
-      <c r="D62" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+      <c r="D66" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>445</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B67" t="s">
         <v>27</v>
       </c>
-      <c r="C63">
+      <c r="C67">
         <v>2</v>
       </c>
-      <c r="D63" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+      <c r="D67" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>443</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B68" t="s">
         <v>28</v>
       </c>
-      <c r="C64">
+      <c r="C68">
         <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>477</v>
+      </c>
+      <c r="G71" t="s">
+        <v>479</v>
+      </c>
+      <c r="H71" t="s">
+        <v>480</v>
+      </c>
+      <c r="K71" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>478</v>
+      </c>
+      <c r="G72" t="s">
+        <v>480</v>
+      </c>
+      <c r="H72" t="s">
+        <v>479</v>
+      </c>
+      <c r="K72" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>479</v>
+      </c>
+      <c r="E73">
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>480</v>
+      </c>
+      <c r="E74">
+        <v>3600000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add opener state and F13-F16 action hotkeys
Expand Monk opener and Perfect Balance logic and adjust Dancer and Scholar burst handling.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA17B238-CB0A-432D-B85C-E31A8C8F41E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A901785-EADC-44A0-B42B-30FBB992F11D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14160" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="497">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1438,9 +1438,6 @@
     <t>Besoin d egérer les charges … Pour le moment Perfect balance reste le seul truc manuel</t>
   </si>
   <si>
-    <t>Balance Buff 3</t>
-  </si>
-  <si>
     <t>Forbidden Meditation</t>
   </si>
   <si>
@@ -1513,9 +1510,6 @@
     <t>Finisher Buff;Force Lunar Buff;Force Solar Buff</t>
   </si>
   <si>
-    <t>Opo-opo Form;Raptor form;Coeurl Form</t>
-  </si>
-  <si>
     <t>Activate Burst</t>
   </si>
   <si>
@@ -1529,6 +1523,18 @@
   </si>
   <si>
     <t>Pot</t>
+  </si>
+  <si>
+    <t>Recent Balance</t>
+  </si>
+  <si>
+    <t>Formless Fist;Recent Balance</t>
+  </si>
+  <si>
+    <t>In Second Balance</t>
+  </si>
+  <si>
+    <t>Opo-opo Form;Raptor Form;Coeurl Form</t>
   </si>
 </sst>
 </file>
@@ -1936,19 +1942,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -1974,7 +1980,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -1985,31 +1991,31 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>488</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" t="s">
         <v>490</v>
       </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D4" t="s">
         <v>33</v>
       </c>
       <c r="G4" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -2018,7 +2024,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>0</v>
       </c>
@@ -2038,7 +2044,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>1</v>
       </c>
@@ -2049,7 +2055,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
         <v>43</v>
       </c>
@@ -2072,7 +2078,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>2</v>
       </c>
@@ -2083,7 +2089,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>3</v>
       </c>
@@ -2103,7 +2109,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>41</v>
       </c>
@@ -2114,7 +2120,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
         <v>40</v>
       </c>
@@ -2134,7 +2140,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
         <v>4</v>
       </c>
@@ -2145,7 +2151,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
         <v>5</v>
       </c>
@@ -2165,7 +2171,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
         <v>6</v>
       </c>
@@ -2176,7 +2182,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
         <v>7</v>
       </c>
@@ -2193,7 +2199,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
         <v>374</v>
       </c>
@@ -2213,7 +2219,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
         <v>373</v>
       </c>
@@ -2227,7 +2233,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
         <v>372</v>
       </c>
@@ -2247,7 +2253,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>8</v>
       </c>
@@ -2258,7 +2264,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>9</v>
       </c>
@@ -2275,7 +2281,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
         <v>371</v>
       </c>
@@ -2289,7 +2295,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
         <v>48</v>
       </c>
@@ -2309,10 +2315,10 @@
         <v>50</v>
       </c>
       <c r="H23" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
         <v>49</v>
       </c>
@@ -2323,7 +2329,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="s">
         <v>11</v>
       </c>
@@ -2334,7 +2340,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
         <v>10</v>
       </c>
@@ -2351,7 +2357,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
         <v>12</v>
       </c>
@@ -2371,7 +2377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
         <v>13</v>
       </c>
@@ -2382,7 +2388,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
         <v>14</v>
       </c>
@@ -2402,7 +2408,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="s">
         <v>15</v>
       </c>
@@ -2413,7 +2419,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
         <v>44</v>
       </c>
@@ -2433,7 +2439,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="10" t="s">
         <v>45</v>
       </c>
@@ -2444,7 +2450,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="s">
         <v>46</v>
       </c>
@@ -2464,7 +2470,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
         <v>16</v>
       </c>
@@ -2475,7 +2481,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
         <v>17</v>
       </c>
@@ -2495,7 +2501,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="s">
         <v>18</v>
       </c>
@@ -2506,7 +2512,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="s">
         <v>19</v>
       </c>
@@ -2523,7 +2529,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="11" t="s">
         <v>20</v>
       </c>
@@ -2540,7 +2546,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="11" t="s">
         <v>21</v>
       </c>
@@ -2557,7 +2563,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="11" t="s">
         <v>22</v>
       </c>
@@ -2571,7 +2577,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>23</v>
       </c>
@@ -2585,7 +2591,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>80</v>
       </c>
@@ -2599,7 +2605,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>379</v>
       </c>
@@ -2619,7 +2625,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>380</v>
       </c>
@@ -2645,16 +2651,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7762502F-9F7A-4AD9-AC88-345A2195334F}">
   <dimension ref="A1:I40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -2683,7 +2689,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -2694,31 +2700,31 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>488</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" t="s">
         <v>490</v>
       </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D4" t="s">
         <v>33</v>
       </c>
       <c r="G4" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -2727,7 +2733,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -2747,7 +2753,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>52</v>
       </c>
@@ -2758,7 +2764,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -2778,7 +2784,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -2789,7 +2795,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>55</v>
       </c>
@@ -2809,7 +2815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>56</v>
       </c>
@@ -2832,7 +2838,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -2843,7 +2849,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>57</v>
       </c>
@@ -2860,7 +2866,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>58</v>
       </c>
@@ -2883,7 +2889,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>59</v>
       </c>
@@ -2909,7 +2915,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>87</v>
       </c>
@@ -2920,7 +2926,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>60</v>
       </c>
@@ -2940,7 +2946,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>61</v>
       </c>
@@ -2951,7 +2957,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -2971,7 +2977,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>90</v>
       </c>
@@ -2982,7 +2988,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>95</v>
       </c>
@@ -2999,7 +3005,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>63</v>
       </c>
@@ -3025,7 +3031,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>64</v>
       </c>
@@ -3036,7 +3042,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -3053,7 +3059,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>66</v>
       </c>
@@ -3064,7 +3070,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -3084,7 +3090,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -3095,7 +3101,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>69</v>
       </c>
@@ -3112,7 +3118,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>70</v>
       </c>
@@ -3123,7 +3129,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>71</v>
       </c>
@@ -3143,7 +3149,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>84</v>
       </c>
@@ -3154,7 +3160,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>72</v>
       </c>
@@ -3171,7 +3177,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>73</v>
       </c>
@@ -3188,7 +3194,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>74</v>
       </c>
@@ -3205,7 +3211,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>75</v>
       </c>
@@ -3225,7 +3231,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>76</v>
       </c>
@@ -3245,7 +3251,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>78</v>
       </c>
@@ -3256,7 +3262,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>88</v>
       </c>
@@ -3267,7 +3273,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>77</v>
       </c>
@@ -3284,7 +3290,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>79</v>
       </c>
@@ -3312,19 +3318,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0983F4B6-DA2C-422A-9A48-B565C13F35E9}">
   <dimension ref="A1:M41"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.1796875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -3359,7 +3365,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -3378,7 +3384,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -3389,31 +3395,31 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>488</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
         <v>490</v>
       </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D5" t="s">
         <v>33</v>
       </c>
       <c r="G5" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D6" t="s">
         <v>31</v>
@@ -3422,7 +3428,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>197</v>
       </c>
@@ -3439,7 +3445,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>199</v>
       </c>
@@ -3450,7 +3456,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>198</v>
       </c>
@@ -3470,7 +3476,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>201</v>
       </c>
@@ -3481,7 +3487,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>200</v>
       </c>
@@ -3501,7 +3507,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>229</v>
       </c>
@@ -3518,7 +3524,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>204</v>
       </c>
@@ -3535,7 +3541,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>202</v>
       </c>
@@ -3564,7 +3570,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>222</v>
       </c>
@@ -3575,7 +3581,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>227</v>
       </c>
@@ -3592,7 +3598,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>206</v>
       </c>
@@ -3609,7 +3615,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>223</v>
       </c>
@@ -3626,7 +3632,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>224</v>
       </c>
@@ -3643,7 +3649,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>205</v>
       </c>
@@ -3660,7 +3666,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>208</v>
       </c>
@@ -3674,7 +3680,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>209</v>
       </c>
@@ -3688,7 +3694,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>210</v>
       </c>
@@ -3702,7 +3708,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>211</v>
       </c>
@@ -3725,7 +3731,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>212</v>
       </c>
@@ -3736,7 +3742,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>213</v>
       </c>
@@ -3753,7 +3759,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>214</v>
       </c>
@@ -3764,7 +3770,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>215</v>
       </c>
@@ -3775,7 +3781,7 @@
         <v>24000</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>216</v>
       </c>
@@ -3795,7 +3801,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>218</v>
       </c>
@@ -3806,7 +3812,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>217</v>
       </c>
@@ -3823,7 +3829,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>219</v>
       </c>
@@ -3846,7 +3852,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>207</v>
       </c>
@@ -3866,7 +3872,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>220</v>
       </c>
@@ -3889,7 +3895,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>225</v>
       </c>
@@ -3908,16 +3914,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E11AA6E-3A21-4E4D-BBE2-CBF8D1A645C0}">
   <dimension ref="A1:M96"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -3949,7 +3955,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="I2" t="s">
         <v>102</v>
       </c>
@@ -3957,7 +3963,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -3968,31 +3974,31 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
         <v>490</v>
       </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -4001,7 +4007,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>104</v>
       </c>
@@ -4018,7 +4024,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>106</v>
       </c>
@@ -4038,7 +4044,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>108</v>
       </c>
@@ -4052,7 +4058,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>109</v>
       </c>
@@ -4066,7 +4072,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>110</v>
       </c>
@@ -4080,7 +4086,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>111</v>
       </c>
@@ -4097,7 +4103,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>112</v>
       </c>
@@ -4114,7 +4120,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>114</v>
       </c>
@@ -4131,7 +4137,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>115</v>
       </c>
@@ -4148,7 +4154,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>116</v>
       </c>
@@ -4174,7 +4180,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>119</v>
       </c>
@@ -4197,7 +4203,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>120</v>
       </c>
@@ -4217,7 +4223,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>122</v>
       </c>
@@ -4237,7 +4243,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>117</v>
       </c>
@@ -4248,7 +4254,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>123</v>
       </c>
@@ -4265,7 +4271,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>124</v>
       </c>
@@ -4279,7 +4285,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>126</v>
       </c>
@@ -4299,7 +4305,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>129</v>
       </c>
@@ -4319,7 +4325,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
         <v>131</v>
       </c>
@@ -4339,7 +4345,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>133</v>
       </c>
@@ -4350,7 +4356,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>134</v>
       </c>
@@ -4361,7 +4367,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
         <v>135</v>
       </c>
@@ -4372,7 +4378,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>136</v>
       </c>
@@ -4383,7 +4389,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>137</v>
       </c>
@@ -4400,7 +4406,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>138</v>
       </c>
@@ -4417,7 +4423,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="s">
         <v>139</v>
       </c>
@@ -4434,7 +4440,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>140</v>
       </c>
@@ -4445,7 +4451,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>141</v>
       </c>
@@ -4462,7 +4468,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
         <v>142</v>
       </c>
@@ -4482,7 +4488,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
         <v>144</v>
       </c>
@@ -4499,7 +4505,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
         <v>145</v>
       </c>
@@ -4510,7 +4516,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
         <v>146</v>
       </c>
@@ -4530,7 +4536,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
         <v>147</v>
       </c>
@@ -4541,7 +4547,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>148</v>
       </c>
@@ -4564,7 +4570,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>151</v>
       </c>
@@ -4575,7 +4581,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
         <v>152</v>
       </c>
@@ -4586,7 +4592,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="6" t="s">
         <v>153</v>
       </c>
@@ -4609,7 +4615,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
         <v>154</v>
       </c>
@@ -4620,7 +4626,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="7" t="s">
         <v>156</v>
       </c>
@@ -4631,7 +4637,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="7" t="s">
         <v>157</v>
       </c>
@@ -4654,7 +4660,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" s="7" t="s">
         <v>160</v>
       </c>
@@ -4665,7 +4671,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>161</v>
       </c>
@@ -4679,7 +4685,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
         <v>162</v>
       </c>
@@ -4702,7 +4708,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A66" s="6" t="s">
         <v>164</v>
       </c>
@@ -4725,7 +4731,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A67" s="7" t="s">
         <v>166</v>
       </c>
@@ -4745,7 +4751,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>167</v>
       </c>
@@ -4759,7 +4765,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
         <v>168</v>
       </c>
@@ -4782,7 +4788,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A71" s="6" t="s">
         <v>169</v>
       </c>
@@ -4805,7 +4811,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A72" s="7" t="s">
         <v>170</v>
       </c>
@@ -4825,12 +4831,12 @@
         <v>370</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
         <v>172</v>
       </c>
@@ -4841,7 +4847,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
         <v>173</v>
       </c>
@@ -4861,7 +4867,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
         <v>174</v>
       </c>
@@ -4872,7 +4878,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
         <v>175</v>
       </c>
@@ -4889,7 +4895,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A79" s="6" t="s">
         <v>165</v>
       </c>
@@ -4900,7 +4906,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A80" s="6" t="s">
         <v>176</v>
       </c>
@@ -4917,7 +4923,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="7" t="s">
         <v>177</v>
       </c>
@@ -4928,7 +4934,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" s="7" t="s">
         <v>178</v>
       </c>
@@ -4945,7 +4951,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>180</v>
       </c>
@@ -4965,10 +4971,10 @@
         <v>181</v>
       </c>
       <c r="H84" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>182</v>
       </c>
@@ -4979,7 +4985,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>183</v>
       </c>
@@ -4990,7 +4996,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>184</v>
       </c>
@@ -5007,7 +5013,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>185</v>
       </c>
@@ -5027,7 +5033,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>105</v>
       </c>
@@ -5038,7 +5044,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>186</v>
       </c>
@@ -5052,7 +5058,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>187</v>
       </c>
@@ -5069,7 +5075,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>188</v>
       </c>
@@ -5086,7 +5092,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>189</v>
       </c>
@@ -5103,7 +5109,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>190</v>
       </c>
@@ -5117,7 +5123,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>191</v>
       </c>
@@ -5139,13 +5145,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF394502-4A59-4E3D-B4CF-5A5D5E1CBE54}">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -5174,12 +5180,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="I2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -5190,31 +5196,31 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
         <v>490</v>
       </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -5223,7 +5229,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>192</v>
       </c>
@@ -5236,14 +5242,11 @@
       <c r="D9" t="s">
         <v>30</v>
       </c>
-      <c r="F9">
-        <v>28500</v>
-      </c>
       <c r="G9" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>367</v>
       </c>
@@ -5254,7 +5257,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>193</v>
       </c>
@@ -5268,7 +5271,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>194</v>
       </c>
@@ -5282,7 +5285,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>382</v>
       </c>
@@ -5296,7 +5299,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>195</v>
       </c>
@@ -5316,7 +5319,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>368</v>
       </c>
@@ -5327,7 +5330,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>364</v>
       </c>
@@ -5338,7 +5341,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>196</v>
       </c>
@@ -5355,7 +5358,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>190</v>
       </c>
@@ -5372,7 +5375,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>365</v>
       </c>
@@ -5392,7 +5395,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>116</v>
       </c>
@@ -5409,7 +5412,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>366</v>
       </c>
@@ -5429,7 +5432,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>383</v>
       </c>
@@ -5451,18 +5454,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD84FEA-D0D3-4F98-B644-3E9C52C4A2B7}">
   <dimension ref="A1:M55"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" customWidth="1"/>
-    <col min="10" max="10" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.453125" customWidth="1"/>
+    <col min="6" max="6" width="13.54296875" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" customWidth="1"/>
+    <col min="10" max="10" width="18.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -5503,7 +5506,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="K2" t="s">
         <v>303</v>
       </c>
@@ -5514,7 +5517,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -5525,31 +5528,31 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
         <v>490</v>
       </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -5558,7 +5561,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>292</v>
       </c>
@@ -5578,7 +5581,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>356</v>
       </c>
@@ -5595,7 +5598,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>293</v>
       </c>
@@ -5618,7 +5621,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>297</v>
       </c>
@@ -5641,7 +5644,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>342</v>
       </c>
@@ -5658,7 +5661,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>298</v>
       </c>
@@ -5681,7 +5684,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>301</v>
       </c>
@@ -5695,7 +5698,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>302</v>
       </c>
@@ -5715,7 +5718,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>344</v>
       </c>
@@ -5723,7 +5726,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>299</v>
       </c>
@@ -5737,7 +5740,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>345</v>
       </c>
@@ -5745,7 +5748,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>300</v>
       </c>
@@ -5759,7 +5762,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>294</v>
       </c>
@@ -5782,7 +5785,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>346</v>
       </c>
@@ -5796,7 +5799,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>295</v>
       </c>
@@ -5819,7 +5822,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>347</v>
       </c>
@@ -5833,7 +5836,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>296</v>
       </c>
@@ -5856,7 +5859,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>361</v>
       </c>
@@ -5885,7 +5888,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>349</v>
       </c>
@@ -5899,7 +5902,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>303</v>
       </c>
@@ -5916,7 +5919,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>362</v>
       </c>
@@ -5945,7 +5948,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>350</v>
       </c>
@@ -5959,7 +5962,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>324</v>
       </c>
@@ -5982,7 +5985,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>304</v>
       </c>
@@ -6005,7 +6008,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>305</v>
       </c>
@@ -6028,7 +6031,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>363</v>
       </c>
@@ -6057,7 +6060,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>351</v>
       </c>
@@ -6071,7 +6074,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>306</v>
       </c>
@@ -6085,7 +6088,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>308</v>
       </c>
@@ -6111,7 +6114,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>340</v>
       </c>
@@ -6122,7 +6125,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>311</v>
       </c>
@@ -6148,7 +6151,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>337</v>
       </c>
@@ -6159,7 +6162,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>309</v>
       </c>
@@ -6185,7 +6188,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>338</v>
       </c>
@@ -6196,7 +6199,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>312</v>
       </c>
@@ -6222,7 +6225,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>339</v>
       </c>
@@ -6233,7 +6236,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>310</v>
       </c>
@@ -6256,7 +6259,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>307</v>
       </c>
@@ -6288,17 +6291,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
   <dimension ref="A1:P72"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" customWidth="1"/>
-    <col min="3" max="3" width="6.140625" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7265625" customWidth="1"/>
+    <col min="3" max="3" width="6.1796875" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="59" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -6330,7 +6333,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="I2" t="s">
         <v>259</v>
       </c>
@@ -6338,7 +6341,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -6349,31 +6352,31 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
         <v>490</v>
       </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -6382,7 +6385,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>230</v>
       </c>
@@ -6399,7 +6402,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>233</v>
       </c>
@@ -6416,7 +6419,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>232</v>
       </c>
@@ -6427,7 +6430,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>231</v>
       </c>
@@ -6444,7 +6447,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>234</v>
       </c>
@@ -6461,7 +6464,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>247</v>
       </c>
@@ -6472,7 +6475,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>283</v>
       </c>
@@ -6483,7 +6486,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>235</v>
       </c>
@@ -6500,7 +6503,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>237</v>
       </c>
@@ -6520,7 +6523,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>248</v>
       </c>
@@ -6531,7 +6534,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>284</v>
       </c>
@@ -6542,7 +6545,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>236</v>
       </c>
@@ -6559,7 +6562,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>238</v>
       </c>
@@ -6576,7 +6579,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>265</v>
       </c>
@@ -6596,7 +6599,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>286</v>
       </c>
@@ -6613,7 +6616,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>266</v>
       </c>
@@ -6624,7 +6627,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>267</v>
       </c>
@@ -6644,7 +6647,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>271</v>
       </c>
@@ -6658,7 +6661,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>269</v>
       </c>
@@ -6672,7 +6675,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>275</v>
       </c>
@@ -6683,7 +6686,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>251</v>
       </c>
@@ -6694,7 +6697,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>252</v>
       </c>
@@ -6711,7 +6714,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>249</v>
       </c>
@@ -6728,10 +6731,10 @@
         <v>280</v>
       </c>
       <c r="H34" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>250</v>
       </c>
@@ -6742,7 +6745,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>253</v>
       </c>
@@ -6765,7 +6768,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>273</v>
       </c>
@@ -6779,7 +6782,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>274</v>
       </c>
@@ -6793,7 +6796,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>270</v>
       </c>
@@ -6807,7 +6810,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>268</v>
       </c>
@@ -6821,7 +6824,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>272</v>
       </c>
@@ -6832,7 +6835,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>277</v>
       </c>
@@ -6843,7 +6846,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>260</v>
       </c>
@@ -6854,7 +6857,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>261</v>
       </c>
@@ -6871,7 +6874,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>254</v>
       </c>
@@ -6888,7 +6891,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>255</v>
       </c>
@@ -6905,7 +6908,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>256</v>
       </c>
@@ -6922,7 +6925,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>257</v>
       </c>
@@ -6939,7 +6942,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>239</v>
       </c>
@@ -6962,7 +6965,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>240</v>
       </c>
@@ -6982,7 +6985,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>262</v>
       </c>
@@ -6993,7 +6996,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>241</v>
       </c>
@@ -7013,7 +7016,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>263</v>
       </c>
@@ -7024,7 +7027,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>242</v>
       </c>
@@ -7044,7 +7047,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>243</v>
       </c>
@@ -7061,7 +7064,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>289</v>
       </c>
@@ -7072,7 +7075,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>288</v>
       </c>
@@ -7092,7 +7095,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>279</v>
       </c>
@@ -7112,7 +7115,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>244</v>
       </c>
@@ -7123,7 +7126,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>246</v>
       </c>
@@ -7134,7 +7137,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>245</v>
       </c>
@@ -7151,7 +7154,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>264</v>
       </c>
@@ -7171,7 +7174,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>285</v>
       </c>
@@ -7182,7 +7185,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>384</v>
       </c>
@@ -7199,7 +7202,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>386</v>
       </c>
@@ -7210,7 +7213,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>385</v>
       </c>
@@ -7235,18 +7238,18 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3261DB23-C434-4F35-8B4F-998D4295A585}">
-  <dimension ref="A1:P80"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P81"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="42.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="42.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.453125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -7281,12 +7284,12 @@
         <v>313</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="I2" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -7300,25 +7303,25 @@
         <v>445</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>488</v>
+      </c>
+      <c r="H4" t="s">
         <v>490</v>
       </c>
-      <c r="H4" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="G5" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D6" t="s">
         <v>31</v>
@@ -7327,15 +7330,15 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B7" t="s">
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="D7" t="s">
         <v>33</v>
@@ -7344,7 +7347,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>446</v>
       </c>
@@ -7355,7 +7358,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>458</v>
       </c>
@@ -7366,7 +7369,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>387</v>
       </c>
@@ -7383,7 +7386,7 @@
         <v>447</v>
       </c>
       <c r="H11" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="K11" t="s">
         <v>395</v>
@@ -7392,7 +7395,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>388</v>
       </c>
@@ -7409,7 +7412,7 @@
         <v>461</v>
       </c>
       <c r="H12" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="K12" t="s">
         <v>396</v>
@@ -7421,7 +7424,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>389</v>
       </c>
@@ -7438,13 +7441,13 @@
         <v>447</v>
       </c>
       <c r="H13" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="K13" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>447</v>
       </c>
@@ -7455,7 +7458,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>459</v>
       </c>
@@ -7466,7 +7469,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>390</v>
       </c>
@@ -7483,7 +7486,7 @@
         <v>448</v>
       </c>
       <c r="H17" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="K17" t="s">
         <v>399</v>
@@ -7492,7 +7495,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>391</v>
       </c>
@@ -7509,7 +7512,7 @@
         <v>462</v>
       </c>
       <c r="H18" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="K18" t="s">
         <v>400</v>
@@ -7518,7 +7521,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>393</v>
       </c>
@@ -7535,13 +7538,13 @@
         <v>448</v>
       </c>
       <c r="H19" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="K19" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>448</v>
       </c>
@@ -7552,7 +7555,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>394</v>
       </c>
@@ -7569,7 +7572,7 @@
         <v>446</v>
       </c>
       <c r="H22" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="I22">
         <v>-1</v>
@@ -7578,7 +7581,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>392</v>
       </c>
@@ -7595,7 +7598,7 @@
         <v>446</v>
       </c>
       <c r="H23" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="I23">
         <v>2</v>
@@ -7607,7 +7610,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>398</v>
       </c>
@@ -7624,13 +7627,13 @@
         <v>446</v>
       </c>
       <c r="H24" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="K24" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>411</v>
       </c>
@@ -7654,9 +7657,9 @@
         <v>413</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B27" t="s">
         <v>27</v>
@@ -7677,9 +7680,9 @@
         <v>413</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B28" t="s">
         <v>27</v>
@@ -7694,7 +7697,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>405</v>
       </c>
@@ -7717,7 +7720,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>406</v>
       </c>
@@ -7734,12 +7737,12 @@
         <v>408</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="N31" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>414</v>
       </c>
@@ -7753,10 +7756,10 @@
         <v>33</v>
       </c>
       <c r="G32" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="H32" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
       <c r="K32" t="s">
         <v>415</v>
@@ -7765,9 +7768,9 @@
         <v>416</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D33" t="s">
         <v>31</v>
@@ -7779,9 +7782,9 @@
         <v>463</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D34" t="s">
         <v>31</v>
@@ -7790,31 +7793,31 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+        <v>493</v>
+      </c>
+      <c r="D35" t="s">
+        <v>31</v>
+      </c>
+      <c r="E35">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
+        <v>495</v>
+      </c>
+      <c r="D36" t="s">
+        <v>31</v>
+      </c>
+      <c r="E36">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>422</v>
-      </c>
-      <c r="B36" t="s">
-        <v>28</v>
-      </c>
-      <c r="C36">
-        <v>8</v>
-      </c>
-      <c r="D36" t="s">
-        <v>30</v>
-      </c>
-      <c r="N36" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>475</v>
       </c>
       <c r="B37" t="s">
         <v>28</v>
@@ -7825,16 +7828,13 @@
       <c r="D37" t="s">
         <v>30</v>
       </c>
-      <c r="G37" t="s">
-        <v>482</v>
-      </c>
-      <c r="H37" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N37" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B38" t="s">
         <v>28</v>
@@ -7846,15 +7846,15 @@
         <v>30</v>
       </c>
       <c r="G38" t="s">
-        <v>482</v>
+        <v>494</v>
       </c>
       <c r="H38" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B39" t="s">
         <v>28</v>
@@ -7866,15 +7866,15 @@
         <v>30</v>
       </c>
       <c r="G39" t="s">
-        <v>482</v>
+        <v>494</v>
       </c>
       <c r="H39" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B40" t="s">
         <v>28</v>
@@ -7886,255 +7886,258 @@
         <v>30</v>
       </c>
       <c r="G40" t="s">
-        <v>482</v>
+        <v>494</v>
       </c>
       <c r="H40" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>473</v>
+      </c>
+      <c r="B41" t="s">
+        <v>28</v>
+      </c>
+      <c r="C41">
+        <v>8</v>
+      </c>
+      <c r="D41" t="s">
+        <v>30</v>
+      </c>
+      <c r="G41" t="s">
+        <v>494</v>
+      </c>
+      <c r="H41" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>423</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>29</v>
       </c>
-      <c r="C42">
+      <c r="C43">
         <v>8</v>
       </c>
-      <c r="D42" t="s">
-        <v>30</v>
-      </c>
-      <c r="G42" t="s">
-        <v>482</v>
-      </c>
-      <c r="K42" t="s">
+      <c r="D43" t="s">
+        <v>30</v>
+      </c>
+      <c r="G43" t="s">
+        <v>481</v>
+      </c>
+      <c r="K43" t="s">
         <v>424</v>
       </c>
-      <c r="N42" t="s">
+      <c r="N43" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>482</v>
-      </c>
-      <c r="D43" t="s">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>481</v>
+      </c>
+      <c r="D44" t="s">
         <v>32</v>
       </c>
-      <c r="E43">
+      <c r="E44">
         <v>30000</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="N44" t="s">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="N45" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>420</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B46" t="s">
         <v>27</v>
       </c>
-      <c r="C45">
+      <c r="C46">
         <v>9</v>
       </c>
-      <c r="D45" t="s">
-        <v>33</v>
-      </c>
-      <c r="F45">
+      <c r="D46" t="s">
+        <v>33</v>
+      </c>
+      <c r="F46">
         <v>60000</v>
       </c>
-      <c r="G45" t="s">
-        <v>428</v>
-      </c>
-      <c r="K45" t="s">
+      <c r="G46" t="s">
+        <v>440</v>
+      </c>
+      <c r="K46" t="s">
         <v>425</v>
       </c>
-      <c r="N45" t="s">
-        <v>440</v>
-      </c>
-      <c r="P45" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="P46" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>438</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D47" t="s">
         <v>32</v>
-      </c>
-      <c r="E46">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>428</v>
-      </c>
-      <c r="D47" t="s">
-        <v>31</v>
       </c>
       <c r="E47">
         <v>20000</v>
       </c>
-      <c r="K47" t="s">
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>428</v>
+      </c>
+      <c r="D48" t="s">
+        <v>31</v>
+      </c>
+      <c r="E48">
+        <v>20000</v>
+      </c>
+      <c r="K48" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>469</v>
-      </c>
-      <c r="B48" t="s">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>468</v>
+      </c>
+      <c r="B49" t="s">
         <v>27</v>
-      </c>
-      <c r="C48">
-        <v>9</v>
-      </c>
-      <c r="D48" t="s">
-        <v>30</v>
-      </c>
-      <c r="G48" t="s">
-        <v>482</v>
-      </c>
-      <c r="H48" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>421</v>
-      </c>
-      <c r="B49" t="s">
-        <v>28</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>33</v>
-      </c>
-      <c r="F49">
+        <v>30</v>
+      </c>
+      <c r="G49" t="s">
+        <v>481</v>
+      </c>
+      <c r="H49" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>421</v>
+      </c>
+      <c r="B50" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50">
+        <v>9</v>
+      </c>
+      <c r="D50" t="s">
+        <v>33</v>
+      </c>
+      <c r="F50">
         <v>90000</v>
       </c>
-      <c r="G49" t="s">
+      <c r="G50" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>431</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D51" t="s">
         <v>32</v>
-      </c>
-      <c r="E50">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>429</v>
-      </c>
-      <c r="D51" t="s">
-        <v>31</v>
       </c>
       <c r="E51">
         <v>15000</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>468</v>
-      </c>
-      <c r="B52" t="s">
+        <v>429</v>
+      </c>
+      <c r="D52" t="s">
+        <v>31</v>
+      </c>
+      <c r="E52">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>467</v>
+      </c>
+      <c r="B53" t="s">
         <v>28</v>
       </c>
-      <c r="C52">
+      <c r="C53">
         <v>9</v>
       </c>
-      <c r="D52" t="s">
-        <v>30</v>
-      </c>
-      <c r="H52" t="s">
+      <c r="D53" t="s">
+        <v>30</v>
+      </c>
+      <c r="H53" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>427</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B55" t="s">
         <v>29</v>
       </c>
-      <c r="C54">
+      <c r="C55">
         <v>9</v>
       </c>
-      <c r="D54" t="s">
+      <c r="D55" t="s">
         <v>453</v>
       </c>
-      <c r="F54">
+      <c r="F55">
         <v>120000</v>
       </c>
-      <c r="G54" t="s">
+      <c r="G55" t="s">
         <v>430</v>
       </c>
-      <c r="H54" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="H55" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>430</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D56" t="s">
         <v>31</v>
       </c>
-      <c r="E55">
+      <c r="E56">
         <v>20000</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>435</v>
-      </c>
-      <c r="B58" t="s">
-        <v>27</v>
-      </c>
-      <c r="C58">
-        <v>10</v>
-      </c>
-      <c r="D58" t="s">
-        <v>33</v>
-      </c>
-      <c r="F58">
-        <v>90000</v>
-      </c>
-      <c r="M58">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>433</v>
       </c>
       <c r="B59" t="s">
         <v>27</v>
       </c>
       <c r="C59">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D59" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="F59">
+        <v>90000</v>
+      </c>
+      <c r="M59">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="B60" t="s">
         <v>27</v>
@@ -8145,50 +8148,44 @@
       <c r="D60" t="s">
         <v>453</v>
       </c>
-      <c r="E60">
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>441</v>
+      </c>
+      <c r="B61" t="s">
+        <v>27</v>
+      </c>
+      <c r="C61">
+        <v>11</v>
+      </c>
+      <c r="D61" t="s">
+        <v>453</v>
+      </c>
+      <c r="E61">
         <v>30000</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>437</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D62" t="s">
         <v>31</v>
       </c>
-      <c r="E61">
+      <c r="E62">
         <v>15000</v>
       </c>
-      <c r="F61">
+      <c r="F62">
         <v>120000</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>432</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B63" t="s">
         <v>28</v>
-      </c>
-      <c r="C62">
-        <v>11</v>
-      </c>
-      <c r="D62" t="s">
-        <v>33</v>
-      </c>
-      <c r="F62">
-        <v>90000</v>
-      </c>
-      <c r="M62">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>434</v>
-      </c>
-      <c r="B63" t="s">
-        <v>29</v>
       </c>
       <c r="C63">
         <v>11</v>
@@ -8197,52 +8194,58 @@
         <v>33</v>
       </c>
       <c r="F63">
+        <v>90000</v>
+      </c>
+      <c r="M63">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>434</v>
+      </c>
+      <c r="B64" t="s">
+        <v>29</v>
+      </c>
+      <c r="C64">
+        <v>11</v>
+      </c>
+      <c r="D64" t="s">
+        <v>33</v>
+      </c>
+      <c r="F64">
         <v>120000</v>
       </c>
-      <c r="M63">
+      <c r="M64">
         <v>6000</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>436</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B65" t="s">
         <v>28</v>
       </c>
-      <c r="C64">
+      <c r="C65">
         <v>12</v>
       </c>
-      <c r="D64" t="s">
-        <v>33</v>
-      </c>
-      <c r="F64">
+      <c r="D65" t="s">
+        <v>33</v>
+      </c>
+      <c r="F65">
         <v>90000</v>
       </c>
-      <c r="M64">
+      <c r="M65">
         <v>10000</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>379</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B70" t="s">
         <v>27</v>
-      </c>
-      <c r="C69">
-        <v>1</v>
-      </c>
-      <c r="D69" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>443</v>
-      </c>
-      <c r="B70" t="s">
-        <v>28</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -8251,78 +8254,92 @@
         <v>33</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
+        <v>443</v>
+      </c>
+      <c r="B71" t="s">
+        <v>28</v>
+      </c>
+      <c r="C71">
+        <v>1</v>
+      </c>
+      <c r="D71" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>444</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B72" t="s">
         <v>27</v>
       </c>
-      <c r="C71">
+      <c r="C72">
         <v>2</v>
       </c>
-      <c r="D71" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+      <c r="D72" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>442</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B73" t="s">
         <v>28</v>
       </c>
-      <c r="C72">
+      <c r="C73">
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>484</v>
-      </c>
-      <c r="G75" t="s">
-        <v>486</v>
-      </c>
-      <c r="H75" t="s">
-        <v>487</v>
-      </c>
-      <c r="K75" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
+        <v>483</v>
+      </c>
+      <c r="G76" t="s">
         <v>485</v>
-      </c>
-      <c r="G76" t="s">
-        <v>487</v>
       </c>
       <c r="H76" t="s">
         <v>486</v>
       </c>
       <c r="K76" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
+        <v>484</v>
+      </c>
+      <c r="G77" t="s">
         <v>486</v>
       </c>
-      <c r="E77">
-        <v>3600000</v>
-      </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H77" t="s">
+        <v>485</v>
+      </c>
+      <c r="K77" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="E78">
         <v>3600000</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="L80" t="s">
-        <v>483</v>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>486</v>
+      </c>
+      <c r="E79">
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="81" spans="12:12" x14ac:dyDescent="0.35">
+      <c r="L81" t="s">
+        <v>482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine Monk Perfect Balance transitions
Require the Balance buff for finishers, adjust opener conditions and remove obsolete Nadi helpers.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A901785-EADC-44A0-B42B-30FBB992F11D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6312425-7D8A-43AB-A1BA-A8AF85B33F49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14160" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -1507,9 +1507,6 @@
     <t>Force Solar Buff</t>
   </si>
   <si>
-    <t>Finisher Buff;Force Lunar Buff;Force Solar Buff</t>
-  </si>
-  <si>
     <t>Activate Burst</t>
   </si>
   <si>
@@ -1535,6 +1532,9 @@
   </si>
   <si>
     <t>Opo-opo Form;Raptor Form;Coeurl Form</t>
+  </si>
+  <si>
+    <t>Finisher Buff;Force Lunar Buff;Force Solar Buff;Balance Buff</t>
   </si>
 </sst>
 </file>
@@ -1942,19 +1942,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -1991,31 +1991,31 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>487</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>488</v>
       </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" t="s">
         <v>489</v>
       </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -2024,7 +2024,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>0</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>1</v>
       </c>
@@ -2055,7 +2055,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>43</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>2</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>3</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>41</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>40</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>4</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>5</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>6</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>7</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>374</v>
       </c>
@@ -2219,7 +2219,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>373</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>372</v>
       </c>
@@ -2253,7 +2253,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>8</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>9</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>371</v>
       </c>
@@ -2295,7 +2295,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>48</v>
       </c>
@@ -2315,10 +2315,10 @@
         <v>50</v>
       </c>
       <c r="H23" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>49</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>11</v>
       </c>
@@ -2340,7 +2340,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>10</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>12</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>13</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>14</v>
       </c>
@@ -2408,7 +2408,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>15</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>44</v>
       </c>
@@ -2439,7 +2439,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>45</v>
       </c>
@@ -2450,7 +2450,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>46</v>
       </c>
@@ -2470,7 +2470,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>16</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>17</v>
       </c>
@@ -2501,7 +2501,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>18</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>19</v>
       </c>
@@ -2529,7 +2529,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>20</v>
       </c>
@@ -2546,7 +2546,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>21</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>22</v>
       </c>
@@ -2577,7 +2577,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>23</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>80</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>379</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>380</v>
       </c>
@@ -2651,16 +2651,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7762502F-9F7A-4AD9-AC88-345A2195334F}">
   <dimension ref="A1:I40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -2700,31 +2700,31 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>487</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>488</v>
       </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" t="s">
         <v>489</v>
       </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -2733,7 +2733,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>52</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>55</v>
       </c>
@@ -2815,7 +2815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>56</v>
       </c>
@@ -2838,7 +2838,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>57</v>
       </c>
@@ -2866,7 +2866,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>58</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>59</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>87</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>60</v>
       </c>
@@ -2946,7 +2946,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>61</v>
       </c>
@@ -2957,7 +2957,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>90</v>
       </c>
@@ -2988,7 +2988,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>95</v>
       </c>
@@ -3005,7 +3005,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>63</v>
       </c>
@@ -3031,7 +3031,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>64</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -3059,7 +3059,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>66</v>
       </c>
@@ -3070,7 +3070,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -3090,7 +3090,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -3101,7 +3101,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>69</v>
       </c>
@@ -3118,7 +3118,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>70</v>
       </c>
@@ -3129,7 +3129,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>71</v>
       </c>
@@ -3149,7 +3149,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>84</v>
       </c>
@@ -3160,7 +3160,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>72</v>
       </c>
@@ -3177,7 +3177,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>73</v>
       </c>
@@ -3194,7 +3194,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>74</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>75</v>
       </c>
@@ -3231,7 +3231,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>76</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>78</v>
       </c>
@@ -3262,7 +3262,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>88</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>77</v>
       </c>
@@ -3290,7 +3290,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>79</v>
       </c>
@@ -3318,19 +3318,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0983F4B6-DA2C-422A-9A48-B565C13F35E9}">
   <dimension ref="A1:M41"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="22.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -3365,7 +3365,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -3384,7 +3384,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -3395,31 +3395,31 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>487</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>488</v>
       </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
         <v>489</v>
       </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D6" t="s">
         <v>31</v>
@@ -3428,7 +3428,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>197</v>
       </c>
@@ -3445,7 +3445,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>199</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>198</v>
       </c>
@@ -3476,7 +3476,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>201</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>200</v>
       </c>
@@ -3507,7 +3507,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>229</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>204</v>
       </c>
@@ -3541,7 +3541,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>202</v>
       </c>
@@ -3570,7 +3570,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>222</v>
       </c>
@@ -3581,7 +3581,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>227</v>
       </c>
@@ -3598,7 +3598,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>206</v>
       </c>
@@ -3615,7 +3615,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>223</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>224</v>
       </c>
@@ -3649,7 +3649,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>205</v>
       </c>
@@ -3666,7 +3666,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>208</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>209</v>
       </c>
@@ -3694,7 +3694,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>210</v>
       </c>
@@ -3708,7 +3708,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>211</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>212</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>213</v>
       </c>
@@ -3759,7 +3759,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>214</v>
       </c>
@@ -3770,7 +3770,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>215</v>
       </c>
@@ -3781,7 +3781,7 @@
         <v>24000</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>216</v>
       </c>
@@ -3801,7 +3801,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>218</v>
       </c>
@@ -3812,7 +3812,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>217</v>
       </c>
@@ -3829,7 +3829,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>219</v>
       </c>
@@ -3852,7 +3852,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>207</v>
       </c>
@@ -3872,7 +3872,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>220</v>
       </c>
@@ -3895,7 +3895,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>225</v>
       </c>
@@ -3914,16 +3914,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E11AA6E-3A21-4E4D-BBE2-CBF8D1A645C0}">
   <dimension ref="A1:M96"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -3955,7 +3955,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
         <v>102</v>
       </c>
@@ -3963,7 +3963,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -3974,31 +3974,31 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>488</v>
       </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
         <v>489</v>
       </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -4007,7 +4007,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>104</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>106</v>
       </c>
@@ -4044,7 +4044,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>108</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>109</v>
       </c>
@@ -4072,7 +4072,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>110</v>
       </c>
@@ -4086,7 +4086,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>111</v>
       </c>
@@ -4103,7 +4103,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>112</v>
       </c>
@@ -4120,7 +4120,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>114</v>
       </c>
@@ -4137,7 +4137,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>115</v>
       </c>
@@ -4154,7 +4154,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>116</v>
       </c>
@@ -4180,7 +4180,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>119</v>
       </c>
@@ -4203,7 +4203,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>120</v>
       </c>
@@ -4223,7 +4223,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>122</v>
       </c>
@@ -4243,7 +4243,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>117</v>
       </c>
@@ -4254,7 +4254,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>123</v>
       </c>
@@ -4271,7 +4271,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>124</v>
       </c>
@@ -4285,7 +4285,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>126</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>129</v>
       </c>
@@ -4325,7 +4325,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>131</v>
       </c>
@@ -4345,7 +4345,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>133</v>
       </c>
@@ -4356,7 +4356,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>134</v>
       </c>
@@ -4367,7 +4367,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>135</v>
       </c>
@@ -4378,7 +4378,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>136</v>
       </c>
@@ -4389,7 +4389,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>137</v>
       </c>
@@ -4406,7 +4406,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>138</v>
       </c>
@@ -4423,7 +4423,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>139</v>
       </c>
@@ -4440,7 +4440,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>140</v>
       </c>
@@ -4451,7 +4451,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>141</v>
       </c>
@@ -4468,7 +4468,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>142</v>
       </c>
@@ -4488,7 +4488,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>144</v>
       </c>
@@ -4505,7 +4505,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>145</v>
       </c>
@@ -4516,7 +4516,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
         <v>146</v>
       </c>
@@ -4536,7 +4536,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>147</v>
       </c>
@@ -4547,7 +4547,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>148</v>
       </c>
@@ -4570,7 +4570,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>151</v>
       </c>
@@ -4581,7 +4581,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>152</v>
       </c>
@@ -4592,7 +4592,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>153</v>
       </c>
@@ -4615,7 +4615,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>154</v>
       </c>
@@ -4626,7 +4626,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
         <v>156</v>
       </c>
@@ -4637,7 +4637,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
         <v>157</v>
       </c>
@@ -4660,7 +4660,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>160</v>
       </c>
@@ -4671,7 +4671,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>161</v>
       </c>
@@ -4685,7 +4685,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>162</v>
       </c>
@@ -4708,7 +4708,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>164</v>
       </c>
@@ -4731,7 +4731,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>166</v>
       </c>
@@ -4751,7 +4751,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>167</v>
       </c>
@@ -4765,7 +4765,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>168</v>
       </c>
@@ -4788,7 +4788,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>169</v>
       </c>
@@ -4811,7 +4811,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>170</v>
       </c>
@@ -4831,12 +4831,12 @@
         <v>370</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
         <v>172</v>
       </c>
@@ -4847,7 +4847,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
         <v>173</v>
       </c>
@@ -4867,7 +4867,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
         <v>174</v>
       </c>
@@ -4878,7 +4878,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
         <v>175</v>
       </c>
@@ -4895,7 +4895,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>165</v>
       </c>
@@ -4906,7 +4906,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>176</v>
       </c>
@@ -4923,7 +4923,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
         <v>177</v>
       </c>
@@ -4934,7 +4934,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="7" t="s">
         <v>178</v>
       </c>
@@ -4951,7 +4951,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>180</v>
       </c>
@@ -4971,10 +4971,10 @@
         <v>181</v>
       </c>
       <c r="H84" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>182</v>
       </c>
@@ -4985,7 +4985,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>183</v>
       </c>
@@ -4996,7 +4996,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>184</v>
       </c>
@@ -5013,7 +5013,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>185</v>
       </c>
@@ -5033,7 +5033,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>105</v>
       </c>
@@ -5044,7 +5044,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>186</v>
       </c>
@@ -5058,7 +5058,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>187</v>
       </c>
@@ -5075,7 +5075,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>188</v>
       </c>
@@ -5092,7 +5092,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>189</v>
       </c>
@@ -5109,7 +5109,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>190</v>
       </c>
@@ -5123,7 +5123,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>191</v>
       </c>
@@ -5145,13 +5145,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF394502-4A59-4E3D-B4CF-5A5D5E1CBE54}">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.26953125" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -5180,12 +5180,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -5196,31 +5196,31 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>488</v>
       </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
         <v>489</v>
       </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -5229,7 +5229,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>192</v>
       </c>
@@ -5246,7 +5246,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>367</v>
       </c>
@@ -5257,7 +5257,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>193</v>
       </c>
@@ -5271,7 +5271,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>194</v>
       </c>
@@ -5285,7 +5285,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>382</v>
       </c>
@@ -5299,7 +5299,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>195</v>
       </c>
@@ -5319,7 +5319,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>368</v>
       </c>
@@ -5330,7 +5330,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>364</v>
       </c>
@@ -5341,7 +5341,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>196</v>
       </c>
@@ -5358,7 +5358,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>190</v>
       </c>
@@ -5375,7 +5375,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>365</v>
       </c>
@@ -5395,7 +5395,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>116</v>
       </c>
@@ -5412,7 +5412,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>366</v>
       </c>
@@ -5432,7 +5432,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>383</v>
       </c>
@@ -5454,18 +5454,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD84FEA-D0D3-4F98-B644-3E9C52C4A2B7}">
   <dimension ref="A1:M55"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.453125" customWidth="1"/>
-    <col min="6" max="6" width="13.54296875" customWidth="1"/>
-    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.1796875" customWidth="1"/>
-    <col min="10" max="10" width="18.54296875" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -5506,7 +5506,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K2" t="s">
         <v>303</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -5528,31 +5528,31 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>488</v>
       </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
         <v>489</v>
       </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -5561,7 +5561,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>292</v>
       </c>
@@ -5581,7 +5581,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>356</v>
       </c>
@@ -5598,7 +5598,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>293</v>
       </c>
@@ -5621,7 +5621,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>297</v>
       </c>
@@ -5644,7 +5644,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>342</v>
       </c>
@@ -5661,7 +5661,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>298</v>
       </c>
@@ -5684,7 +5684,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>301</v>
       </c>
@@ -5698,7 +5698,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>302</v>
       </c>
@@ -5718,7 +5718,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>344</v>
       </c>
@@ -5726,7 +5726,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>299</v>
       </c>
@@ -5740,7 +5740,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>345</v>
       </c>
@@ -5748,7 +5748,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>300</v>
       </c>
@@ -5762,7 +5762,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>294</v>
       </c>
@@ -5785,7 +5785,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>346</v>
       </c>
@@ -5799,7 +5799,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>295</v>
       </c>
@@ -5822,7 +5822,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>347</v>
       </c>
@@ -5836,7 +5836,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>296</v>
       </c>
@@ -5859,7 +5859,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>361</v>
       </c>
@@ -5888,7 +5888,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>349</v>
       </c>
@@ -5902,7 +5902,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>303</v>
       </c>
@@ -5919,7 +5919,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>362</v>
       </c>
@@ -5948,7 +5948,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>350</v>
       </c>
@@ -5962,7 +5962,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>324</v>
       </c>
@@ -5985,7 +5985,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>304</v>
       </c>
@@ -6008,7 +6008,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>305</v>
       </c>
@@ -6031,7 +6031,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>363</v>
       </c>
@@ -6060,7 +6060,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>351</v>
       </c>
@@ -6074,7 +6074,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>306</v>
       </c>
@@ -6088,7 +6088,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>308</v>
       </c>
@@ -6114,7 +6114,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>340</v>
       </c>
@@ -6125,7 +6125,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>311</v>
       </c>
@@ -6151,7 +6151,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>337</v>
       </c>
@@ -6162,7 +6162,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>309</v>
       </c>
@@ -6188,7 +6188,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>338</v>
       </c>
@@ -6199,7 +6199,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>312</v>
       </c>
@@ -6225,7 +6225,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>339</v>
       </c>
@@ -6236,7 +6236,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>310</v>
       </c>
@@ -6259,7 +6259,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>307</v>
       </c>
@@ -6291,17 +6291,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
   <dimension ref="A1:P72"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.7265625" customWidth="1"/>
-    <col min="3" max="3" width="6.1796875" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" customWidth="1"/>
+    <col min="3" max="3" width="6.140625" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="59" customWidth="1"/>
-    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -6333,7 +6333,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
         <v>259</v>
       </c>
@@ -6341,7 +6341,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -6352,31 +6352,31 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>488</v>
       </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
         <v>489</v>
       </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -6385,7 +6385,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>230</v>
       </c>
@@ -6402,7 +6402,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>233</v>
       </c>
@@ -6419,7 +6419,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>232</v>
       </c>
@@ -6430,7 +6430,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>231</v>
       </c>
@@ -6447,7 +6447,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>234</v>
       </c>
@@ -6464,7 +6464,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>247</v>
       </c>
@@ -6475,7 +6475,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>283</v>
       </c>
@@ -6486,7 +6486,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>235</v>
       </c>
@@ -6503,7 +6503,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>237</v>
       </c>
@@ -6523,7 +6523,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>248</v>
       </c>
@@ -6534,7 +6534,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>284</v>
       </c>
@@ -6545,7 +6545,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>236</v>
       </c>
@@ -6562,7 +6562,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>238</v>
       </c>
@@ -6579,7 +6579,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>265</v>
       </c>
@@ -6599,7 +6599,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>286</v>
       </c>
@@ -6616,7 +6616,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>266</v>
       </c>
@@ -6627,7 +6627,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>267</v>
       </c>
@@ -6647,7 +6647,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>271</v>
       </c>
@@ -6661,7 +6661,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>269</v>
       </c>
@@ -6675,7 +6675,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>275</v>
       </c>
@@ -6686,7 +6686,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>251</v>
       </c>
@@ -6697,7 +6697,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>252</v>
       </c>
@@ -6714,7 +6714,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>249</v>
       </c>
@@ -6731,10 +6731,10 @@
         <v>280</v>
       </c>
       <c r="H34" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>250</v>
       </c>
@@ -6745,7 +6745,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>253</v>
       </c>
@@ -6768,7 +6768,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>273</v>
       </c>
@@ -6782,7 +6782,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>274</v>
       </c>
@@ -6796,7 +6796,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>270</v>
       </c>
@@ -6810,7 +6810,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>268</v>
       </c>
@@ -6824,7 +6824,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>272</v>
       </c>
@@ -6835,7 +6835,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>277</v>
       </c>
@@ -6846,7 +6846,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>260</v>
       </c>
@@ -6857,7 +6857,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>261</v>
       </c>
@@ -6874,7 +6874,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>254</v>
       </c>
@@ -6891,7 +6891,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>255</v>
       </c>
@@ -6908,7 +6908,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>256</v>
       </c>
@@ -6925,7 +6925,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>257</v>
       </c>
@@ -6942,7 +6942,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>239</v>
       </c>
@@ -6965,7 +6965,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>240</v>
       </c>
@@ -6985,7 +6985,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>262</v>
       </c>
@@ -6996,7 +6996,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>241</v>
       </c>
@@ -7016,7 +7016,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>263</v>
       </c>
@@ -7027,7 +7027,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>242</v>
       </c>
@@ -7047,7 +7047,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>243</v>
       </c>
@@ -7064,7 +7064,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>289</v>
       </c>
@@ -7075,7 +7075,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>288</v>
       </c>
@@ -7095,7 +7095,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>279</v>
       </c>
@@ -7115,7 +7115,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>244</v>
       </c>
@@ -7126,7 +7126,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>246</v>
       </c>
@@ -7137,7 +7137,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>245</v>
       </c>
@@ -7154,7 +7154,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>264</v>
       </c>
@@ -7174,7 +7174,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>285</v>
       </c>
@@ -7185,7 +7185,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>384</v>
       </c>
@@ -7202,7 +7202,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>386</v>
       </c>
@@ -7213,7 +7213,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>385</v>
       </c>
@@ -7239,17 +7239,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3261DB23-C434-4F35-8B4F-998D4295A585}">
   <dimension ref="A1:P81"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="42.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="42.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -7284,12 +7284,12 @@
         <v>313</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -7303,25 +7303,25 @@
         <v>445</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>487</v>
+      </c>
+      <c r="H4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>488</v>
       </c>
-      <c r="H4" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="G5" t="s">
         <v>489</v>
       </c>
-      <c r="G5" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D6" t="s">
         <v>31</v>
@@ -7330,15 +7330,15 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B7" t="s">
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D7" t="s">
         <v>33</v>
@@ -7347,7 +7347,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>446</v>
       </c>
@@ -7358,7 +7358,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>458</v>
       </c>
@@ -7369,7 +7369,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>387</v>
       </c>
@@ -7395,7 +7395,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>388</v>
       </c>
@@ -7424,7 +7424,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>389</v>
       </c>
@@ -7447,7 +7447,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>447</v>
       </c>
@@ -7458,7 +7458,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>459</v>
       </c>
@@ -7469,7 +7469,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>390</v>
       </c>
@@ -7495,7 +7495,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>391</v>
       </c>
@@ -7521,7 +7521,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>393</v>
       </c>
@@ -7544,7 +7544,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>448</v>
       </c>
@@ -7555,7 +7555,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>394</v>
       </c>
@@ -7581,7 +7581,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>392</v>
       </c>
@@ -7610,7 +7610,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>398</v>
       </c>
@@ -7633,7 +7633,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>411</v>
       </c>
@@ -7657,7 +7657,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>464</v>
       </c>
@@ -7680,7 +7680,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>465</v>
       </c>
@@ -7697,7 +7697,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>405</v>
       </c>
@@ -7720,7 +7720,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>406</v>
       </c>
@@ -7737,12 +7737,12 @@
         <v>408</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N31" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>414</v>
       </c>
@@ -7759,7 +7759,7 @@
         <v>470</v>
       </c>
       <c r="H32" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="K32" t="s">
         <v>415</v>
@@ -7768,7 +7768,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>470</v>
       </c>
@@ -7782,7 +7782,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>471</v>
       </c>
@@ -7793,9 +7793,9 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="D35" t="s">
         <v>31</v>
@@ -7804,9 +7804,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="D36" t="s">
         <v>31</v>
@@ -7815,7 +7815,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>422</v>
       </c>
@@ -7832,7 +7832,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>474</v>
       </c>
@@ -7846,13 +7846,13 @@
         <v>30</v>
       </c>
       <c r="G38" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="H38" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>475</v>
       </c>
@@ -7866,13 +7866,13 @@
         <v>30</v>
       </c>
       <c r="G39" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="H39" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>472</v>
       </c>
@@ -7886,13 +7886,13 @@
         <v>30</v>
       </c>
       <c r="G40" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="H40" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>473</v>
       </c>
@@ -7906,13 +7906,13 @@
         <v>30</v>
       </c>
       <c r="G41" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="H41" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>423</v>
       </c>
@@ -7935,7 +7935,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>481</v>
       </c>
@@ -7946,12 +7946,12 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="N45" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>420</v>
       </c>
@@ -7977,7 +7977,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>438</v>
       </c>
@@ -7988,7 +7988,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>428</v>
       </c>
@@ -8002,7 +8002,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>468</v>
       </c>
@@ -8022,7 +8022,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>421</v>
       </c>
@@ -8042,7 +8042,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>431</v>
       </c>
@@ -8053,7 +8053,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>429</v>
       </c>
@@ -8064,7 +8064,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>467</v>
       </c>
@@ -8081,7 +8081,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>427</v>
       </c>
@@ -8101,10 +8101,10 @@
         <v>430</v>
       </c>
       <c r="H55" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>430</v>
       </c>
@@ -8115,7 +8115,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>435</v>
       </c>
@@ -8135,7 +8135,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>433</v>
       </c>
@@ -8149,7 +8149,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>441</v>
       </c>
@@ -8166,7 +8166,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>437</v>
       </c>
@@ -8180,7 +8180,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>432</v>
       </c>
@@ -8200,7 +8200,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>434</v>
       </c>
@@ -8220,7 +8220,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>436</v>
       </c>
@@ -8240,7 +8240,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>379</v>
       </c>
@@ -8254,7 +8254,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>443</v>
       </c>
@@ -8268,7 +8268,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>444</v>
       </c>
@@ -8282,7 +8282,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>442</v>
       </c>
@@ -8293,7 +8293,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>483</v>
       </c>
@@ -8307,7 +8307,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>484</v>
       </c>
@@ -8321,7 +8321,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>485</v>
       </c>
@@ -8329,7 +8329,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>486</v>
       </c>
@@ -8337,7 +8337,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="81" spans="12:12" x14ac:dyDescent="0.35">
+    <row r="81" spans="12:12" x14ac:dyDescent="0.25">
       <c r="L81" t="s">
         <v>482</v>
       </c>

</xml_diff>

<commit_message>
Configure charges for Paladin Intervene
Update Intervene in the spell workbook to use the new maximum-charge field.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE515DAB-C384-440D-922E-C751703F5339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D2934C-6B32-4CD1-B5AB-62C4F4D956A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21150" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="498">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1535,6 +1535,9 @@
   </si>
   <si>
     <t>Finisher Buff;Force Lunar Buff;Force Solar Buff;Balance Buff</t>
+  </si>
+  <si>
+    <t>max_charges</t>
   </si>
 </sst>
 </file>
@@ -1979,6 +1982,9 @@
       <c r="H1" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>497</v>
+      </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -2450,7 +2456,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>46</v>
       </c>
@@ -2470,7 +2476,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>16</v>
       </c>
@@ -2481,7 +2487,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>17</v>
       </c>
@@ -2501,7 +2507,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>18</v>
       </c>
@@ -2512,7 +2518,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>19</v>
       </c>
@@ -2529,7 +2535,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>20</v>
       </c>
@@ -2546,7 +2552,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>21</v>
       </c>
@@ -2563,7 +2569,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>22</v>
       </c>
@@ -2576,8 +2582,14 @@
       <c r="D40" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F40">
+        <v>3000</v>
+      </c>
+      <c r="I40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>23</v>
       </c>
@@ -2591,7 +2603,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>80</v>
       </c>
@@ -2605,7 +2617,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>379</v>
       </c>
@@ -2625,7 +2637,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>380</v>
       </c>

</xml_diff>

<commit_message>
Track spell charge recovery timers
Calculate current and future charge availability and expose overcap helpers. In-game validation remains pending.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\lavender_keys\lavender_moogle\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D2934C-6B32-4CD1-B5AB-62C4F4D956A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F979FD-45BB-4E8E-9380-5F3A7A6B039D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15495" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="MNK" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="500">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1538,6 +1538,12 @@
   </si>
   <si>
     <t>max_charges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloodfest Buff </t>
+  </si>
+  <si>
+    <t>Ready to Reign;Bloodfest Buff</t>
   </si>
 </sst>
 </file>
@@ -2662,7 +2668,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7762502F-9F7A-4AD9-AC88-345A2195334F}">
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
@@ -2918,7 +2924,7 @@
         <v>120000</v>
       </c>
       <c r="G15" t="s">
-        <v>87</v>
+        <v>499</v>
       </c>
       <c r="H15" t="s">
         <v>86</v>
@@ -2929,7 +2935,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>498</v>
       </c>
       <c r="D16" t="s">
         <v>32</v>
@@ -2940,278 +2946,272 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>60</v>
-      </c>
-      <c r="B17" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17">
-        <v>8</v>
+        <v>87</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
-      </c>
-      <c r="G17" t="s">
-        <v>61</v>
-      </c>
-      <c r="H17" t="s">
-        <v>93</v>
+        <v>32</v>
+      </c>
+      <c r="E17">
+        <v>30000</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18">
+        <v>8</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="G18" t="s">
         <v>61</v>
       </c>
-      <c r="D18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18">
-        <v>30000</v>
+      <c r="H18" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19">
-        <v>8</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>30</v>
-      </c>
-      <c r="G19" t="s">
-        <v>90</v>
-      </c>
-      <c r="H19" t="s">
-        <v>94</v>
+        <v>31</v>
+      </c>
+      <c r="E19">
+        <v>30000</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+      <c r="G20" t="s">
         <v>90</v>
       </c>
-      <c r="D20" t="s">
-        <v>31</v>
-      </c>
-      <c r="E20">
-        <v>30000</v>
+      <c r="H20" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>95</v>
-      </c>
-      <c r="B21" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="D21" t="s">
-        <v>30</v>
-      </c>
-      <c r="H21" t="s">
-        <v>96</v>
+        <v>31</v>
+      </c>
+      <c r="E21">
+        <v>30000</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="B22" t="s">
         <v>28</v>
       </c>
       <c r="C22">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D22" t="s">
         <v>30</v>
       </c>
-      <c r="F22">
-        <v>30000</v>
-      </c>
-      <c r="G22" t="s">
-        <v>82</v>
-      </c>
       <c r="H22" t="s">
-        <v>97</v>
-      </c>
-      <c r="I22">
-        <v>-1</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23">
+        <v>4</v>
       </c>
       <c r="D23" t="s">
-        <v>32</v>
-      </c>
-      <c r="E23">
-        <v>10000</v>
+        <v>30</v>
+      </c>
+      <c r="F23">
+        <v>30000</v>
+      </c>
+      <c r="G23" t="s">
+        <v>82</v>
+      </c>
+      <c r="H23" t="s">
+        <v>97</v>
+      </c>
+      <c r="I23">
+        <v>-1</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>65</v>
-      </c>
-      <c r="B24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>33</v>
-      </c>
-      <c r="H24" t="s">
-        <v>86</v>
+        <v>32</v>
+      </c>
+      <c r="E24">
+        <v>10000</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>65</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25">
+        <v>5</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
-      </c>
-      <c r="E25">
-        <v>30000</v>
+        <v>33</v>
+      </c>
+      <c r="H25" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>67</v>
-      </c>
-      <c r="B26" t="s">
-        <v>28</v>
-      </c>
-      <c r="C26">
-        <v>4</v>
+        <v>66</v>
       </c>
       <c r="D26" t="s">
-        <v>30</v>
-      </c>
-      <c r="G26" t="s">
-        <v>83</v>
-      </c>
-      <c r="H26" t="s">
-        <v>98</v>
+        <v>31</v>
+      </c>
+      <c r="E26">
+        <v>30000</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>68</v>
+        <v>67</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
       </c>
       <c r="D27" t="s">
-        <v>32</v>
-      </c>
-      <c r="E27">
-        <v>10000</v>
+        <v>30</v>
+      </c>
+      <c r="G27" t="s">
+        <v>83</v>
+      </c>
+      <c r="H27" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B28" t="s">
-        <v>28</v>
-      </c>
-      <c r="C28">
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="D28" t="s">
-        <v>33</v>
-      </c>
-      <c r="H28" t="s">
-        <v>86</v>
+        <v>32</v>
+      </c>
+      <c r="E28">
+        <v>10000</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>69</v>
+      </c>
+      <c r="B29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29">
+        <v>5</v>
       </c>
       <c r="D29" t="s">
-        <v>31</v>
-      </c>
-      <c r="E29">
-        <v>30000</v>
+        <v>33</v>
+      </c>
+      <c r="H29" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>71</v>
-      </c>
-      <c r="B30" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="D30" t="s">
-        <v>30</v>
-      </c>
-      <c r="G30" t="s">
-        <v>84</v>
-      </c>
-      <c r="H30" t="s">
-        <v>99</v>
+        <v>31</v>
+      </c>
+      <c r="E30">
+        <v>30000</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31">
+        <v>4</v>
+      </c>
+      <c r="D31" t="s">
+        <v>30</v>
+      </c>
+      <c r="G31" t="s">
         <v>84</v>
       </c>
-      <c r="D31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E31">
-        <v>10000</v>
+      <c r="H31" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>72</v>
-      </c>
-      <c r="B32" t="s">
-        <v>28</v>
-      </c>
-      <c r="C32">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="D32" t="s">
-        <v>33</v>
-      </c>
-      <c r="H32" t="s">
-        <v>86</v>
+        <v>32</v>
+      </c>
+      <c r="E32">
+        <v>10000</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B33" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C33">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D33" t="s">
         <v>33</v>
       </c>
-      <c r="F33">
-        <v>30000</v>
+      <c r="H33" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C34">
         <v>9</v>
@@ -3220,105 +3220,122 @@
         <v>33</v>
       </c>
       <c r="F34">
-        <v>60000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B35" t="s">
         <v>29</v>
       </c>
       <c r="C35">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D35" t="s">
-        <v>30</v>
-      </c>
-      <c r="G35" t="s">
-        <v>84</v>
-      </c>
-      <c r="H35" t="s">
-        <v>86</v>
+        <v>33</v>
+      </c>
+      <c r="F35">
+        <v>60000</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B36" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D36" t="s">
-        <v>33</v>
-      </c>
-      <c r="F36">
-        <v>60000</v>
+        <v>30</v>
       </c>
       <c r="G36" t="s">
-        <v>89</v>
+        <v>84</v>
+      </c>
+      <c r="H36" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>76</v>
+      </c>
+      <c r="B37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
       </c>
       <c r="D37" t="s">
-        <v>32</v>
-      </c>
-      <c r="E37">
-        <v>20000</v>
+        <v>33</v>
+      </c>
+      <c r="F37">
+        <v>60000</v>
+      </c>
+      <c r="G37" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D38" t="s">
         <v>32</v>
       </c>
       <c r="E38">
-        <v>30000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>77</v>
-      </c>
-      <c r="B39" t="s">
-        <v>28</v>
-      </c>
-      <c r="C39">
-        <v>2</v>
+        <v>88</v>
       </c>
       <c r="D39" t="s">
-        <v>30</v>
-      </c>
-      <c r="H39" t="s">
-        <v>100</v>
+        <v>32</v>
+      </c>
+      <c r="E39">
+        <v>30000</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>77</v>
+      </c>
+      <c r="B40" t="s">
+        <v>28</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40" t="s">
+        <v>30</v>
+      </c>
+      <c r="H40" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>79</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>29</v>
       </c>
-      <c r="C40">
+      <c r="C41">
         <v>8</v>
       </c>
-      <c r="D40" t="s">
-        <v>30</v>
-      </c>
-      <c r="H40" t="s">
+      <c r="D41" t="s">
+        <v>30</v>
+      </c>
+      <c r="H41" t="s">
         <v>99</v>
       </c>
-      <c r="I40">
+      <c r="I41">
         <v>-1</v>
       </c>
     </row>
@@ -7255,6 +7272,7 @@
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="27.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="42.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Add ANY-job events and resource-dump state
Resolve generic events against the active job, track dump mode and refine Dancer spending priorities.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0D1C660-3123-4D7E-B0B5-710AE1F9061B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F99915-CBED-4467-B39E-1CD58A564D61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1453" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1470" uniqueCount="513">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1565,6 +1565,24 @@
   </si>
   <si>
     <t>Potion Buff</t>
+  </si>
+  <si>
+    <t>Shower Ready</t>
+  </si>
+  <si>
+    <t>Fountain Ready;Shower Ready</t>
+  </si>
+  <si>
+    <t>En Avant</t>
+  </si>
+  <si>
+    <t>Curing Waltz</t>
+  </si>
+  <si>
+    <t>Shield Samba</t>
+  </si>
+  <si>
+    <t>Second Wind</t>
   </si>
 </sst>
 </file>
@@ -6604,7 +6622,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9448C388-C543-449D-8B21-6D32E03898B2}">
-  <dimension ref="A1:P74"/>
+  <dimension ref="A1:P82"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -6746,6 +6764,9 @@
       <c r="G12" t="s">
         <v>222</v>
       </c>
+      <c r="H12" t="s">
+        <v>507</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -6761,12 +6782,15 @@
         <v>30</v>
       </c>
       <c r="G13" t="s">
+        <v>507</v>
+      </c>
+      <c r="H13" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>222</v>
+        <v>507</v>
       </c>
       <c r="D14" t="s">
         <v>31</v>
@@ -6777,27 +6801,21 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>221</v>
-      </c>
-      <c r="B15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15">
-        <v>5</v>
+        <v>222</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
-      </c>
-      <c r="H15" t="s">
-        <v>222</v>
+        <v>31</v>
+      </c>
+      <c r="E15">
+        <v>30000</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C16">
         <v>5</v>
@@ -6806,23 +6824,29 @@
         <v>30</v>
       </c>
       <c r="H16" t="s">
-        <v>222</v>
+        <v>508</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>237</v>
+        <v>224</v>
+      </c>
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17">
+        <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E17">
-        <v>30000</v>
+        <v>30</v>
+      </c>
+      <c r="H17" t="s">
+        <v>508</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>273</v>
+        <v>237</v>
       </c>
       <c r="D18" t="s">
         <v>32</v>
@@ -6833,27 +6857,21 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>225</v>
-      </c>
-      <c r="B19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19">
-        <v>7</v>
+        <v>273</v>
       </c>
       <c r="D19" t="s">
-        <v>30</v>
-      </c>
-      <c r="P19" t="s">
-        <v>444</v>
+        <v>32</v>
+      </c>
+      <c r="E19">
+        <v>30000</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C20">
         <v>7</v>
@@ -6861,27 +6879,33 @@
       <c r="D20" t="s">
         <v>30</v>
       </c>
-      <c r="O20" t="s">
-        <v>446</v>
-      </c>
       <c r="P20" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>238</v>
+        <v>227</v>
+      </c>
+      <c r="B21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21">
+        <v>7</v>
       </c>
       <c r="D21" t="s">
-        <v>32</v>
-      </c>
-      <c r="E21">
-        <v>30000</v>
+        <v>30</v>
+      </c>
+      <c r="O21" t="s">
+        <v>446</v>
+      </c>
+      <c r="P21" t="s">
+        <v>444</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>274</v>
+        <v>238</v>
       </c>
       <c r="D22" t="s">
         <v>32</v>
@@ -6892,27 +6916,21 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>226</v>
-      </c>
-      <c r="B23" t="s">
-        <v>27</v>
-      </c>
-      <c r="C23">
-        <v>8</v>
+        <v>274</v>
       </c>
       <c r="D23" t="s">
-        <v>30</v>
-      </c>
-      <c r="P23" t="s">
-        <v>445</v>
+        <v>32</v>
+      </c>
+      <c r="E23">
+        <v>30000</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C24">
         <v>8</v>
@@ -6924,29 +6942,32 @@
         <v>445</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>255</v>
-      </c>
-      <c r="B26" t="s">
-        <v>27</v>
-      </c>
-      <c r="C26">
-        <v>9</v>
-      </c>
-      <c r="D26" t="s">
-        <v>30</v>
-      </c>
-      <c r="F26">
-        <v>30000</v>
-      </c>
-      <c r="G26" t="s">
-        <v>271</v>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>228</v>
+      </c>
+      <c r="B25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25">
+        <v>8</v>
+      </c>
+      <c r="D25" t="s">
+        <v>30</v>
+      </c>
+      <c r="P25" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>276</v>
+        <v>255</v>
+      </c>
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27">
+        <v>9</v>
       </c>
       <c r="D27" t="s">
         <v>30</v>
@@ -6955,46 +6976,46 @@
         <v>30000</v>
       </c>
       <c r="G27" t="s">
-        <v>277</v>
-      </c>
-      <c r="H27" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>256</v>
+        <v>276</v>
       </c>
       <c r="D28" t="s">
-        <v>31</v>
-      </c>
-      <c r="E28">
-        <v>15000</v>
+        <v>30</v>
+      </c>
+      <c r="F28">
+        <v>30000</v>
+      </c>
+      <c r="G28" t="s">
+        <v>277</v>
+      </c>
+      <c r="H28" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>257</v>
-      </c>
-      <c r="B29" t="s">
-        <v>27</v>
-      </c>
-      <c r="C29">
-        <v>9</v>
+        <v>256</v>
       </c>
       <c r="D29" t="s">
-        <v>248</v>
-      </c>
-      <c r="G29" t="s">
-        <v>241</v>
-      </c>
-      <c r="H29" t="s">
-        <v>256</v>
+        <v>31</v>
+      </c>
+      <c r="E29">
+        <v>15000</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>261</v>
+        <v>257</v>
+      </c>
+      <c r="B30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30">
+        <v>9</v>
       </c>
       <c r="D30" t="s">
         <v>248</v>
@@ -7008,7 +7029,7 @@
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D31" t="s">
         <v>248</v>
@@ -7022,21 +7043,24 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="D32" t="s">
-        <v>31</v>
-      </c>
-      <c r="E32">
-        <v>30000</v>
+        <v>248</v>
+      </c>
+      <c r="G32" t="s">
+        <v>241</v>
+      </c>
+      <c r="H32" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>241</v>
+        <v>265</v>
       </c>
       <c r="D33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E33">
         <v>30000</v>
@@ -7044,78 +7068,72 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>241</v>
+      </c>
+      <c r="D34" t="s">
+        <v>32</v>
+      </c>
+      <c r="E34">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>242</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>29</v>
       </c>
-      <c r="C34">
+      <c r="C35">
         <v>9</v>
       </c>
-      <c r="D34" t="s">
-        <v>30</v>
-      </c>
-      <c r="H34" t="s">
+      <c r="D35" t="s">
+        <v>30</v>
+      </c>
+      <c r="H35" t="s">
         <v>241</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>239</v>
-      </c>
-      <c r="B36" t="s">
-        <v>28</v>
-      </c>
-      <c r="C36">
-        <v>9</v>
-      </c>
-      <c r="D36" t="s">
-        <v>30</v>
-      </c>
-      <c r="G36" t="s">
-        <v>270</v>
-      </c>
-      <c r="H36" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>240</v>
+        <v>239</v>
+      </c>
+      <c r="B37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37">
+        <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>31</v>
-      </c>
-      <c r="E37">
-        <v>15000</v>
+        <v>30</v>
+      </c>
+      <c r="G37" t="s">
+        <v>270</v>
+      </c>
+      <c r="H37" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>243</v>
-      </c>
-      <c r="B38" t="s">
-        <v>28</v>
-      </c>
-      <c r="C38">
-        <v>9</v>
+        <v>240</v>
       </c>
       <c r="D38" t="s">
-        <v>248</v>
-      </c>
-      <c r="G38" t="s">
-        <v>280</v>
-      </c>
-      <c r="H38" t="s">
-        <v>240</v>
-      </c>
-      <c r="K38" t="s">
-        <v>272</v>
+        <v>31</v>
+      </c>
+      <c r="E38">
+        <v>15000</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>263</v>
+        <v>243</v>
+      </c>
+      <c r="B39" t="s">
+        <v>28</v>
+      </c>
+      <c r="C39">
+        <v>9</v>
       </c>
       <c r="D39" t="s">
         <v>248</v>
@@ -7126,10 +7144,13 @@
       <c r="H39" t="s">
         <v>240</v>
       </c>
+      <c r="K39" t="s">
+        <v>272</v>
+      </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D40" t="s">
         <v>248</v>
@@ -7143,7 +7164,7 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D41" t="s">
         <v>248</v>
@@ -7157,7 +7178,7 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D42" t="s">
         <v>248</v>
@@ -7171,80 +7192,77 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D43" t="s">
-        <v>31</v>
-      </c>
-      <c r="E43">
-        <v>120000</v>
+        <v>248</v>
+      </c>
+      <c r="G43" t="s">
+        <v>280</v>
+      </c>
+      <c r="H43" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="D44" t="s">
         <v>31</v>
       </c>
       <c r="E44">
-        <v>20000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>250</v>
+        <v>267</v>
       </c>
       <c r="D45" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E45">
-        <v>30000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>251</v>
-      </c>
-      <c r="B46" t="s">
-        <v>28</v>
-      </c>
-      <c r="C46">
-        <v>9</v>
+        <v>250</v>
       </c>
       <c r="D46" t="s">
-        <v>30</v>
-      </c>
-      <c r="H46" t="s">
-        <v>250</v>
+        <v>32</v>
+      </c>
+      <c r="E46">
+        <v>30000</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="B47" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C47">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D47" t="s">
-        <v>248</v>
-      </c>
-      <c r="F47">
-        <v>1000</v>
+        <v>30</v>
+      </c>
+      <c r="H47" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B48" t="s">
         <v>27</v>
       </c>
       <c r="C48">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D48" t="s">
         <v>248</v>
@@ -7255,13 +7273,13 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B49" t="s">
         <v>27</v>
       </c>
       <c r="C49">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D49" t="s">
         <v>248</v>
@@ -7272,13 +7290,13 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B50" t="s">
         <v>27</v>
       </c>
       <c r="C50">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D50" t="s">
         <v>248</v>
@@ -7287,35 +7305,29 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>229</v>
-      </c>
-      <c r="B53" t="s">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>247</v>
+      </c>
+      <c r="B51" t="s">
         <v>27</v>
       </c>
-      <c r="C53">
-        <v>6</v>
-      </c>
-      <c r="D53" t="s">
-        <v>33</v>
-      </c>
-      <c r="E53">
+      <c r="C51">
+        <v>8</v>
+      </c>
+      <c r="D51" t="s">
+        <v>248</v>
+      </c>
+      <c r="F51">
         <v>1000</v>
-      </c>
-      <c r="F53">
-        <v>1000</v>
-      </c>
-      <c r="I53">
-        <v>-1</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B54" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C54">
         <v>6</v>
@@ -7323,6 +7335,9 @@
       <c r="D54" t="s">
         <v>33</v>
       </c>
+      <c r="E54">
+        <v>1000</v>
+      </c>
       <c r="F54">
         <v>1000</v>
       </c>
@@ -7332,151 +7347,160 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>252</v>
+        <v>230</v>
+      </c>
+      <c r="B55" t="s">
+        <v>29</v>
+      </c>
+      <c r="C55">
+        <v>6</v>
       </c>
       <c r="D55" t="s">
-        <v>32</v>
-      </c>
-      <c r="E55">
-        <v>30000</v>
+        <v>33</v>
+      </c>
+      <c r="F55">
+        <v>1000</v>
+      </c>
+      <c r="I55">
+        <v>-1</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>231</v>
-      </c>
-      <c r="B56" t="s">
-        <v>28</v>
-      </c>
-      <c r="C56">
-        <v>6</v>
+        <v>252</v>
       </c>
       <c r="D56" t="s">
-        <v>33</v>
-      </c>
-      <c r="F56">
-        <v>1000</v>
-      </c>
-      <c r="H56" t="s">
-        <v>252</v>
+        <v>32</v>
+      </c>
+      <c r="E56">
+        <v>30000</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>253</v>
+        <v>231</v>
+      </c>
+      <c r="B57" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57">
+        <v>6</v>
       </c>
       <c r="D57" t="s">
-        <v>32</v>
-      </c>
-      <c r="E57">
-        <v>30000</v>
+        <v>33</v>
+      </c>
+      <c r="F57">
+        <v>1000</v>
+      </c>
+      <c r="H57" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>253</v>
+      </c>
+      <c r="D58" t="s">
+        <v>32</v>
+      </c>
+      <c r="E58">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>232</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B59" t="s">
         <v>28</v>
       </c>
-      <c r="C58">
+      <c r="C59">
         <v>5</v>
       </c>
-      <c r="D58" t="s">
-        <v>33</v>
-      </c>
-      <c r="F58">
+      <c r="D59" t="s">
+        <v>33</v>
+      </c>
+      <c r="F59">
         <v>1000</v>
       </c>
-      <c r="H58" t="s">
+      <c r="H59" t="s">
         <v>253</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>233</v>
-      </c>
-      <c r="B60" t="s">
-        <v>28</v>
-      </c>
-      <c r="C60">
-        <v>4</v>
-      </c>
-      <c r="D60" t="s">
-        <v>30</v>
-      </c>
-      <c r="J60">
-        <v>-50</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>279</v>
+        <v>233</v>
+      </c>
+      <c r="B61" t="s">
+        <v>28</v>
+      </c>
+      <c r="C61">
+        <v>4</v>
       </c>
       <c r="D61" t="s">
-        <v>32</v>
-      </c>
-      <c r="E61">
-        <v>30000</v>
+        <v>30</v>
+      </c>
+      <c r="J61">
+        <v>-50</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>279</v>
+      </c>
+      <c r="D62" t="s">
+        <v>32</v>
+      </c>
+      <c r="E62">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>278</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B63" t="s">
         <v>28</v>
       </c>
-      <c r="C62">
+      <c r="C63">
         <v>4</v>
       </c>
-      <c r="D62" t="s">
-        <v>30</v>
-      </c>
-      <c r="H62" t="s">
+      <c r="D63" t="s">
+        <v>30</v>
+      </c>
+      <c r="H63" t="s">
         <v>279</v>
       </c>
-      <c r="J62">
+      <c r="J63">
         <v>-50</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>269</v>
-      </c>
-      <c r="B64" t="s">
-        <v>28</v>
-      </c>
-      <c r="C64">
-        <v>2</v>
-      </c>
-      <c r="D64" t="s">
-        <v>33</v>
-      </c>
-      <c r="F64">
-        <v>120000</v>
-      </c>
-      <c r="G64" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>234</v>
+        <v>269</v>
+      </c>
+      <c r="B65" t="s">
+        <v>28</v>
+      </c>
+      <c r="C65">
+        <v>2</v>
       </c>
       <c r="D65" t="s">
-        <v>31</v>
-      </c>
-      <c r="E65">
-        <v>20000</v>
+        <v>33</v>
+      </c>
+      <c r="F65">
+        <v>120000</v>
+      </c>
+      <c r="G65" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D66" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E66">
         <v>20000</v>
@@ -7484,95 +7508,164 @@
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>236</v>
+      </c>
+      <c r="D67" t="s">
+        <v>32</v>
+      </c>
+      <c r="E67">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>235</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B68" t="s">
         <v>28</v>
       </c>
-      <c r="C67">
+      <c r="C68">
         <v>7</v>
       </c>
-      <c r="D67" t="s">
-        <v>30</v>
-      </c>
-      <c r="H67" t="s">
+      <c r="D68" t="s">
+        <v>30</v>
+      </c>
+      <c r="H68" t="s">
         <v>236</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>254</v>
-      </c>
-      <c r="B69" t="s">
-        <v>27</v>
-      </c>
-      <c r="C69">
-        <v>12</v>
-      </c>
-      <c r="D69" t="s">
-        <v>33</v>
-      </c>
-      <c r="F69">
-        <v>60000</v>
-      </c>
-      <c r="G69" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>254</v>
+      </c>
+      <c r="B70" t="s">
+        <v>27</v>
+      </c>
+      <c r="C70">
+        <v>12</v>
+      </c>
+      <c r="D70" t="s">
+        <v>33</v>
+      </c>
+      <c r="F70">
+        <v>60000</v>
+      </c>
+      <c r="G70" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>275</v>
       </c>
-      <c r="D70" t="s">
+      <c r="D71" t="s">
         <v>32</v>
       </c>
-      <c r="E70">
+      <c r="E71">
         <v>30000</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>374</v>
-      </c>
-      <c r="B72" t="s">
-        <v>28</v>
-      </c>
-      <c r="C72">
-        <v>11</v>
-      </c>
-      <c r="D72" t="s">
-        <v>33</v>
-      </c>
-      <c r="G72" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>374</v>
+      </c>
+      <c r="B73" t="s">
+        <v>28</v>
+      </c>
+      <c r="C73">
+        <v>11</v>
+      </c>
+      <c r="D73" t="s">
+        <v>33</v>
+      </c>
+      <c r="G73" t="s">
         <v>376</v>
-      </c>
-      <c r="D73" t="s">
-        <v>31</v>
-      </c>
-      <c r="E73">
-        <v>15000</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>376</v>
+      </c>
+      <c r="D74" t="s">
+        <v>31</v>
+      </c>
+      <c r="E74">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>375</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B75" t="s">
         <v>28</v>
       </c>
-      <c r="C74">
+      <c r="C75">
         <v>11</v>
       </c>
-      <c r="D74" t="s">
-        <v>33</v>
-      </c>
-      <c r="H74" t="s">
+      <c r="D75" t="s">
+        <v>33</v>
+      </c>
+      <c r="H75" t="s">
         <v>376</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>509</v>
+      </c>
+      <c r="B77" t="s">
+        <v>28</v>
+      </c>
+      <c r="C77">
+        <v>1</v>
+      </c>
+      <c r="D77" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>510</v>
+      </c>
+      <c r="D79" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>511</v>
+      </c>
+      <c r="D80" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>424</v>
+      </c>
+      <c r="B81" t="s">
+        <v>29</v>
+      </c>
+      <c r="C81">
+        <v>11</v>
+      </c>
+      <c r="D81" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>512</v>
+      </c>
+      <c r="B82" t="s">
+        <v>28</v>
+      </c>
+      <c r="C82">
+        <v>10</v>
+      </c>
+      <c r="D82" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand Bard and Dancer priorities and add Black Mage spell data
Refine Bard opener, AoE and gauge handling and restrict weaving after Dancer steps. BLM has spell data only.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F99915-CBED-4467-B39E-1CD58A564D61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF037F1-95AB-4FAC-BF70-B34C82CD5175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="14160" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,8 @@
     <sheet name="SCH" sheetId="4" r:id="rId5"/>
     <sheet name="BRD" sheetId="7" r:id="rId6"/>
     <sheet name="DNC" sheetId="6" r:id="rId7"/>
-    <sheet name="MNK" sheetId="8" r:id="rId8"/>
+    <sheet name="BLM" sheetId="9" r:id="rId8"/>
+    <sheet name="MNK" sheetId="8" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">GNB!$D$1:$D$61</definedName>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1470" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1665" uniqueCount="588">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1583,13 +1584,238 @@
   </si>
   <si>
     <t>Second Wind</t>
+  </si>
+  <si>
+    <t>specific_gcd</t>
+  </si>
+  <si>
+    <t>Blizzard</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>MP</t>
+  </si>
+  <si>
+    <t>Transpose</t>
+  </si>
+  <si>
+    <t>Thunder</t>
+  </si>
+  <si>
+    <t>Blizzard II</t>
+  </si>
+  <si>
+    <t>Scathe</t>
+  </si>
+  <si>
+    <t>cast_time</t>
+  </si>
+  <si>
+    <t>Fire II</t>
+  </si>
+  <si>
+    <t>AOE</t>
+  </si>
+  <si>
+    <t>Thunder II</t>
+  </si>
+  <si>
+    <t>DOT</t>
+  </si>
+  <si>
+    <t>Thunder II DOT</t>
+  </si>
+  <si>
+    <t>Thunder DOT</t>
+  </si>
+  <si>
+    <t>Manaward</t>
+  </si>
+  <si>
+    <t>Manafont</t>
+  </si>
+  <si>
+    <t>Astral Fire III</t>
+  </si>
+  <si>
+    <t>Fire III</t>
+  </si>
+  <si>
+    <t>Blizzard III</t>
+  </si>
+  <si>
+    <t>Grants Umbral Ice III and removes Astral Fire</t>
+  </si>
+  <si>
+    <t>TODO</t>
+  </si>
+  <si>
+    <t>Additional Effect: Grants Umbral Ice III and removes Astral Fire</t>
+  </si>
+  <si>
+    <t>Umbral Soul</t>
+  </si>
+  <si>
+    <t>A LOT</t>
+  </si>
+  <si>
+    <t>Freeze</t>
+  </si>
+  <si>
+    <t>Thunder III</t>
+  </si>
+  <si>
+    <t>Thunder III DOT</t>
+  </si>
+  <si>
+    <t>Can only be cast while under the effect of Thunderhead, granted when gaining Astral Fire or Umbral Ice from an unaspected state, or changing between their influences.</t>
+  </si>
+  <si>
+    <t>Aetherial Manipulation</t>
+  </si>
+  <si>
+    <t>Flare</t>
+  </si>
+  <si>
+    <t>Ley Lines</t>
+  </si>
+  <si>
+    <t>Duration 20000</t>
+  </si>
+  <si>
+    <t>A PLANIFIER et PAS AUTO CAST</t>
+  </si>
+  <si>
+    <t>Blizzard IV</t>
+  </si>
+  <si>
+    <t>Grants 3 Umbral Hearts</t>
+  </si>
+  <si>
+    <t>Between the Lines</t>
+  </si>
+  <si>
+    <t>Thunder IV</t>
+  </si>
+  <si>
+    <t>Thunder IV DOT</t>
+  </si>
+  <si>
+    <t>Can only be cast while under the effect of Thunderhead</t>
+  </si>
+  <si>
+    <t>Foul</t>
+  </si>
+  <si>
+    <t>Despair</t>
+  </si>
+  <si>
+    <t>Xenoglossy</t>
+  </si>
+  <si>
+    <t>Polyglot Cost: 1</t>
+  </si>
+  <si>
+    <t>Grants Astral Fire III</t>
+  </si>
+  <si>
+    <t>Fire IV</t>
+  </si>
+  <si>
+    <t>Grants Astral Fire III, 3 Astral Souls</t>
+  </si>
+  <si>
+    <t>Astral Fire III, 3 Umbral Hearts, Paradox / requires astral fire</t>
+  </si>
+  <si>
+    <t>Astral Fire I</t>
+  </si>
+  <si>
+    <t>Astral Fire II</t>
+  </si>
+  <si>
+    <t>Umbral Ice III</t>
+  </si>
+  <si>
+    <t>Umbral Ice I</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Astral Fire III</t>
+  </si>
+  <si>
+    <t>Astral Soul</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Astral Fire III;Astral Soul III</t>
+  </si>
+  <si>
+    <t>Astral Soul I</t>
+  </si>
+  <si>
+    <t>High Fire II</t>
+  </si>
+  <si>
+    <t>High Blizzard II</t>
+  </si>
+  <si>
+    <t>Amplifier</t>
+  </si>
+  <si>
+    <t>Grant Polyglot</t>
+  </si>
+  <si>
+    <t>Umbral Ice I;Umbral Ice II;Umbral Ice III; Astral Fire I; Astral FireII;Astral Fire III</t>
+  </si>
+  <si>
+    <t>Paradox</t>
+  </si>
+  <si>
+    <t>This action cannot be assigned to a hotbar</t>
+  </si>
+  <si>
+    <t>High Thunder</t>
+  </si>
+  <si>
+    <t>High Thunder DOT</t>
+  </si>
+  <si>
+    <t>High Thunder II</t>
+  </si>
+  <si>
+    <t>High Thunder II DOT</t>
+  </si>
+  <si>
+    <t>Triplecast</t>
+  </si>
+  <si>
+    <t>Retrace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucid Dreaming	</t>
+  </si>
+  <si>
+    <t>Surecast</t>
+  </si>
+  <si>
+    <t>Flare Star</t>
+  </si>
+  <si>
+    <t>Astral Gauge Full</t>
+  </si>
+  <si>
+    <t>todo</t>
+  </si>
+  <si>
+    <t>Todo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1614,8 +1840,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1682,6 +1916,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2D9FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1695,7 +1941,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1709,12 +1955,30 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF2D9FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -5754,7 +6018,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD84FEA-D0D3-4F98-B644-3E9C52C4A2B7}">
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -5764,9 +6028,11 @@
     <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.140625" customWidth="1"/>
     <col min="10" max="10" width="18.5703125" customWidth="1"/>
+    <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -5806,8 +6072,12 @@
       <c r="M1" s="1" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="K2" t="s">
         <v>293</v>
       </c>
@@ -5818,7 +6088,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -5829,7 +6099,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>477</v>
       </c>
@@ -5840,7 +6110,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>478</v>
       </c>
@@ -5851,7 +6121,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>479</v>
       </c>
@@ -5862,7 +6132,7 @@
         <v>3600000</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>505</v>
       </c>
@@ -5882,7 +6152,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>506</v>
       </c>
@@ -5893,7 +6163,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>282</v>
       </c>
@@ -5913,7 +6183,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>346</v>
       </c>
@@ -5930,7 +6200,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>283</v>
       </c>
@@ -5953,7 +6223,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>287</v>
       </c>
@@ -5964,10 +6234,10 @@
         <v>349</v>
       </c>
       <c r="D15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E15">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F15" t="s">
         <v>30</v>
@@ -5976,7 +6246,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>332</v>
       </c>
@@ -6024,7 +6294,13 @@
         <v>324</v>
       </c>
       <c r="C18" t="s">
-        <v>350</v>
+        <v>586</v>
+      </c>
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+      <c r="E18">
+        <v>5</v>
       </c>
       <c r="F18" t="s">
         <v>30</v>
@@ -6038,7 +6314,7 @@
         <v>323</v>
       </c>
       <c r="C19" t="s">
-        <v>350</v>
+        <v>586</v>
       </c>
       <c r="D19" t="s">
         <v>29</v>
@@ -6048,6 +6324,9 @@
       </c>
       <c r="F19" t="s">
         <v>30</v>
+      </c>
+      <c r="J19" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -6087,6 +6366,12 @@
       <c r="B24" t="s">
         <v>322</v>
       </c>
+      <c r="D24" t="s">
+        <v>29</v>
+      </c>
+      <c r="E24">
+        <v>3</v>
+      </c>
       <c r="F24" t="s">
         <v>30</v>
       </c>
@@ -6220,7 +6505,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>339</v>
       </c>
@@ -6234,7 +6519,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>293</v>
       </c>
@@ -6251,7 +6536,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>352</v>
       </c>
@@ -6280,7 +6565,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>340</v>
       </c>
@@ -6294,7 +6579,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>314</v>
       </c>
@@ -6317,7 +6602,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>294</v>
       </c>
@@ -6339,8 +6624,11 @@
       <c r="H39">
         <v>1500</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L39">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>295</v>
       </c>
@@ -6348,7 +6636,7 @@
         <v>307</v>
       </c>
       <c r="C40" t="s">
-        <v>350</v>
+        <v>587</v>
       </c>
       <c r="D40" t="s">
         <v>29</v>
@@ -6362,8 +6650,11 @@
       <c r="H40">
         <v>1500</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L40">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>353</v>
       </c>
@@ -6392,7 +6683,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>341</v>
       </c>
@@ -6406,7 +6697,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>296</v>
       </c>
@@ -6420,7 +6711,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>298</v>
       </c>
@@ -6446,7 +6737,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>330</v>
       </c>
@@ -6542,10 +6833,10 @@
         <v>349</v>
       </c>
       <c r="D53" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E53">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F53" t="s">
         <v>33</v>
@@ -7525,7 +7816,7 @@
         <v>28</v>
       </c>
       <c r="C68">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D68" t="s">
         <v>30</v>
@@ -7675,6 +7966,1092 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F698799-D664-4BA4-8D34-0E7AC088D617}">
+  <dimension ref="A1:P77"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" customWidth="1"/>
+    <col min="9" max="9" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>477</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>478</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>479</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5">
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>505</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>480</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6">
+        <v>300000</v>
+      </c>
+      <c r="I6" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>506</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>369</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8">
+        <v>10000</v>
+      </c>
+      <c r="F8">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>583</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>175</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>176</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>582</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>179</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G17">
+        <v>2000</v>
+      </c>
+      <c r="H17">
+        <v>2500</v>
+      </c>
+      <c r="L17">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="18" t="s">
+        <v>519</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G18" s="17">
+        <v>3000</v>
+      </c>
+      <c r="H18" s="17">
+        <v>2500</v>
+      </c>
+      <c r="L18" s="17">
+        <v>800</v>
+      </c>
+      <c r="M18" s="17" t="s">
+        <v>523</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="G19">
+        <v>3000</v>
+      </c>
+      <c r="H19">
+        <v>2500</v>
+      </c>
+      <c r="I19" t="s">
+        <v>563</v>
+      </c>
+      <c r="J19" s="17" t="s">
+        <v>573</v>
+      </c>
+      <c r="L19">
+        <v>800</v>
+      </c>
+      <c r="M19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+      <c r="G20">
+        <v>3500</v>
+      </c>
+      <c r="H20">
+        <v>2500</v>
+      </c>
+      <c r="L20">
+        <v>800</v>
+      </c>
+      <c r="N20" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+      <c r="G21">
+        <v>2000</v>
+      </c>
+      <c r="H21">
+        <v>2500</v>
+      </c>
+      <c r="L21">
+        <v>1000</v>
+      </c>
+      <c r="M21" t="s">
+        <v>523</v>
+      </c>
+      <c r="N21" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="D22" t="s">
+        <v>30</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>2500</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="N22" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
+        <v>547</v>
+      </c>
+      <c r="B23" s="14"/>
+      <c r="D23" t="s">
+        <v>30</v>
+      </c>
+      <c r="G23">
+        <v>2000</v>
+      </c>
+      <c r="H23">
+        <v>2500</v>
+      </c>
+      <c r="L23">
+        <v>800</v>
+      </c>
+      <c r="N23" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="B24" s="14"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B25" s="14"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B26" s="14"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="14"/>
+      <c r="B27" s="14"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>515</v>
+      </c>
+      <c r="B30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30">
+        <v>5</v>
+      </c>
+      <c r="D30" t="s">
+        <v>30</v>
+      </c>
+      <c r="G30">
+        <v>2000</v>
+      </c>
+      <c r="H30">
+        <v>2500</v>
+      </c>
+      <c r="L30">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="18" t="s">
+        <v>522</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G31" s="17">
+        <v>3000</v>
+      </c>
+      <c r="H31" s="17">
+        <v>2500</v>
+      </c>
+      <c r="I31" s="17" t="s">
+        <v>565</v>
+      </c>
+      <c r="J31" s="17" t="s">
+        <v>573</v>
+      </c>
+      <c r="L31" s="17">
+        <v>1500</v>
+      </c>
+      <c r="M31" s="17" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="B32" t="s">
+        <v>29</v>
+      </c>
+      <c r="C32">
+        <v>5</v>
+      </c>
+      <c r="G32">
+        <v>3000</v>
+      </c>
+      <c r="H32">
+        <v>2500</v>
+      </c>
+      <c r="I32" t="s">
+        <v>565</v>
+      </c>
+      <c r="J32" t="s">
+        <v>573</v>
+      </c>
+      <c r="L32" s="17">
+        <v>1500</v>
+      </c>
+      <c r="M32" s="17" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33">
+        <v>5</v>
+      </c>
+      <c r="D33" t="s">
+        <v>30</v>
+      </c>
+      <c r="I33" t="s">
+        <v>565</v>
+      </c>
+      <c r="J33" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="D34" t="s">
+        <v>30</v>
+      </c>
+      <c r="G34">
+        <v>2000</v>
+      </c>
+      <c r="H34">
+        <v>2500</v>
+      </c>
+      <c r="I34" t="s">
+        <v>567</v>
+      </c>
+      <c r="J34" t="s">
+        <v>573</v>
+      </c>
+      <c r="L34">
+        <v>10000</v>
+      </c>
+      <c r="N34" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="D35" t="s">
+        <v>33</v>
+      </c>
+      <c r="F35">
+        <v>120000</v>
+      </c>
+      <c r="G35">
+        <v>2000</v>
+      </c>
+      <c r="H35">
+        <v>2500</v>
+      </c>
+      <c r="I35" t="s">
+        <v>565</v>
+      </c>
+      <c r="J35" t="s">
+        <v>573</v>
+      </c>
+      <c r="N35" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
+        <v>558</v>
+      </c>
+      <c r="D36" t="s">
+        <v>30</v>
+      </c>
+      <c r="I36" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>554</v>
+      </c>
+      <c r="D37" t="s">
+        <v>30</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>2500</v>
+      </c>
+      <c r="I37" t="s">
+        <v>565</v>
+      </c>
+      <c r="J37" t="s">
+        <v>573</v>
+      </c>
+      <c r="L37">
+        <v>10000</v>
+      </c>
+      <c r="N37" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
+        <v>584</v>
+      </c>
+      <c r="D38" t="s">
+        <v>30</v>
+      </c>
+      <c r="G38">
+        <v>2000</v>
+      </c>
+      <c r="H38">
+        <v>2500</v>
+      </c>
+      <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="M38" t="s">
+        <v>523</v>
+      </c>
+      <c r="N38" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>561</v>
+      </c>
+      <c r="D39" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D40" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="D41" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A42" s="16" t="s">
+        <v>566</v>
+      </c>
+      <c r="D42" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A43" s="14"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="D45" t="s">
+        <v>30</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45">
+        <v>2500</v>
+      </c>
+      <c r="L45">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
+        <v>553</v>
+      </c>
+      <c r="D46" t="s">
+        <v>30</v>
+      </c>
+      <c r="G46">
+        <v>0</v>
+      </c>
+      <c r="H46">
+        <v>2500</v>
+      </c>
+      <c r="L46">
+        <v>0</v>
+      </c>
+      <c r="M46" t="s">
+        <v>523</v>
+      </c>
+      <c r="N46" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="D47" t="s">
+        <v>30</v>
+      </c>
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47">
+        <v>2500</v>
+      </c>
+      <c r="L47">
+        <v>0</v>
+      </c>
+      <c r="N47" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="19" t="s">
+        <v>574</v>
+      </c>
+      <c r="D48" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G48" s="17">
+        <v>0</v>
+      </c>
+      <c r="H48" s="17">
+        <v>2500</v>
+      </c>
+      <c r="L48" s="17">
+        <v>1600</v>
+      </c>
+      <c r="N48" s="17" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50" s="18" t="s">
+        <v>518</v>
+      </c>
+      <c r="B50" s="17"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E50" s="17"/>
+      <c r="F50" s="17"/>
+      <c r="G50" s="17">
+        <v>0</v>
+      </c>
+      <c r="H50" s="17">
+        <v>2500</v>
+      </c>
+      <c r="I50" s="17"/>
+      <c r="J50" s="17"/>
+      <c r="K50" s="17"/>
+      <c r="L50" s="17">
+        <v>0</v>
+      </c>
+      <c r="M50" s="17" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A51" s="18" t="s">
+        <v>527</v>
+      </c>
+      <c r="B51" s="17"/>
+      <c r="C51" s="17"/>
+      <c r="D51" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E51" s="17">
+        <v>24000</v>
+      </c>
+      <c r="F51" s="17"/>
+      <c r="G51" s="17"/>
+      <c r="H51" s="17"/>
+      <c r="I51" s="17"/>
+      <c r="J51" s="17"/>
+      <c r="K51" s="17"/>
+      <c r="L51" s="17"/>
+      <c r="M51" s="17"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A52" s="18" t="s">
+        <v>524</v>
+      </c>
+      <c r="B52" s="17"/>
+      <c r="C52" s="17"/>
+      <c r="D52" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E52" s="17"/>
+      <c r="F52" s="17"/>
+      <c r="G52" s="17">
+        <v>0</v>
+      </c>
+      <c r="H52" s="17">
+        <v>2500</v>
+      </c>
+      <c r="I52" s="17"/>
+      <c r="J52" s="17"/>
+      <c r="K52" s="17"/>
+      <c r="L52" s="17">
+        <v>0</v>
+      </c>
+      <c r="M52" s="17" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A53" s="18" t="s">
+        <v>526</v>
+      </c>
+      <c r="B53" s="17"/>
+      <c r="C53" s="17"/>
+      <c r="D53" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E53" s="17">
+        <v>18000</v>
+      </c>
+      <c r="F53" s="17"/>
+      <c r="G53" s="17"/>
+      <c r="H53" s="17"/>
+      <c r="I53" s="17"/>
+      <c r="J53" s="17"/>
+      <c r="K53" s="17"/>
+      <c r="L53" s="17"/>
+      <c r="M53" s="17"/>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A54" s="18" t="s">
+        <v>539</v>
+      </c>
+      <c r="D54" t="s">
+        <v>30</v>
+      </c>
+      <c r="G54">
+        <v>0</v>
+      </c>
+      <c r="H54">
+        <v>2500</v>
+      </c>
+      <c r="L54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A55" s="18" t="s">
+        <v>540</v>
+      </c>
+      <c r="D55" t="s">
+        <v>31</v>
+      </c>
+      <c r="E55">
+        <v>27000</v>
+      </c>
+      <c r="N55" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A56" s="18" t="s">
+        <v>550</v>
+      </c>
+      <c r="D56" t="s">
+        <v>30</v>
+      </c>
+      <c r="G56">
+        <v>0</v>
+      </c>
+      <c r="H56">
+        <v>2500</v>
+      </c>
+      <c r="L56">
+        <v>400</v>
+      </c>
+      <c r="M56" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A57" s="18" t="s">
+        <v>551</v>
+      </c>
+      <c r="D57" t="s">
+        <v>31</v>
+      </c>
+      <c r="N57" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A58" s="13" t="s">
+        <v>576</v>
+      </c>
+      <c r="D58" t="s">
+        <v>30</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58">
+        <v>2500</v>
+      </c>
+      <c r="L58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A59" s="13" t="s">
+        <v>577</v>
+      </c>
+      <c r="D59" t="s">
+        <v>31</v>
+      </c>
+      <c r="E59">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A60" s="13" t="s">
+        <v>578</v>
+      </c>
+      <c r="D60" t="s">
+        <v>30</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60">
+        <v>2500</v>
+      </c>
+      <c r="L60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A61" s="13" t="s">
+        <v>579</v>
+      </c>
+      <c r="D61" t="s">
+        <v>31</v>
+      </c>
+      <c r="E61">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
+        <v>517</v>
+      </c>
+      <c r="D63" t="s">
+        <v>33</v>
+      </c>
+      <c r="F63">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A64" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="D64" t="s">
+        <v>33</v>
+      </c>
+      <c r="F64">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A65" s="7" t="s">
+        <v>542</v>
+      </c>
+      <c r="D65" t="s">
+        <v>33</v>
+      </c>
+      <c r="F65">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A66" s="7" t="s">
+        <v>544</v>
+      </c>
+      <c r="D66" t="s">
+        <v>33</v>
+      </c>
+      <c r="F66">
+        <v>120000</v>
+      </c>
+      <c r="K66">
+        <v>2</v>
+      </c>
+      <c r="N66" t="s">
+        <v>545</v>
+      </c>
+      <c r="P66" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A67" s="7" t="s">
+        <v>549</v>
+      </c>
+      <c r="D67" t="s">
+        <v>33</v>
+      </c>
+      <c r="F67">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A68" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="D68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F68">
+        <v>120000</v>
+      </c>
+      <c r="N68" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A69" s="7" t="s">
+        <v>581</v>
+      </c>
+      <c r="B69" t="s">
+        <v>28</v>
+      </c>
+      <c r="C69">
+        <v>2</v>
+      </c>
+      <c r="D69" t="s">
+        <v>33</v>
+      </c>
+      <c r="F69">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A70" s="7" t="s">
+        <v>580</v>
+      </c>
+      <c r="B70" t="s">
+        <v>28</v>
+      </c>
+      <c r="C70">
+        <v>11</v>
+      </c>
+      <c r="D70" t="s">
+        <v>33</v>
+      </c>
+      <c r="F70">
+        <v>60000</v>
+      </c>
+      <c r="K70">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>564</v>
+      </c>
+      <c r="D75" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>563</v>
+      </c>
+      <c r="D76" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>563</v>
+      </c>
+      <c r="D77" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3261DB23-C434-4F35-8B4F-998D4295A585}">
   <dimension ref="A1:P83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Adjust Bard opener weave accounting
Set the opener weave counter to three in the additional spell-effect logic and update spell data.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF037F1-95AB-4FAC-BF70-B34C82CD5175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8286EEB4-616C-4AD3-BEEA-82FFC004ACAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="14160" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="0" windowWidth="12800" windowHeight="13940" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1665" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1670" uniqueCount="588">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -6344,6 +6344,12 @@
       <c r="B22" t="s">
         <v>321</v>
       </c>
+      <c r="D22" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22">
+        <v>7</v>
+      </c>
       <c r="F22" t="s">
         <v>30</v>
       </c>
@@ -6367,10 +6373,10 @@
         <v>322</v>
       </c>
       <c r="D24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E24">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F24" t="s">
         <v>30</v>
@@ -6722,7 +6728,7 @@
         <v>349</v>
       </c>
       <c r="D47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E47">
         <v>7</v>
@@ -6744,6 +6750,9 @@
       <c r="C48" t="s">
         <v>349</v>
       </c>
+      <c r="F48" t="s">
+        <v>312</v>
+      </c>
       <c r="G48">
         <v>10000</v>
       </c>
@@ -6781,6 +6790,9 @@
       <c r="C50" t="s">
         <v>349</v>
       </c>
+      <c r="F50" t="s">
+        <v>312</v>
+      </c>
       <c r="G50">
         <v>20000</v>
       </c>
@@ -6818,6 +6830,9 @@
       <c r="C52" t="s">
         <v>349</v>
       </c>
+      <c r="F52" t="s">
+        <v>312</v>
+      </c>
       <c r="G52">
         <v>20000</v>
       </c>
@@ -6833,10 +6848,10 @@
         <v>349</v>
       </c>
       <c r="D53" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E53">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F53" t="s">
         <v>33</v>
@@ -6854,6 +6869,9 @@
       </c>
       <c r="C54" t="s">
         <v>349</v>
+      </c>
+      <c r="F54" t="s">
+        <v>312</v>
       </c>
       <c r="G54">
         <v>20000</v>

</xml_diff>

<commit_message>
Sequence the Bard opener and prioritize Empyreal Arrow
Select opening actions from tracked state and refine song and Pitch Perfect decisions.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8286EEB4-616C-4AD3-BEEA-82FFC004ACAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8731C99E-5496-44A1-8527-5815BB2A22D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="0" windowWidth="12800" windowHeight="13940" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1670" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1679" uniqueCount="591">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1001,9 +1001,6 @@
     <t>DoT</t>
   </si>
   <si>
-    <t>Hawk’s Eye procs</t>
-  </si>
-  <si>
     <t>80+, No overcap unless 2m burst soon</t>
   </si>
   <si>
@@ -1061,9 +1058,6 @@
     <t>Caustic DoT</t>
   </si>
   <si>
-    <t>Storm DoT;Caustic DoT</t>
-  </si>
-  <si>
     <t>Wanderer song</t>
   </si>
   <si>
@@ -1805,10 +1799,25 @@
     <t>Astral Gauge Full</t>
   </si>
   <si>
-    <t>todo</t>
-  </si>
-  <si>
-    <t>Todo</t>
+    <t>Storm DoT;Caustic DoT;Recent Refresh</t>
+  </si>
+  <si>
+    <t>Recent refresh</t>
+  </si>
+  <si>
+    <t>10y jump - 12 y  aoe - 25 y range -30 y buff</t>
+  </si>
+  <si>
+    <t>Radiant Finale Buff;Radiant Encore Ready</t>
+  </si>
+  <si>
+    <t>Barrage Buff;Resonant Arrow Ready</t>
+  </si>
+  <si>
+    <t>special refulgent arrow</t>
+  </si>
+  <si>
+    <t>Hawk’s Eye procs (treated in special section because 2 procs)</t>
   </si>
 </sst>
 </file>
@@ -2292,7 +2301,7 @@
         <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -2308,29 +2317,29 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>475</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" t="s">
         <v>477</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D4" t="s">
         <v>33</v>
       </c>
       <c r="G4" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -2341,13 +2350,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
@@ -2356,12 +2365,12 @@
         <v>300000</v>
       </c>
       <c r="G6" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -2387,7 +2396,7 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -2418,7 +2427,7 @@
         <v>2</v>
       </c>
       <c r="H10" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="I10" t="s">
         <v>47</v>
@@ -2452,7 +2461,7 @@
         <v>42</v>
       </c>
       <c r="H12" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -2547,7 +2556,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B19" t="s">
         <v>29</v>
@@ -2559,15 +2568,15 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H19" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D20" t="s">
         <v>31</v>
@@ -2576,12 +2585,12 @@
         <v>30000</v>
       </c>
       <c r="H20" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B21" t="s">
         <v>29</v>
@@ -2596,7 +2605,7 @@
         <v>8</v>
       </c>
       <c r="H21" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -2629,7 +2638,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B24" t="s">
         <v>29</v>
@@ -2661,7 +2670,7 @@
         <v>50</v>
       </c>
       <c r="H25" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -2959,7 +2968,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B45" t="s">
         <v>27</v>
@@ -2979,7 +2988,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B46" t="s">
         <v>27</v>
@@ -2991,7 +3000,7 @@
         <v>30</v>
       </c>
       <c r="H46" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
   </sheetData>
@@ -3054,29 +3063,29 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>475</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" t="s">
         <v>477</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D4" t="s">
         <v>33</v>
       </c>
       <c r="G4" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -3087,13 +3096,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
@@ -3102,12 +3111,12 @@
         <v>300000</v>
       </c>
       <c r="G6" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -3133,7 +3142,7 @@
         <v>52</v>
       </c>
       <c r="H9" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3164,7 +3173,7 @@
         <v>54</v>
       </c>
       <c r="H11" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -3192,7 +3201,7 @@
         <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="I13">
         <v>1</v>
@@ -3215,7 +3224,7 @@
         <v>84</v>
       </c>
       <c r="H15" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="I15">
         <v>-1</v>
@@ -3266,7 +3275,7 @@
         <v>60000</v>
       </c>
       <c r="H19" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="I19">
         <v>-1</v>
@@ -3289,10 +3298,10 @@
         <v>60000</v>
       </c>
       <c r="G21" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="H21" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="I21">
         <v>3</v>
@@ -3300,7 +3309,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="D22" t="s">
         <v>32</v>
@@ -3337,7 +3346,7 @@
         <v>61</v>
       </c>
       <c r="H25" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -3368,7 +3377,7 @@
         <v>88</v>
       </c>
       <c r="H27" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -3396,7 +3405,7 @@
         <v>30</v>
       </c>
       <c r="H29" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -3450,7 +3459,7 @@
         <v>33</v>
       </c>
       <c r="H33" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -3481,7 +3490,7 @@
         <v>82</v>
       </c>
       <c r="H35" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -3509,7 +3518,7 @@
         <v>33</v>
       </c>
       <c r="H37" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -3540,7 +3549,7 @@
         <v>83</v>
       </c>
       <c r="H39" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -3568,7 +3577,7 @@
         <v>33</v>
       </c>
       <c r="H41" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -3607,7 +3616,7 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B46" t="s">
         <v>29</v>
@@ -3619,7 +3628,7 @@
         <v>30</v>
       </c>
       <c r="H46" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
@@ -3678,12 +3687,12 @@
         <v>30</v>
       </c>
       <c r="H52" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B56" t="s">
         <v>29</v>
@@ -3695,15 +3704,15 @@
         <v>30</v>
       </c>
       <c r="G56" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="H56" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D57" t="s">
         <v>31</v>
@@ -3714,7 +3723,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B58" t="s">
         <v>29</v>
@@ -3726,15 +3735,15 @@
         <v>30</v>
       </c>
       <c r="G58" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="H58" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D59" t="s">
         <v>32</v>
@@ -3745,7 +3754,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B60" t="s">
         <v>28</v>
@@ -3757,7 +3766,7 @@
         <v>33</v>
       </c>
       <c r="H60" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -3774,7 +3783,7 @@
         <v>30</v>
       </c>
       <c r="H61" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="I61">
         <v>-1</v>
@@ -3867,29 +3876,29 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>475</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
         <v>477</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D5" t="s">
         <v>33</v>
       </c>
       <c r="G5" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D6" t="s">
         <v>31</v>
@@ -3900,13 +3909,13 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B7" t="s">
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D7" t="s">
         <v>33</v>
@@ -3915,12 +3924,12 @@
         <v>300000</v>
       </c>
       <c r="G7" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D8" t="s">
         <v>31</v>
@@ -4479,29 +4488,29 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>475</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
         <v>477</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -4512,13 +4521,13 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D8" t="s">
         <v>33</v>
@@ -4527,12 +4536,12 @@
         <v>300000</v>
       </c>
       <c r="G8" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
@@ -5319,7 +5328,7 @@
         <v>-1</v>
       </c>
       <c r="M71" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.25">
@@ -5342,7 +5351,7 @@
         <v>-1</v>
       </c>
       <c r="M72" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
@@ -5362,7 +5371,7 @@
         <v>-1</v>
       </c>
       <c r="M73" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
@@ -5505,7 +5514,7 @@
         <v>171</v>
       </c>
       <c r="H85" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -5732,29 +5741,29 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>475</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
         <v>477</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -5765,13 +5774,13 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D8" t="s">
         <v>33</v>
@@ -5780,12 +5789,12 @@
         <v>300000</v>
       </c>
       <c r="G8" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
@@ -5808,12 +5817,12 @@
         <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D13" t="s">
         <v>31</v>
@@ -5852,7 +5861,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
@@ -5881,12 +5890,12 @@
         <v>120000</v>
       </c>
       <c r="G17" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D18" t="s">
         <v>31</v>
@@ -5897,7 +5906,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D19" t="s">
         <v>32</v>
@@ -5920,7 +5929,7 @@
         <v>33</v>
       </c>
       <c r="H20" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -5942,7 +5951,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B22" t="s">
         <v>27</v>
@@ -5979,7 +5988,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B24" t="s">
         <v>29</v>
@@ -5999,7 +6008,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B25" t="s">
         <v>27</v>
@@ -6018,7 +6027,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD84FEA-D0D3-4F98-B644-3E9C52C4A2B7}">
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -6040,7 +6049,7 @@
         <v>303</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>25</v>
@@ -6073,11 +6082,14 @@
         <v>216</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="O1" s="1"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>586</v>
+      </c>
       <c r="K2" t="s">
         <v>293</v>
       </c>
@@ -6085,7 +6097,7 @@
         <v>314</v>
       </c>
       <c r="M2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -6096,70 +6108,73 @@
         <v>31</v>
       </c>
       <c r="G4">
-        <v>2450</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>475</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" t="s">
         <v>477</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>478</v>
-      </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" t="s">
-        <v>479</v>
+        <v>476</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>479</v>
-      </c>
-      <c r="D7" t="s">
+        <v>477</v>
+      </c>
+      <c r="F7" t="s">
         <v>31</v>
       </c>
-      <c r="E7">
+      <c r="G7">
         <v>3600000</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>505</v>
-      </c>
-      <c r="B8" t="s">
-        <v>27</v>
+        <v>503</v>
       </c>
       <c r="C8" t="s">
-        <v>480</v>
+        <v>347</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8">
+        <v>29</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8">
         <v>300000</v>
       </c>
-      <c r="G8" t="s">
-        <v>506</v>
+      <c r="I8" t="s">
+        <v>504</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>506</v>
-      </c>
-      <c r="D9" t="s">
+        <v>504</v>
+      </c>
+      <c r="F9" t="s">
         <v>31</v>
       </c>
-      <c r="E9">
+      <c r="G9">
         <v>30000</v>
       </c>
     </row>
@@ -6171,7 +6186,7 @@
         <v>313</v>
       </c>
       <c r="C12" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D12" t="s">
         <v>27</v>
@@ -6185,13 +6200,13 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B13" t="s">
+        <v>345</v>
+      </c>
+      <c r="C13" t="s">
         <v>347</v>
-      </c>
-      <c r="C13" t="s">
-        <v>349</v>
       </c>
       <c r="F13" t="s">
         <v>32</v>
@@ -6205,10 +6220,10 @@
         <v>283</v>
       </c>
       <c r="B14" t="s">
-        <v>318</v>
+        <v>590</v>
       </c>
       <c r="C14" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D14" t="s">
         <v>27</v>
@@ -6219,8 +6234,8 @@
       <c r="F14" t="s">
         <v>30</v>
       </c>
-      <c r="J14" t="s">
-        <v>346</v>
+      <c r="O14" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -6228,10 +6243,10 @@
         <v>287</v>
       </c>
       <c r="B15" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C15" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D15" t="s">
         <v>28</v>
@@ -6248,13 +6263,13 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>331</v>
+      </c>
+      <c r="B16" t="s">
         <v>332</v>
       </c>
-      <c r="B16" t="s">
-        <v>333</v>
-      </c>
       <c r="C16" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="F16" t="s">
         <v>32</v>
@@ -6268,22 +6283,22 @@
         <v>288</v>
       </c>
       <c r="B17" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C17" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E17">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F17" t="s">
         <v>30</v>
       </c>
       <c r="J17" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -6291,10 +6306,10 @@
         <v>291</v>
       </c>
       <c r="B18" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C18" t="s">
-        <v>586</v>
+        <v>347</v>
       </c>
       <c r="D18" t="s">
         <v>29</v>
@@ -6311,10 +6326,10 @@
         <v>292</v>
       </c>
       <c r="B19" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C19" t="s">
-        <v>586</v>
+        <v>347</v>
       </c>
       <c r="D19" t="s">
         <v>29</v>
@@ -6326,63 +6341,7 @@
         <v>30</v>
       </c>
       <c r="J19" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>334</v>
-      </c>
-      <c r="F21" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>289</v>
-      </c>
-      <c r="B22" t="s">
-        <v>321</v>
-      </c>
-      <c r="D22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E22">
-        <v>7</v>
-      </c>
-      <c r="F22" t="s">
-        <v>30</v>
-      </c>
-      <c r="J22" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>335</v>
-      </c>
-      <c r="F23" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>290</v>
-      </c>
-      <c r="B24" t="s">
-        <v>322</v>
-      </c>
-      <c r="D24" t="s">
-        <v>27</v>
-      </c>
-      <c r="E24">
-        <v>7</v>
-      </c>
-      <c r="F24" t="s">
-        <v>30</v>
-      </c>
-      <c r="J24" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -6393,7 +6352,7 @@
         <v>317</v>
       </c>
       <c r="C26" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -6405,15 +6364,15 @@
         <v>30</v>
       </c>
       <c r="I26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C27" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="F27" t="s">
         <v>312</v>
@@ -6430,7 +6389,7 @@
         <v>317</v>
       </c>
       <c r="C28" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D28" t="s">
         <v>27</v>
@@ -6442,15 +6401,15 @@
         <v>30</v>
       </c>
       <c r="I28" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C29" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="F29" t="s">
         <v>312</v>
@@ -6467,7 +6426,7 @@
         <v>316</v>
       </c>
       <c r="C30" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D30" t="s">
         <v>29</v>
@@ -6479,144 +6438,135 @@
         <v>30</v>
       </c>
       <c r="I30" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>351</v>
-      </c>
-      <c r="B32" t="s">
-        <v>304</v>
-      </c>
-      <c r="C32" t="s">
-        <v>349</v>
-      </c>
-      <c r="D32" t="s">
-        <v>27</v>
-      </c>
-      <c r="E32">
-        <v>8</v>
-      </c>
-      <c r="F32" t="s">
-        <v>33</v>
-      </c>
-      <c r="H32">
-        <v>120000</v>
-      </c>
-      <c r="I32" t="s">
-        <v>339</v>
-      </c>
-      <c r="J32" t="s">
-        <v>344</v>
+        <v>584</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>585</v>
+      </c>
+      <c r="F31" t="s">
+        <v>312</v>
+      </c>
+      <c r="G31">
+        <v>18000</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>339</v>
+        <v>349</v>
+      </c>
+      <c r="B33" t="s">
+        <v>304</v>
       </c>
       <c r="C33" t="s">
-        <v>349</v>
+        <v>347</v>
+      </c>
+      <c r="D33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E33">
+        <v>8</v>
       </c>
       <c r="F33" t="s">
-        <v>312</v>
-      </c>
-      <c r="G33">
-        <v>45000</v>
+        <v>33</v>
+      </c>
+      <c r="H33">
+        <v>120000</v>
+      </c>
+      <c r="I33" t="s">
+        <v>337</v>
+      </c>
+      <c r="J33" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>337</v>
+      </c>
+      <c r="C34" t="s">
+        <v>347</v>
+      </c>
+      <c r="F34" t="s">
+        <v>312</v>
+      </c>
+      <c r="G34">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>293</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>305</v>
       </c>
-      <c r="D34" t="s">
+      <c r="C35" t="s">
+        <v>347</v>
+      </c>
+      <c r="D35" t="s">
         <v>27</v>
       </c>
-      <c r="E34">
+      <c r="E35">
         <v>8</v>
       </c>
-      <c r="F34" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>352</v>
-      </c>
-      <c r="B36" t="s">
-        <v>309</v>
-      </c>
-      <c r="C36" t="s">
-        <v>349</v>
-      </c>
-      <c r="D36" t="s">
-        <v>28</v>
-      </c>
-      <c r="E36">
-        <v>8</v>
-      </c>
-      <c r="F36" t="s">
-        <v>33</v>
-      </c>
-      <c r="H36">
-        <v>120000</v>
-      </c>
-      <c r="I36" t="s">
-        <v>340</v>
-      </c>
-      <c r="J36" t="s">
-        <v>343</v>
+      <c r="F35" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>340</v>
+        <v>350</v>
+      </c>
+      <c r="B37" t="s">
+        <v>309</v>
       </c>
       <c r="C37" t="s">
-        <v>349</v>
+        <v>347</v>
+      </c>
+      <c r="D37" t="s">
+        <v>28</v>
+      </c>
+      <c r="E37">
+        <v>8</v>
       </c>
       <c r="F37" t="s">
-        <v>312</v>
-      </c>
-      <c r="G37">
-        <v>45000</v>
+        <v>33</v>
+      </c>
+      <c r="H37">
+        <v>120000</v>
+      </c>
+      <c r="I37" t="s">
+        <v>338</v>
+      </c>
+      <c r="J37" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>314</v>
-      </c>
-      <c r="B38" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
       <c r="C38" t="s">
-        <v>349</v>
-      </c>
-      <c r="D38" t="s">
-        <v>27</v>
-      </c>
-      <c r="E38">
-        <v>6</v>
+        <v>347</v>
       </c>
       <c r="F38" t="s">
-        <v>33</v>
-      </c>
-      <c r="H38">
-        <v>1500</v>
+        <v>312</v>
+      </c>
+      <c r="G38">
+        <v>45000</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>294</v>
+        <v>314</v>
       </c>
       <c r="B39" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="C39" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D39" t="s">
         <v>27</v>
@@ -6630,22 +6580,19 @@
       <c r="H39">
         <v>1500</v>
       </c>
-      <c r="L39">
-        <v>-1</v>
-      </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B40" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C40" t="s">
-        <v>587</v>
+        <v>347</v>
       </c>
       <c r="D40" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E40">
         <v>6</v>
@@ -6660,266 +6607,369 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>353</v>
-      </c>
-      <c r="B42" t="s">
-        <v>310</v>
-      </c>
-      <c r="C42" t="s">
-        <v>349</v>
-      </c>
-      <c r="D42" t="s">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>295</v>
+      </c>
+      <c r="B41" t="s">
+        <v>307</v>
+      </c>
+      <c r="C41" t="s">
+        <v>347</v>
+      </c>
+      <c r="D41" t="s">
         <v>29</v>
       </c>
-      <c r="E42">
-        <v>8</v>
-      </c>
-      <c r="F42" t="s">
-        <v>33</v>
-      </c>
-      <c r="H42">
-        <v>120000</v>
-      </c>
-      <c r="I42" t="s">
-        <v>341</v>
-      </c>
-      <c r="J42" t="s">
-        <v>342</v>
+      <c r="E41">
+        <v>6</v>
+      </c>
+      <c r="F41" t="s">
+        <v>33</v>
+      </c>
+      <c r="H41">
+        <v>1500</v>
+      </c>
+      <c r="L41">
+        <v>-1</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>341</v>
+        <v>351</v>
+      </c>
+      <c r="B43" t="s">
+        <v>310</v>
       </c>
       <c r="C43" t="s">
-        <v>349</v>
+        <v>347</v>
+      </c>
+      <c r="D43" t="s">
+        <v>29</v>
+      </c>
+      <c r="E43">
+        <v>8</v>
       </c>
       <c r="F43" t="s">
-        <v>312</v>
-      </c>
-      <c r="G43">
-        <v>45000</v>
+        <v>33</v>
+      </c>
+      <c r="H43">
+        <v>120000</v>
+      </c>
+      <c r="I43" t="s">
+        <v>339</v>
+      </c>
+      <c r="J43" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>339</v>
+      </c>
+      <c r="C44" t="s">
+        <v>347</v>
+      </c>
+      <c r="F44" t="s">
+        <v>312</v>
+      </c>
+      <c r="G44">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>296</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B45" t="s">
         <v>311</v>
       </c>
-      <c r="C44" t="s">
-        <v>350</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="C45" t="s">
+        <v>348</v>
+      </c>
+      <c r="F45" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>298</v>
-      </c>
-      <c r="B47" t="s">
-        <v>325</v>
-      </c>
-      <c r="C47" t="s">
-        <v>349</v>
-      </c>
-      <c r="D47" t="s">
-        <v>28</v>
-      </c>
-      <c r="E47">
-        <v>7</v>
-      </c>
-      <c r="F47" t="s">
-        <v>33</v>
-      </c>
-      <c r="H47">
-        <v>120000</v>
-      </c>
-      <c r="I47" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>298</v>
+      </c>
+      <c r="B48" t="s">
+        <v>324</v>
+      </c>
+      <c r="C48" t="s">
+        <v>347</v>
+      </c>
+      <c r="D48" t="s">
+        <v>28</v>
+      </c>
+      <c r="E48">
+        <v>7</v>
+      </c>
+      <c r="F48" t="s">
+        <v>33</v>
+      </c>
+      <c r="H48">
+        <v>120000</v>
+      </c>
+      <c r="I48" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>329</v>
+      </c>
+      <c r="B49" t="s">
+        <v>589</v>
+      </c>
+      <c r="C49" t="s">
+        <v>347</v>
+      </c>
+      <c r="F49" t="s">
+        <v>312</v>
+      </c>
+      <c r="G49">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>301</v>
+      </c>
+      <c r="B50" t="s">
+        <v>325</v>
+      </c>
+      <c r="C50" t="s">
+        <v>347</v>
+      </c>
+      <c r="D50" t="s">
+        <v>28</v>
+      </c>
+      <c r="E50">
+        <v>2</v>
+      </c>
+      <c r="F50" t="s">
+        <v>33</v>
+      </c>
+      <c r="H50">
+        <v>120000</v>
+      </c>
+      <c r="I50" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>326</v>
+      </c>
+      <c r="C51" t="s">
+        <v>347</v>
+      </c>
+      <c r="F51" t="s">
+        <v>312</v>
+      </c>
+      <c r="G51">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>299</v>
+      </c>
+      <c r="B52" t="s">
+        <v>324</v>
+      </c>
+      <c r="C52" t="s">
+        <v>347</v>
+      </c>
+      <c r="D52" t="s">
+        <v>29</v>
+      </c>
+      <c r="E52">
+        <v>2</v>
+      </c>
+      <c r="F52" t="s">
+        <v>33</v>
+      </c>
+      <c r="H52">
+        <v>120000</v>
+      </c>
+      <c r="I52" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>327</v>
+      </c>
+      <c r="C53" t="s">
+        <v>347</v>
+      </c>
+      <c r="F53" t="s">
+        <v>312</v>
+      </c>
+      <c r="G53">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>302</v>
+      </c>
+      <c r="B54" t="s">
+        <v>324</v>
+      </c>
+      <c r="C54" t="s">
+        <v>347</v>
+      </c>
+      <c r="D54" t="s">
+        <v>27</v>
+      </c>
+      <c r="E54">
+        <v>7</v>
+      </c>
+      <c r="F54" t="s">
+        <v>33</v>
+      </c>
+      <c r="H54">
+        <v>110000</v>
+      </c>
+      <c r="I54" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>328</v>
+      </c>
+      <c r="C55" t="s">
+        <v>347</v>
+      </c>
+      <c r="F55" t="s">
+        <v>312</v>
+      </c>
+      <c r="G55">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>333</v>
+      </c>
+      <c r="C57" t="s">
+        <v>347</v>
+      </c>
+      <c r="F57" t="s">
+        <v>32</v>
+      </c>
+      <c r="G57">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>289</v>
+      </c>
+      <c r="B58" t="s">
+        <v>320</v>
+      </c>
+      <c r="C58" t="s">
+        <v>347</v>
+      </c>
+      <c r="D58" t="s">
+        <v>28</v>
+      </c>
+      <c r="E58">
+        <v>7</v>
+      </c>
+      <c r="F58" t="s">
+        <v>30</v>
+      </c>
+      <c r="J58" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>334</v>
+      </c>
+      <c r="C59" t="s">
+        <v>347</v>
+      </c>
+      <c r="F59" t="s">
+        <v>32</v>
+      </c>
+      <c r="G59">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>290</v>
+      </c>
+      <c r="B60" t="s">
+        <v>321</v>
+      </c>
+      <c r="C60" t="s">
+        <v>347</v>
+      </c>
+      <c r="D60" t="s">
+        <v>27</v>
+      </c>
+      <c r="E60">
+        <v>7</v>
+      </c>
+      <c r="F60" t="s">
+        <v>30</v>
+      </c>
+      <c r="J60" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>300</v>
+      </c>
+      <c r="B62" t="s">
         <v>330</v>
       </c>
-      <c r="C48" t="s">
-        <v>349</v>
-      </c>
-      <c r="F48" t="s">
-        <v>312</v>
-      </c>
-      <c r="G48">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>301</v>
-      </c>
-      <c r="B49" t="s">
-        <v>326</v>
-      </c>
-      <c r="C49" t="s">
-        <v>349</v>
-      </c>
-      <c r="D49" t="s">
+      <c r="C62" t="s">
+        <v>347</v>
+      </c>
+      <c r="D62" t="s">
         <v>28</v>
       </c>
-      <c r="E49">
-        <v>2</v>
-      </c>
-      <c r="F49" t="s">
-        <v>33</v>
-      </c>
-      <c r="H49">
-        <v>120000</v>
-      </c>
-      <c r="I49" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>327</v>
-      </c>
-      <c r="C50" t="s">
-        <v>349</v>
-      </c>
-      <c r="F50" t="s">
-        <v>312</v>
-      </c>
-      <c r="G50">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>299</v>
-      </c>
-      <c r="B51" t="s">
-        <v>325</v>
-      </c>
-      <c r="C51" t="s">
-        <v>349</v>
-      </c>
-      <c r="D51" t="s">
-        <v>29</v>
-      </c>
-      <c r="E51">
-        <v>2</v>
-      </c>
-      <c r="F51" t="s">
-        <v>33</v>
-      </c>
-      <c r="H51">
-        <v>120000</v>
-      </c>
-      <c r="I51" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>328</v>
-      </c>
-      <c r="C52" t="s">
-        <v>349</v>
-      </c>
-      <c r="F52" t="s">
-        <v>312</v>
-      </c>
-      <c r="G52">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>302</v>
-      </c>
-      <c r="B53" t="s">
-        <v>325</v>
-      </c>
-      <c r="C53" t="s">
-        <v>349</v>
-      </c>
-      <c r="D53" t="s">
-        <v>27</v>
-      </c>
-      <c r="E53">
-        <v>7</v>
-      </c>
-      <c r="F53" t="s">
-        <v>33</v>
-      </c>
-      <c r="H53">
-        <v>110000</v>
-      </c>
-      <c r="I53" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>329</v>
-      </c>
-      <c r="C54" t="s">
-        <v>349</v>
-      </c>
-      <c r="F54" t="s">
-        <v>312</v>
-      </c>
-      <c r="G54">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>300</v>
-      </c>
-      <c r="B56" t="s">
-        <v>331</v>
-      </c>
-      <c r="C56" t="s">
-        <v>349</v>
-      </c>
-      <c r="D56" t="s">
+      <c r="E62">
+        <v>6</v>
+      </c>
+      <c r="F62" t="s">
+        <v>33</v>
+      </c>
+      <c r="H62">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>297</v>
+      </c>
+      <c r="B63" t="s">
+        <v>308</v>
+      </c>
+      <c r="C63" t="s">
+        <v>347</v>
+      </c>
+      <c r="D63" t="s">
         <v>28</v>
       </c>
-      <c r="E56">
-        <v>6</v>
-      </c>
-      <c r="F56" t="s">
-        <v>33</v>
-      </c>
-      <c r="H56">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>297</v>
-      </c>
-      <c r="B57" t="s">
-        <v>308</v>
-      </c>
-      <c r="C57" t="s">
-        <v>349</v>
-      </c>
-      <c r="D57" t="s">
-        <v>28</v>
-      </c>
-      <c r="E57">
+      <c r="E63">
         <v>5</v>
       </c>
-      <c r="F57" t="s">
-        <v>33</v>
-      </c>
-      <c r="H57">
+      <c r="F63" t="s">
+        <v>33</v>
+      </c>
+      <c r="H63">
         <v>15000</v>
       </c>
     </row>
@@ -6995,29 +7045,29 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>475</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
         <v>477</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -7028,13 +7078,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D8" t="s">
         <v>33</v>
@@ -7043,12 +7093,12 @@
         <v>300000</v>
       </c>
       <c r="G8" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
@@ -7074,7 +7124,7 @@
         <v>222</v>
       </c>
       <c r="H12" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -7091,7 +7141,7 @@
         <v>30</v>
       </c>
       <c r="G13" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="H13" t="s">
         <v>222</v>
@@ -7099,7 +7149,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="D14" t="s">
         <v>31</v>
@@ -7133,7 +7183,7 @@
         <v>30</v>
       </c>
       <c r="H16" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
@@ -7150,7 +7200,7 @@
         <v>30</v>
       </c>
       <c r="H17" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
@@ -7189,7 +7239,7 @@
         <v>30</v>
       </c>
       <c r="P20" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
@@ -7206,10 +7256,10 @@
         <v>30</v>
       </c>
       <c r="O21" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="P21" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
@@ -7248,7 +7298,7 @@
         <v>30</v>
       </c>
       <c r="P24" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
@@ -7265,7 +7315,7 @@
         <v>30</v>
       </c>
       <c r="P25" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
@@ -7420,7 +7470,7 @@
         <v>270</v>
       </c>
       <c r="H37" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -7860,7 +7910,7 @@
         <v>60000</v>
       </c>
       <c r="G70" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -7876,7 +7926,7 @@
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B73" t="s">
         <v>28</v>
@@ -7888,12 +7938,12 @@
         <v>33</v>
       </c>
       <c r="G73" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D74" t="s">
         <v>31</v>
@@ -7904,7 +7954,7 @@
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B75" t="s">
         <v>28</v>
@@ -7916,12 +7966,12 @@
         <v>33</v>
       </c>
       <c r="H75" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B77" t="s">
         <v>28</v>
@@ -7935,7 +7985,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="D79" t="s">
         <v>33</v>
@@ -7943,7 +7993,7 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="D80" t="s">
         <v>33</v>
@@ -7951,7 +8001,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B81" t="s">
         <v>29</v>
@@ -7965,7 +8015,7 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="B82" t="s">
         <v>28</v>
@@ -8021,10 +8071,10 @@
         <v>35</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>38</v>
@@ -8033,16 +8083,16 @@
         <v>39</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>303</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -8058,29 +8108,29 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>475</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" t="s">
         <v>477</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J3" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D4" t="s">
         <v>33</v>
       </c>
       <c r="I4" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -8091,13 +8141,13 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
@@ -8106,12 +8156,12 @@
         <v>300000</v>
       </c>
       <c r="I6" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -8122,7 +8172,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
@@ -8142,7 +8192,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B10" t="s">
         <v>27</v>
@@ -8190,7 +8240,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B13" t="s">
         <v>29</v>
@@ -8218,7 +8268,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="D17" t="s">
         <v>30</v>
@@ -8235,7 +8285,7 @@
     </row>
     <row r="18" spans="1:14" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="D18" s="17" t="s">
         <v>30</v>
@@ -8250,15 +8300,15 @@
         <v>800</v>
       </c>
       <c r="M18" s="17" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="N18" s="17" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="G19">
         <v>3000</v>
@@ -8267,21 +8317,21 @@
         <v>2500</v>
       </c>
       <c r="I19" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="J19" s="17" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="L19">
         <v>800</v>
       </c>
       <c r="M19" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="D20" t="s">
         <v>30</v>
@@ -8296,12 +8346,12 @@
         <v>800</v>
       </c>
       <c r="N20" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="D21" t="s">
         <v>30</v>
@@ -8316,15 +8366,15 @@
         <v>1000</v>
       </c>
       <c r="M21" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="N21" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="D22" t="s">
         <v>30</v>
@@ -8339,12 +8389,12 @@
         <v>0</v>
       </c>
       <c r="N22" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="B23" s="14"/>
       <c r="D23" t="s">
@@ -8360,24 +8410,24 @@
         <v>800</v>
       </c>
       <c r="N23" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="B24" s="14"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B25" s="14"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B26" s="14"/>
     </row>
@@ -8387,7 +8437,7 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B30" t="s">
         <v>27</v>
@@ -8410,7 +8460,7 @@
     </row>
     <row r="31" spans="1:14" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="18" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="D31" s="17" t="s">
         <v>30</v>
@@ -8422,21 +8472,21 @@
         <v>2500</v>
       </c>
       <c r="I31" s="17" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="J31" s="17" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="L31" s="17">
         <v>1500</v>
       </c>
       <c r="M31" s="17" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="B32" t="s">
         <v>29</v>
@@ -8451,21 +8501,21 @@
         <v>2500</v>
       </c>
       <c r="I32" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="J32" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="L32" s="17">
         <v>1500</v>
       </c>
       <c r="M32" s="17" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="B33" t="s">
         <v>28</v>
@@ -8477,15 +8527,15 @@
         <v>30</v>
       </c>
       <c r="I33" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="J33" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="D34" t="s">
         <v>30</v>
@@ -8497,21 +8547,21 @@
         <v>2500</v>
       </c>
       <c r="I34" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="J34" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="L34">
         <v>10000</v>
       </c>
       <c r="N34" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="D35" t="s">
         <v>33</v>
@@ -8526,29 +8576,29 @@
         <v>2500</v>
       </c>
       <c r="I35" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="J35" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="N35" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="D36" t="s">
         <v>30</v>
       </c>
       <c r="I36" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="D37" t="s">
         <v>30</v>
@@ -8560,21 +8610,21 @@
         <v>2500</v>
       </c>
       <c r="I37" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="J37" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="L37">
         <v>10000</v>
       </c>
       <c r="N37" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D38" t="s">
         <v>30</v>
@@ -8589,15 +8639,15 @@
         <v>0</v>
       </c>
       <c r="M38" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="N38" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="D39" t="s">
         <v>31</v>
@@ -8605,7 +8655,7 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="D40" t="s">
         <v>31</v>
@@ -8613,7 +8663,7 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="D41" t="s">
         <v>31</v>
@@ -8621,7 +8671,7 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="D42" t="s">
         <v>31</v>
@@ -8632,7 +8682,7 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="D45" t="s">
         <v>30</v>
@@ -8649,7 +8699,7 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="D46" t="s">
         <v>30</v>
@@ -8664,15 +8714,15 @@
         <v>0</v>
       </c>
       <c r="M46" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="N46" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="D47" t="s">
         <v>30</v>
@@ -8687,12 +8737,12 @@
         <v>0</v>
       </c>
       <c r="N47" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="48" spans="1:14" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="19" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="D48" s="17" t="s">
         <v>30</v>
@@ -8707,12 +8757,12 @@
         <v>1600</v>
       </c>
       <c r="N48" s="17" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="18" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="B50" s="17"/>
       <c r="C50" s="17"/>
@@ -8734,12 +8784,12 @@
         <v>0</v>
       </c>
       <c r="M50" s="17" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="18" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B51" s="17"/>
       <c r="C51" s="17"/>
@@ -8760,7 +8810,7 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="18" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="B52" s="17"/>
       <c r="C52" s="17"/>
@@ -8782,12 +8832,12 @@
         <v>0</v>
       </c>
       <c r="M52" s="17" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="18" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="B53" s="17"/>
       <c r="C53" s="17"/>
@@ -8808,7 +8858,7 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="18" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="D54" t="s">
         <v>30</v>
@@ -8825,7 +8875,7 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="18" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="D55" t="s">
         <v>31</v>
@@ -8834,12 +8884,12 @@
         <v>27000</v>
       </c>
       <c r="N55" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="18" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="D56" t="s">
         <v>30</v>
@@ -8854,23 +8904,23 @@
         <v>400</v>
       </c>
       <c r="M56" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="18" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="D57" t="s">
         <v>31</v>
       </c>
       <c r="N57" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="13" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D58" t="s">
         <v>30</v>
@@ -8887,7 +8937,7 @@
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D59" t="s">
         <v>31</v>
@@ -8898,7 +8948,7 @@
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="D60" t="s">
         <v>30</v>
@@ -8915,7 +8965,7 @@
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="D61" t="s">
         <v>31</v>
@@ -8926,7 +8976,7 @@
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D63" t="s">
         <v>33</v>
@@ -8937,7 +8987,7 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="D64" t="s">
         <v>33</v>
@@ -8948,7 +8998,7 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="D65" t="s">
         <v>33</v>
@@ -8959,7 +9009,7 @@
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="D66" t="s">
         <v>33</v>
@@ -8971,15 +9021,15 @@
         <v>2</v>
       </c>
       <c r="N66" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="P66" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="D67" t="s">
         <v>33</v>
@@ -8990,7 +9040,7 @@
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="D68" t="s">
         <v>33</v>
@@ -8999,12 +9049,12 @@
         <v>120000</v>
       </c>
       <c r="N68" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="B69" t="s">
         <v>28</v>
@@ -9021,7 +9071,7 @@
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B70" t="s">
         <v>28</v>
@@ -9041,7 +9091,7 @@
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="D75" t="s">
         <v>31</v>
@@ -9049,7 +9099,7 @@
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="D76" t="s">
         <v>31</v>
@@ -9057,7 +9107,7 @@
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="D77" t="s">
         <v>31</v>
@@ -9120,7 +9170,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="I2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -9134,28 +9184,28 @@
         <v>1960</v>
       </c>
       <c r="K3" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>475</v>
+      </c>
+      <c r="H4" t="s">
         <v>477</v>
-      </c>
-      <c r="H4" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="G5" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D6" t="s">
         <v>31</v>
@@ -9166,13 +9216,13 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B7" t="s">
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D7" t="s">
         <v>33</v>
@@ -9181,12 +9231,12 @@
         <v>300000</v>
       </c>
       <c r="G7" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D8" t="s">
         <v>31</v>
@@ -9197,7 +9247,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D11" t="s">
         <v>32</v>
@@ -9208,7 +9258,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D12" t="s">
         <v>31</v>
@@ -9219,7 +9269,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B13" t="s">
         <v>27</v>
@@ -9231,21 +9281,21 @@
         <v>30</v>
       </c>
       <c r="G13" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="H13" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="K13" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="N13" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B14" t="s">
         <v>28</v>
@@ -9257,24 +9307,24 @@
         <v>30</v>
       </c>
       <c r="G14" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="H14" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="K14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="M14" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="N14" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B15" t="s">
         <v>29</v>
@@ -9286,18 +9336,18 @@
         <v>30</v>
       </c>
       <c r="G15" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="H15" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="K15" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="D17" t="s">
         <v>32</v>
@@ -9308,7 +9358,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="D18" t="s">
         <v>31</v>
@@ -9319,7 +9369,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B19" t="s">
         <v>27</v>
@@ -9331,21 +9381,21 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="H19" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="K19" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="N19" s="12" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B20" t="s">
         <v>28</v>
@@ -9357,21 +9407,21 @@
         <v>30</v>
       </c>
       <c r="G20" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="H20" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="K20" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="M20" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B21" t="s">
         <v>29</v>
@@ -9383,18 +9433,18 @@
         <v>30</v>
       </c>
       <c r="G21" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="H21" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="K21" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D23" t="s">
         <v>32</v>
@@ -9405,7 +9455,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B24" t="s">
         <v>27</v>
@@ -9417,21 +9467,21 @@
         <v>30</v>
       </c>
       <c r="G24" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="H24" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="I24">
         <v>-1</v>
       </c>
       <c r="K24" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B25" t="s">
         <v>28</v>
@@ -9443,24 +9493,24 @@
         <v>30</v>
       </c>
       <c r="G25" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="H25" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="I25">
         <v>2</v>
       </c>
       <c r="K25" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="M25" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B26" t="s">
         <v>29</v>
@@ -9472,18 +9522,18 @@
         <v>30</v>
       </c>
       <c r="G26" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="H26" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="K26" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B28" t="s">
         <v>27</v>
@@ -9499,15 +9549,15 @@
         <v>3920</v>
       </c>
       <c r="K28" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="N28" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B29" t="s">
         <v>27</v>
@@ -9522,15 +9572,15 @@
         <v>1000</v>
       </c>
       <c r="K29" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="N29" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="B30" t="s">
         <v>27</v>
@@ -9542,12 +9592,12 @@
         <v>33</v>
       </c>
       <c r="K30" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B31" t="s">
         <v>29</v>
@@ -9562,15 +9612,15 @@
         <v>1000</v>
       </c>
       <c r="K31" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="N31" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B32" t="s">
         <v>29</v>
@@ -9582,17 +9632,17 @@
         <v>33</v>
       </c>
       <c r="K32" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="N33" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B34" t="s">
         <v>27</v>
@@ -9604,21 +9654,21 @@
         <v>33</v>
       </c>
       <c r="G34" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="H34" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="K34" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="N34" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="D35" t="s">
         <v>31</v>
@@ -9627,12 +9677,12 @@
         <v>20000</v>
       </c>
       <c r="N35" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="D36" t="s">
         <v>31</v>
@@ -9643,7 +9693,7 @@
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D37" t="s">
         <v>31</v>
@@ -9654,7 +9704,7 @@
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="D38" t="s">
         <v>31</v>
@@ -9665,7 +9715,7 @@
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B39" t="s">
         <v>28</v>
@@ -9677,12 +9727,12 @@
         <v>30</v>
       </c>
       <c r="N39" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="B40" t="s">
         <v>28</v>
@@ -9694,15 +9744,15 @@
         <v>30</v>
       </c>
       <c r="G40" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="H40" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="B41" t="s">
         <v>28</v>
@@ -9714,15 +9764,15 @@
         <v>30</v>
       </c>
       <c r="G41" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="H41" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B42" t="s">
         <v>28</v>
@@ -9734,15 +9784,15 @@
         <v>30</v>
       </c>
       <c r="G42" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="H42" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="B43" t="s">
         <v>28</v>
@@ -9754,15 +9804,15 @@
         <v>30</v>
       </c>
       <c r="G43" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="H43" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B45" t="s">
         <v>29</v>
@@ -9774,18 +9824,18 @@
         <v>30</v>
       </c>
       <c r="G45" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="K45" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="N45" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D46" t="s">
         <v>32</v>
@@ -9796,12 +9846,12 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="N47" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B48" t="s">
         <v>27</v>
@@ -9816,18 +9866,18 @@
         <v>60000</v>
       </c>
       <c r="G48" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="K48" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="P48" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D49" t="s">
         <v>32</v>
@@ -9838,7 +9888,7 @@
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D50" t="s">
         <v>31</v>
@@ -9847,12 +9897,12 @@
         <v>20000</v>
       </c>
       <c r="K50" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B51" t="s">
         <v>27</v>
@@ -9864,15 +9914,15 @@
         <v>30</v>
       </c>
       <c r="G51" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="H51" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B52" t="s">
         <v>28</v>
@@ -9887,12 +9937,12 @@
         <v>90000</v>
       </c>
       <c r="G52" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D53" t="s">
         <v>32</v>
@@ -9903,7 +9953,7 @@
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D54" t="s">
         <v>31</v>
@@ -9914,7 +9964,7 @@
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B55" t="s">
         <v>28</v>
@@ -9926,12 +9976,12 @@
         <v>30</v>
       </c>
       <c r="H55" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B57" t="s">
         <v>29</v>
@@ -9940,21 +9990,21 @@
         <v>9</v>
       </c>
       <c r="D57" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="F57">
         <v>120000</v>
       </c>
       <c r="G57" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="H57" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D58" t="s">
         <v>31</v>
@@ -9965,7 +10015,7 @@
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B61" t="s">
         <v>27</v>
@@ -9985,7 +10035,7 @@
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B62" t="s">
         <v>27</v>
@@ -9994,12 +10044,12 @@
         <v>11</v>
       </c>
       <c r="D62" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B63" t="s">
         <v>27</v>
@@ -10008,7 +10058,7 @@
         <v>11</v>
       </c>
       <c r="D63" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="E63">
         <v>30000</v>
@@ -10016,7 +10066,7 @@
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D64" t="s">
         <v>31</v>
@@ -10030,7 +10080,7 @@
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B65" t="s">
         <v>28</v>
@@ -10050,7 +10100,7 @@
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B66" t="s">
         <v>29</v>
@@ -10070,7 +10120,7 @@
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B67" t="s">
         <v>28</v>
@@ -10090,7 +10140,7 @@
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B72" t="s">
         <v>27</v>
@@ -10104,7 +10154,7 @@
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B73" t="s">
         <v>28</v>
@@ -10118,7 +10168,7 @@
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B74" t="s">
         <v>27</v>
@@ -10132,7 +10182,7 @@
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B75" t="s">
         <v>28</v>
@@ -10143,35 +10193,35 @@
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>471</v>
+      </c>
+      <c r="G78" t="s">
         <v>473</v>
       </c>
-      <c r="G78" t="s">
-        <v>475</v>
-      </c>
       <c r="H78" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="K78" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>472</v>
+      </c>
+      <c r="G79" t="s">
         <v>474</v>
       </c>
-      <c r="G79" t="s">
-        <v>476</v>
-      </c>
       <c r="H79" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K79" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="E80">
         <v>3600000</v>
@@ -10179,7 +10229,7 @@
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E81">
         <v>3600000</v>
@@ -10187,7 +10237,7 @@
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="L83" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine Bard DoT, burst and late-weave decisions
Track the last cast and status activation names and add helpers for burst readiness and Iron Jaws.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8731C99E-5496-44A1-8527-5815BB2A22D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3C191D2-141D-4270-AF08-6562154AD23E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1679" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1692" uniqueCount="598">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1818,6 +1818,27 @@
   </si>
   <si>
     <t>Hawk’s Eye procs (treated in special section because 2 procs)</t>
+  </si>
+  <si>
+    <t>Avoid double refresh in burst ! To be replaced by a test on the Dot Buffs because it doesn't account redot sceanrr</t>
+  </si>
+  <si>
+    <t>reDOT Storm</t>
+  </si>
+  <si>
+    <t>reDOT Caustic</t>
+  </si>
+  <si>
+    <t>Custom spell to force a redot without breaking other stuff</t>
+  </si>
+  <si>
+    <t>Actually useless</t>
+  </si>
+  <si>
+    <t>Storm DoT;Caustic DoT</t>
+  </si>
+  <si>
+    <t>DOT Again</t>
   </si>
 </sst>
 </file>
@@ -6027,7 +6048,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD84FEA-D0D3-4F98-B644-3E9C52C4A2B7}">
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -6366,6 +6387,9 @@
       <c r="I26" t="s">
         <v>335</v>
       </c>
+      <c r="J26" t="s">
+        <v>592</v>
+      </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -6403,6 +6427,9 @@
       <c r="I28" t="s">
         <v>336</v>
       </c>
+      <c r="J28" t="s">
+        <v>593</v>
+      </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -6445,6 +6472,9 @@
       <c r="A31" t="s">
         <v>585</v>
       </c>
+      <c r="B31" t="s">
+        <v>591</v>
+      </c>
       <c r="F31" t="s">
         <v>312</v>
       </c>
@@ -6452,81 +6482,54 @@
         <v>18000</v>
       </c>
     </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>592</v>
+      </c>
+      <c r="B32" t="s">
+        <v>595</v>
+      </c>
+      <c r="F32" t="s">
+        <v>312</v>
+      </c>
+    </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>349</v>
+        <v>593</v>
       </c>
       <c r="B33" t="s">
-        <v>304</v>
-      </c>
-      <c r="C33" t="s">
-        <v>347</v>
-      </c>
-      <c r="D33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E33">
-        <v>8</v>
+        <v>595</v>
       </c>
       <c r="F33" t="s">
-        <v>33</v>
-      </c>
-      <c r="H33">
-        <v>120000</v>
-      </c>
-      <c r="I33" t="s">
-        <v>337</v>
-      </c>
-      <c r="J33" t="s">
-        <v>342</v>
+        <v>312</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>337</v>
-      </c>
-      <c r="C34" t="s">
-        <v>347</v>
+        <v>597</v>
+      </c>
+      <c r="B34" t="s">
+        <v>594</v>
       </c>
       <c r="F34" t="s">
-        <v>312</v>
-      </c>
-      <c r="G34">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>293</v>
-      </c>
-      <c r="B35" t="s">
-        <v>305</v>
-      </c>
-      <c r="C35" t="s">
-        <v>347</v>
-      </c>
-      <c r="D35" t="s">
-        <v>27</v>
-      </c>
-      <c r="E35">
-        <v>8</v>
-      </c>
-      <c r="F35" t="s">
-        <v>33</v>
+        <v>33</v>
+      </c>
+      <c r="J34" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B37" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C37" t="s">
         <v>347</v>
       </c>
       <c r="D37" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E37">
         <v>8</v>
@@ -6538,15 +6541,15 @@
         <v>120000</v>
       </c>
       <c r="I37" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="J37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C38" t="s">
         <v>347</v>
@@ -6560,10 +6563,10 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>314</v>
+        <v>293</v>
       </c>
       <c r="B39" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="C39" t="s">
         <v>347</v>
@@ -6572,210 +6575,190 @@
         <v>27</v>
       </c>
       <c r="E39">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F39" t="s">
         <v>33</v>
-      </c>
-      <c r="H39">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>294</v>
-      </c>
-      <c r="B40" t="s">
-        <v>306</v>
-      </c>
-      <c r="C40" t="s">
-        <v>347</v>
-      </c>
-      <c r="D40" t="s">
-        <v>27</v>
-      </c>
-      <c r="E40">
-        <v>6</v>
-      </c>
-      <c r="F40" t="s">
-        <v>33</v>
-      </c>
-      <c r="H40">
-        <v>1500</v>
-      </c>
-      <c r="L40">
-        <v>-1</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>295</v>
+        <v>350</v>
       </c>
       <c r="B41" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C41" t="s">
         <v>347</v>
       </c>
       <c r="D41" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E41">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F41" t="s">
         <v>33</v>
       </c>
       <c r="H41">
-        <v>1500</v>
-      </c>
-      <c r="L41">
-        <v>-1</v>
+        <v>120000</v>
+      </c>
+      <c r="I41" t="s">
+        <v>338</v>
+      </c>
+      <c r="J41" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>338</v>
+      </c>
+      <c r="C42" t="s">
+        <v>347</v>
+      </c>
+      <c r="F42" t="s">
+        <v>312</v>
+      </c>
+      <c r="G42">
+        <v>45000</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>351</v>
+        <v>314</v>
       </c>
       <c r="B43" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="C43" t="s">
         <v>347</v>
       </c>
       <c r="D43" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E43">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F43" t="s">
         <v>33</v>
       </c>
       <c r="H43">
-        <v>120000</v>
-      </c>
-      <c r="I43" t="s">
-        <v>339</v>
-      </c>
-      <c r="J43" t="s">
-        <v>340</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>339</v>
+        <v>294</v>
+      </c>
+      <c r="B44" t="s">
+        <v>306</v>
       </c>
       <c r="C44" t="s">
         <v>347</v>
       </c>
+      <c r="D44" t="s">
+        <v>27</v>
+      </c>
+      <c r="E44">
+        <v>6</v>
+      </c>
       <c r="F44" t="s">
-        <v>312</v>
-      </c>
-      <c r="G44">
-        <v>45000</v>
+        <v>33</v>
+      </c>
+      <c r="H44">
+        <v>1500</v>
+      </c>
+      <c r="L44">
+        <v>-1</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B45" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C45" t="s">
-        <v>348</v>
+        <v>347</v>
+      </c>
+      <c r="D45" t="s">
+        <v>29</v>
+      </c>
+      <c r="E45">
+        <v>6</v>
       </c>
       <c r="F45" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="H45">
+        <v>1500</v>
+      </c>
+      <c r="L45">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>351</v>
+      </c>
+      <c r="B47" t="s">
+        <v>310</v>
+      </c>
+      <c r="C47" t="s">
+        <v>347</v>
+      </c>
+      <c r="D47" t="s">
+        <v>29</v>
+      </c>
+      <c r="E47">
+        <v>8</v>
+      </c>
+      <c r="F47" t="s">
+        <v>33</v>
+      </c>
+      <c r="H47">
+        <v>120000</v>
+      </c>
+      <c r="I47" t="s">
+        <v>339</v>
+      </c>
+      <c r="J47" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>298</v>
-      </c>
-      <c r="B48" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="C48" t="s">
         <v>347</v>
       </c>
-      <c r="D48" t="s">
-        <v>28</v>
-      </c>
-      <c r="E48">
-        <v>7</v>
-      </c>
       <c r="F48" t="s">
-        <v>33</v>
-      </c>
-      <c r="H48">
-        <v>120000</v>
-      </c>
-      <c r="I48" t="s">
-        <v>588</v>
+        <v>312</v>
+      </c>
+      <c r="G48">
+        <v>45000</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>329</v>
+        <v>296</v>
       </c>
       <c r="B49" t="s">
-        <v>589</v>
+        <v>311</v>
       </c>
       <c r="C49" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F49" t="s">
-        <v>312</v>
-      </c>
-      <c r="G49">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>301</v>
-      </c>
-      <c r="B50" t="s">
-        <v>325</v>
-      </c>
-      <c r="C50" t="s">
-        <v>347</v>
-      </c>
-      <c r="D50" t="s">
-        <v>28</v>
-      </c>
-      <c r="E50">
-        <v>2</v>
-      </c>
-      <c r="F50" t="s">
-        <v>33</v>
-      </c>
-      <c r="H50">
-        <v>120000</v>
-      </c>
-      <c r="I50" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>326</v>
-      </c>
-      <c r="C51" t="s">
-        <v>347</v>
-      </c>
-      <c r="F51" t="s">
-        <v>312</v>
-      </c>
-      <c r="G51">
-        <v>20000</v>
+        <v>32</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B52" t="s">
         <v>324</v>
@@ -6787,7 +6770,7 @@
         <v>29</v>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F52" t="s">
         <v>33</v>
@@ -6796,12 +6779,15 @@
         <v>120000</v>
       </c>
       <c r="I52" t="s">
-        <v>327</v>
+        <v>588</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>327</v>
+        <v>329</v>
+      </c>
+      <c r="B53" t="s">
+        <v>589</v>
       </c>
       <c r="C53" t="s">
         <v>347</v>
@@ -6810,38 +6796,38 @@
         <v>312</v>
       </c>
       <c r="G53">
-        <v>20000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B54" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C54" t="s">
         <v>347</v>
       </c>
       <c r="D54" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E54">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F54" t="s">
         <v>33</v>
       </c>
       <c r="H54">
-        <v>110000</v>
+        <v>120000</v>
       </c>
       <c r="I54" t="s">
-        <v>587</v>
+        <v>326</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C55" t="s">
         <v>347</v>
@@ -6853,123 +6839,203 @@
         <v>20000</v>
       </c>
     </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>299</v>
+      </c>
+      <c r="B56" t="s">
+        <v>324</v>
+      </c>
+      <c r="C56" t="s">
+        <v>347</v>
+      </c>
+      <c r="D56" t="s">
+        <v>28</v>
+      </c>
+      <c r="E56">
+        <v>7</v>
+      </c>
+      <c r="F56" t="s">
+        <v>33</v>
+      </c>
+      <c r="H56">
+        <v>120000</v>
+      </c>
+      <c r="I56" t="s">
+        <v>327</v>
+      </c>
+    </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="C57" t="s">
         <v>347</v>
       </c>
       <c r="F57" t="s">
-        <v>32</v>
+        <v>312</v>
       </c>
       <c r="G57">
-        <v>30000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="B58" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C58" t="s">
         <v>347</v>
       </c>
       <c r="D58" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E58">
         <v>7</v>
       </c>
       <c r="F58" t="s">
-        <v>30</v>
-      </c>
-      <c r="J58" t="s">
-        <v>333</v>
+        <v>33</v>
+      </c>
+      <c r="H58">
+        <v>110000</v>
+      </c>
+      <c r="I58" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="C59" t="s">
         <v>347</v>
       </c>
       <c r="F59" t="s">
+        <v>312</v>
+      </c>
+      <c r="G59">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>333</v>
+      </c>
+      <c r="C61" t="s">
+        <v>347</v>
+      </c>
+      <c r="F61" t="s">
         <v>32</v>
       </c>
-      <c r="G59">
+      <c r="G61">
         <v>30000</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>290</v>
-      </c>
-      <c r="B60" t="s">
-        <v>321</v>
-      </c>
-      <c r="C60" t="s">
-        <v>347</v>
-      </c>
-      <c r="D60" t="s">
-        <v>27</v>
-      </c>
-      <c r="E60">
-        <v>7</v>
-      </c>
-      <c r="F60" t="s">
-        <v>30</v>
-      </c>
-      <c r="J60" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="B62" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="C62" t="s">
         <v>347</v>
       </c>
       <c r="D62" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E62">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F62" t="s">
-        <v>33</v>
-      </c>
-      <c r="H62">
-        <v>60000</v>
+        <v>30</v>
+      </c>
+      <c r="J62" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>297</v>
-      </c>
-      <c r="B63" t="s">
-        <v>308</v>
+        <v>334</v>
       </c>
       <c r="C63" t="s">
         <v>347</v>
       </c>
-      <c r="D63" t="s">
+      <c r="F63" t="s">
+        <v>32</v>
+      </c>
+      <c r="G63">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>290</v>
+      </c>
+      <c r="B64" t="s">
+        <v>321</v>
+      </c>
+      <c r="C64" t="s">
+        <v>347</v>
+      </c>
+      <c r="D64" t="s">
+        <v>27</v>
+      </c>
+      <c r="E64">
+        <v>7</v>
+      </c>
+      <c r="F64" t="s">
+        <v>30</v>
+      </c>
+      <c r="J64" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>300</v>
+      </c>
+      <c r="B66" t="s">
+        <v>330</v>
+      </c>
+      <c r="C66" t="s">
+        <v>347</v>
+      </c>
+      <c r="D66" t="s">
         <v>28</v>
       </c>
-      <c r="E63">
+      <c r="E66">
+        <v>6</v>
+      </c>
+      <c r="F66" t="s">
+        <v>33</v>
+      </c>
+      <c r="H66">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>297</v>
+      </c>
+      <c r="B67" t="s">
+        <v>308</v>
+      </c>
+      <c r="C67" t="s">
+        <v>347</v>
+      </c>
+      <c r="D67" t="s">
+        <v>28</v>
+      </c>
+      <c r="E67">
         <v>5</v>
       </c>
-      <c r="F63" t="s">
-        <v>33</v>
-      </c>
-      <c r="H63">
+      <c r="F67" t="s">
+        <v>33</v>
+      </c>
+      <c r="H67">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Limit Bard weaving during Army's Paeon
Restrict late or second weaves during Paeon, revise song selection and adjust DoT permissions.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3C191D2-141D-4270-AF08-6562154AD23E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802C9060-45A3-4F60-BC51-F941FFD1D856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1692" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1697" uniqueCount="600">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1835,10 +1835,16 @@
     <t>Actually useless</t>
   </si>
   <si>
-    <t>Storm DoT;Caustic DoT</t>
-  </si>
-  <si>
     <t>DOT Again</t>
+  </si>
+  <si>
+    <t>DOT Stop</t>
+  </si>
+  <si>
+    <t>Do Not Dot</t>
+  </si>
+  <si>
+    <t>Storm DoT;Caustic DoT;Do Not Dot</t>
   </si>
 </sst>
 </file>
@@ -6048,7 +6054,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD84FEA-D0D3-4F98-B644-3E9C52C4A2B7}">
-  <dimension ref="A1:O67"/>
+  <dimension ref="A1:O68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -6506,7 +6512,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B34" t="s">
         <v>594</v>
@@ -6515,144 +6521,143 @@
         <v>33</v>
       </c>
       <c r="J34" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>349</v>
-      </c>
-      <c r="B37" t="s">
-        <v>304</v>
-      </c>
-      <c r="C37" t="s">
-        <v>347</v>
-      </c>
-      <c r="D37" t="s">
-        <v>27</v>
-      </c>
-      <c r="E37">
-        <v>8</v>
-      </c>
-      <c r="F37" t="s">
-        <v>33</v>
-      </c>
-      <c r="H37">
-        <v>120000</v>
-      </c>
-      <c r="I37" t="s">
-        <v>337</v>
-      </c>
-      <c r="J37" t="s">
-        <v>342</v>
+        <v>599</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>597</v>
+      </c>
+      <c r="F35" t="s">
+        <v>33</v>
+      </c>
+      <c r="I35" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>598</v>
+      </c>
+      <c r="F36" t="s">
+        <v>312</v>
+      </c>
+      <c r="G36">
+        <v>1200000</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>337</v>
+        <v>349</v>
+      </c>
+      <c r="B38" t="s">
+        <v>304</v>
       </c>
       <c r="C38" t="s">
         <v>347</v>
       </c>
+      <c r="D38" t="s">
+        <v>27</v>
+      </c>
+      <c r="E38">
+        <v>8</v>
+      </c>
       <c r="F38" t="s">
-        <v>312</v>
-      </c>
-      <c r="G38">
-        <v>45000</v>
+        <v>33</v>
+      </c>
+      <c r="H38">
+        <v>120000</v>
+      </c>
+      <c r="I38" t="s">
+        <v>337</v>
+      </c>
+      <c r="J38" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>293</v>
-      </c>
-      <c r="B39" t="s">
-        <v>305</v>
+        <v>337</v>
       </c>
       <c r="C39" t="s">
         <v>347</v>
       </c>
-      <c r="D39" t="s">
+      <c r="F39" t="s">
+        <v>312</v>
+      </c>
+      <c r="G39">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>293</v>
+      </c>
+      <c r="B40" t="s">
+        <v>305</v>
+      </c>
+      <c r="C40" t="s">
+        <v>347</v>
+      </c>
+      <c r="D40" t="s">
         <v>27</v>
       </c>
-      <c r="E39">
+      <c r="E40">
         <v>8</v>
       </c>
-      <c r="F39" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>350</v>
-      </c>
-      <c r="B41" t="s">
-        <v>309</v>
-      </c>
-      <c r="C41" t="s">
-        <v>347</v>
-      </c>
-      <c r="D41" t="s">
-        <v>28</v>
-      </c>
-      <c r="E41">
-        <v>8</v>
-      </c>
-      <c r="F41" t="s">
-        <v>33</v>
-      </c>
-      <c r="H41">
-        <v>120000</v>
-      </c>
-      <c r="I41" t="s">
-        <v>338</v>
-      </c>
-      <c r="J41" t="s">
-        <v>341</v>
+      <c r="F40" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>338</v>
+        <v>350</v>
+      </c>
+      <c r="B42" t="s">
+        <v>309</v>
       </c>
       <c r="C42" t="s">
         <v>347</v>
       </c>
+      <c r="D42" t="s">
+        <v>28</v>
+      </c>
+      <c r="E42">
+        <v>8</v>
+      </c>
       <c r="F42" t="s">
-        <v>312</v>
-      </c>
-      <c r="G42">
-        <v>45000</v>
+        <v>33</v>
+      </c>
+      <c r="H42">
+        <v>120000</v>
+      </c>
+      <c r="I42" t="s">
+        <v>338</v>
+      </c>
+      <c r="J42" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>314</v>
-      </c>
-      <c r="B43" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
       <c r="C43" t="s">
         <v>347</v>
       </c>
-      <c r="D43" t="s">
-        <v>27</v>
-      </c>
-      <c r="E43">
-        <v>6</v>
-      </c>
       <c r="F43" t="s">
-        <v>33</v>
-      </c>
-      <c r="H43">
-        <v>1500</v>
+        <v>312</v>
+      </c>
+      <c r="G43">
+        <v>45000</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>294</v>
+        <v>314</v>
       </c>
       <c r="B44" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="C44" t="s">
         <v>347</v>
@@ -6669,22 +6674,19 @@
       <c r="H44">
         <v>1500</v>
       </c>
-      <c r="L44">
-        <v>-1</v>
-      </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B45" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C45" t="s">
         <v>347</v>
       </c>
       <c r="D45" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E45">
         <v>6</v>
@@ -6699,329 +6701,332 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>351</v>
-      </c>
-      <c r="B47" t="s">
-        <v>310</v>
-      </c>
-      <c r="C47" t="s">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>295</v>
+      </c>
+      <c r="B46" t="s">
+        <v>307</v>
+      </c>
+      <c r="C46" t="s">
         <v>347</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D46" t="s">
         <v>29</v>
       </c>
-      <c r="E47">
-        <v>8</v>
-      </c>
-      <c r="F47" t="s">
-        <v>33</v>
-      </c>
-      <c r="H47">
-        <v>120000</v>
-      </c>
-      <c r="I47" t="s">
-        <v>339</v>
-      </c>
-      <c r="J47" t="s">
-        <v>340</v>
+      <c r="E46">
+        <v>6</v>
+      </c>
+      <c r="F46" t="s">
+        <v>33</v>
+      </c>
+      <c r="H46">
+        <v>1500</v>
+      </c>
+      <c r="L46">
+        <v>-1</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>339</v>
+        <v>351</v>
+      </c>
+      <c r="B48" t="s">
+        <v>310</v>
       </c>
       <c r="C48" t="s">
         <v>347</v>
       </c>
+      <c r="D48" t="s">
+        <v>29</v>
+      </c>
+      <c r="E48">
+        <v>8</v>
+      </c>
       <c r="F48" t="s">
-        <v>312</v>
-      </c>
-      <c r="G48">
-        <v>45000</v>
+        <v>33</v>
+      </c>
+      <c r="H48">
+        <v>120000</v>
+      </c>
+      <c r="I48" t="s">
+        <v>339</v>
+      </c>
+      <c r="J48" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>339</v>
+      </c>
+      <c r="C49" t="s">
+        <v>347</v>
+      </c>
+      <c r="F49" t="s">
+        <v>312</v>
+      </c>
+      <c r="G49">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>296</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>311</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C50" t="s">
         <v>348</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F50" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>298</v>
-      </c>
-      <c r="B52" t="s">
-        <v>324</v>
-      </c>
-      <c r="C52" t="s">
-        <v>347</v>
-      </c>
-      <c r="D52" t="s">
-        <v>29</v>
-      </c>
-      <c r="E52">
-        <v>7</v>
-      </c>
-      <c r="F52" t="s">
-        <v>33</v>
-      </c>
-      <c r="H52">
-        <v>120000</v>
-      </c>
-      <c r="I52" t="s">
-        <v>588</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>329</v>
+        <v>298</v>
       </c>
       <c r="B53" t="s">
-        <v>589</v>
+        <v>324</v>
       </c>
       <c r="C53" t="s">
         <v>347</v>
       </c>
+      <c r="D53" t="s">
+        <v>29</v>
+      </c>
+      <c r="E53">
+        <v>7</v>
+      </c>
       <c r="F53" t="s">
-        <v>312</v>
-      </c>
-      <c r="G53">
-        <v>10000</v>
+        <v>33</v>
+      </c>
+      <c r="H53">
+        <v>120000</v>
+      </c>
+      <c r="I53" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>301</v>
+        <v>329</v>
       </c>
       <c r="B54" t="s">
-        <v>325</v>
+        <v>589</v>
       </c>
       <c r="C54" t="s">
         <v>347</v>
       </c>
-      <c r="D54" t="s">
-        <v>28</v>
-      </c>
-      <c r="E54">
-        <v>2</v>
-      </c>
       <c r="F54" t="s">
-        <v>33</v>
-      </c>
-      <c r="H54">
-        <v>120000</v>
-      </c>
-      <c r="I54" t="s">
-        <v>326</v>
+        <v>312</v>
+      </c>
+      <c r="G54">
+        <v>10000</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>326</v>
+        <v>301</v>
+      </c>
+      <c r="B55" t="s">
+        <v>325</v>
       </c>
       <c r="C55" t="s">
         <v>347</v>
       </c>
+      <c r="D55" t="s">
+        <v>28</v>
+      </c>
+      <c r="E55">
+        <v>2</v>
+      </c>
       <c r="F55" t="s">
-        <v>312</v>
-      </c>
-      <c r="G55">
-        <v>20000</v>
+        <v>33</v>
+      </c>
+      <c r="H55">
+        <v>120000</v>
+      </c>
+      <c r="I55" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>299</v>
-      </c>
-      <c r="B56" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C56" t="s">
         <v>347</v>
       </c>
-      <c r="D56" t="s">
-        <v>28</v>
-      </c>
-      <c r="E56">
-        <v>7</v>
-      </c>
       <c r="F56" t="s">
-        <v>33</v>
-      </c>
-      <c r="H56">
-        <v>120000</v>
-      </c>
-      <c r="I56" t="s">
-        <v>327</v>
+        <v>312</v>
+      </c>
+      <c r="G56">
+        <v>20000</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>327</v>
+        <v>299</v>
+      </c>
+      <c r="B57" t="s">
+        <v>324</v>
       </c>
       <c r="C57" t="s">
         <v>347</v>
       </c>
+      <c r="D57" t="s">
+        <v>28</v>
+      </c>
+      <c r="E57">
+        <v>7</v>
+      </c>
       <c r="F57" t="s">
-        <v>312</v>
-      </c>
-      <c r="G57">
-        <v>20000</v>
+        <v>33</v>
+      </c>
+      <c r="H57">
+        <v>120000</v>
+      </c>
+      <c r="I57" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>302</v>
-      </c>
-      <c r="B58" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C58" t="s">
         <v>347</v>
       </c>
-      <c r="D58" t="s">
-        <v>27</v>
-      </c>
-      <c r="E58">
-        <v>7</v>
-      </c>
       <c r="F58" t="s">
-        <v>33</v>
-      </c>
-      <c r="H58">
-        <v>110000</v>
-      </c>
-      <c r="I58" t="s">
-        <v>587</v>
+        <v>312</v>
+      </c>
+      <c r="G58">
+        <v>20000</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>328</v>
+        <v>302</v>
+      </c>
+      <c r="B59" t="s">
+        <v>324</v>
       </c>
       <c r="C59" t="s">
         <v>347</v>
       </c>
+      <c r="D59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E59">
+        <v>7</v>
+      </c>
       <c r="F59" t="s">
+        <v>33</v>
+      </c>
+      <c r="H59">
+        <v>110000</v>
+      </c>
+      <c r="I59" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>328</v>
+      </c>
+      <c r="C60" t="s">
+        <v>347</v>
+      </c>
+      <c r="F60" t="s">
         <v>312</v>
       </c>
-      <c r="G59">
+      <c r="G60">
         <v>20000</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>333</v>
-      </c>
-      <c r="C61" t="s">
-        <v>347</v>
-      </c>
-      <c r="F61" t="s">
-        <v>32</v>
-      </c>
-      <c r="G61">
-        <v>30000</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>289</v>
-      </c>
-      <c r="B62" t="s">
-        <v>320</v>
+        <v>333</v>
       </c>
       <c r="C62" t="s">
         <v>347</v>
       </c>
-      <c r="D62" t="s">
-        <v>29</v>
-      </c>
-      <c r="E62">
-        <v>7</v>
-      </c>
       <c r="F62" t="s">
-        <v>30</v>
-      </c>
-      <c r="J62" t="s">
-        <v>333</v>
+        <v>32</v>
+      </c>
+      <c r="G62">
+        <v>30000</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>334</v>
+        <v>289</v>
+      </c>
+      <c r="B63" t="s">
+        <v>320</v>
       </c>
       <c r="C63" t="s">
         <v>347</v>
       </c>
+      <c r="D63" t="s">
+        <v>29</v>
+      </c>
+      <c r="E63">
+        <v>7</v>
+      </c>
       <c r="F63" t="s">
-        <v>32</v>
-      </c>
-      <c r="G63">
-        <v>30000</v>
+        <v>30</v>
+      </c>
+      <c r="J63" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>290</v>
-      </c>
-      <c r="B64" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
       <c r="C64" t="s">
         <v>347</v>
       </c>
-      <c r="D64" t="s">
+      <c r="F64" t="s">
+        <v>32</v>
+      </c>
+      <c r="G64">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>290</v>
+      </c>
+      <c r="B65" t="s">
+        <v>321</v>
+      </c>
+      <c r="C65" t="s">
+        <v>347</v>
+      </c>
+      <c r="D65" t="s">
         <v>27</v>
       </c>
-      <c r="E64">
+      <c r="E65">
         <v>7</v>
       </c>
-      <c r="F64" t="s">
-        <v>30</v>
-      </c>
-      <c r="J64" t="s">
+      <c r="F65" t="s">
+        <v>30</v>
+      </c>
+      <c r="J65" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>300</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B67" t="s">
         <v>330</v>
-      </c>
-      <c r="C66" t="s">
-        <v>347</v>
-      </c>
-      <c r="D66" t="s">
-        <v>28</v>
-      </c>
-      <c r="E66">
-        <v>6</v>
-      </c>
-      <c r="F66" t="s">
-        <v>33</v>
-      </c>
-      <c r="H66">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>297</v>
-      </c>
-      <c r="B67" t="s">
-        <v>308</v>
       </c>
       <c r="C67" t="s">
         <v>347</v>
@@ -7030,12 +7035,35 @@
         <v>28</v>
       </c>
       <c r="E67">
+        <v>6</v>
+      </c>
+      <c r="F67" t="s">
+        <v>33</v>
+      </c>
+      <c r="H67">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>297</v>
+      </c>
+      <c r="B68" t="s">
+        <v>308</v>
+      </c>
+      <c r="C68" t="s">
+        <v>347</v>
+      </c>
+      <c r="D68" t="s">
+        <v>28</v>
+      </c>
+      <c r="E68">
         <v>5</v>
       </c>
-      <c r="F67" t="s">
-        <v>33</v>
-      </c>
-      <c r="H67">
+      <c r="F68" t="s">
+        <v>33</v>
+      </c>
+      <c r="H68">
         <v>15000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace fixed AoE flags with numbered rotation variants
Rename the four shared-memory spell slots and introduce Scholar instant, AoE and unrestricted variants.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802C9060-45A3-4F60-BC51-F941FFD1D856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BB111E-7C62-4D29-850A-9A05C3421553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="14160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1697" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1705" uniqueCount="601">
   <si>
     <t>Fast Blade</t>
   </si>
@@ -1845,6 +1845,9 @@
   </si>
   <si>
     <t>Storm DoT;Caustic DoT;Do Not Dot</t>
+  </si>
+  <si>
+    <t>Do Not Dot;Dot</t>
   </si>
 </sst>
 </file>
@@ -5714,7 +5717,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF394502-4A59-4E3D-B4CF-5A5D5E1CBE54}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -6045,6 +6048,39 @@
       </c>
       <c r="D25" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>596</v>
+      </c>
+      <c r="D27" t="s">
+        <v>33</v>
+      </c>
+      <c r="H27" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>597</v>
+      </c>
+      <c r="D28" t="s">
+        <v>33</v>
+      </c>
+      <c r="G28" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>598</v>
+      </c>
+      <c r="D29" t="s">
+        <v>312</v>
+      </c>
+      <c r="F29">
+        <v>1200000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Define job-specific rotation variants and movement state
Adapt all rotations to numbered choices and add initial movement-control fields and memory bytes.
</commit_message>
<xml_diff>
--- a/lavender_moogle/moogle_spell_list.xlsx
+++ b/lavender_moogle/moogle_spell_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\lavender_keys\lavender_moogle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BB111E-7C62-4D29-850A-9A05C3421553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E63B2AA9-09B0-46F2-9F2C-2D06049CD9D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="14160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="14160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLD" sheetId="1" r:id="rId1"/>
@@ -3764,9 +3764,6 @@
       <c r="D58" t="s">
         <v>30</v>
       </c>
-      <c r="G58" t="s">
-        <v>488</v>
-      </c>
       <c r="H58" t="s">
         <v>502</v>
       </c>
@@ -3811,6 +3808,9 @@
       </c>
       <c r="D61" t="s">
         <v>30</v>
+      </c>
+      <c r="G61" t="s">
+        <v>488</v>
       </c>
       <c r="H61" t="s">
         <v>495</v>

</xml_diff>